<commit_message>
Publish privacy-safe request status v9
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7a08fc293b844387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R615b51d48add4edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R0097626e82464e5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc14394fc64534c0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R70c475a9e9fb4e36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8d966a285e0b4d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R77e1e5cf808e401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4dc8966a098d4621"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bad63682b8740c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3840d42438b478f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.22-8</x:v>
+        <x:v>2026.07.22-9</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde4b255b8c304a1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ca9d604d2e04907"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17427105aebc468b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2db133f5ba344d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish privacy-safe request status v9 (#7)
Publish the privacy-safe three-sent/seventeen-draft ledger, refresh all FI/EN lender downloads, and enforce deterministic public-boundary checks.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7a08fc293b844387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R615b51d48add4edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R0097626e82464e5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc14394fc64534c0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R70c475a9e9fb4e36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8d966a285e0b4d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R77e1e5cf808e401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4dc8966a098d4621"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bad63682b8740c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3840d42438b478f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.22-8</x:v>
+        <x:v>2026.07.22-9</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde4b255b8c304a1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ca9d604d2e04907"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17427105aebc468b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2db133f5ba344d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish bankability gates and Top 10 matrix v10
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R70c475a9e9fb4e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8d966a285e0b4d37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R77e1e5cf808e401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4dc8966a098d4621"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R2c23e6164a0b4e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rfba8e55d240f4e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3b7a7b88adbd4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R788424a8fc324018"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3840d42438b478f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c28a3399e234f2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.22-9</x:v>
+        <x:v>2026.07.23-10</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ca9d604d2e04907"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35aec4c1c50c42c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2db133f5ba344d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb68607c562584d0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Pixan bankability gates and Top 10 matrix v10
Adds the bilingual public HOLD/gate view, Top 10 market/right matrix, and release-locked v10 lender downloads after full validation.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R70c475a9e9fb4e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8d966a285e0b4d37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R77e1e5cf808e401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4dc8966a098d4621"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R2c23e6164a0b4e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rfba8e55d240f4e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3b7a7b88adbd4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R788424a8fc324018"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3840d42438b478f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c28a3399e234f2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.22-9</x:v>
+        <x:v>2026.07.23-10</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ca9d604d2e04907"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35aec4c1c50c42c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2db133f5ba344d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb68607c562584d0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish paid data procurement shortlist v11
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R2c23e6164a0b4e46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rfba8e55d240f4e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3b7a7b88adbd4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R788424a8fc324018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6e38c9b692d94899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rac4dd6666f8142a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R6e971f01fde54011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4933dcd71bfe41d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c28a3399e234f2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf23d572179044f04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-10</x:v>
+        <x:v>2026.07.23-11</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35aec4c1c50c42c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbb579c6b481496c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb68607c562584d0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32c2b77e8ff34551"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Canada and vendor outreach status
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6e38c9b692d94899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rac4dd6666f8142a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R6e971f01fde54011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4933dcd71bfe41d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R9e9932283cd748ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7341f910fbf24bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R2b8ddff2d40c46ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R05f8b4f2ec034630"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf23d572179044f04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa21daa13fa4154"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-11</x:v>
+        <x:v>2026.07.23-12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbb579c6b481496c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7d61efdbcf64a2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32c2b77e8ff34551"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6e08aac5bb3421b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Canada and vendor outreach status (#10)
Publish the privacy-safe Canada dispatch and commercial outreach states, refresh the bilingual v12 evidence package, and keep all no-response and no-purchase boundaries explicit.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6e38c9b692d94899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rac4dd6666f8142a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R6e971f01fde54011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R4933dcd71bfe41d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R9e9932283cd748ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7341f910fbf24bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R2b8ddff2d40c46ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R05f8b4f2ec034630"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf23d572179044f04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa21daa13fa4154"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-11</x:v>
+        <x:v>2026.07.23-12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbb579c6b481496c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7d61efdbcf64a2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32c2b77e8ff34551"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6e08aac5bb3421b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add vendor response control center
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R9e9932283cd748ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7341f910fbf24bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R2b8ddff2d40c46ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R05f8b4f2ec034630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R0b969f81a992443d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9e5e4d278daa4382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf518ce7961864731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra30d69b207084321"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa21daa13fa4154"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9603e6380ed47a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-12</x:v>
+        <x:v>2026.07.23-13</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7d61efdbcf64a2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5db7b8e1449a4007"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6e08aac5bb3421b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race02e8e1b8443ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add privacy-safe vendor response control center (v13)
Publishes the bilingual vendor-response control, release-locked workbook privacy controls, and refreshed v13 lender package after all required checks passed.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R9e9932283cd748ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7341f910fbf24bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R2b8ddff2d40c46ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R05f8b4f2ec034630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R0b969f81a992443d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9e5e4d278daa4382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf518ce7961864731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra30d69b207084321"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa21daa13fa4154"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9603e6380ed47a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-12</x:v>
+        <x:v>2026.07.23-13</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7d61efdbcf64a2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5db7b8e1449a4007"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6e08aac5bb3421b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race02e8e1b8443ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record administrative vendor response
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R0b969f81a992443d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9e5e4d278daa4382"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf518ce7961864731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra30d69b207084321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7658dd8789dc4bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rd1f57ec70a8f45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rbc3f8fcd4b614584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R881f294505f544f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9603e6380ed47a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95a22d0a48084a86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-13</x:v>
+        <x:v>2026.07.23-14</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5db7b8e1449a4007"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a41facb81b24c89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race02e8e1b8443ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc60141271f4d4ae0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record authority process responses
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7658dd8789dc4bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rd1f57ec70a8f45b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rbc3f8fcd4b614584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R881f294505f544f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R63e77dd9bad6470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rce7b54a016484df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1a9a5dc553c94b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9730d1b5b3a94177"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95a22d0a48084a86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33402335d43d431e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-14</x:v>
+        <x:v>2026.07.23-15</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a41facb81b24c89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b8413f546634b2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc60141271f4d4ae0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a0092d4542844fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add v16 decision cockpit and audit trail
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R63e77dd9bad6470c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rce7b54a016484df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1a9a5dc553c94b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9730d1b5b3a94177"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R1d39198ddcba4f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5e0168769b7c48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rd343844462834d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9c1d13f81a7f46ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33402335d43d431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc80918f9d44b21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-15</x:v>
+        <x:v>2026.07.23-16</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b8413f546634b2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f1c04221b984c34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a0092d4542844fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a9905480a7a466b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add v16 Decision Cockpit and audit trail (#14)
Publish the bilingual decision review, separated Research Operations view, Germany calculation waterfall, deterministic source ledger, and v16 release-locked bank package.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R63e77dd9bad6470c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rce7b54a016484df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1a9a5dc553c94b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9730d1b5b3a94177"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R1d39198ddcba4f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5e0168769b7c48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rd343844462834d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9c1d13f81a7f46ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1862,7 +1862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33402335d43d431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc80918f9d44b21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +1920,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-15</x:v>
+        <x:v>2026.07.23-16</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2167,7 +2167,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b8413f546634b2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f1c04221b984c34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a0092d4542844fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a9905480a7a466b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add v17 donor market sprint
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R1d39198ddcba4f9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5e0168769b7c48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rd343844462834d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9c1d13f81a7f46ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7d985d1cc4da4c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R86a2a7edaf7a4034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1d256bdff4b94488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R0b4bfd41f6974a2b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -266,8 +266,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I50"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -296,7 +296,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -557,7 +557,7 @@
         <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=main</x:v>
       </x:c>
       <x:c r="E2" s="13" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F2" s="13" t="str">
         <x:v>Direct observation from the register.</x:v>
@@ -673,7 +673,7 @@
         <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
         <x:v>Count of EPO family publications; the count does not represent active rights.</x:v>
@@ -789,7 +789,7 @@
         <x:v>https://www.un.org/en/about-us/member-states ; https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
         <x:v>193 UN Member States + Holy See + State of Palestine.</x:v>
@@ -806,312 +806,312 @@
     </x:row>
     <x:row r="11" ht="55.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>Accepted annual official quantitative observations are available from five countries.</x:v>
+        <x:v>Accepted annual official quantitative observations are available from six countries.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The accepted countries are Canada, Germany, Finland, Poland and Sweden.</x:v>
+        <x:v>The accepted countries are Canada, Germany, Finland, New Zealand, Poland and Sweden. The 20 official records include different transaction levels, currencies and product scopes.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Count of unique countries represented among accepted annual official observations.</x:v>
+        <x:v>Count of unique countries represented among annual observations whose evidenceStatus begins official_.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>The metrics are not automatically comparable across countries.</x:v>
+        <x:v>Official publication does not make the metrics automatically comparable across countries.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Comparable annual device and liquid sales series are required from additional countries.</x:v>
+        <x:v>Comparable annual device and liquid consumer-retail series are required from additional countries.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="55.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>There are zero accepted official full-year national consumer-retail-value donor markets.</x:v>
+        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Four candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness)</x:v>
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>Application of the published acceptance criterion to the current evidence register.</x:v>
+        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>Shipment value, tax receipts and physical volume are not treated as consumer retail value.</x:v>
+        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>At least three comparable donor markets are required, with regional and regulatory coverage.</x:v>
+        <x:v>At least three accepted donors are required, with regional and regulatory coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="55.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
+        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
+        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>Sum of the four reported product categories.</x:v>
+        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
-        <x:v>Shipment value is not treated as consumer retail value.</x:v>
+        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
+        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="55.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
+        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
+        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Sum of the reported liquid-containing product categories.</x:v>
+        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>Physical volume is not treated as market value.</x:v>
+        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
+        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="55.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>A conservative text classification identifies NZD 274,180,410.21 as New Zealand 2024 vaping-product-row raw sales.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>NZD 2,137,085.24 is identified as adjacent notifiable products and NZD 4,367,017.37 as unresolved product type. The vaping exact-row-de-duplication sensitivity is NZD 258,327,110.88, but it is not a corrected estimate.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>Conservative Product type text classification of product rows in the official XLSX files; classification and repeated-row sensitivities are reported separately.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Product-type corruption and unresolved rows prevent interpretation as a complete vaping market.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+        <x:v>Obtain the authority's product-code dictionary, repeat-row semantics, complete channel coverage and GST basis. The figure is not donor-eligible.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="55.5" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="55.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the four reported product categories.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Shipment value is not treated as consumer retail value.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="55.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the reported liquid-containing product categories.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>Physical volume is not treated as market value.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
+        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="55.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Poland reported 805,441 litres in 2023.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>A newer series and observed retail value are required.</x:v>
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="55.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>The tax amount is not treated as retail value.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>Finality and reconciliation to the tax base are required.</x:v>
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="55.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
         <x:v>The observation is not treated as the full market.</x:v>
@@ -1120,749 +1120,865 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Observed retail value and device data are required.</x:v>
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="55.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+        <x:v>Observed retail sales and price evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="55.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Poland reported 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+        <x:v>A newer series and observed retail value are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="55.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>The tax amount is not treated as retail value.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
+        <x:v>Finality and reconciliation to the tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="55.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>The public data does not contain an independent IVS valuation.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Direct use of the calculation basis stated by the government.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The observation is not treated as the full market.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+        <x:v>Observed retail value and device data are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="55.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="55.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2025 volume / 2026 prices</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="55.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Validation</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
+        <x:v>site/data/atlas.json (readiness)</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="55.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+        <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>IP status</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="55.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I30" s="14" t="str">
-        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="55.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>Total market value is not automatically the royalty base.</x:v>
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>Application of the valuation boundary stated in the framework.</x:v>
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
+        <x:v>A patent publication is not treated as a product test report.</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I31" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="55.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Validation</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>site/data/evidence.csv</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
+        <x:v>Absence check against the public evidence register.</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I32" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="55.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>IP status</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="55.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Financing principle.</x:v>
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="55.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+        <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
+        <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="55.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="55.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
-        <x:v>2026-12-04</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Check of the official maintenance-fee window.</x:v>
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I37" s="14" t="str">
-        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="55.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Financing principle.</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>No company-level financial conclusion is drawn.</x:v>
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="55.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="55.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Direct observation from the official register.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="55.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>Competition</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
+        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-12-04</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I41" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="55.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>Customers</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+        <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="55.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+        <x:v>No amount, maturity or security package is assumed.</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I43" s="14" t="str">
-        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="55.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+        <x:v>The public package is limited to market and patent material.</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>Count of countries in each evidence grade.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="55.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+      </x:c>
+      <x:c r="B45" s="14" t="str">
+        <x:v>Competition</x:v>
+      </x:c>
+      <x:c r="C45" s="14" t="str">
+        <x:v>Patent and case materials are not a competition map.</x:v>
+      </x:c>
+      <x:c r="D45" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E45" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F45" s="14" t="str">
+        <x:v>Absence check against the public package.</x:v>
+      </x:c>
+      <x:c r="G45" s="14" t="str">
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+      </x:c>
+      <x:c r="H45" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I45" s="14" t="str">
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="55.5" customHeight="1">
+      <x:c r="A46" s="14" t="str">
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>Customers</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+      </x:c>
+      <x:c r="G46" s="14" t="str">
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+      </x:c>
+      <x:c r="H46" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I46" s="14" t="str">
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="55.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="str">
+        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="str">
+        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+      </x:c>
+      <x:c r="G47" s="14" t="str">
+        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+      </x:c>
+      <x:c r="H47" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I47" s="14" t="str">
+        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="55.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>Count of countries in each evidence grade.</x:v>
+      </x:c>
+      <x:c r="G48" s="14" t="str">
+        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+      </x:c>
+      <x:c r="H48" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="str">
+        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="55.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
         <x:v>No global atlas estimate has been approved for publication.</x:v>
       </x:c>
-      <x:c r="B45" s="14" t="str">
+      <x:c r="B49" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C45" s="14" t="str">
-        <x:v>Zero comparable retail-value donor markets is below the minimum threshold of three donor markets.</x:v>
-      </x:c>
-      <x:c r="D45" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness)</x:v>
-      </x:c>
-      <x:c r="E45" s="14" t="str">
-        <x:v>2026-07-22</x:v>
-      </x:c>
-      <x:c r="F45" s="14" t="str">
-        <x:v>Hard gate: at least three compatible donor markets plus regional validation.</x:v>
-      </x:c>
-      <x:c r="G45" s="14" t="str">
-        <x:v>Commercial global estimates are used only as a reasonableness-check range.</x:v>
-      </x:c>
-      <x:c r="H45" s="14" t="str">
+      <x:c r="C49" s="14" t="str">
+        <x:v>Zero accepted donor markets is below the minimum threshold of three. The published New Zealand, EU, Canada and Germany candidate tests each have at least one failed criterion.</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>Hard gate: each donor must pass D1–D10, and at least three compatible donors plus regional validation are required.</x:v>
+      </x:c>
+      <x:c r="G49" s="14" t="str">
+        <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
+      </x:c>
+      <x:c r="H49" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I45" s="14" t="str">
+      <x:c r="I49" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="55.5" customHeight="1">
-      <x:c r="A46" s="15" t="str">
+    <x:row r="50" ht="55.5" customHeight="1">
+      <x:c r="A50" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B46" s="15" t="str">
+      <x:c r="B50" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C46" s="15" t="str">
+      <x:c r="C50" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D46" s="15" t="str">
+      <x:c r="D50" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E46" s="15" t="str">
-        <x:v>2026-07-22</x:v>
-      </x:c>
-      <x:c r="F46" s="15" t="str">
+      <x:c r="E50" s="15" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F50" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G46" s="15" t="str">
+      <x:c r="G50" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H46" s="15" t="str">
+      <x:c r="H50" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I46" s="15" t="str">
+      <x:c r="I50" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H46">
+  <x:conditionalFormatting sqref="H2:H50">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H46">
+    <x:dataValidation type="list" sqref="H2:H50">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc80918f9d44b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebd05d810aae4cd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +2036,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-16</x:v>
+        <x:v>2026.07.24-17</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -1928,7 +2044,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -1944,7 +2060,7 @@
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:v>45</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
@@ -1959,7 +2075,7 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -1967,7 +2083,7 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2167,7 +2283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f1c04221b984c34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569dfe6a03374efd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2474,50 +2590,50 @@
     </x:row>
     <x:row r="18" ht="31.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>EU-TPLF-MAPPING</x:v>
+        <x:v>EU-EC-SWD-2025-560</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>European Commission</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>official_policy_study</x:v>
+        <x:v>official_secondary</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://commission.europa.eu/strategy-and-policy/policies/justice-and-fundamental-rights/civil-justice/civil-and-commercial-law/third-party-litigation-funding-tplf_en</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="31.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>FI-TAX-EXCISE-VVT-010-2025</x:v>
+        <x:v>EU-EC-SWD-2026-111</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>Finnish Tax Administration</x:v>
+        <x:v>European Commission</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>official</x:v>
+        <x:v>official_secondary</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="31.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>FORTUNE-GLOBAL-2025</x:v>
+        <x:v>EU-TPLF-MAPPING</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>Fortune Business Insights</x:v>
+        <x:v>European Commission</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>commercial_estimate</x:v>
+        <x:v>official_policy_study</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://commission.europa.eu/strategy-and-policy/policies/justice-and-fundamental-rights/civil-justice/civil-and-commercial-law/third-party-litigation-funding-tplf_en</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2525,16 +2641,16 @@
     </x:row>
     <x:row r="21" ht="31.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>GVR-GLOBAL-2025</x:v>
+        <x:v>FI-TAX-EXCISE-VVT-010-2025</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>Grand View Research</x:v>
+        <x:v>Finnish Tax Administration</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>commercial_estimate</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2542,16 +2658,16 @@
     </x:row>
     <x:row r="22" ht="31.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>IMARC-GLOBAL-2025</x:v>
+        <x:v>FORTUNE-GLOBAL-2025</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>IMARC Group</x:v>
+        <x:v>Fortune Business Insights</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
         <x:v>commercial_estimate</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market</x:v>
+        <x:v>https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2559,16 +2675,16 @@
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>INTASTE-GERMANFLAVOURS-2026</x:v>
+        <x:v>GVR-GLOBAL-2025</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>inTaste.de</x:v>
+        <x:v>Grand View Research</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>retail_listing</x:v>
+        <x:v>commercial_estimate</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid</x:v>
+        <x:v>https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2576,16 +2692,16 @@
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>INTASTE-REVOLTAGE-2026</x:v>
+        <x:v>IMARC-GLOBAL-2025</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>inTaste.de</x:v>
+        <x:v>IMARC Group</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>retail_listing</x:v>
+        <x:v>commercial_estimate</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2593,7 +2709,7 @@
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>INTASTE-SAMURAI-2026</x:v>
+        <x:v>INTASTE-GERMANFLAVOURS-2026</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>inTaste.de</x:v>
@@ -2602,7 +2718,7 @@
         <x:v>retail_listing</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://www.intaste.de/anstand-liquid-samurai-liquid</x:v>
+        <x:v>https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2610,16 +2726,16 @@
     </x:row>
     <x:row r="26" ht="31.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>IPAU-PATENT-API</x:v>
+        <x:v>INTASTE-REVOLTAGE-2026</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>IP Australia</x:v>
+        <x:v>inTaste.de</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>official_national_api</x:v>
+        <x:v>retail_listing</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2627,16 +2743,16 @@
     </x:row>
     <x:row r="27" ht="31.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>KIPRIS-REGISTER</x:v>
+        <x:v>INTASTE-SAMURAI-2026</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>Korean Intellectual Property Office / KIPRIS</x:v>
+        <x:v>inTaste.de</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>official_national_register</x:v>
+        <x:v>retail_listing</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://www.kipris.or.kr/khome/search/searchResult.do</x:v>
+        <x:v>https://www.intaste.de/anstand-liquid-samurai-liquid</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2644,16 +2760,16 @@
     </x:row>
     <x:row r="28" ht="31.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>PL-SEJM-I07255-O1</x:v>
+        <x:v>IPAU-PATENT-API</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Sejm of the Republic of Poland</x:v>
+        <x:v>IP Australia</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>official</x:v>
+        <x:v>official_national_api</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2661,16 +2777,16 @@
     </x:row>
     <x:row r="29" ht="31.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>PL-SEJM-I17526-O1</x:v>
+        <x:v>KIPRIS-REGISTER</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>Sejm of the Republic of Poland</x:v>
+        <x:v>Korean Intellectual Property Office / KIPRIS</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>official</x:v>
+        <x:v>official_national_register</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://www.kipris.or.kr/khome/search/searchResult.do</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2678,67 +2794,67 @@
     </x:row>
     <x:row r="30" ht="31.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>PRH-FI-REGISTER</x:v>
+        <x:v>NZ-MOH-ANNUAL-RETURNS-2022</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>Finnish Patent and Registration Office</x:v>
+        <x:v>New Zealand Ministry of Health</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>official_national_register</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2022</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="31.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>ROSPATENT-REGISTER</x:v>
+        <x:v>NZ-MOH-ANNUAL-RETURNS-2023</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>Federal Service for Intellectual Property (Rospatent)</x:v>
+        <x:v>New Zealand Ministry of Health</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>official_national_register</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://new.fips.ru/registers-doc-view/fips_servlet?DB=RUPAT&amp;DocNumber=2600093&amp;TypeFile=html</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="31.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>RPAD-KANANEN-2013</x:v>
+        <x:v>NZ-MOH-ANNUAL-RETURNS-2024</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>RPad.tv</x:v>
+        <x:v>New Zealand Ministry of Health</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>secondary_interview</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>https://rpad.tv/2013/09/23/vaping-diaries-108-electric-angel-owner-mika-kananen-interview/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="31.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>RPX-CN-225669</x:v>
+        <x:v>PL-SEJM-I07255-O1</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>RPX Insight</x:v>
+        <x:v>Sejm of the Republic of Poland</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>secondary_litigation_database</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2746,16 +2862,16 @@
     </x:row>
     <x:row r="34" ht="31.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>SE-GOV-BERAKNINGSKONVENTIONER-2026</x:v>
+        <x:v>PL-SEJM-I17526-O1</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Government Offices of Sweden</x:v>
+        <x:v>Sejm of the Republic of Poland</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
         <x:v>official</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2763,16 +2879,16 @@
     </x:row>
     <x:row r="35" ht="31.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>UPCA-ARTICLE-83</x:v>
+        <x:v>PRH-FI-REGISTER</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>European Patent Office / Agreement on a Unified Patent Court</x:v>
+        <x:v>Finnish Patent and Registration Office</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>official_treaty_text</x:v>
+        <x:v>official_national_register</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>https://www.epo.org/en/legal/up-upc/2022/upca_83.html</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2780,16 +2896,16 @@
     </x:row>
     <x:row r="36" ht="31.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>USPTO-ASSIGNMENT</x:v>
+        <x:v>ROSPATENT-REGISTER</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>United States Patent and Trademark Office</x:v>
+        <x:v>Federal Service for Intellectual Property (Rospatent)</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>official_national_assignment_route</x:v>
+        <x:v>official_national_register</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://new.fips.ru/registers-doc-view/fips_servlet?DB=RUPAT&amp;DocNumber=2600093&amp;TypeFile=html</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2797,16 +2913,16 @@
     </x:row>
     <x:row r="37" ht="31.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>USPTO-MAINTENANCE</x:v>
+        <x:v>RPAD-KANANEN-2013</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>United States Patent and Trademark Office</x:v>
+        <x:v>RPad.tv</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>official_national_fee_route</x:v>
+        <x:v>secondary_interview</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923</x:v>
+        <x:v>https://rpad.tv/2013/09/23/vaping-diaries-108-electric-angel-owner-mika-kananen-interview/</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2814,16 +2930,16 @@
     </x:row>
     <x:row r="38" ht="31.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>USPTO-PATENT-CENTER</x:v>
+        <x:v>RPX-CN-225669</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>United States Patent and Trademark Office</x:v>
+        <x:v>RPX Insight</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>official_national_register_route</x:v>
+        <x:v>secondary_litigation_database</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>https://patentcenter.uspto.gov/applications/14911851</x:v>
+        <x:v>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2831,16 +2947,16 @@
     </x:row>
     <x:row r="39" ht="31.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>WAYBACK-EA-ABOUT-2012</x:v>
+        <x:v>SE-GOV-BERAKNINGSKONVENTIONER-2026</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
+        <x:v>Government Offices of Sweden</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>archived_company_statement</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>https://web.archive.org/web/20121206055248/http://www.electricangel.fi:80/page/4/about-us</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2848,16 +2964,16 @@
     </x:row>
     <x:row r="40" ht="31.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>WAYBACK-EA-INVICTUS-2013</x:v>
+        <x:v>UPCA-ARTICLE-83</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
+        <x:v>European Patent Office / Agreement on a Unified Patent Court</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>archived_company_statement</x:v>
+        <x:v>official_treaty_text</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://web.archive.org/web/20131216064916/http://www.electricangel.fi:80/news/3/ea-invictus</x:v>
+        <x:v>https://www.epo.org/en/legal/up-upc/2022/upca_83.html</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2865,16 +2981,16 @@
     </x:row>
     <x:row r="41" ht="31.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>WIPO-ASSIGNMENT-LICENSING</x:v>
+        <x:v>USPTO-ASSIGNMENT</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>United States Patent and Trademark Office</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>official_national_assignment_route</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing</x:v>
+        <x:v>https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2882,16 +2998,16 @@
     </x:row>
     <x:row r="42" ht="31.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>WIPO-DISPUTE-RESOLUTION</x:v>
+        <x:v>USPTO-MAINTENANCE</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>United States Patent and Trademark Office</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>official_national_fee_route</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/settle-ip-disputes</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2899,16 +3015,16 @@
     </x:row>
     <x:row r="43" ht="31.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>WIPO-IP-FINANCE</x:v>
+        <x:v>USPTO-PATENT-CENTER</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>United States Patent and Trademark Office</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>official_national_register_route</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>https://patentcenter.uspto.gov/applications/14911851</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2916,16 +3032,16 @@
     </x:row>
     <x:row r="44" ht="31.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>WIPO-IP-VALUATION</x:v>
+        <x:v>WAYBACK-EA-ABOUT-2012</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>archived_company_statement</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://web.archive.org/web/20121206055248/http://www.electricangel.fi:80/page/4/about-us</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2933,16 +3049,16 @@
     </x:row>
     <x:row r="45" ht="31.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
-        <x:v>WIPO-PCT-NATIONAL-PHASE</x:v>
+        <x:v>WAYBACK-EA-INVICTUS-2013</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
       </x:c>
       <x:c r="C45" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>archived_company_statement</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/pct-system/national-phase</x:v>
+        <x:v>https://web.archive.org/web/20131216064916/http://www.electricangel.fi:80/news/3/ea-invictus</x:v>
       </x:c>
       <x:c r="E45" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2950,42 +3066,127 @@
     </x:row>
     <x:row r="46" ht="31.5" customHeight="1">
       <x:c r="A46" s="14" t="str">
+        <x:v>WIPO-ASSIGNMENT-LICENSING</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="31.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
+        <x:v>WIPO-DISPUTE-RESOLUTION</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/business/settle-ip-disputes</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="31.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>WIPO-IP-FINANCE</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="31.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>WIPO-IP-VALUATION</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="31.5" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>WIPO-PCT-NATIONAL-PHASE</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/pct-system/national-phase</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="31.5" customHeight="1">
+      <x:c r="A51" s="14" t="str">
         <x:v>YTJ-ELECTRIC-ANGEL</x:v>
       </x:c>
-      <x:c r="B46" s="14" t="str">
+      <x:c r="B51" s="14" t="str">
         <x:v>Finnish Patent and Registration Office / Finnish Tax Administration</x:v>
       </x:c>
-      <x:c r="C46" s="14" t="str">
+      <x:c r="C51" s="14" t="str">
         <x:v>official_company_register</x:v>
       </x:c>
-      <x:c r="D46" s="14" t="str">
+      <x:c r="D51" s="14" t="str">
         <x:v>https://avoindata.prh.fi/opendata-ytj-api/v3/companies?businessId=2498114-9</x:v>
       </x:c>
-      <x:c r="E46" s="14" t="str">
-        <x:v>2026-07-22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="31.5" customHeight="1">
-      <x:c r="A47" s="15" t="str">
+      <x:c r="E51" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="31.5" customHeight="1">
+      <x:c r="A52" s="15" t="str">
         <x:v>YTJ-PIXAN</x:v>
       </x:c>
-      <x:c r="B47" s="15" t="str">
+      <x:c r="B52" s="15" t="str">
         <x:v>Finnish Patent and Registration Office / Finnish Tax Administration</x:v>
       </x:c>
-      <x:c r="C47" s="15" t="str">
+      <x:c r="C52" s="15" t="str">
         <x:v>official_company_register</x:v>
       </x:c>
-      <x:c r="D47" s="15" t="str">
+      <x:c r="D52" s="15" t="str">
         <x:v>https://avoindata.prh.fi/opendata-ytj-api/v3/companies?businessId=2632380-1</x:v>
       </x:c>
-      <x:c r="E47" s="15" t="str">
+      <x:c r="E52" s="15" t="str">
         <x:v>2026-07-22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a9905480a7a466b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8787a1611fab4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add v17 donor market sprint (#15)
Co-authored-by: jounirautio78-ops <jounirautio78-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R1d39198ddcba4f9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5e0168769b7c48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rd343844462834d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9c1d13f81a7f46ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7d985d1cc4da4c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R86a2a7edaf7a4034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1d256bdff4b94488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R0b4bfd41f6974a2b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -266,8 +266,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I50"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -296,7 +296,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -557,7 +557,7 @@
         <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=main</x:v>
       </x:c>
       <x:c r="E2" s="13" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F2" s="13" t="str">
         <x:v>Direct observation from the register.</x:v>
@@ -673,7 +673,7 @@
         <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
         <x:v>Count of EPO family publications; the count does not represent active rights.</x:v>
@@ -789,7 +789,7 @@
         <x:v>https://www.un.org/en/about-us/member-states ; https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
         <x:v>193 UN Member States + Holy See + State of Palestine.</x:v>
@@ -806,312 +806,312 @@
     </x:row>
     <x:row r="11" ht="55.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>Accepted annual official quantitative observations are available from five countries.</x:v>
+        <x:v>Accepted annual official quantitative observations are available from six countries.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The accepted countries are Canada, Germany, Finland, Poland and Sweden.</x:v>
+        <x:v>The accepted countries are Canada, Germany, Finland, New Zealand, Poland and Sweden. The 20 official records include different transaction levels, currencies and product scopes.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Count of unique countries represented among accepted annual official observations.</x:v>
+        <x:v>Count of unique countries represented among annual observations whose evidenceStatus begins official_.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>The metrics are not automatically comparable across countries.</x:v>
+        <x:v>Official publication does not make the metrics automatically comparable across countries.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Comparable annual device and liquid sales series are required from additional countries.</x:v>
+        <x:v>Comparable annual device and liquid consumer-retail series are required from additional countries.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="55.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>There are zero accepted official full-year national consumer-retail-value donor markets.</x:v>
+        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Four candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness)</x:v>
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>Application of the published acceptance criterion to the current evidence register.</x:v>
+        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>Shipment value, tax receipts and physical volume are not treated as consumer retail value.</x:v>
+        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>At least three comparable donor markets are required, with regional and regulatory coverage.</x:v>
+        <x:v>At least three accepted donors are required, with regional and regulatory coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="55.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
+        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
+        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>Sum of the four reported product categories.</x:v>
+        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
-        <x:v>Shipment value is not treated as consumer retail value.</x:v>
+        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
+        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="55.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
+        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
+        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Sum of the reported liquid-containing product categories.</x:v>
+        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>Physical volume is not treated as market value.</x:v>
+        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
+        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="55.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>A conservative text classification identifies NZD 274,180,410.21 as New Zealand 2024 vaping-product-row raw sales.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>NZD 2,137,085.24 is identified as adjacent notifiable products and NZD 4,367,017.37 as unresolved product type. The vaping exact-row-de-duplication sensitivity is NZD 258,327,110.88, but it is not a corrected estimate.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>Conservative Product type text classification of product rows in the official XLSX files; classification and repeated-row sensitivities are reported separately.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Product-type corruption and unresolved rows prevent interpretation as a complete vaping market.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+        <x:v>Obtain the authority's product-code dictionary, repeat-row semantics, complete channel coverage and GST basis. The figure is not donor-eligible.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="55.5" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="55.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the four reported product categories.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Shipment value is not treated as consumer retail value.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="55.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the reported liquid-containing product categories.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>Physical volume is not treated as market value.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
+        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="55.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Poland reported 805,441 litres in 2023.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>A newer series and observed retail value are required.</x:v>
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="55.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>The tax amount is not treated as retail value.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>Finality and reconciliation to the tax base are required.</x:v>
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="55.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
         <x:v>The observation is not treated as the full market.</x:v>
@@ -1120,749 +1120,865 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Observed retail value and device data are required.</x:v>
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="55.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+        <x:v>Observed retail sales and price evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="55.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Poland reported 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+        <x:v>A newer series and observed retail value are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="55.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>The tax amount is not treated as retail value.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
+        <x:v>Finality and reconciliation to the tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="55.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>The public data does not contain an independent IVS valuation.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Direct use of the calculation basis stated by the government.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The observation is not treated as the full market.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+        <x:v>Observed retail value and device data are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="55.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="55.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2025 volume / 2026 prices</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="55.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Validation</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
+        <x:v>site/data/atlas.json (readiness)</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="55.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+        <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>IP status</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="55.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I30" s="14" t="str">
-        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="55.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>Total market value is not automatically the royalty base.</x:v>
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>Application of the valuation boundary stated in the framework.</x:v>
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
+        <x:v>A patent publication is not treated as a product test report.</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I31" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="55.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Validation</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>site/data/evidence.csv</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
+        <x:v>Absence check against the public evidence register.</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I32" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="55.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>IP status</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="55.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Financing principle.</x:v>
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="55.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+        <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
+        <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="55.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="55.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
-        <x:v>2026-12-04</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Check of the official maintenance-fee window.</x:v>
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I37" s="14" t="str">
-        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="55.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Financing principle.</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>No company-level financial conclusion is drawn.</x:v>
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="55.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="55.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Direct observation from the official register.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="55.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>Competition</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
+        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-12-04</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I41" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="55.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>Customers</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+        <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="55.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+        <x:v>No amount, maturity or security package is assumed.</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I43" s="14" t="str">
-        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="55.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+        <x:v>The public package is limited to market and patent material.</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>Count of countries in each evidence grade.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="55.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+      </x:c>
+      <x:c r="B45" s="14" t="str">
+        <x:v>Competition</x:v>
+      </x:c>
+      <x:c r="C45" s="14" t="str">
+        <x:v>Patent and case materials are not a competition map.</x:v>
+      </x:c>
+      <x:c r="D45" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E45" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F45" s="14" t="str">
+        <x:v>Absence check against the public package.</x:v>
+      </x:c>
+      <x:c r="G45" s="14" t="str">
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+      </x:c>
+      <x:c r="H45" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I45" s="14" t="str">
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="55.5" customHeight="1">
+      <x:c r="A46" s="14" t="str">
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>Customers</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+      </x:c>
+      <x:c r="G46" s="14" t="str">
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+      </x:c>
+      <x:c r="H46" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I46" s="14" t="str">
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="55.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="str">
+        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="str">
+        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+      </x:c>
+      <x:c r="G47" s="14" t="str">
+        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+      </x:c>
+      <x:c r="H47" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I47" s="14" t="str">
+        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="55.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>Count of countries in each evidence grade.</x:v>
+      </x:c>
+      <x:c r="G48" s="14" t="str">
+        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+      </x:c>
+      <x:c r="H48" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="str">
+        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="55.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
         <x:v>No global atlas estimate has been approved for publication.</x:v>
       </x:c>
-      <x:c r="B45" s="14" t="str">
+      <x:c r="B49" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C45" s="14" t="str">
-        <x:v>Zero comparable retail-value donor markets is below the minimum threshold of three donor markets.</x:v>
-      </x:c>
-      <x:c r="D45" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness)</x:v>
-      </x:c>
-      <x:c r="E45" s="14" t="str">
-        <x:v>2026-07-22</x:v>
-      </x:c>
-      <x:c r="F45" s="14" t="str">
-        <x:v>Hard gate: at least three compatible donor markets plus regional validation.</x:v>
-      </x:c>
-      <x:c r="G45" s="14" t="str">
-        <x:v>Commercial global estimates are used only as a reasonableness-check range.</x:v>
-      </x:c>
-      <x:c r="H45" s="14" t="str">
+      <x:c r="C49" s="14" t="str">
+        <x:v>Zero accepted donor markets is below the minimum threshold of three. The published New Zealand, EU, Canada and Germany candidate tests each have at least one failed criterion.</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>Hard gate: each donor must pass D1–D10, and at least three compatible donors plus regional validation are required.</x:v>
+      </x:c>
+      <x:c r="G49" s="14" t="str">
+        <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
+      </x:c>
+      <x:c r="H49" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I45" s="14" t="str">
+      <x:c r="I49" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="55.5" customHeight="1">
-      <x:c r="A46" s="15" t="str">
+    <x:row r="50" ht="55.5" customHeight="1">
+      <x:c r="A50" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B46" s="15" t="str">
+      <x:c r="B50" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C46" s="15" t="str">
+      <x:c r="C50" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D46" s="15" t="str">
+      <x:c r="D50" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E46" s="15" t="str">
-        <x:v>2026-07-22</x:v>
-      </x:c>
-      <x:c r="F46" s="15" t="str">
+      <x:c r="E50" s="15" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F50" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G46" s="15" t="str">
+      <x:c r="G50" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H46" s="15" t="str">
+      <x:c r="H50" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I46" s="15" t="str">
+      <x:c r="I50" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H46">
+  <x:conditionalFormatting sqref="H2:H50">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H46">
+    <x:dataValidation type="list" sqref="H2:H50">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc80918f9d44b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebd05d810aae4cd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1920,7 +2036,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.23-16</x:v>
+        <x:v>2026.07.24-17</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -1928,7 +2044,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -1944,7 +2060,7 @@
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:v>45</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
@@ -1959,7 +2075,7 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -1967,7 +2083,7 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2167,7 +2283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f1c04221b984c34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569dfe6a03374efd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2474,50 +2590,50 @@
     </x:row>
     <x:row r="18" ht="31.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>EU-TPLF-MAPPING</x:v>
+        <x:v>EU-EC-SWD-2025-560</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>European Commission</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>official_policy_study</x:v>
+        <x:v>official_secondary</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://commission.europa.eu/strategy-and-policy/policies/justice-and-fundamental-rights/civil-justice/civil-and-commercial-law/third-party-litigation-funding-tplf_en</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="31.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>FI-TAX-EXCISE-VVT-010-2025</x:v>
+        <x:v>EU-EC-SWD-2026-111</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>Finnish Tax Administration</x:v>
+        <x:v>European Commission</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>official</x:v>
+        <x:v>official_secondary</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="31.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>FORTUNE-GLOBAL-2025</x:v>
+        <x:v>EU-TPLF-MAPPING</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>Fortune Business Insights</x:v>
+        <x:v>European Commission</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>commercial_estimate</x:v>
+        <x:v>official_policy_study</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://commission.europa.eu/strategy-and-policy/policies/justice-and-fundamental-rights/civil-justice/civil-and-commercial-law/third-party-litigation-funding-tplf_en</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2525,16 +2641,16 @@
     </x:row>
     <x:row r="21" ht="31.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>GVR-GLOBAL-2025</x:v>
+        <x:v>FI-TAX-EXCISE-VVT-010-2025</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>Grand View Research</x:v>
+        <x:v>Finnish Tax Administration</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>commercial_estimate</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2542,16 +2658,16 @@
     </x:row>
     <x:row r="22" ht="31.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>IMARC-GLOBAL-2025</x:v>
+        <x:v>FORTUNE-GLOBAL-2025</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>IMARC Group</x:v>
+        <x:v>Fortune Business Insights</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
         <x:v>commercial_estimate</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market</x:v>
+        <x:v>https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2559,16 +2675,16 @@
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>INTASTE-GERMANFLAVOURS-2026</x:v>
+        <x:v>GVR-GLOBAL-2025</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>inTaste.de</x:v>
+        <x:v>Grand View Research</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>retail_listing</x:v>
+        <x:v>commercial_estimate</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid</x:v>
+        <x:v>https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2576,16 +2692,16 @@
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>INTASTE-REVOLTAGE-2026</x:v>
+        <x:v>IMARC-GLOBAL-2025</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>inTaste.de</x:v>
+        <x:v>IMARC Group</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>retail_listing</x:v>
+        <x:v>commercial_estimate</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2593,7 +2709,7 @@
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>INTASTE-SAMURAI-2026</x:v>
+        <x:v>INTASTE-GERMANFLAVOURS-2026</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>inTaste.de</x:v>
@@ -2602,7 +2718,7 @@
         <x:v>retail_listing</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://www.intaste.de/anstand-liquid-samurai-liquid</x:v>
+        <x:v>https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2610,16 +2726,16 @@
     </x:row>
     <x:row r="26" ht="31.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>IPAU-PATENT-API</x:v>
+        <x:v>INTASTE-REVOLTAGE-2026</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>IP Australia</x:v>
+        <x:v>inTaste.de</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>official_national_api</x:v>
+        <x:v>retail_listing</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2627,16 +2743,16 @@
     </x:row>
     <x:row r="27" ht="31.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>KIPRIS-REGISTER</x:v>
+        <x:v>INTASTE-SAMURAI-2026</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>Korean Intellectual Property Office / KIPRIS</x:v>
+        <x:v>inTaste.de</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>official_national_register</x:v>
+        <x:v>retail_listing</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://www.kipris.or.kr/khome/search/searchResult.do</x:v>
+        <x:v>https://www.intaste.de/anstand-liquid-samurai-liquid</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2644,16 +2760,16 @@
     </x:row>
     <x:row r="28" ht="31.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>PL-SEJM-I07255-O1</x:v>
+        <x:v>IPAU-PATENT-API</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Sejm of the Republic of Poland</x:v>
+        <x:v>IP Australia</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>official</x:v>
+        <x:v>official_national_api</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2661,16 +2777,16 @@
     </x:row>
     <x:row r="29" ht="31.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>PL-SEJM-I17526-O1</x:v>
+        <x:v>KIPRIS-REGISTER</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>Sejm of the Republic of Poland</x:v>
+        <x:v>Korean Intellectual Property Office / KIPRIS</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>official</x:v>
+        <x:v>official_national_register</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://www.kipris.or.kr/khome/search/searchResult.do</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2678,67 +2794,67 @@
     </x:row>
     <x:row r="30" ht="31.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>PRH-FI-REGISTER</x:v>
+        <x:v>NZ-MOH-ANNUAL-RETURNS-2022</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>Finnish Patent and Registration Office</x:v>
+        <x:v>New Zealand Ministry of Health</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>official_national_register</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2022</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="31.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>ROSPATENT-REGISTER</x:v>
+        <x:v>NZ-MOH-ANNUAL-RETURNS-2023</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>Federal Service for Intellectual Property (Rospatent)</x:v>
+        <x:v>New Zealand Ministry of Health</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>official_national_register</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://new.fips.ru/registers-doc-view/fips_servlet?DB=RUPAT&amp;DocNumber=2600093&amp;TypeFile=html</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="31.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>RPAD-KANANEN-2013</x:v>
+        <x:v>NZ-MOH-ANNUAL-RETURNS-2024</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>RPad.tv</x:v>
+        <x:v>New Zealand Ministry of Health</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>secondary_interview</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>https://rpad.tv/2013/09/23/vaping-diaries-108-electric-angel-owner-mika-kananen-interview/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="31.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>RPX-CN-225669</x:v>
+        <x:v>PL-SEJM-I07255-O1</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>RPX Insight</x:v>
+        <x:v>Sejm of the Republic of Poland</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>secondary_litigation_database</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2746,16 +2862,16 @@
     </x:row>
     <x:row r="34" ht="31.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>SE-GOV-BERAKNINGSKONVENTIONER-2026</x:v>
+        <x:v>PL-SEJM-I17526-O1</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Government Offices of Sweden</x:v>
+        <x:v>Sejm of the Republic of Poland</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
         <x:v>official</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2763,16 +2879,16 @@
     </x:row>
     <x:row r="35" ht="31.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>UPCA-ARTICLE-83</x:v>
+        <x:v>PRH-FI-REGISTER</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>European Patent Office / Agreement on a Unified Patent Court</x:v>
+        <x:v>Finnish Patent and Registration Office</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>official_treaty_text</x:v>
+        <x:v>official_national_register</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>https://www.epo.org/en/legal/up-upc/2022/upca_83.html</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2780,16 +2896,16 @@
     </x:row>
     <x:row r="36" ht="31.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>USPTO-ASSIGNMENT</x:v>
+        <x:v>ROSPATENT-REGISTER</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>United States Patent and Trademark Office</x:v>
+        <x:v>Federal Service for Intellectual Property (Rospatent)</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>official_national_assignment_route</x:v>
+        <x:v>official_national_register</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://new.fips.ru/registers-doc-view/fips_servlet?DB=RUPAT&amp;DocNumber=2600093&amp;TypeFile=html</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2797,16 +2913,16 @@
     </x:row>
     <x:row r="37" ht="31.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>USPTO-MAINTENANCE</x:v>
+        <x:v>RPAD-KANANEN-2013</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>United States Patent and Trademark Office</x:v>
+        <x:v>RPad.tv</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>official_national_fee_route</x:v>
+        <x:v>secondary_interview</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923</x:v>
+        <x:v>https://rpad.tv/2013/09/23/vaping-diaries-108-electric-angel-owner-mika-kananen-interview/</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2814,16 +2930,16 @@
     </x:row>
     <x:row r="38" ht="31.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>USPTO-PATENT-CENTER</x:v>
+        <x:v>RPX-CN-225669</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>United States Patent and Trademark Office</x:v>
+        <x:v>RPX Insight</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>official_national_register_route</x:v>
+        <x:v>secondary_litigation_database</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>https://patentcenter.uspto.gov/applications/14911851</x:v>
+        <x:v>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2831,16 +2947,16 @@
     </x:row>
     <x:row r="39" ht="31.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>WAYBACK-EA-ABOUT-2012</x:v>
+        <x:v>SE-GOV-BERAKNINGSKONVENTIONER-2026</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
+        <x:v>Government Offices of Sweden</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>archived_company_statement</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>https://web.archive.org/web/20121206055248/http://www.electricangel.fi:80/page/4/about-us</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2848,16 +2964,16 @@
     </x:row>
     <x:row r="40" ht="31.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>WAYBACK-EA-INVICTUS-2013</x:v>
+        <x:v>UPCA-ARTICLE-83</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
+        <x:v>European Patent Office / Agreement on a Unified Patent Court</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>archived_company_statement</x:v>
+        <x:v>official_treaty_text</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://web.archive.org/web/20131216064916/http://www.electricangel.fi:80/news/3/ea-invictus</x:v>
+        <x:v>https://www.epo.org/en/legal/up-upc/2022/upca_83.html</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2865,16 +2981,16 @@
     </x:row>
     <x:row r="41" ht="31.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>WIPO-ASSIGNMENT-LICENSING</x:v>
+        <x:v>USPTO-ASSIGNMENT</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>United States Patent and Trademark Office</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>official_national_assignment_route</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing</x:v>
+        <x:v>https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2882,16 +2998,16 @@
     </x:row>
     <x:row r="42" ht="31.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>WIPO-DISPUTE-RESOLUTION</x:v>
+        <x:v>USPTO-MAINTENANCE</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>United States Patent and Trademark Office</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>official_national_fee_route</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/settle-ip-disputes</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2899,16 +3015,16 @@
     </x:row>
     <x:row r="43" ht="31.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>WIPO-IP-FINANCE</x:v>
+        <x:v>USPTO-PATENT-CENTER</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>United States Patent and Trademark Office</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>official_national_register_route</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>https://patentcenter.uspto.gov/applications/14911851</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2916,16 +3032,16 @@
     </x:row>
     <x:row r="44" ht="31.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>WIPO-IP-VALUATION</x:v>
+        <x:v>WAYBACK-EA-ABOUT-2012</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>archived_company_statement</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://web.archive.org/web/20121206055248/http://www.electricangel.fi:80/page/4/about-us</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2933,16 +3049,16 @@
     </x:row>
     <x:row r="45" ht="31.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
-        <x:v>WIPO-PCT-NATIONAL-PHASE</x:v>
+        <x:v>WAYBACK-EA-INVICTUS-2013</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
-        <x:v>World Intellectual Property Organization</x:v>
+        <x:v>Electric Angel Oy webpage archived by Internet Archive</x:v>
       </x:c>
       <x:c r="C45" s="14" t="str">
-        <x:v>official_guidance</x:v>
+        <x:v>archived_company_statement</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/pct-system/national-phase</x:v>
+        <x:v>https://web.archive.org/web/20131216064916/http://www.electricangel.fi:80/news/3/ea-invictus</x:v>
       </x:c>
       <x:c r="E45" s="14" t="str">
         <x:v>2026-07-22</x:v>
@@ -2950,42 +3066,127 @@
     </x:row>
     <x:row r="46" ht="31.5" customHeight="1">
       <x:c r="A46" s="14" t="str">
+        <x:v>WIPO-ASSIGNMENT-LICENSING</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="31.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
+        <x:v>WIPO-DISPUTE-RESOLUTION</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/business/settle-ip-disputes</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="31.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>WIPO-IP-FINANCE</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="31.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>WIPO-IP-VALUATION</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="31.5" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>WIPO-PCT-NATIONAL-PHASE</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>World Intellectual Property Organization</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>official_guidance</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/pct-system/national-phase</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="31.5" customHeight="1">
+      <x:c r="A51" s="14" t="str">
         <x:v>YTJ-ELECTRIC-ANGEL</x:v>
       </x:c>
-      <x:c r="B46" s="14" t="str">
+      <x:c r="B51" s="14" t="str">
         <x:v>Finnish Patent and Registration Office / Finnish Tax Administration</x:v>
       </x:c>
-      <x:c r="C46" s="14" t="str">
+      <x:c r="C51" s="14" t="str">
         <x:v>official_company_register</x:v>
       </x:c>
-      <x:c r="D46" s="14" t="str">
+      <x:c r="D51" s="14" t="str">
         <x:v>https://avoindata.prh.fi/opendata-ytj-api/v3/companies?businessId=2498114-9</x:v>
       </x:c>
-      <x:c r="E46" s="14" t="str">
-        <x:v>2026-07-22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="31.5" customHeight="1">
-      <x:c r="A47" s="15" t="str">
+      <x:c r="E51" s="14" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="31.5" customHeight="1">
+      <x:c r="A52" s="15" t="str">
         <x:v>YTJ-PIXAN</x:v>
       </x:c>
-      <x:c r="B47" s="15" t="str">
+      <x:c r="B52" s="15" t="str">
         <x:v>Finnish Patent and Registration Office / Finnish Tax Administration</x:v>
       </x:c>
-      <x:c r="C47" s="15" t="str">
+      <x:c r="C52" s="15" t="str">
         <x:v>official_company_register</x:v>
       </x:c>
-      <x:c r="D47" s="15" t="str">
+      <x:c r="D52" s="15" t="str">
         <x:v>https://avoindata.prh.fi/opendata-ytj-api/v3/companies?businessId=2632380-1</x:v>
       </x:c>
-      <x:c r="E47" s="15" t="str">
+      <x:c r="E52" s="15" t="str">
         <x:v>2026-07-22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a9905480a7a466b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8787a1611fab4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish donor-conversion cockpit v18
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7d985d1cc4da4c16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R86a2a7edaf7a4034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1d256bdff4b94488"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R0b4bfd41f6974a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R74cba888082f4021"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5c44fee1a80f4349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R4261d945d76e4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R17ceb104cfe849c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6263184a042843fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,6 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0.00000000000000"/>
+  </x:numFmts>
   <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
@@ -34,15 +38,15 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF182935"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="22"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos Display"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="9"/>
-      <x:color rgb="FF182935"/>
-      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
@@ -63,7 +67,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,6 +77,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF071A2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE3F6F3"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -135,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -168,48 +177,81 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -266,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I50"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I54"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -296,13 +338,35 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
     <x:tableColumn id="3" name="Source class"/>
     <x:tableColumn id="4" name="URL"/>
     <x:tableColumn id="5" name="Retrieved / data as of"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="14">
+    <x:tableColumn id="1" name="Record type"/>
+    <x:tableColumn id="2" name="Record ID"/>
+    <x:tableColumn id="3" name="Item / component"/>
+    <x:tableColumn id="4" name="Country / geography"/>
+    <x:tableColumn id="5" name="Year"/>
+    <x:tableColumn id="6" name="Period"/>
+    <x:tableColumn id="7" name="Original amount"/>
+    <x:tableColumn id="8" name="Currency"/>
+    <x:tableColumn id="9" name="ECB rate (currency units / EUR)"/>
+    <x:tableColumn id="10" name="EUR equivalent (full precision)"/>
+    <x:tableColumn id="11" name="Rate ID"/>
+    <x:tableColumn id="12" name="ECB source URL"/>
+    <x:tableColumn id="13" name="Status"/>
+    <x:tableColumn id="14" name="Reason / method"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -543,7 +607,7 @@
         <x:v>Gaps / additional evidence needed</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="55.5" customHeight="1">
+    <x:row r="2" ht="58.5" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>Public register data records Pixan Oy as the proprietor.</x:v>
       </x:c>
@@ -572,7 +636,7 @@
         <x:v>The complete chain of title, deeds of assignment and possible encumbrances must be reviewed separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="55.5" customHeight="1">
+    <x:row r="3" ht="58.5" customHeight="1">
       <x:c r="A3" s="14" t="str">
         <x:v>The earliest priority is FI20135829 dated 2013-08-14.</x:v>
       </x:c>
@@ -601,7 +665,7 @@
         <x:v>No material gap for the priority claim.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="55.5" customHeight="1">
+    <x:row r="4" ht="58.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>The central EPO opposition and appeal proceedings concluded with the patent maintained in amended form.</x:v>
       </x:c>
@@ -630,7 +694,7 @@
         <x:v>Current status in each national register is still required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="55.5" customHeight="1">
+    <x:row r="5" ht="58.5" customHeight="1">
       <x:c r="A5" s="14" t="str">
         <x:v>The amended EP3032975B2 contains nine claims.</x:v>
       </x:c>
@@ -659,7 +723,7 @@
         <x:v>Country-specific expert claim construction and product mapping are required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="55.5" customHeight="1">
+    <x:row r="6" ht="58.5" customHeight="1">
       <x:c r="A6" s="14" t="str">
         <x:v>The patent family contains 22 publication-based records.</x:v>
       </x:c>
@@ -688,7 +752,7 @@
         <x:v>Title, fee status, operative claims and legal status must be verified country by country.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="55.5" customHeight="1">
+    <x:row r="7" ht="58.5" customHeight="1">
       <x:c r="A7" s="14" t="str">
         <x:v>The German nullity action was dismissed on 14 January 2026, and an appeal is pending.</x:v>
       </x:c>
@@ -717,7 +781,7 @@
         <x:v>Monitor the progress and outcome of the Federal Court of Justice appeal X ZR 21/26.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="55.5" customHeight="1">
+    <x:row r="8" ht="58.5" customHeight="1">
       <x:c r="A8" s="14" t="str">
         <x:v>The Munich court found that the products examined in the case infringed claims 1 and 6.</x:v>
       </x:c>
@@ -746,7 +810,7 @@
         <x:v>Appeal status, finality, enforcement and any damages actually paid remain to be verified.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="55.5" customHeight="1">
+    <x:row r="9" ht="58.5" customHeight="1">
       <x:c r="A9" s="14" t="str">
         <x:v>The identified Chinese matter is an applicant-side re-examination, not infringement litigation.</x:v>
       </x:c>
@@ -775,7 +839,7 @@
         <x:v>The official CNIPA decision and its reasoning are required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="55.5" customHeight="1">
+    <x:row r="10" ht="58.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
         <x:v>The public atlas contains a fixed research universe of 195 countries.</x:v>
       </x:c>
@@ -804,15 +868,15 @@
         <x:v>There is no gap in the universe definition; evidence coverage is assessed separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="55.5" customHeight="1">
+    <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>Accepted annual official quantitative observations are available from six countries.</x:v>
+        <x:v>The public package contains 27 annual observations sourced from official routes across seven countries.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The accepted countries are Canada, Germany, Finland, New Zealand, Poland and Sweden. The 20 official records include different transaction levels, currencies and product scopes.</x:v>
+        <x:v>The countries are Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. Transaction levels, currencies and product scopes differ.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
@@ -821,19 +885,19 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Count of unique countries represented among annual observations whose evidenceStatus begins official_.</x:v>
+        <x:v>Count of annual observations whose evidenceStatus begins official_.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>Official publication does not make the metrics automatically comparable across countries.</x:v>
+        <x:v>Official publication does not make the metrics automatically comparable.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Comparable annual device and liquid consumer-retail series are required from additional countries.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="55.5" customHeight="1">
+        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
         <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
@@ -841,7 +905,7 @@
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0. Four candidate tests are published against the same ten-criterion protocol.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
@@ -859,10 +923,10 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>At least three accepted donors are required, with regional and regulatory coverage.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="55.5" customHeight="1">
+        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
         <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
@@ -891,7 +955,7 @@
         <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="55.5" customHeight="1">
+    <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
@@ -920,7 +984,7 @@
         <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="55.5" customHeight="1">
+    <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
         <x:v>A conservative text classification identifies NZD 274,180,410.21 as New Zealand 2024 vaping-product-row raw sales.</x:v>
       </x:c>
@@ -949,285 +1013,285 @@
         <x:v>Obtain the authority's product-code dictionary, repeat-row semantics, complete channel coverage and GST basis. The figure is not donor-eligible.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="55.5" customHeight="1">
+    <x:row r="16" ht="93" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
+        <x:v>New Zealand's supported 2024 identified-vaping retail sensitivity is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="F16" s="14" t="str">
-        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F16" s="17" t="str">
+        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
+        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="55.5" customHeight="1">
+        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
+        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
+        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Sum of the four reported product categories.</x:v>
+        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>Shipment value is not treated as consumer retail value.</x:v>
+        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="55.5" customHeight="1">
+        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Sum of the reported liquid-containing product categories.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Physical volume is not treated as market value.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="55.5" customHeight="1">
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="55.5" customHeight="1">
+        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="55.5" customHeight="1">
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the four reported product categories.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Shipment value is not treated as consumer retail value.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="55.5" customHeight="1">
+        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="58.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the reported liquid-containing product categories.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>Physical volume is not treated as market value.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="55.5" customHeight="1">
+        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Poland reported 805,441 litres in 2023.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>A newer series and observed retail value are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="55.5" customHeight="1">
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>The tax amount is not treated as retail value.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Finality and reconciliation to the tax base are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="55.5" customHeight="1">
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
         <x:v>The observation is not treated as the full market.</x:v>
@@ -1236,749 +1300,865 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Observed retail value and device data are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="55.5" customHeight="1">
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="58.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="55.5" customHeight="1">
+        <x:v>Observed retail sales and price evidence are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Poland reported 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="55.5" customHeight="1">
+        <x:v>A newer series and observed retail value are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>The tax amount is not treated as retail value.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
+        <x:v>Finality and reconciliation to the tax base are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="58.5" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="str">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F29" s="14" t="str">
+        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+      </x:c>
+      <x:c r="G29" s="14" t="str">
+        <x:v>The observation is not treated as the full market.</x:v>
+      </x:c>
+      <x:c r="H29" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I29" s="14" t="str">
+        <x:v>Observed retail value and device data are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="58.5" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+      </x:c>
+      <x:c r="G30" s="14" t="str">
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+      </x:c>
+      <x:c r="H30" s="14" t="str">
+        <x:v>Supported</x:v>
+      </x:c>
+      <x:c r="I30" s="14" t="str">
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="58.5" customHeight="1">
+      <x:c r="A31" s="14" t="str">
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>Financial model</x:v>
+      </x:c>
+      <x:c r="C31" s="14" t="str">
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+      </x:c>
+      <x:c r="D31" s="14" t="str">
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+      </x:c>
+      <x:c r="E31" s="14" t="str">
+        <x:v>2025 volume / 2026 prices</x:v>
+      </x:c>
+      <x:c r="F31" s="14" t="str">
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+      </x:c>
+      <x:c r="G31" s="14" t="str">
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+      </x:c>
+      <x:c r="H31" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I31" s="14" t="str">
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="58.5" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+      </x:c>
+      <x:c r="D32" s="14" t="str">
+        <x:v>site/data/atlas.json (readiness)</x:v>
+      </x:c>
+      <x:c r="E32" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F32" s="14" t="str">
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
+      </x:c>
+      <x:c r="G32" s="14" t="str">
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
+      </x:c>
+      <x:c r="H32" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I32" s="14" t="str">
         <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="55.5" customHeight="1">
-      <x:c r="A29" s="14" t="str">
+    <x:row r="33" ht="58.5" customHeight="1">
+      <x:c r="A33" s="14" t="str">
         <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
-      <x:c r="B29" s="14" t="str">
+      <x:c r="B33" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
-      <x:c r="C29" s="14" t="str">
+      <x:c r="C33" s="14" t="str">
         <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
-      <x:c r="D29" s="14" t="str">
+      <x:c r="D33" s="14" t="str">
         <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
-      <x:c r="E29" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F29" s="14" t="str">
+      <x:c r="E33" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F33" s="14" t="str">
         <x:v>Absence check against the public package.</x:v>
       </x:c>
-      <x:c r="G29" s="14" t="str">
+      <x:c r="G33" s="14" t="str">
         <x:v>No assumptions.</x:v>
-      </x:c>
-      <x:c r="H29" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I29" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="55.5" customHeight="1">
-      <x:c r="A30" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
-      </x:c>
-      <x:c r="B30" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
-      </x:c>
-      <x:c r="C30" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
-      </x:c>
-      <x:c r="D30" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
-      </x:c>
-      <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F30" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
-      </x:c>
-      <x:c r="G30" s="14" t="str">
-        <x:v>No assumptions.</x:v>
-      </x:c>
-      <x:c r="H30" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I30" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="55.5" customHeight="1">
-      <x:c r="A31" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
-      </x:c>
-      <x:c r="B31" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
-      </x:c>
-      <x:c r="C31" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
-      </x:c>
-      <x:c r="D31" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
-      </x:c>
-      <x:c r="E31" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F31" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
-      </x:c>
-      <x:c r="G31" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
-      </x:c>
-      <x:c r="H31" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I31" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="55.5" customHeight="1">
-      <x:c r="A32" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
-      </x:c>
-      <x:c r="B32" s="14" t="str">
-        <x:v>Validation</x:v>
-      </x:c>
-      <x:c r="C32" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
-      </x:c>
-      <x:c r="D32" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
-      </x:c>
-      <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F32" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
-      </x:c>
-      <x:c r="G32" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
-      </x:c>
-      <x:c r="H32" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I32" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="55.5" customHeight="1">
-      <x:c r="A33" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
-      </x:c>
-      <x:c r="B33" s="14" t="str">
-        <x:v>IP status</x:v>
-      </x:c>
-      <x:c r="C33" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
-      </x:c>
-      <x:c r="D33" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
-      </x:c>
-      <x:c r="E33" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F33" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
-      </x:c>
-      <x:c r="G33" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="55.5" customHeight="1">
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="58.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="58.5" customHeight="1">
+      <x:c r="A35" s="14" t="str">
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+      </x:c>
+      <x:c r="B35" s="14" t="str">
+        <x:v>Technical differentiation</x:v>
+      </x:c>
+      <x:c r="C35" s="14" t="str">
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+      </x:c>
+      <x:c r="D35" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E35" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F35" s="14" t="str">
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
+      </x:c>
+      <x:c r="G35" s="14" t="str">
+        <x:v>A patent publication is not treated as a product test report.</x:v>
+      </x:c>
+      <x:c r="H35" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I35" s="14" t="str">
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="58.5" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>site/data/evidence.csv</x:v>
+      </x:c>
+      <x:c r="E36" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>Absence check against the public evidence register.</x:v>
+      </x:c>
+      <x:c r="G36" s="14" t="str">
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+      </x:c>
+      <x:c r="H36" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I36" s="14" t="str">
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="58.5" customHeight="1">
+      <x:c r="A37" s="14" t="str">
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+      </x:c>
+      <x:c r="B37" s="14" t="str">
+        <x:v>IP status</x:v>
+      </x:c>
+      <x:c r="C37" s="14" t="str">
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
+      </x:c>
+      <x:c r="D37" s="14" t="str">
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+      </x:c>
+      <x:c r="E37" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F37" s="14" t="str">
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
+      </x:c>
+      <x:c r="G37" s="14" t="str">
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+      </x:c>
+      <x:c r="H37" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I37" s="14" t="str">
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="58.5" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>Technical differentiation</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+      </x:c>
+      <x:c r="G38" s="14" t="str">
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+      </x:c>
+      <x:c r="H38" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I38" s="14" t="str">
         <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="55.5" customHeight="1">
-      <x:c r="A35" s="14" t="str">
+    <x:row r="39" ht="58.5" customHeight="1">
+      <x:c r="A39" s="14" t="str">
         <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
-      <x:c r="B35" s="14" t="str">
+      <x:c r="B39" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
-      <x:c r="C35" s="14" t="str">
+      <x:c r="C39" s="14" t="str">
         <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
-      <x:c r="D35" s="14" t="str">
+      <x:c r="D39" s="14" t="str">
         <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
-      <x:c r="E35" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F35" s="14" t="str">
+      <x:c r="E39" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F39" s="14" t="str">
         <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
-      <x:c r="G35" s="14" t="str">
+      <x:c r="G39" s="14" t="str">
         <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
-      </x:c>
-      <x:c r="H35" s="14" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="I35" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="55.5" customHeight="1">
-      <x:c r="A36" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
-      </x:c>
-      <x:c r="B36" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C36" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
-      </x:c>
-      <x:c r="D36" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
-      </x:c>
-      <x:c r="E36" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F36" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
-      </x:c>
-      <x:c r="G36" s="14" t="str">
-        <x:v>No assumptions.</x:v>
-      </x:c>
-      <x:c r="H36" s="14" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="I36" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="55.5" customHeight="1">
-      <x:c r="A37" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
-      </x:c>
-      <x:c r="B37" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
-      </x:c>
-      <x:c r="C37" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
-      </x:c>
-      <x:c r="D37" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
-      </x:c>
-      <x:c r="E37" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F37" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
-      </x:c>
-      <x:c r="G37" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
-      </x:c>
-      <x:c r="H37" s="14" t="str">
-        <x:v>Assumption</x:v>
-      </x:c>
-      <x:c r="I37" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="55.5" customHeight="1">
-      <x:c r="A38" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
-      </x:c>
-      <x:c r="B38" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C38" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
-      </x:c>
-      <x:c r="D38" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
-      </x:c>
-      <x:c r="E38" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F38" s="14" t="str">
-        <x:v>Financing principle.</x:v>
-      </x:c>
-      <x:c r="G38" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
-      </x:c>
-      <x:c r="H38" s="14" t="str">
-        <x:v>Supported</x:v>
-      </x:c>
-      <x:c r="I38" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="55.5" customHeight="1">
-      <x:c r="A39" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
-      </x:c>
-      <x:c r="B39" s="14" t="str">
-        <x:v>Risks</x:v>
-      </x:c>
-      <x:c r="C39" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
-      </x:c>
-      <x:c r="D39" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
-      </x:c>
-      <x:c r="E39" s="14" t="str">
-        <x:v>2026-08-14</x:v>
-      </x:c>
-      <x:c r="F39" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
-      </x:c>
-      <x:c r="G39" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="55.5" customHeight="1">
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="58.5" customHeight="1">
+      <x:c r="A41" s="14" t="str">
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+      </x:c>
+      <x:c r="B41" s="14" t="str">
+        <x:v>Commercialisation model</x:v>
+      </x:c>
+      <x:c r="C41" s="14" t="str">
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+      </x:c>
+      <x:c r="D41" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+      </x:c>
+      <x:c r="E41" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F41" s="14" t="str">
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+      </x:c>
+      <x:c r="G41" s="14" t="str">
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+      </x:c>
+      <x:c r="H41" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I41" s="14" t="str">
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="58.5" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+      </x:c>
+      <x:c r="D42" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+      </x:c>
+      <x:c r="E42" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>Financing principle.</x:v>
+      </x:c>
+      <x:c r="G42" s="14" t="str">
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+      </x:c>
+      <x:c r="H42" s="14" t="str">
+        <x:v>Supported</x:v>
+      </x:c>
+      <x:c r="I42" s="14" t="str">
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="58.5" customHeight="1">
+      <x:c r="A43" s="14" t="str">
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+      </x:c>
+      <x:c r="B43" s="14" t="str">
+        <x:v>Risks</x:v>
+      </x:c>
+      <x:c r="C43" s="14" t="str">
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+      </x:c>
+      <x:c r="D43" s="14" t="str">
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+      </x:c>
+      <x:c r="E43" s="14" t="str">
+        <x:v>2026-08-14</x:v>
+      </x:c>
+      <x:c r="F43" s="14" t="str">
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
+      </x:c>
+      <x:c r="G43" s="14" t="str">
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+      </x:c>
+      <x:c r="H43" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I43" s="14" t="str">
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="58.5" customHeight="1">
+      <x:c r="A44" s="14" t="str">
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+      </x:c>
+      <x:c r="B44" s="14" t="str">
+        <x:v>Risks</x:v>
+      </x:c>
+      <x:c r="C44" s="14" t="str">
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+      </x:c>
+      <x:c r="D44" s="14" t="str">
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+      </x:c>
+      <x:c r="E44" s="14" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="F44" s="14" t="str">
+        <x:v>Direct observation from the official register.</x:v>
+      </x:c>
+      <x:c r="G44" s="14" t="str">
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+      </x:c>
+      <x:c r="H44" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I44" s="14" t="str">
         <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="55.5" customHeight="1">
-      <x:c r="A41" s="14" t="str">
+    <x:row r="45" ht="58.5" customHeight="1">
+      <x:c r="A45" s="14" t="str">
         <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
-      <x:c r="B41" s="14" t="str">
+      <x:c r="B45" s="14" t="str">
         <x:v>Risks</x:v>
       </x:c>
-      <x:c r="C41" s="14" t="str">
+      <x:c r="C45" s="14" t="str">
         <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
-      <x:c r="D41" s="14" t="str">
+      <x:c r="D45" s="14" t="str">
         <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
-      <x:c r="E41" s="14" t="str">
+      <x:c r="E45" s="14" t="str">
         <x:v>2026-12-04</x:v>
       </x:c>
-      <x:c r="F41" s="14" t="str">
+      <x:c r="F45" s="14" t="str">
         <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
-      <x:c r="G41" s="14" t="str">
+      <x:c r="G45" s="14" t="str">
         <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
-      <x:c r="H41" s="14" t="str">
+      <x:c r="H45" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I41" s="14" t="str">
+      <x:c r="I45" s="14" t="str">
         <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="55.5" customHeight="1">
-      <x:c r="A42" s="14" t="str">
+    <x:row r="46" ht="58.5" customHeight="1">
+      <x:c r="A46" s="14" t="str">
         <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
-      <x:c r="B42" s="14" t="str">
+      <x:c r="B46" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
-      <x:c r="C42" s="14" t="str">
+      <x:c r="C46" s="14" t="str">
         <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
-      <x:c r="D42" s="14" t="str">
+      <x:c r="D46" s="14" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E42" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F42" s="14" t="str">
+      <x:c r="E46" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
         <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
-      <x:c r="G42" s="14" t="str">
+      <x:c r="G46" s="14" t="str">
         <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
-      <x:c r="H42" s="14" t="str">
+      <x:c r="H46" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="I42" s="14" t="str">
+      <x:c r="I46" s="14" t="str">
         <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="55.5" customHeight="1">
-      <x:c r="A43" s="14" t="str">
+    <x:row r="47" ht="58.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
         <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
-      </x:c>
-      <x:c r="B43" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C43" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
-      </x:c>
-      <x:c r="D43" s="14" t="str">
-        <x:v>Public package scope</x:v>
-      </x:c>
-      <x:c r="E43" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F43" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
-      </x:c>
-      <x:c r="G43" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
-      </x:c>
-      <x:c r="H43" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I43" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="55.5" customHeight="1">
-      <x:c r="A44" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
-      </x:c>
-      <x:c r="B44" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C44" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
-      </x:c>
-      <x:c r="D44" s="14" t="str">
-        <x:v>Public package scope</x:v>
-      </x:c>
-      <x:c r="E44" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F44" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
-      </x:c>
-      <x:c r="G44" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
-      </x:c>
-      <x:c r="H44" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I44" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="55.5" customHeight="1">
-      <x:c r="A45" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
-      </x:c>
-      <x:c r="B45" s="14" t="str">
-        <x:v>Competition</x:v>
-      </x:c>
-      <x:c r="C45" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
-      </x:c>
-      <x:c r="D45" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
-      </x:c>
-      <x:c r="E45" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F45" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
-      </x:c>
-      <x:c r="G45" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
-      </x:c>
-      <x:c r="H45" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I45" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="55.5" customHeight="1">
-      <x:c r="A46" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
-      </x:c>
-      <x:c r="B46" s="14" t="str">
-        <x:v>Customers</x:v>
-      </x:c>
-      <x:c r="C46" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
-      </x:c>
-      <x:c r="D46" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
-      </x:c>
-      <x:c r="E46" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F46" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
-      </x:c>
-      <x:c r="G46" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
-      </x:c>
-      <x:c r="H46" s="14" t="str">
-        <x:v>Assumption</x:v>
-      </x:c>
-      <x:c r="I46" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="55.5" customHeight="1">
-      <x:c r="A47" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G47" s="14" t="str">
+        <x:v>No amount, maturity or security package is assumed.</x:v>
+      </x:c>
+      <x:c r="H47" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I47" s="14" t="str">
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="58.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>The public package is limited to market and patent material.</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G48" s="14" t="str">
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+      </x:c>
+      <x:c r="H48" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="str">
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="58.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="str">
+        <x:v>Competition</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="str">
+        <x:v>Patent and case materials are not a competition map.</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>Absence check against the public package.</x:v>
+      </x:c>
+      <x:c r="G49" s="14" t="str">
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+      </x:c>
+      <x:c r="H49" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I49" s="14" t="str">
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="58.5" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>Customers</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+      </x:c>
+      <x:c r="G50" s="14" t="str">
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+      </x:c>
+      <x:c r="H50" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I50" s="14" t="str">
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="58.5" customHeight="1">
+      <x:c r="A51" s="14" t="str">
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+      </x:c>
+      <x:c r="B51" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C51" s="14" t="str">
         <x:v>The decisions are limited to a country, products, parties and period.</x:v>
       </x:c>
-      <x:c r="D47" s="14" t="str">
+      <x:c r="D51" s="14" t="str">
         <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
-      <x:c r="E47" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F47" s="14" t="str">
+      <x:c r="E51" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F51" s="14" t="str">
         <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
       </x:c>
-      <x:c r="G47" s="14" t="str">
+      <x:c r="G51" s="14" t="str">
         <x:v>Other countries depend on local rights and the products examined there.</x:v>
       </x:c>
-      <x:c r="H47" s="14" t="str">
+      <x:c r="H51" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I47" s="14" t="str">
+      <x:c r="I51" s="14" t="str">
         <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="55.5" customHeight="1">
-      <x:c r="A48" s="14" t="str">
+    <x:row r="52" ht="58.5" customHeight="1">
+      <x:c r="A52" s="14" t="str">
         <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
       </x:c>
-      <x:c r="B48" s="14" t="str">
+      <x:c r="B52" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C48" s="14" t="str">
+      <x:c r="C52" s="14" t="str">
         <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
       </x:c>
-      <x:c r="D48" s="14" t="str">
+      <x:c r="D52" s="14" t="str">
         <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
       </x:c>
-      <x:c r="E48" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F48" s="14" t="str">
+      <x:c r="E52" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F52" s="14" t="str">
         <x:v>Count of countries in each evidence grade.</x:v>
       </x:c>
-      <x:c r="G48" s="14" t="str">
+      <x:c r="G52" s="14" t="str">
         <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
       </x:c>
-      <x:c r="H48" s="14" t="str">
+      <x:c r="H52" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I48" s="14" t="str">
+      <x:c r="I52" s="14" t="str">
         <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="55.5" customHeight="1">
-      <x:c r="A49" s="14" t="str">
+    <x:row r="53" ht="58.5" customHeight="1">
+      <x:c r="A53" s="14" t="str">
         <x:v>No global atlas estimate has been approved for publication.</x:v>
       </x:c>
-      <x:c r="B49" s="14" t="str">
+      <x:c r="B53" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C49" s="14" t="str">
-        <x:v>Zero accepted donor markets is below the minimum threshold of three. The published New Zealand, EU, Canada and Germany candidate tests each have at least one failed criterion.</x:v>
-      </x:c>
-      <x:c r="D49" s="14" t="str">
+      <x:c r="C53" s="14" t="str">
+        <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
+      </x:c>
+      <x:c r="D53" s="14" t="str">
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
-      <x:c r="E49" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F49" s="14" t="str">
-        <x:v>Hard gate: each donor must pass D1–D10, and at least three compatible donors plus regional validation are required.</x:v>
-      </x:c>
-      <x:c r="G49" s="14" t="str">
+      <x:c r="E53" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F53" s="14" t="str">
+        <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
+      </x:c>
+      <x:c r="G53" s="14" t="str">
         <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
       </x:c>
-      <x:c r="H49" s="14" t="str">
+      <x:c r="H53" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I49" s="14" t="str">
+      <x:c r="I53" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="55.5" customHeight="1">
-      <x:c r="A50" s="15" t="str">
+    <x:row r="54" ht="58.5" customHeight="1">
+      <x:c r="A54" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B50" s="15" t="str">
+      <x:c r="B54" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C50" s="15" t="str">
+      <x:c r="C54" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D50" s="15" t="str">
+      <x:c r="D54" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E50" s="15" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F50" s="15" t="str">
+      <x:c r="E54" s="15" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F54" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G50" s="15" t="str">
+      <x:c r="G54" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H50" s="15" t="str">
+      <x:c r="H54" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I50" s="15" t="str">
+      <x:c r="I54" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H50">
+  <x:conditionalFormatting sqref="H2:H54">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H50">
+    <x:dataValidation type="list" sqref="H2:H54">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebd05d810aae4cd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7aa4f32e5298488c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1998,49 +2178,49 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="17" t="str">
+      <x:c r="A1" s="20" t="str">
         <x:v>Pixan · public evidence package summary</x:v>
       </x:c>
-      <x:c r="B1" s="17"/>
-      <x:c r="C1" s="17"/>
-      <x:c r="D1" s="17"/>
-      <x:c r="E1" s="17"/>
-      <x:c r="F1" s="17"/>
-      <x:c r="G1" s="17"/>
-      <x:c r="H1" s="17"/>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
-      <x:c r="A2" s="17"/>
-      <x:c r="B2" s="17"/>
-      <x:c r="C2" s="17"/>
-      <x:c r="D2" s="17"/>
-      <x:c r="E2" s="17"/>
-      <x:c r="F2" s="17"/>
-      <x:c r="G2" s="17"/>
-      <x:c r="H2" s="17"/>
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+      <x:c r="H2" s="20"/>
     </x:row>
     <x:row r="3" ht="28.5" customHeight="1">
-      <x:c r="A3" s="22" t="str">
+      <x:c r="A3" s="25" t="str">
         <x:v>Independent public evidence summary. Not Pixan Oy's official position; not an audit, valuation, legal opinion, investment recommendation or lending recommendation.</x:v>
       </x:c>
-      <x:c r="B3" s="22"/>
-      <x:c r="C3" s="22"/>
-      <x:c r="D3" s="22"/>
-      <x:c r="E3" s="22"/>
-      <x:c r="F3" s="22"/>
-      <x:c r="G3" s="22"/>
-      <x:c r="H3" s="22"/>
+      <x:c r="B3" s="25"/>
+      <x:c r="C3" s="25"/>
+      <x:c r="D3" s="25"/>
+      <x:c r="E3" s="25"/>
+      <x:c r="F3" s="25"/>
+      <x:c r="G3" s="25"/>
+      <x:c r="H3" s="25"/>
     </x:row>
     <x:row r="5" ht="20.25" customHeight="1">
-      <x:c r="A5" s="25" t="str">
+      <x:c r="A5" s="29" t="str">
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-17</x:v>
+        <x:v>2026.07.24-18</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
-      <x:c r="A6" s="25" t="str">
+      <x:c r="A6" s="29" t="str">
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
@@ -2048,7 +2228,7 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
-      <x:c r="A7" s="25" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
@@ -2056,59 +2236,64 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="20.25" customHeight="1">
-      <x:c r="A8" s="25" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:v>49</x:v>
+        <x:f>COUNTA('Evidence Register'!$A$2:$A$54)</x:f>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
     <x:row r="10" ht="20.25" customHeight="1">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="A10" s="31" t="str">
         <x:v>Evidence distribution</x:v>
       </x:c>
-      <x:c r="B10" s="27"/>
+      <x:c r="B10" s="31"/>
     </x:row>
     <x:row r="11" ht="20.25" customHeight="1">
-      <x:c r="A11" s="32" t="str">
+      <x:c r="A11" s="36" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:v>28</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
-      <x:c r="A12" s="33" t="str">
+      <x:c r="A12" s="37" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:v>8</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
-      <x:c r="A13" s="34" t="str">
+      <x:c r="A13" s="38" t="str">
         <x:v>Assumption</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A13)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="20.25" customHeight="1">
-      <x:c r="A14" s="35" t="str">
+      <x:c r="A14" s="39" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="20.25" customHeight="1"/>
     <x:row r="16" ht="20.25" customHeight="1"/>
     <x:row r="17" ht="20.25" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>Three strongest financing grounds</x:v>
       </x:c>
-      <x:c r="B17" s="27"/>
+      <x:c r="B17" s="31"/>
     </x:row>
     <x:row r="18" ht="28.5" customHeight="1">
       <x:c r="A18" s="13" t="n">
@@ -2137,10 +2322,10 @@
     <x:row r="21" ht="20.25" customHeight="1"/>
     <x:row r="22" ht="20.25" customHeight="1"/>
     <x:row r="23" ht="20.25" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="31" t="str">
         <x:v>Four corrections required for lender readiness</x:v>
       </x:c>
-      <x:c r="B23" s="27"/>
+      <x:c r="B23" s="31"/>
     </x:row>
     <x:row r="24" ht="27" customHeight="1">
       <x:c r="A24" s="13" t="n">
@@ -2190,14 +2375,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="47.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="44.439998626708984" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="25.559999465942383" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="31.5" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="40" t="str">
         <x:v>Priority</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
@@ -2211,7 +2396,7 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="40.5" customHeight="1">
-      <x:c r="A2" s="13" t="n">
+      <x:c r="A2" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
@@ -2225,7 +2410,7 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="40.5" customHeight="1">
-      <x:c r="A3" s="14" t="n">
+      <x:c r="A3" s="42" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
@@ -2239,7 +2424,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="40.5" customHeight="1">
-      <x:c r="A4" s="14" t="n">
+      <x:c r="A4" s="42" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
@@ -2253,7 +2438,7 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="40.5" customHeight="1">
-      <x:c r="A5" s="14" t="n">
+      <x:c r="A5" s="42" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
@@ -2267,7 +2452,7 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="40.5" customHeight="1">
-      <x:c r="A6" s="15" t="n">
+      <x:c r="A6" s="43" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
@@ -2283,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569dfe6a03374efd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a790b47859497e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3167,26 +3352,2097 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="31.5" customHeight="1">
-      <x:c r="A52" s="15" t="str">
+      <x:c r="A52" s="14" t="str">
         <x:v>YTJ-PIXAN</x:v>
       </x:c>
-      <x:c r="B52" s="15" t="str">
+      <x:c r="B52" s="14" t="str">
         <x:v>Finnish Patent and Registration Office / Finnish Tax Administration</x:v>
       </x:c>
-      <x:c r="C52" s="15" t="str">
+      <x:c r="C52" s="14" t="str">
         <x:v>official_company_register</x:v>
       </x:c>
-      <x:c r="D52" s="15" t="str">
+      <x:c r="D52" s="14" t="str">
         <x:v>https://avoindata.prh.fi/opendata-ytj-api/v3/companies?businessId=2632380-1</x:v>
       </x:c>
-      <x:c r="E52" s="15" t="str">
+      <x:c r="E52" s="14" t="str">
         <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="31.5" customHeight="1">
+      <x:c r="A53" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
+      </x:c>
+      <x:c r="B53" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C53" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D53" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E53" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="31.5" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="31.5" customHeight="1">
+      <x:c r="A55" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
+      </x:c>
+      <x:c r="B55" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C55" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D55" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E55" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="31.5" customHeight="1">
+      <x:c r="A56" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
+      </x:c>
+      <x:c r="B56" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C56" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D56" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E56" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="31.5" customHeight="1">
+      <x:c r="A57" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="31.5" customHeight="1">
+      <x:c r="A58" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="31.5" customHeight="1">
+      <x:c r="A59" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="31.5" customHeight="1">
+      <x:c r="A60" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+      </x:c>
+      <x:c r="B60" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C60" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D60" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E60" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="31.5" customHeight="1">
+      <x:c r="A61" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+      </x:c>
+      <x:c r="B61" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C61" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D61" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E61" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="31.5" customHeight="1">
+      <x:c r="A62" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+      </x:c>
+      <x:c r="B62" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C62" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D62" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E62" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="31.5" customHeight="1">
+      <x:c r="A63" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+      </x:c>
+      <x:c r="B63" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C63" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D63" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E63" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="31.5" customHeight="1">
+      <x:c r="A64" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+      </x:c>
+      <x:c r="B64" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C64" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D64" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E64" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="31.5" customHeight="1">
+      <x:c r="A65" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+      </x:c>
+      <x:c r="B65" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C65" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D65" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E65" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="31.5" customHeight="1">
+      <x:c r="A66" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+      </x:c>
+      <x:c r="B66" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C66" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D66" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E66" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="31.5" customHeight="1">
+      <x:c r="A67" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+      </x:c>
+      <x:c r="B67" s="14" t="str">
+        <x:v>data.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C67" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D67" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="E67" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="31.5" customHeight="1">
+      <x:c r="A68" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+      </x:c>
+      <x:c r="B68" s="14" t="str">
+        <x:v>ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C68" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D68" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="E68" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="31.5" customHeight="1">
+      <x:c r="A69" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+      </x:c>
+      <x:c r="B69" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C69" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D69" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+      </x:c>
+      <x:c r="E69" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="31.5" customHeight="1">
+      <x:c r="A70" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+      </x:c>
+      <x:c r="B70" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C70" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D70" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+      </x:c>
+      <x:c r="E70" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="31.5" customHeight="1">
+      <x:c r="A71" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B71" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C71" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D71" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E71" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="31.5" customHeight="1">
+      <x:c r="A72" s="15" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B72" s="15" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C72" s="15" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D72" s="15" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E72" s="15" t="str">
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8787a1611fab4583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dcf706411294d0a"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="32.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="68.88999938964844" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="36.66999816894531" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="37.5" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>Record type</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>Record ID</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Item / component</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Country / geography</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Period</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>Original amount</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>ECB rate (currency units / EUR)</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>EUR equivalent (full precision)</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>Rate ID</x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>ECB source URL</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="N1" s="5" t="str">
+        <x:v>Reason / method</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25.5" customHeight="1">
+      <x:c r="A2" s="13" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="str">
+        <x:v>CA-2024-MANUFACTURER-IMPORTER-SHIPMENTS-VALUE</x:v>
+      </x:c>
+      <x:c r="C2" s="13" t="str">
+        <x:v>manufacturer_importer_shipments_value</x:v>
+      </x:c>
+      <x:c r="D2" s="13" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E2" s="13" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F2" s="13" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G2" s="44" t="n">
+        <x:v>1160753796.78</x:v>
+      </x:c>
+      <x:c r="H2" s="44" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I2" s="44" t="n">
+        <x:v>1.482110546875</x:v>
+      </x:c>
+      <x:c r="J2" s="44" t="n">
+        <x:f>G2/I2</x:f>
+        <x:v>783176261.1955132</x:v>
+      </x:c>
+      <x:c r="K2" s="13" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L2" s="13" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M2" s="13" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N2" s="13" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="25.5" customHeight="1">
+      <x:c r="A3" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>NZ-2022-NOTIFIABLE-PRODUCT-REPORTED-REVENUE</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+      </x:c>
+      <x:c r="D3" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E3" s="14" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="F3" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G3" s="45" t="n">
+        <x:v>404000000</x:v>
+      </x:c>
+      <x:c r="H3" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I3" s="45" t="n">
+        <x:v>1.6582474708171</x:v>
+      </x:c>
+      <x:c r="J3" s="45" t="n">
+        <x:f>G3/I3</x:f>
+        <x:v>243630704.7710613</x:v>
+      </x:c>
+      <x:c r="K3" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2022</x:v>
+      </x:c>
+      <x:c r="L3" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M3" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N3" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="25.5" customHeight="1">
+      <x:c r="A4" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>NZ-2023-NOTIFIABLE-PRODUCT-REPORTED-REVENUE-LOWER-BOUND</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+      </x:c>
+      <x:c r="D4" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G4" s="45" t="n">
+        <x:v>374000000</x:v>
+      </x:c>
+      <x:c r="H4" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I4" s="45" t="n">
+        <x:v>1.762151372549</x:v>
+      </x:c>
+      <x:c r="J4" s="45" t="n">
+        <x:f>G4/I4</x:f>
+        <x:v>212240563.33991262</x:v>
+      </x:c>
+      <x:c r="K4" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2023</x:v>
+      </x:c>
+      <x:c r="L4" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M4" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N4" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="25.5" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>NZ-2024-SPECIALIST-RETAIL-SALES-LOWER-BOUND</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>official_specialist_retail_sales_lower_bound</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="n">
+        <x:v>280000000</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="n">
+        <x:f>G5/I5</x:f>
+        <x:v>156595276.14445302</x:v>
+      </x:c>
+      <x:c r="K5" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L5" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M5" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N5" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="25.5" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>NZ-2024-SPECIALIST-RETAIL-PRODUCT-SALES-RAW-FILE-SUM</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>derived_official_workbook_sales_raw_sum</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="n">
+        <x:v>280684512.81</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J6" s="45" t="n">
+        <x:f>G6/I6</x:f>
+        <x:v>156978102.83197576</x:v>
+      </x:c>
+      <x:c r="K6" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L6" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M6" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N6" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="25.5" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>NZ-2024-IDENTIFIED-VAPING-PRODUCT-SALES-RAW-SUM</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>derived_identified_vaping_product_sales_raw_sum</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="n">
+        <x:f>G7/I7</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K7" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L7" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M7" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N7" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="25.5" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>EU-2023-EC-E-CIGARETTE-MARKET-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>institutional_market_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>European Union</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="n">
+        <x:v>4990000000</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J8" s="45" t="n">
+        <x:f>G8</x:f>
+        <x:v>4990000000</x:v>
+      </x:c>
+      <x:c r="K8" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L8" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M8" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N8" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="25.5" customHeight="1">
+      <x:c r="A9" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>DE-2023-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>substitutes_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="n">
+        <x:v>201000000</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="n">
+        <x:f>G9</x:f>
+        <x:v>201000000</x:v>
+      </x:c>
+      <x:c r="K9" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L9" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M9" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N9" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="25.5" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>DE-2024-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>substitutes_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F10" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="n">
+        <x:v>266000000</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J10" s="45" t="n">
+        <x:f>G10</x:f>
+        <x:v>266000000</x:v>
+      </x:c>
+      <x:c r="K10" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L10" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M10" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N10" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="25.5" customHeight="1">
+      <x:c r="A11" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>DE-2025-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>substitutes_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F11" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="n">
+        <x:v>404000000</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="n">
+        <x:f>G11</x:f>
+        <x:v>404000000</x:v>
+      </x:c>
+      <x:c r="K11" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L11" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M11" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N11" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="25.5" customHeight="1">
+      <x:c r="A12" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C12" s="14" t="str">
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>Finland</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="n">
+        <x:v>3540319</x:v>
+      </x:c>
+      <x:c r="H12" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I12" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="45" t="n">
+        <x:f>G12</x:f>
+        <x:v>3540319</x:v>
+      </x:c>
+      <x:c r="K12" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L12" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M12" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N12" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="25.5" customHeight="1">
+      <x:c r="A13" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>e_liquid_excise_amount</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="n">
+        <x:v>993100000</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I13" s="45" t="n">
+        <x:v>4.2396576470588</x:v>
+      </x:c>
+      <x:c r="J13" s="45" t="n">
+        <x:f>G13/I13</x:f>
+        <x:v>234240611.54771507</x:v>
+      </x:c>
+      <x:c r="K13" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L13" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M13" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N13" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="25.5" customHeight="1">
+      <x:c r="A14" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>vaping_device_excise_amount</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F14" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="n">
+        <x:v>175300000</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I14" s="45" t="n">
+        <x:v>4.2396576470588</x:v>
+      </x:c>
+      <x:c r="J14" s="45" t="n">
+        <x:f>G14/I14</x:f>
+        <x:v>41347678.183782555</x:v>
+      </x:c>
+      <x:c r="K14" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L14" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M14" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N14" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="25.5" customHeight="1">
+      <x:c r="A15" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>vaping_component_sets_excise_amount</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="n">
+        <x:v>2500000</x:v>
+      </x:c>
+      <x:c r="H15" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I15" s="45" t="n">
+        <x:v>4.2396576470588</x:v>
+      </x:c>
+      <x:c r="J15" s="45" t="n">
+        <x:f>G15/I15</x:f>
+        <x:v>589670.2536192606</x:v>
+      </x:c>
+      <x:c r="K15" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L15" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M15" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N15" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="25.5" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Sweden</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G16" s="45" t="n">
+        <x:v>80000000</x:v>
+      </x:c>
+      <x:c r="H16" s="45" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="I16" s="45" t="n">
+        <x:v>11.432519140625</x:v>
+      </x:c>
+      <x:c r="J16" s="45" t="n">
+        <x:f>G16/I16</x:f>
+        <x:v>6997582.861306848</x:v>
+      </x:c>
+      <x:c r="K16" s="14" t="str">
+        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L16" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M16" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N16" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="25.5" customHeight="1">
+      <x:c r="A17" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>commercial_market_estimate</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
+        <x:v>calendar_year_estimate</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="n">
+        <x:v>26000000000</x:v>
+      </x:c>
+      <x:c r="H17" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I17" s="45" t="n">
+        <x:v>1.1299831372549</x:v>
+      </x:c>
+      <x:c r="J17" s="45" t="n">
+        <x:f>G17/I17</x:f>
+        <x:v>23009192918.721367</x:v>
+      </x:c>
+      <x:c r="K17" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L17" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M17" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N17" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="25.5" customHeight="1">
+      <x:c r="A18" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>commercial_market_estimate</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F18" s="14" t="str">
+        <x:v>calendar_year_estimate</x:v>
+      </x:c>
+      <x:c r="G18" s="45" t="n">
+        <x:v>45700000000</x:v>
+      </x:c>
+      <x:c r="H18" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I18" s="45" t="n">
+        <x:v>1.1299831372549</x:v>
+      </x:c>
+      <x:c r="J18" s="45" t="n">
+        <x:f>G18/I18</x:f>
+        <x:v>40443081399.44486</x:v>
+      </x:c>
+      <x:c r="K18" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L18" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M18" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N18" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="25.5" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>commercial_market_estimate</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>calendar_year_estimate</x:v>
+      </x:c>
+      <x:c r="G19" s="45" t="n">
+        <x:v>46320000000</x:v>
+      </x:c>
+      <x:c r="H19" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I19" s="45" t="n">
+        <x:v>1.1299831372549</x:v>
+      </x:c>
+      <x:c r="J19" s="45" t="n">
+        <x:f>G19/I19</x:f>
+        <x:v>40991762153.66052</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L19" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M19" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N19" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="25.5" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="n">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G20" s="45" t="n">
+        <x:v>304170046</x:v>
+      </x:c>
+      <x:c r="H20" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I20" s="45" t="n">
+        <x:v>1.109512890625</x:v>
+      </x:c>
+      <x:c r="J20" s="45" t="n">
+        <x:f>G20/I20</x:f>
+        <x:v>274147374.5552049</x:v>
+      </x:c>
+      <x:c r="K20" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
+      </x:c>
+      <x:c r="L20" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M20" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N20" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="25.5" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E21" s="14" t="n">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G21" s="45" t="n">
+        <x:v>485707484</x:v>
+      </x:c>
+      <x:c r="H21" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I21" s="45" t="n">
+        <x:v>1.1069031128405</x:v>
+      </x:c>
+      <x:c r="J21" s="45" t="n">
+        <x:f>G21/I21</x:f>
+        <x:v>438798552.7961817</x:v>
+      </x:c>
+      <x:c r="K21" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
+      </x:c>
+      <x:c r="L21" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M21" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N21" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="25.5" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="n">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F22" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G22" s="45" t="n">
+        <x:v>779836399</x:v>
+      </x:c>
+      <x:c r="H22" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I22" s="45" t="n">
+        <x:v>1.1296811764706</x:v>
+      </x:c>
+      <x:c r="J22" s="45" t="n">
+        <x:f>G22/I22</x:f>
+        <x:v>690315475.943752</x:v>
+      </x:c>
+      <x:c r="K22" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
+      </x:c>
+      <x:c r="L22" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M22" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N22" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="25.5" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="n">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G23" s="45" t="n">
+        <x:v>2043703005</x:v>
+      </x:c>
+      <x:c r="H23" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I23" s="45" t="n">
+        <x:v>1.1809545098039</x:v>
+      </x:c>
+      <x:c r="J23" s="45" t="n">
+        <x:f>G23/I23</x:f>
+        <x:v>1730551844.3207107</x:v>
+      </x:c>
+      <x:c r="K23" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
+      </x:c>
+      <x:c r="L23" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M23" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N23" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="25.5" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G24" s="45" t="n">
+        <x:v>2702608307</x:v>
+      </x:c>
+      <x:c r="H24" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I24" s="45" t="n">
+        <x:v>1.1194745098039</x:v>
+      </x:c>
+      <x:c r="J24" s="45" t="n">
+        <x:f>G24/I24</x:f>
+        <x:v>2414175832.796246</x:v>
+      </x:c>
+      <x:c r="K24" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
+      </x:c>
+      <x:c r="L24" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M24" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N24" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="25.5" customHeight="1">
+      <x:c r="A25" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F25" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G25" s="45" t="n">
+        <x:v>2394423105</x:v>
+      </x:c>
+      <x:c r="H25" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I25" s="45" t="n">
+        <x:v>1.1421961089494</x:v>
+      </x:c>
+      <x:c r="J25" s="45" t="n">
+        <x:f>G25/I25</x:f>
+        <x:v>2096332745.523365</x:v>
+      </x:c>
+      <x:c r="K25" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
+      </x:c>
+      <x:c r="L25" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M25" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N25" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="25.5" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G26" s="45" t="n">
+        <x:v>2763284338</x:v>
+      </x:c>
+      <x:c r="H26" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I26" s="45" t="n">
+        <x:v>1.1827403100775</x:v>
+      </x:c>
+      <x:c r="J26" s="45" t="n">
+        <x:f>G26/I26</x:f>
+        <x:v>2336340711.866778</x:v>
+      </x:c>
+      <x:c r="K26" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L26" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M26" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N26" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="25.5" customHeight="1">
+      <x:c r="A27" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>low.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D27" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E27" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F27" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G27" s="45" t="n">
+        <x:v>258327110.88</x:v>
+      </x:c>
+      <x:c r="H27" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I27" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J27" s="45" t="n">
+        <x:f>G27/I27</x:f>
+        <x:v>144474304.51375833</x:v>
+      </x:c>
+      <x:c r="K27" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L27" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M27" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N27" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="25.5" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>low.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G28" s="45" t="n">
+        <x:v>275335272.8</x:v>
+      </x:c>
+      <x:c r="H28" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I28" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J28" s="45" t="n">
+        <x:f>G28/I28</x:f>
+        <x:v>153986439.55865824</x:v>
+      </x:c>
+      <x:c r="K28" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L28" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M28" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N28" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="25.5" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>low.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F29" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G29" s="45" t="n">
+        <x:v>533662383.68</x:v>
+      </x:c>
+      <x:c r="H29" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I29" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J29" s="45" t="n">
+        <x:f>G29/I29</x:f>
+        <x:v>298460744.0724166</x:v>
+      </x:c>
+      <x:c r="K29" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L29" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M29" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N29" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="25.5" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>base.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G30" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H30" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I30" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J30" s="45" t="n">
+        <x:f>G30/I30</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K30" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L30" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M30" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N30" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="25.5" customHeight="1">
+      <x:c r="A31" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C31" s="14" t="str">
+        <x:v>base.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D31" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E31" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F31" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G31" s="45" t="n">
+        <x:v>367631277.68</x:v>
+      </x:c>
+      <x:c r="H31" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I31" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J31" s="45" t="n">
+        <x:f>G31/I31</x:f>
+        <x:v>205604719.4558489</x:v>
+      </x:c>
+      <x:c r="K31" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L31" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M31" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N31" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="25.5" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>base.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D32" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E32" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F32" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G32" s="45" t="n">
+        <x:v>641811687.89</x:v>
+      </x:c>
+      <x:c r="H32" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I32" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J32" s="45" t="n">
+        <x:f>G32/I32</x:f>
+        <x:v>358945280.34954304</x:v>
+      </x:c>
+      <x:c r="K32" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L32" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M32" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N32" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="25.5" customHeight="1">
+      <x:c r="A33" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B33" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C33" s="14" t="str">
+        <x:v>high.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D33" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E33" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F33" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G33" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H33" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I33" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J33" s="45" t="n">
+        <x:f>G33/I33</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K33" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L33" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M33" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N33" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="25.5" customHeight="1">
+      <x:c r="A34" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B34" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
+        <x:v>high.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D34" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E34" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F34" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G34" s="45" t="n">
+        <x:v>456995382.29</x:v>
+      </x:c>
+      <x:c r="H34" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I34" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J34" s="45" t="n">
+        <x:f>G34/I34</x:f>
+        <x:v>255583278.88015154</x:v>
+      </x:c>
+      <x:c r="K34" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L34" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M34" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N34" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="25.5" customHeight="1">
+      <x:c r="A35" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B35" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C35" s="14" t="str">
+        <x:v>high.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D35" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E35" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F35" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G35" s="45" t="n">
+        <x:v>731175792.5</x:v>
+      </x:c>
+      <x:c r="H35" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I35" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J35" s="45" t="n">
+        <x:f>G35/I35</x:f>
+        <x:v>408923839.7738457</x:v>
+      </x:c>
+      <x:c r="K35" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L35" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M35" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N35" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="25.5" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="D36" s="14"/>
+      <x:c r="E36" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G36" s="45" t="n">
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="H36" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I36" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J36" s="45" t="n">
+        <x:f>G36</x:f>
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="K36" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L36" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M36" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N36" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="25.5" customHeight="1">
+      <x:c r="A37" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B37" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C37" s="14" t="str">
+        <x:v>central</x:v>
+      </x:c>
+      <x:c r="D37" s="14"/>
+      <x:c r="E37" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F37" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G37" s="45" t="n">
+        <x:v>1199220000</x:v>
+      </x:c>
+      <x:c r="H37" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I37" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J37" s="45" t="n">
+        <x:f>G37</x:f>
+        <x:v>1199220000</x:v>
+      </x:c>
+      <x:c r="K37" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L37" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M37" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N37" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="25.5" customHeight="1">
+      <x:c r="A38" s="15" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B38" s="15" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C38" s="15" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="D38" s="15"/>
+      <x:c r="E38" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F38" s="15" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G38" s="46" t="n">
+        <x:v>1654620000</x:v>
+      </x:c>
+      <x:c r="H38" s="46" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I38" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J38" s="46" t="n">
+        <x:f>G38</x:f>
+        <x:v>1654620000</x:v>
+      </x:c>
+      <x:c r="K38" s="15" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L38" s="15" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M38" s="15" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N38" s="15" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a0407373924926"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish donor-conversion cockpit v18 (#16)
Adds the D1-D10 donor gate, fail-closed scenario lab, source-linked ECB EUR equivalents, refreshed New Zealand and FTC evidence routes, and bilingual review artifacts.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7d985d1cc4da4c16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R86a2a7edaf7a4034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1d256bdff4b94488"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R0b4bfd41f6974a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R74cba888082f4021"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5c44fee1a80f4349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R4261d945d76e4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R17ceb104cfe849c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6263184a042843fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,6 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0.00000000000000"/>
+  </x:numFmts>
   <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
@@ -34,15 +38,15 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF182935"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="22"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos Display"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="9"/>
-      <x:color rgb="FF182935"/>
-      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
@@ -63,7 +67,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,6 +77,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF071A2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE3F6F3"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -135,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -168,48 +177,81 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -266,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I50"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I54"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -296,13 +338,35 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
     <x:tableColumn id="3" name="Source class"/>
     <x:tableColumn id="4" name="URL"/>
     <x:tableColumn id="5" name="Retrieved / data as of"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="14">
+    <x:tableColumn id="1" name="Record type"/>
+    <x:tableColumn id="2" name="Record ID"/>
+    <x:tableColumn id="3" name="Item / component"/>
+    <x:tableColumn id="4" name="Country / geography"/>
+    <x:tableColumn id="5" name="Year"/>
+    <x:tableColumn id="6" name="Period"/>
+    <x:tableColumn id="7" name="Original amount"/>
+    <x:tableColumn id="8" name="Currency"/>
+    <x:tableColumn id="9" name="ECB rate (currency units / EUR)"/>
+    <x:tableColumn id="10" name="EUR equivalent (full precision)"/>
+    <x:tableColumn id="11" name="Rate ID"/>
+    <x:tableColumn id="12" name="ECB source URL"/>
+    <x:tableColumn id="13" name="Status"/>
+    <x:tableColumn id="14" name="Reason / method"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -543,7 +607,7 @@
         <x:v>Gaps / additional evidence needed</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="55.5" customHeight="1">
+    <x:row r="2" ht="58.5" customHeight="1">
       <x:c r="A2" s="13" t="str">
         <x:v>Public register data records Pixan Oy as the proprietor.</x:v>
       </x:c>
@@ -572,7 +636,7 @@
         <x:v>The complete chain of title, deeds of assignment and possible encumbrances must be reviewed separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="55.5" customHeight="1">
+    <x:row r="3" ht="58.5" customHeight="1">
       <x:c r="A3" s="14" t="str">
         <x:v>The earliest priority is FI20135829 dated 2013-08-14.</x:v>
       </x:c>
@@ -601,7 +665,7 @@
         <x:v>No material gap for the priority claim.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="55.5" customHeight="1">
+    <x:row r="4" ht="58.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>The central EPO opposition and appeal proceedings concluded with the patent maintained in amended form.</x:v>
       </x:c>
@@ -630,7 +694,7 @@
         <x:v>Current status in each national register is still required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="55.5" customHeight="1">
+    <x:row r="5" ht="58.5" customHeight="1">
       <x:c r="A5" s="14" t="str">
         <x:v>The amended EP3032975B2 contains nine claims.</x:v>
       </x:c>
@@ -659,7 +723,7 @@
         <x:v>Country-specific expert claim construction and product mapping are required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="55.5" customHeight="1">
+    <x:row r="6" ht="58.5" customHeight="1">
       <x:c r="A6" s="14" t="str">
         <x:v>The patent family contains 22 publication-based records.</x:v>
       </x:c>
@@ -688,7 +752,7 @@
         <x:v>Title, fee status, operative claims and legal status must be verified country by country.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="55.5" customHeight="1">
+    <x:row r="7" ht="58.5" customHeight="1">
       <x:c r="A7" s="14" t="str">
         <x:v>The German nullity action was dismissed on 14 January 2026, and an appeal is pending.</x:v>
       </x:c>
@@ -717,7 +781,7 @@
         <x:v>Monitor the progress and outcome of the Federal Court of Justice appeal X ZR 21/26.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="55.5" customHeight="1">
+    <x:row r="8" ht="58.5" customHeight="1">
       <x:c r="A8" s="14" t="str">
         <x:v>The Munich court found that the products examined in the case infringed claims 1 and 6.</x:v>
       </x:c>
@@ -746,7 +810,7 @@
         <x:v>Appeal status, finality, enforcement and any damages actually paid remain to be verified.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="55.5" customHeight="1">
+    <x:row r="9" ht="58.5" customHeight="1">
       <x:c r="A9" s="14" t="str">
         <x:v>The identified Chinese matter is an applicant-side re-examination, not infringement litigation.</x:v>
       </x:c>
@@ -775,7 +839,7 @@
         <x:v>The official CNIPA decision and its reasoning are required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="55.5" customHeight="1">
+    <x:row r="10" ht="58.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
         <x:v>The public atlas contains a fixed research universe of 195 countries.</x:v>
       </x:c>
@@ -804,15 +868,15 @@
         <x:v>There is no gap in the universe definition; evidence coverage is assessed separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="55.5" customHeight="1">
+    <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>Accepted annual official quantitative observations are available from six countries.</x:v>
+        <x:v>The public package contains 27 annual observations sourced from official routes across seven countries.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The accepted countries are Canada, Germany, Finland, New Zealand, Poland and Sweden. The 20 official records include different transaction levels, currencies and product scopes.</x:v>
+        <x:v>The countries are Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. Transaction levels, currencies and product scopes differ.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
@@ -821,19 +885,19 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Count of unique countries represented among annual observations whose evidenceStatus begins official_.</x:v>
+        <x:v>Count of annual observations whose evidenceStatus begins official_.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>Official publication does not make the metrics automatically comparable across countries.</x:v>
+        <x:v>Official publication does not make the metrics automatically comparable.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Comparable annual device and liquid consumer-retail series are required from additional countries.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="55.5" customHeight="1">
+        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
         <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
@@ -841,7 +905,7 @@
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0. Four candidate tests are published against the same ten-criterion protocol.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
@@ -859,10 +923,10 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>At least three accepted donors are required, with regional and regulatory coverage.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="55.5" customHeight="1">
+        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
         <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
@@ -891,7 +955,7 @@
         <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="55.5" customHeight="1">
+    <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
@@ -920,7 +984,7 @@
         <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="55.5" customHeight="1">
+    <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
         <x:v>A conservative text classification identifies NZD 274,180,410.21 as New Zealand 2024 vaping-product-row raw sales.</x:v>
       </x:c>
@@ -949,285 +1013,285 @@
         <x:v>Obtain the authority's product-code dictionary, repeat-row semantics, complete channel coverage and GST basis. The figure is not donor-eligible.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="55.5" customHeight="1">
+    <x:row r="16" ht="93" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
+        <x:v>New Zealand's supported 2024 identified-vaping retail sensitivity is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="F16" s="14" t="str">
-        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F16" s="17" t="str">
+        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
+        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="55.5" customHeight="1">
+        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
+        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
+        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Sum of the four reported product categories.</x:v>
+        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>Shipment value is not treated as consumer retail value.</x:v>
+        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="55.5" customHeight="1">
+        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Sum of the reported liquid-containing product categories.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Physical volume is not treated as market value.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="55.5" customHeight="1">
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="55.5" customHeight="1">
+        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="55.5" customHeight="1">
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the four reported product categories.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Shipment value is not treated as consumer retail value.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="55.5" customHeight="1">
+        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="58.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Sum of the reported liquid-containing product categories.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>Physical volume is not treated as market value.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="55.5" customHeight="1">
+        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Poland reported 805,441 litres in 2023.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>A newer series and observed retail value are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="55.5" customHeight="1">
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>The tax amount is not treated as retail value.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Finality and reconciliation to the tax base are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="55.5" customHeight="1">
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
         <x:v>The observation is not treated as the full market.</x:v>
@@ -1236,749 +1300,865 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Observed retail value and device data are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="55.5" customHeight="1">
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="58.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="55.5" customHeight="1">
+        <x:v>Observed retail sales and price evidence are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Poland reported 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="55.5" customHeight="1">
+        <x:v>A newer series and observed retail value are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>Direct use of the amount reported in the official response.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>The tax amount is not treated as retail value.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
+        <x:v>Finality and reconciliation to the tax base are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="58.5" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="str">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F29" s="14" t="str">
+        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+      </x:c>
+      <x:c r="G29" s="14" t="str">
+        <x:v>The observation is not treated as the full market.</x:v>
+      </x:c>
+      <x:c r="H29" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I29" s="14" t="str">
+        <x:v>Observed retail value and device data are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="58.5" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+      </x:c>
+      <x:c r="G30" s="14" t="str">
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+      </x:c>
+      <x:c r="H30" s="14" t="str">
+        <x:v>Supported</x:v>
+      </x:c>
+      <x:c r="I30" s="14" t="str">
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="58.5" customHeight="1">
+      <x:c r="A31" s="14" t="str">
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>Financial model</x:v>
+      </x:c>
+      <x:c r="C31" s="14" t="str">
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+      </x:c>
+      <x:c r="D31" s="14" t="str">
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+      </x:c>
+      <x:c r="E31" s="14" t="str">
+        <x:v>2025 volume / 2026 prices</x:v>
+      </x:c>
+      <x:c r="F31" s="14" t="str">
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+      </x:c>
+      <x:c r="G31" s="14" t="str">
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+      </x:c>
+      <x:c r="H31" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I31" s="14" t="str">
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="58.5" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+      </x:c>
+      <x:c r="D32" s="14" t="str">
+        <x:v>site/data/atlas.json (readiness)</x:v>
+      </x:c>
+      <x:c r="E32" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F32" s="14" t="str">
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
+      </x:c>
+      <x:c r="G32" s="14" t="str">
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
+      </x:c>
+      <x:c r="H32" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I32" s="14" t="str">
         <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="55.5" customHeight="1">
-      <x:c r="A29" s="14" t="str">
+    <x:row r="33" ht="58.5" customHeight="1">
+      <x:c r="A33" s="14" t="str">
         <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
-      <x:c r="B29" s="14" t="str">
+      <x:c r="B33" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
-      <x:c r="C29" s="14" t="str">
+      <x:c r="C33" s="14" t="str">
         <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
-      <x:c r="D29" s="14" t="str">
+      <x:c r="D33" s="14" t="str">
         <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
-      <x:c r="E29" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F29" s="14" t="str">
+      <x:c r="E33" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F33" s="14" t="str">
         <x:v>Absence check against the public package.</x:v>
       </x:c>
-      <x:c r="G29" s="14" t="str">
+      <x:c r="G33" s="14" t="str">
         <x:v>No assumptions.</x:v>
-      </x:c>
-      <x:c r="H29" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I29" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="55.5" customHeight="1">
-      <x:c r="A30" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
-      </x:c>
-      <x:c r="B30" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
-      </x:c>
-      <x:c r="C30" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
-      </x:c>
-      <x:c r="D30" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
-      </x:c>
-      <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F30" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
-      </x:c>
-      <x:c r="G30" s="14" t="str">
-        <x:v>No assumptions.</x:v>
-      </x:c>
-      <x:c r="H30" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I30" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="55.5" customHeight="1">
-      <x:c r="A31" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
-      </x:c>
-      <x:c r="B31" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
-      </x:c>
-      <x:c r="C31" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
-      </x:c>
-      <x:c r="D31" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
-      </x:c>
-      <x:c r="E31" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F31" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
-      </x:c>
-      <x:c r="G31" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
-      </x:c>
-      <x:c r="H31" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I31" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="55.5" customHeight="1">
-      <x:c r="A32" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
-      </x:c>
-      <x:c r="B32" s="14" t="str">
-        <x:v>Validation</x:v>
-      </x:c>
-      <x:c r="C32" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
-      </x:c>
-      <x:c r="D32" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
-      </x:c>
-      <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F32" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
-      </x:c>
-      <x:c r="G32" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
-      </x:c>
-      <x:c r="H32" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I32" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="55.5" customHeight="1">
-      <x:c r="A33" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
-      </x:c>
-      <x:c r="B33" s="14" t="str">
-        <x:v>IP status</x:v>
-      </x:c>
-      <x:c r="C33" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
-      </x:c>
-      <x:c r="D33" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
-      </x:c>
-      <x:c r="E33" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F33" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
-      </x:c>
-      <x:c r="G33" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="55.5" customHeight="1">
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="58.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="58.5" customHeight="1">
+      <x:c r="A35" s="14" t="str">
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+      </x:c>
+      <x:c r="B35" s="14" t="str">
+        <x:v>Technical differentiation</x:v>
+      </x:c>
+      <x:c r="C35" s="14" t="str">
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+      </x:c>
+      <x:c r="D35" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E35" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F35" s="14" t="str">
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
+      </x:c>
+      <x:c r="G35" s="14" t="str">
+        <x:v>A patent publication is not treated as a product test report.</x:v>
+      </x:c>
+      <x:c r="H35" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I35" s="14" t="str">
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="58.5" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>site/data/evidence.csv</x:v>
+      </x:c>
+      <x:c r="E36" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>Absence check against the public evidence register.</x:v>
+      </x:c>
+      <x:c r="G36" s="14" t="str">
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+      </x:c>
+      <x:c r="H36" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I36" s="14" t="str">
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="58.5" customHeight="1">
+      <x:c r="A37" s="14" t="str">
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+      </x:c>
+      <x:c r="B37" s="14" t="str">
+        <x:v>IP status</x:v>
+      </x:c>
+      <x:c r="C37" s="14" t="str">
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
+      </x:c>
+      <x:c r="D37" s="14" t="str">
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+      </x:c>
+      <x:c r="E37" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F37" s="14" t="str">
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
+      </x:c>
+      <x:c r="G37" s="14" t="str">
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+      </x:c>
+      <x:c r="H37" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I37" s="14" t="str">
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="58.5" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>Technical differentiation</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+      </x:c>
+      <x:c r="G38" s="14" t="str">
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+      </x:c>
+      <x:c r="H38" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I38" s="14" t="str">
         <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="55.5" customHeight="1">
-      <x:c r="A35" s="14" t="str">
+    <x:row r="39" ht="58.5" customHeight="1">
+      <x:c r="A39" s="14" t="str">
         <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
-      <x:c r="B35" s="14" t="str">
+      <x:c r="B39" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
-      <x:c r="C35" s="14" t="str">
+      <x:c r="C39" s="14" t="str">
         <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
-      <x:c r="D35" s="14" t="str">
+      <x:c r="D39" s="14" t="str">
         <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
-      <x:c r="E35" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F35" s="14" t="str">
+      <x:c r="E39" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F39" s="14" t="str">
         <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
-      <x:c r="G35" s="14" t="str">
+      <x:c r="G39" s="14" t="str">
         <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
-      </x:c>
-      <x:c r="H35" s="14" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="I35" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="55.5" customHeight="1">
-      <x:c r="A36" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
-      </x:c>
-      <x:c r="B36" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C36" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
-      </x:c>
-      <x:c r="D36" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
-      </x:c>
-      <x:c r="E36" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F36" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
-      </x:c>
-      <x:c r="G36" s="14" t="str">
-        <x:v>No assumptions.</x:v>
-      </x:c>
-      <x:c r="H36" s="14" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="I36" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="55.5" customHeight="1">
-      <x:c r="A37" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
-      </x:c>
-      <x:c r="B37" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
-      </x:c>
-      <x:c r="C37" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
-      </x:c>
-      <x:c r="D37" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
-      </x:c>
-      <x:c r="E37" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F37" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
-      </x:c>
-      <x:c r="G37" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
-      </x:c>
-      <x:c r="H37" s="14" t="str">
-        <x:v>Assumption</x:v>
-      </x:c>
-      <x:c r="I37" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="55.5" customHeight="1">
-      <x:c r="A38" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
-      </x:c>
-      <x:c r="B38" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C38" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
-      </x:c>
-      <x:c r="D38" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
-      </x:c>
-      <x:c r="E38" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F38" s="14" t="str">
-        <x:v>Financing principle.</x:v>
-      </x:c>
-      <x:c r="G38" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
-      </x:c>
-      <x:c r="H38" s="14" t="str">
-        <x:v>Supported</x:v>
-      </x:c>
-      <x:c r="I38" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="55.5" customHeight="1">
-      <x:c r="A39" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
-      </x:c>
-      <x:c r="B39" s="14" t="str">
-        <x:v>Risks</x:v>
-      </x:c>
-      <x:c r="C39" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
-      </x:c>
-      <x:c r="D39" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
-      </x:c>
-      <x:c r="E39" s="14" t="str">
-        <x:v>2026-08-14</x:v>
-      </x:c>
-      <x:c r="F39" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
-      </x:c>
-      <x:c r="G39" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="55.5" customHeight="1">
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="58.5" customHeight="1">
+      <x:c r="A41" s="14" t="str">
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+      </x:c>
+      <x:c r="B41" s="14" t="str">
+        <x:v>Commercialisation model</x:v>
+      </x:c>
+      <x:c r="C41" s="14" t="str">
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+      </x:c>
+      <x:c r="D41" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+      </x:c>
+      <x:c r="E41" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F41" s="14" t="str">
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+      </x:c>
+      <x:c r="G41" s="14" t="str">
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+      </x:c>
+      <x:c r="H41" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I41" s="14" t="str">
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="58.5" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+      </x:c>
+      <x:c r="D42" s="14" t="str">
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+      </x:c>
+      <x:c r="E42" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>Financing principle.</x:v>
+      </x:c>
+      <x:c r="G42" s="14" t="str">
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+      </x:c>
+      <x:c r="H42" s="14" t="str">
+        <x:v>Supported</x:v>
+      </x:c>
+      <x:c r="I42" s="14" t="str">
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="58.5" customHeight="1">
+      <x:c r="A43" s="14" t="str">
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+      </x:c>
+      <x:c r="B43" s="14" t="str">
+        <x:v>Risks</x:v>
+      </x:c>
+      <x:c r="C43" s="14" t="str">
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+      </x:c>
+      <x:c r="D43" s="14" t="str">
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+      </x:c>
+      <x:c r="E43" s="14" t="str">
+        <x:v>2026-08-14</x:v>
+      </x:c>
+      <x:c r="F43" s="14" t="str">
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
+      </x:c>
+      <x:c r="G43" s="14" t="str">
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+      </x:c>
+      <x:c r="H43" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I43" s="14" t="str">
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="58.5" customHeight="1">
+      <x:c r="A44" s="14" t="str">
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+      </x:c>
+      <x:c r="B44" s="14" t="str">
+        <x:v>Risks</x:v>
+      </x:c>
+      <x:c r="C44" s="14" t="str">
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+      </x:c>
+      <x:c r="D44" s="14" t="str">
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+      </x:c>
+      <x:c r="E44" s="14" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="F44" s="14" t="str">
+        <x:v>Direct observation from the official register.</x:v>
+      </x:c>
+      <x:c r="G44" s="14" t="str">
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+      </x:c>
+      <x:c r="H44" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I44" s="14" t="str">
         <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="55.5" customHeight="1">
-      <x:c r="A41" s="14" t="str">
+    <x:row r="45" ht="58.5" customHeight="1">
+      <x:c r="A45" s="14" t="str">
         <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
-      <x:c r="B41" s="14" t="str">
+      <x:c r="B45" s="14" t="str">
         <x:v>Risks</x:v>
       </x:c>
-      <x:c r="C41" s="14" t="str">
+      <x:c r="C45" s="14" t="str">
         <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
-      <x:c r="D41" s="14" t="str">
+      <x:c r="D45" s="14" t="str">
         <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
-      <x:c r="E41" s="14" t="str">
+      <x:c r="E45" s="14" t="str">
         <x:v>2026-12-04</x:v>
       </x:c>
-      <x:c r="F41" s="14" t="str">
+      <x:c r="F45" s="14" t="str">
         <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
-      <x:c r="G41" s="14" t="str">
+      <x:c r="G45" s="14" t="str">
         <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
-      <x:c r="H41" s="14" t="str">
+      <x:c r="H45" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I41" s="14" t="str">
+      <x:c r="I45" s="14" t="str">
         <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="55.5" customHeight="1">
-      <x:c r="A42" s="14" t="str">
+    <x:row r="46" ht="58.5" customHeight="1">
+      <x:c r="A46" s="14" t="str">
         <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
-      <x:c r="B42" s="14" t="str">
+      <x:c r="B46" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
-      <x:c r="C42" s="14" t="str">
+      <x:c r="C46" s="14" t="str">
         <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
-      <x:c r="D42" s="14" t="str">
+      <x:c r="D46" s="14" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E42" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F42" s="14" t="str">
+      <x:c r="E46" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
         <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
-      <x:c r="G42" s="14" t="str">
+      <x:c r="G46" s="14" t="str">
         <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
-      <x:c r="H42" s="14" t="str">
+      <x:c r="H46" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
-      <x:c r="I42" s="14" t="str">
+      <x:c r="I46" s="14" t="str">
         <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="55.5" customHeight="1">
-      <x:c r="A43" s="14" t="str">
+    <x:row r="47" ht="58.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
         <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
-      </x:c>
-      <x:c r="B43" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C43" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
-      </x:c>
-      <x:c r="D43" s="14" t="str">
-        <x:v>Public package scope</x:v>
-      </x:c>
-      <x:c r="E43" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F43" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
-      </x:c>
-      <x:c r="G43" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
-      </x:c>
-      <x:c r="H43" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I43" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="55.5" customHeight="1">
-      <x:c r="A44" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
-      </x:c>
-      <x:c r="B44" s="14" t="str">
-        <x:v>Financing thesis</x:v>
-      </x:c>
-      <x:c r="C44" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
-      </x:c>
-      <x:c r="D44" s="14" t="str">
-        <x:v>Public package scope</x:v>
-      </x:c>
-      <x:c r="E44" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F44" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
-      </x:c>
-      <x:c r="G44" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
-      </x:c>
-      <x:c r="H44" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I44" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="55.5" customHeight="1">
-      <x:c r="A45" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
-      </x:c>
-      <x:c r="B45" s="14" t="str">
-        <x:v>Competition</x:v>
-      </x:c>
-      <x:c r="C45" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
-      </x:c>
-      <x:c r="D45" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
-      </x:c>
-      <x:c r="E45" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F45" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
-      </x:c>
-      <x:c r="G45" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
-      </x:c>
-      <x:c r="H45" s="14" t="str">
-        <x:v>Missing</x:v>
-      </x:c>
-      <x:c r="I45" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="55.5" customHeight="1">
-      <x:c r="A46" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
-      </x:c>
-      <x:c r="B46" s="14" t="str">
-        <x:v>Customers</x:v>
-      </x:c>
-      <x:c r="C46" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
-      </x:c>
-      <x:c r="D46" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
-      </x:c>
-      <x:c r="E46" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F46" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
-      </x:c>
-      <x:c r="G46" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
-      </x:c>
-      <x:c r="H46" s="14" t="str">
-        <x:v>Assumption</x:v>
-      </x:c>
-      <x:c r="I46" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="55.5" customHeight="1">
-      <x:c r="A47" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G47" s="14" t="str">
+        <x:v>No amount, maturity or security package is assumed.</x:v>
+      </x:c>
+      <x:c r="H47" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I47" s="14" t="str">
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="58.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>The public package is limited to market and patent material.</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G48" s="14" t="str">
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+      </x:c>
+      <x:c r="H48" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="str">
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="58.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="str">
+        <x:v>Competition</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="str">
+        <x:v>Patent and case materials are not a competition map.</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>Absence check against the public package.</x:v>
+      </x:c>
+      <x:c r="G49" s="14" t="str">
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+      </x:c>
+      <x:c r="H49" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I49" s="14" t="str">
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="58.5" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>Customers</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+      </x:c>
+      <x:c r="G50" s="14" t="str">
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+      </x:c>
+      <x:c r="H50" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I50" s="14" t="str">
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="58.5" customHeight="1">
+      <x:c r="A51" s="14" t="str">
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+      </x:c>
+      <x:c r="B51" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C51" s="14" t="str">
         <x:v>The decisions are limited to a country, products, parties and period.</x:v>
       </x:c>
-      <x:c r="D47" s="14" t="str">
+      <x:c r="D51" s="14" t="str">
         <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
-      <x:c r="E47" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F47" s="14" t="str">
+      <x:c r="E51" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F51" s="14" t="str">
         <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
       </x:c>
-      <x:c r="G47" s="14" t="str">
+      <x:c r="G51" s="14" t="str">
         <x:v>Other countries depend on local rights and the products examined there.</x:v>
       </x:c>
-      <x:c r="H47" s="14" t="str">
+      <x:c r="H51" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I47" s="14" t="str">
+      <x:c r="I51" s="14" t="str">
         <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="55.5" customHeight="1">
-      <x:c r="A48" s="14" t="str">
+    <x:row r="52" ht="58.5" customHeight="1">
+      <x:c r="A52" s="14" t="str">
         <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
       </x:c>
-      <x:c r="B48" s="14" t="str">
+      <x:c r="B52" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C48" s="14" t="str">
+      <x:c r="C52" s="14" t="str">
         <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
       </x:c>
-      <x:c r="D48" s="14" t="str">
+      <x:c r="D52" s="14" t="str">
         <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
       </x:c>
-      <x:c r="E48" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F48" s="14" t="str">
+      <x:c r="E52" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F52" s="14" t="str">
         <x:v>Count of countries in each evidence grade.</x:v>
       </x:c>
-      <x:c r="G48" s="14" t="str">
+      <x:c r="G52" s="14" t="str">
         <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
       </x:c>
-      <x:c r="H48" s="14" t="str">
+      <x:c r="H52" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I48" s="14" t="str">
+      <x:c r="I52" s="14" t="str">
         <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="55.5" customHeight="1">
-      <x:c r="A49" s="14" t="str">
+    <x:row r="53" ht="58.5" customHeight="1">
+      <x:c r="A53" s="14" t="str">
         <x:v>No global atlas estimate has been approved for publication.</x:v>
       </x:c>
-      <x:c r="B49" s="14" t="str">
+      <x:c r="B53" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C49" s="14" t="str">
-        <x:v>Zero accepted donor markets is below the minimum threshold of three. The published New Zealand, EU, Canada and Germany candidate tests each have at least one failed criterion.</x:v>
-      </x:c>
-      <x:c r="D49" s="14" t="str">
+      <x:c r="C53" s="14" t="str">
+        <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
+      </x:c>
+      <x:c r="D53" s="14" t="str">
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
-      <x:c r="E49" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F49" s="14" t="str">
-        <x:v>Hard gate: each donor must pass D1–D10, and at least three compatible donors plus regional validation are required.</x:v>
-      </x:c>
-      <x:c r="G49" s="14" t="str">
+      <x:c r="E53" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F53" s="14" t="str">
+        <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
+      </x:c>
+      <x:c r="G53" s="14" t="str">
         <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
       </x:c>
-      <x:c r="H49" s="14" t="str">
+      <x:c r="H53" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I49" s="14" t="str">
+      <x:c r="I53" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="55.5" customHeight="1">
-      <x:c r="A50" s="15" t="str">
+    <x:row r="54" ht="58.5" customHeight="1">
+      <x:c r="A54" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B50" s="15" t="str">
+      <x:c r="B54" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C50" s="15" t="str">
+      <x:c r="C54" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D50" s="15" t="str">
+      <x:c r="D54" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E50" s="15" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F50" s="15" t="str">
+      <x:c r="E54" s="15" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F54" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G50" s="15" t="str">
+      <x:c r="G54" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H50" s="15" t="str">
+      <x:c r="H54" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I50" s="15" t="str">
+      <x:c r="I54" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H50">
+  <x:conditionalFormatting sqref="H2:H54">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H50">
+    <x:dataValidation type="list" sqref="H2:H54">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebd05d810aae4cd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7aa4f32e5298488c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1998,49 +2178,49 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="17" t="str">
+      <x:c r="A1" s="20" t="str">
         <x:v>Pixan · public evidence package summary</x:v>
       </x:c>
-      <x:c r="B1" s="17"/>
-      <x:c r="C1" s="17"/>
-      <x:c r="D1" s="17"/>
-      <x:c r="E1" s="17"/>
-      <x:c r="F1" s="17"/>
-      <x:c r="G1" s="17"/>
-      <x:c r="H1" s="17"/>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
     </x:row>
     <x:row r="2" ht="25.5" customHeight="1">
-      <x:c r="A2" s="17"/>
-      <x:c r="B2" s="17"/>
-      <x:c r="C2" s="17"/>
-      <x:c r="D2" s="17"/>
-      <x:c r="E2" s="17"/>
-      <x:c r="F2" s="17"/>
-      <x:c r="G2" s="17"/>
-      <x:c r="H2" s="17"/>
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+      <x:c r="H2" s="20"/>
     </x:row>
     <x:row r="3" ht="28.5" customHeight="1">
-      <x:c r="A3" s="22" t="str">
+      <x:c r="A3" s="25" t="str">
         <x:v>Independent public evidence summary. Not Pixan Oy's official position; not an audit, valuation, legal opinion, investment recommendation or lending recommendation.</x:v>
       </x:c>
-      <x:c r="B3" s="22"/>
-      <x:c r="C3" s="22"/>
-      <x:c r="D3" s="22"/>
-      <x:c r="E3" s="22"/>
-      <x:c r="F3" s="22"/>
-      <x:c r="G3" s="22"/>
-      <x:c r="H3" s="22"/>
+      <x:c r="B3" s="25"/>
+      <x:c r="C3" s="25"/>
+      <x:c r="D3" s="25"/>
+      <x:c r="E3" s="25"/>
+      <x:c r="F3" s="25"/>
+      <x:c r="G3" s="25"/>
+      <x:c r="H3" s="25"/>
     </x:row>
     <x:row r="5" ht="20.25" customHeight="1">
-      <x:c r="A5" s="25" t="str">
+      <x:c r="A5" s="29" t="str">
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-17</x:v>
+        <x:v>2026.07.24-18</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
-      <x:c r="A6" s="25" t="str">
+      <x:c r="A6" s="29" t="str">
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
@@ -2048,7 +2228,7 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
-      <x:c r="A7" s="25" t="str">
+      <x:c r="A7" s="29" t="str">
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
@@ -2056,59 +2236,64 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="20.25" customHeight="1">
-      <x:c r="A8" s="25" t="str">
+      <x:c r="A8" s="29" t="str">
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:v>49</x:v>
+        <x:f>COUNTA('Evidence Register'!$A$2:$A$54)</x:f>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
     <x:row r="10" ht="20.25" customHeight="1">
-      <x:c r="A10" s="27" t="str">
+      <x:c r="A10" s="31" t="str">
         <x:v>Evidence distribution</x:v>
       </x:c>
-      <x:c r="B10" s="27"/>
+      <x:c r="B10" s="31"/>
     </x:row>
     <x:row r="11" ht="20.25" customHeight="1">
-      <x:c r="A11" s="32" t="str">
+      <x:c r="A11" s="36" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:v>28</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
-      <x:c r="A12" s="33" t="str">
+      <x:c r="A12" s="37" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:v>8</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
-      <x:c r="A13" s="34" t="str">
+      <x:c r="A13" s="38" t="str">
         <x:v>Assumption</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A13)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="20.25" customHeight="1">
-      <x:c r="A14" s="35" t="str">
+      <x:c r="A14" s="39" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="20.25" customHeight="1"/>
     <x:row r="16" ht="20.25" customHeight="1"/>
     <x:row r="17" ht="20.25" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="31" t="str">
         <x:v>Three strongest financing grounds</x:v>
       </x:c>
-      <x:c r="B17" s="27"/>
+      <x:c r="B17" s="31"/>
     </x:row>
     <x:row r="18" ht="28.5" customHeight="1">
       <x:c r="A18" s="13" t="n">
@@ -2137,10 +2322,10 @@
     <x:row r="21" ht="20.25" customHeight="1"/>
     <x:row r="22" ht="20.25" customHeight="1"/>
     <x:row r="23" ht="20.25" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="31" t="str">
         <x:v>Four corrections required for lender readiness</x:v>
       </x:c>
-      <x:c r="B23" s="27"/>
+      <x:c r="B23" s="31"/>
     </x:row>
     <x:row r="24" ht="27" customHeight="1">
       <x:c r="A24" s="13" t="n">
@@ -2190,14 +2375,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="47.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="44.439998626708984" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="25.559999465942383" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="31.5" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="40" t="str">
         <x:v>Priority</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
@@ -2211,7 +2396,7 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="40.5" customHeight="1">
-      <x:c r="A2" s="13" t="n">
+      <x:c r="A2" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
@@ -2225,7 +2410,7 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="40.5" customHeight="1">
-      <x:c r="A3" s="14" t="n">
+      <x:c r="A3" s="42" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
@@ -2239,7 +2424,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="40.5" customHeight="1">
-      <x:c r="A4" s="14" t="n">
+      <x:c r="A4" s="42" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
@@ -2253,7 +2438,7 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="40.5" customHeight="1">
-      <x:c r="A5" s="14" t="n">
+      <x:c r="A5" s="42" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
@@ -2267,7 +2452,7 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="40.5" customHeight="1">
-      <x:c r="A6" s="15" t="n">
+      <x:c r="A6" s="43" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
@@ -2283,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569dfe6a03374efd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a790b47859497e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3167,26 +3352,2097 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="31.5" customHeight="1">
-      <x:c r="A52" s="15" t="str">
+      <x:c r="A52" s="14" t="str">
         <x:v>YTJ-PIXAN</x:v>
       </x:c>
-      <x:c r="B52" s="15" t="str">
+      <x:c r="B52" s="14" t="str">
         <x:v>Finnish Patent and Registration Office / Finnish Tax Administration</x:v>
       </x:c>
-      <x:c r="C52" s="15" t="str">
+      <x:c r="C52" s="14" t="str">
         <x:v>official_company_register</x:v>
       </x:c>
-      <x:c r="D52" s="15" t="str">
+      <x:c r="D52" s="14" t="str">
         <x:v>https://avoindata.prh.fi/opendata-ytj-api/v3/companies?businessId=2632380-1</x:v>
       </x:c>
-      <x:c r="E52" s="15" t="str">
+      <x:c r="E52" s="14" t="str">
         <x:v>2026-07-22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="31.5" customHeight="1">
+      <x:c r="A53" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
+      </x:c>
+      <x:c r="B53" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C53" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D53" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E53" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="31.5" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="31.5" customHeight="1">
+      <x:c r="A55" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
+      </x:c>
+      <x:c r="B55" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C55" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D55" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E55" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="31.5" customHeight="1">
+      <x:c r="A56" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
+      </x:c>
+      <x:c r="B56" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C56" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D56" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E56" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="31.5" customHeight="1">
+      <x:c r="A57" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="31.5" customHeight="1">
+      <x:c r="A58" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="31.5" customHeight="1">
+      <x:c r="A59" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="31.5" customHeight="1">
+      <x:c r="A60" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+      </x:c>
+      <x:c r="B60" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C60" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D60" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E60" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="31.5" customHeight="1">
+      <x:c r="A61" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+      </x:c>
+      <x:c r="B61" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C61" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D61" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E61" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="31.5" customHeight="1">
+      <x:c r="A62" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+      </x:c>
+      <x:c r="B62" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C62" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D62" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E62" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="31.5" customHeight="1">
+      <x:c r="A63" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+      </x:c>
+      <x:c r="B63" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C63" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D63" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E63" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="31.5" customHeight="1">
+      <x:c r="A64" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+      </x:c>
+      <x:c r="B64" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C64" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D64" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E64" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="31.5" customHeight="1">
+      <x:c r="A65" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+      </x:c>
+      <x:c r="B65" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C65" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D65" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E65" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="31.5" customHeight="1">
+      <x:c r="A66" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+      </x:c>
+      <x:c r="B66" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C66" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D66" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E66" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="31.5" customHeight="1">
+      <x:c r="A67" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+      </x:c>
+      <x:c r="B67" s="14" t="str">
+        <x:v>data.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C67" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D67" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="E67" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="31.5" customHeight="1">
+      <x:c r="A68" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+      </x:c>
+      <x:c r="B68" s="14" t="str">
+        <x:v>ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C68" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D68" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="E68" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="31.5" customHeight="1">
+      <x:c r="A69" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+      </x:c>
+      <x:c r="B69" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C69" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D69" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+      </x:c>
+      <x:c r="E69" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="31.5" customHeight="1">
+      <x:c r="A70" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+      </x:c>
+      <x:c r="B70" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C70" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D70" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+      </x:c>
+      <x:c r="E70" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="31.5" customHeight="1">
+      <x:c r="A71" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B71" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C71" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D71" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E71" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="31.5" customHeight="1">
+      <x:c r="A72" s="15" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B72" s="15" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C72" s="15" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D72" s="15" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E72" s="15" t="str">
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8787a1611fab4583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dcf706411294d0a"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="32.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="68.88999938964844" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="36.66999816894531" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="37.5" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>Record type</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>Record ID</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Item / component</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Country / geography</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Period</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>Original amount</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>ECB rate (currency units / EUR)</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>EUR equivalent (full precision)</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>Rate ID</x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>ECB source URL</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="N1" s="5" t="str">
+        <x:v>Reason / method</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="25.5" customHeight="1">
+      <x:c r="A2" s="13" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="str">
+        <x:v>CA-2024-MANUFACTURER-IMPORTER-SHIPMENTS-VALUE</x:v>
+      </x:c>
+      <x:c r="C2" s="13" t="str">
+        <x:v>manufacturer_importer_shipments_value</x:v>
+      </x:c>
+      <x:c r="D2" s="13" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E2" s="13" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F2" s="13" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G2" s="44" t="n">
+        <x:v>1160753796.78</x:v>
+      </x:c>
+      <x:c r="H2" s="44" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I2" s="44" t="n">
+        <x:v>1.482110546875</x:v>
+      </x:c>
+      <x:c r="J2" s="44" t="n">
+        <x:f>G2/I2</x:f>
+        <x:v>783176261.1955132</x:v>
+      </x:c>
+      <x:c r="K2" s="13" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L2" s="13" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M2" s="13" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N2" s="13" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="25.5" customHeight="1">
+      <x:c r="A3" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>NZ-2022-NOTIFIABLE-PRODUCT-REPORTED-REVENUE</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+      </x:c>
+      <x:c r="D3" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E3" s="14" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="F3" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G3" s="45" t="n">
+        <x:v>404000000</x:v>
+      </x:c>
+      <x:c r="H3" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I3" s="45" t="n">
+        <x:v>1.6582474708171</x:v>
+      </x:c>
+      <x:c r="J3" s="45" t="n">
+        <x:f>G3/I3</x:f>
+        <x:v>243630704.7710613</x:v>
+      </x:c>
+      <x:c r="K3" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2022</x:v>
+      </x:c>
+      <x:c r="L3" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M3" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N3" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="25.5" customHeight="1">
+      <x:c r="A4" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>NZ-2023-NOTIFIABLE-PRODUCT-REPORTED-REVENUE-LOWER-BOUND</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+      </x:c>
+      <x:c r="D4" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G4" s="45" t="n">
+        <x:v>374000000</x:v>
+      </x:c>
+      <x:c r="H4" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I4" s="45" t="n">
+        <x:v>1.762151372549</x:v>
+      </x:c>
+      <x:c r="J4" s="45" t="n">
+        <x:f>G4/I4</x:f>
+        <x:v>212240563.33991262</x:v>
+      </x:c>
+      <x:c r="K4" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2023</x:v>
+      </x:c>
+      <x:c r="L4" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M4" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N4" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="25.5" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>NZ-2024-SPECIALIST-RETAIL-SALES-LOWER-BOUND</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>official_specialist_retail_sales_lower_bound</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="n">
+        <x:v>280000000</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="n">
+        <x:f>G5/I5</x:f>
+        <x:v>156595276.14445302</x:v>
+      </x:c>
+      <x:c r="K5" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L5" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M5" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N5" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="25.5" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>NZ-2024-SPECIALIST-RETAIL-PRODUCT-SALES-RAW-FILE-SUM</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>derived_official_workbook_sales_raw_sum</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="n">
+        <x:v>280684512.81</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J6" s="45" t="n">
+        <x:f>G6/I6</x:f>
+        <x:v>156978102.83197576</x:v>
+      </x:c>
+      <x:c r="K6" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L6" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M6" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N6" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="25.5" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>NZ-2024-IDENTIFIED-VAPING-PRODUCT-SALES-RAW-SUM</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>derived_identified_vaping_product_sales_raw_sum</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="n">
+        <x:f>G7/I7</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K7" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L7" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M7" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N7" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="25.5" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>EU-2023-EC-E-CIGARETTE-MARKET-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>institutional_market_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>European Union</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="n">
+        <x:v>4990000000</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J8" s="45" t="n">
+        <x:f>G8</x:f>
+        <x:v>4990000000</x:v>
+      </x:c>
+      <x:c r="K8" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L8" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M8" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N8" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="25.5" customHeight="1">
+      <x:c r="A9" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>DE-2023-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>substitutes_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="n">
+        <x:v>201000000</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="n">
+        <x:f>G9</x:f>
+        <x:v>201000000</x:v>
+      </x:c>
+      <x:c r="K9" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L9" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M9" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N9" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="25.5" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>DE-2024-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>substitutes_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F10" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="n">
+        <x:v>266000000</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J10" s="45" t="n">
+        <x:f>G10</x:f>
+        <x:v>266000000</x:v>
+      </x:c>
+      <x:c r="K10" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L10" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M10" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N10" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="25.5" customHeight="1">
+      <x:c r="A11" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>DE-2025-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>substitutes_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F11" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="n">
+        <x:v>404000000</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="n">
+        <x:f>G11</x:f>
+        <x:v>404000000</x:v>
+      </x:c>
+      <x:c r="K11" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L11" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M11" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N11" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="25.5" customHeight="1">
+      <x:c r="A12" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C12" s="14" t="str">
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>Finland</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="n">
+        <x:v>3540319</x:v>
+      </x:c>
+      <x:c r="H12" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I12" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="45" t="n">
+        <x:f>G12</x:f>
+        <x:v>3540319</x:v>
+      </x:c>
+      <x:c r="K12" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L12" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M12" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N12" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="25.5" customHeight="1">
+      <x:c r="A13" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>e_liquid_excise_amount</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="n">
+        <x:v>993100000</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I13" s="45" t="n">
+        <x:v>4.2396576470588</x:v>
+      </x:c>
+      <x:c r="J13" s="45" t="n">
+        <x:f>G13/I13</x:f>
+        <x:v>234240611.54771507</x:v>
+      </x:c>
+      <x:c r="K13" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L13" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M13" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N13" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="25.5" customHeight="1">
+      <x:c r="A14" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>vaping_device_excise_amount</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F14" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="n">
+        <x:v>175300000</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I14" s="45" t="n">
+        <x:v>4.2396576470588</x:v>
+      </x:c>
+      <x:c r="J14" s="45" t="n">
+        <x:f>G14/I14</x:f>
+        <x:v>41347678.183782555</x:v>
+      </x:c>
+      <x:c r="K14" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L14" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M14" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N14" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="25.5" customHeight="1">
+      <x:c r="A15" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>vaping_component_sets_excise_amount</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="n">
+        <x:v>2500000</x:v>
+      </x:c>
+      <x:c r="H15" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I15" s="45" t="n">
+        <x:v>4.2396576470588</x:v>
+      </x:c>
+      <x:c r="J15" s="45" t="n">
+        <x:f>G15/I15</x:f>
+        <x:v>589670.2536192606</x:v>
+      </x:c>
+      <x:c r="K15" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L15" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M15" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N15" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="25.5" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Sweden</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G16" s="45" t="n">
+        <x:v>80000000</x:v>
+      </x:c>
+      <x:c r="H16" s="45" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="I16" s="45" t="n">
+        <x:v>11.432519140625</x:v>
+      </x:c>
+      <x:c r="J16" s="45" t="n">
+        <x:f>G16/I16</x:f>
+        <x:v>6997582.861306848</x:v>
+      </x:c>
+      <x:c r="K16" s="14" t="str">
+        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L16" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M16" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N16" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="25.5" customHeight="1">
+      <x:c r="A17" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>commercial_market_estimate</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
+        <x:v>calendar_year_estimate</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="n">
+        <x:v>26000000000</x:v>
+      </x:c>
+      <x:c r="H17" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I17" s="45" t="n">
+        <x:v>1.1299831372549</x:v>
+      </x:c>
+      <x:c r="J17" s="45" t="n">
+        <x:f>G17/I17</x:f>
+        <x:v>23009192918.721367</x:v>
+      </x:c>
+      <x:c r="K17" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L17" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M17" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N17" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="25.5" customHeight="1">
+      <x:c r="A18" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>commercial_market_estimate</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F18" s="14" t="str">
+        <x:v>calendar_year_estimate</x:v>
+      </x:c>
+      <x:c r="G18" s="45" t="n">
+        <x:v>45700000000</x:v>
+      </x:c>
+      <x:c r="H18" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I18" s="45" t="n">
+        <x:v>1.1299831372549</x:v>
+      </x:c>
+      <x:c r="J18" s="45" t="n">
+        <x:f>G18/I18</x:f>
+        <x:v>40443081399.44486</x:v>
+      </x:c>
+      <x:c r="K18" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L18" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M18" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N18" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="25.5" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>commercial_market_estimate</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Global</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>calendar_year_estimate</x:v>
+      </x:c>
+      <x:c r="G19" s="45" t="n">
+        <x:v>46320000000</x:v>
+      </x:c>
+      <x:c r="H19" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I19" s="45" t="n">
+        <x:v>1.1299831372549</x:v>
+      </x:c>
+      <x:c r="J19" s="45" t="n">
+        <x:f>G19/I19</x:f>
+        <x:v>40991762153.66052</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+      </x:c>
+      <x:c r="L19" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M19" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N19" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="25.5" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="n">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G20" s="45" t="n">
+        <x:v>304170046</x:v>
+      </x:c>
+      <x:c r="H20" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I20" s="45" t="n">
+        <x:v>1.109512890625</x:v>
+      </x:c>
+      <x:c r="J20" s="45" t="n">
+        <x:f>G20/I20</x:f>
+        <x:v>274147374.5552049</x:v>
+      </x:c>
+      <x:c r="K20" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
+      </x:c>
+      <x:c r="L20" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M20" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N20" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="25.5" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E21" s="14" t="n">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G21" s="45" t="n">
+        <x:v>485707484</x:v>
+      </x:c>
+      <x:c r="H21" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I21" s="45" t="n">
+        <x:v>1.1069031128405</x:v>
+      </x:c>
+      <x:c r="J21" s="45" t="n">
+        <x:f>G21/I21</x:f>
+        <x:v>438798552.7961817</x:v>
+      </x:c>
+      <x:c r="K21" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
+      </x:c>
+      <x:c r="L21" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M21" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N21" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="25.5" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="n">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F22" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G22" s="45" t="n">
+        <x:v>779836399</x:v>
+      </x:c>
+      <x:c r="H22" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I22" s="45" t="n">
+        <x:v>1.1296811764706</x:v>
+      </x:c>
+      <x:c r="J22" s="45" t="n">
+        <x:f>G22/I22</x:f>
+        <x:v>690315475.943752</x:v>
+      </x:c>
+      <x:c r="K22" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
+      </x:c>
+      <x:c r="L22" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M22" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N22" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="25.5" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="n">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G23" s="45" t="n">
+        <x:v>2043703005</x:v>
+      </x:c>
+      <x:c r="H23" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I23" s="45" t="n">
+        <x:v>1.1809545098039</x:v>
+      </x:c>
+      <x:c r="J23" s="45" t="n">
+        <x:f>G23/I23</x:f>
+        <x:v>1730551844.3207107</x:v>
+      </x:c>
+      <x:c r="K23" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
+      </x:c>
+      <x:c r="L23" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M23" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N23" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="25.5" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G24" s="45" t="n">
+        <x:v>2702608307</x:v>
+      </x:c>
+      <x:c r="H24" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I24" s="45" t="n">
+        <x:v>1.1194745098039</x:v>
+      </x:c>
+      <x:c r="J24" s="45" t="n">
+        <x:f>G24/I24</x:f>
+        <x:v>2414175832.796246</x:v>
+      </x:c>
+      <x:c r="K24" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
+      </x:c>
+      <x:c r="L24" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M24" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N24" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="25.5" customHeight="1">
+      <x:c r="A25" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F25" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G25" s="45" t="n">
+        <x:v>2394423105</x:v>
+      </x:c>
+      <x:c r="H25" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I25" s="45" t="n">
+        <x:v>1.1421961089494</x:v>
+      </x:c>
+      <x:c r="J25" s="45" t="n">
+        <x:f>G25/I25</x:f>
+        <x:v>2096332745.523365</x:v>
+      </x:c>
+      <x:c r="K25" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
+      </x:c>
+      <x:c r="L25" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M25" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N25" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="25.5" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G26" s="45" t="n">
+        <x:v>2763284338</x:v>
+      </x:c>
+      <x:c r="H26" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I26" s="45" t="n">
+        <x:v>1.1827403100775</x:v>
+      </x:c>
+      <x:c r="J26" s="45" t="n">
+        <x:f>G26/I26</x:f>
+        <x:v>2336340711.866778</x:v>
+      </x:c>
+      <x:c r="K26" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L26" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M26" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N26" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="25.5" customHeight="1">
+      <x:c r="A27" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>low.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D27" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E27" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F27" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G27" s="45" t="n">
+        <x:v>258327110.88</x:v>
+      </x:c>
+      <x:c r="H27" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I27" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J27" s="45" t="n">
+        <x:f>G27/I27</x:f>
+        <x:v>144474304.51375833</x:v>
+      </x:c>
+      <x:c r="K27" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L27" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M27" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N27" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="25.5" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>low.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G28" s="45" t="n">
+        <x:v>275335272.8</x:v>
+      </x:c>
+      <x:c r="H28" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I28" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J28" s="45" t="n">
+        <x:f>G28/I28</x:f>
+        <x:v>153986439.55865824</x:v>
+      </x:c>
+      <x:c r="K28" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L28" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M28" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N28" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="25.5" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>low.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F29" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G29" s="45" t="n">
+        <x:v>533662383.68</x:v>
+      </x:c>
+      <x:c r="H29" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I29" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J29" s="45" t="n">
+        <x:f>G29/I29</x:f>
+        <x:v>298460744.0724166</x:v>
+      </x:c>
+      <x:c r="K29" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L29" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M29" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N29" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="25.5" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>base.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G30" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H30" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I30" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J30" s="45" t="n">
+        <x:f>G30/I30</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K30" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L30" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M30" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N30" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="25.5" customHeight="1">
+      <x:c r="A31" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C31" s="14" t="str">
+        <x:v>base.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D31" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E31" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F31" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G31" s="45" t="n">
+        <x:v>367631277.68</x:v>
+      </x:c>
+      <x:c r="H31" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I31" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J31" s="45" t="n">
+        <x:f>G31/I31</x:f>
+        <x:v>205604719.4558489</x:v>
+      </x:c>
+      <x:c r="K31" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L31" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M31" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N31" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="25.5" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>base.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D32" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E32" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F32" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G32" s="45" t="n">
+        <x:v>641811687.89</x:v>
+      </x:c>
+      <x:c r="H32" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I32" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J32" s="45" t="n">
+        <x:f>G32/I32</x:f>
+        <x:v>358945280.34954304</x:v>
+      </x:c>
+      <x:c r="K32" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L32" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M32" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N32" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="25.5" customHeight="1">
+      <x:c r="A33" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B33" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C33" s="14" t="str">
+        <x:v>high.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D33" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E33" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F33" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G33" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H33" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I33" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J33" s="45" t="n">
+        <x:f>G33/I33</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K33" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L33" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M33" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N33" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="25.5" customHeight="1">
+      <x:c r="A34" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B34" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
+        <x:v>high.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D34" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E34" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F34" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G34" s="45" t="n">
+        <x:v>456995382.29</x:v>
+      </x:c>
+      <x:c r="H34" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I34" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J34" s="45" t="n">
+        <x:f>G34/I34</x:f>
+        <x:v>255583278.88015154</x:v>
+      </x:c>
+      <x:c r="K34" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L34" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M34" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N34" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="25.5" customHeight="1">
+      <x:c r="A35" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B35" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C35" s="14" t="str">
+        <x:v>high.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D35" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E35" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F35" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G35" s="45" t="n">
+        <x:v>731175792.5</x:v>
+      </x:c>
+      <x:c r="H35" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I35" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J35" s="45" t="n">
+        <x:f>G35/I35</x:f>
+        <x:v>408923839.7738457</x:v>
+      </x:c>
+      <x:c r="K35" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L35" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M35" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N35" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="25.5" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="D36" s="14"/>
+      <x:c r="E36" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G36" s="45" t="n">
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="H36" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I36" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J36" s="45" t="n">
+        <x:f>G36</x:f>
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="K36" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L36" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M36" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N36" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="25.5" customHeight="1">
+      <x:c r="A37" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B37" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C37" s="14" t="str">
+        <x:v>central</x:v>
+      </x:c>
+      <x:c r="D37" s="14"/>
+      <x:c r="E37" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F37" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G37" s="45" t="n">
+        <x:v>1199220000</x:v>
+      </x:c>
+      <x:c r="H37" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I37" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J37" s="45" t="n">
+        <x:f>G37</x:f>
+        <x:v>1199220000</x:v>
+      </x:c>
+      <x:c r="K37" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L37" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M37" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N37" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="25.5" customHeight="1">
+      <x:c r="A38" s="15" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B38" s="15" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C38" s="15" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="D38" s="15"/>
+      <x:c r="E38" s="15" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F38" s="15" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G38" s="46" t="n">
+        <x:v>1654620000</x:v>
+      </x:c>
+      <x:c r="H38" s="46" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I38" s="46" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J38" s="46" t="n">
+        <x:f>G38</x:f>
+        <x:v>1654620000</x:v>
+      </x:c>
+      <x:c r="K38" s="15" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L38" s="15" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M38" s="15" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N38" s="15" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a0407373924926"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Canada retail donor sprint v19
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R74cba888082f4021"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5c44fee1a80f4349"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R4261d945d76e4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R17ceb104cfe849c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6263184a042843fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R0be318fc6c234b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7a21837fe5764959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1da2b31e28be48eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R39e5335d567a405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re44a4e909c2a433c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -351,7 +351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Record type"/>
     <x:tableColumn id="2" name="Record ID"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public package contains 27 annual observations sourced from official routes across seven countries.</x:v>
+        <x:v>The public package contains 34 annual observations sourced from official routes across seven countries.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
@@ -1160,31 +1160,31 @@
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
+        <x:v>Statistics Canada's Canada series contains seven full-year consumer-retail estimates for 2019–2025; the 2024 value is CAD 1,219,160,000.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
+        <x:v>The annual estimate is the sum of four RCS quarters for NAPCS 5619122. Health Canada's 2024 manufacturer/importer shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_RCS_2019_2025_RETAIL_SALES.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Sum of the four reported product categories.</x:v>
+        <x:v>CAD 1,219,160,000 − CAD 1,160,753,796.78 = CAD 58,406,203.22; RCS / Health Canada = 1.0503175, or +5.03%.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>Shipment value is not treated as consumer retail value.</x:v>
+        <x:v>Every 2024 quarter carries quality flag E. Vaping-specific channel completeness is not quantified and the vaping-excise basis is not confirmed.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
+        <x:v>The retail-to-shipment bridge does not yet explain margin, inventory, returns, timing, product scope or tax treatment; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58.5" customHeight="1">
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7aa4f32e5298488c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb43a70f44cfa4102"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-18</x:v>
+        <x:v>2026.07.24-19</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2257,7 +2257,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2266,7 +2266,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a790b47859497e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R362dc33430c844c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3370,7 +3370,7 @@
     </x:row>
     <x:row r="53" ht="31.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
+        <x:v>REGISTER-REFERENCE-BC2CDD0708D5</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3379,7 +3379,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3387,7 +3387,7 @@
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
       <x:c r="A54" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
+        <x:v>REGISTER-REFERENCE-7264539499F0</x:v>
       </x:c>
       <x:c r="B54" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3396,7 +3396,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D54" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3404,7 +3404,7 @@
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
       <x:c r="A55" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
+        <x:v>REGISTER-REFERENCE-2580DD0733C9</x:v>
       </x:c>
       <x:c r="B55" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3413,7 +3413,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D55" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3421,7 +3421,7 @@
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
       <x:c r="A56" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
+        <x:v>REGISTER-REFERENCE-38DD93023815</x:v>
       </x:c>
       <x:c r="B56" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3430,7 +3430,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D56" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3438,7 +3438,7 @@
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
       <x:c r="A57" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+        <x:v>REGISTER-REFERENCE-72D82058EA8A</x:v>
       </x:c>
       <x:c r="B57" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3447,7 +3447,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D57" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3455,7 +3455,7 @@
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
       <x:c r="A58" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
       </x:c>
       <x:c r="B58" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3464,7 +3464,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D58" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3472,7 +3472,7 @@
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
       <x:c r="A59" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+        <x:v>REGISTER-REFERENCE-ACB549D404B8</x:v>
       </x:c>
       <x:c r="B59" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3481,7 +3481,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D59" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3489,7 +3489,7 @@
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
       <x:c r="A60" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
       </x:c>
       <x:c r="B60" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3498,7 +3498,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D60" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3506,7 +3506,7 @@
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
       <x:c r="A61" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
       </x:c>
       <x:c r="B61" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3515,7 +3515,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D61" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3523,7 +3523,7 @@
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
       <x:c r="A62" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
       </x:c>
       <x:c r="B62" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3532,7 +3532,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D62" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3540,7 +3540,7 @@
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
       <x:c r="A63" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
       </x:c>
       <x:c r="B63" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3549,7 +3549,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D63" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3557,7 +3557,7 @@
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
       <x:c r="A64" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
       </x:c>
       <x:c r="B64" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3566,7 +3566,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D64" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3574,7 +3574,7 @@
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
       <x:c r="A65" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
       </x:c>
       <x:c r="B65" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3583,7 +3583,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D65" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3591,7 +3591,7 @@
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
       <x:c r="A66" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
       </x:c>
       <x:c r="B66" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3600,7 +3600,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D66" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3608,16 +3608,16 @@
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
       </x:c>
       <x:c r="B67" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C67" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D67" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3625,16 +3625,16 @@
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
       <x:c r="A68" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
       </x:c>
       <x:c r="B68" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C68" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D68" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3642,16 +3642,16 @@
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
       </x:c>
       <x:c r="B69" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C69" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D69" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3659,16 +3659,16 @@
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
       <x:c r="A70" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
       </x:c>
       <x:c r="B70" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C70" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D70" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3676,42 +3676,161 @@
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
       <x:c r="A71" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+      </x:c>
+      <x:c r="B71" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C71" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D71" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E71" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="31.5" customHeight="1">
+      <x:c r="A72" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+      </x:c>
+      <x:c r="B72" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C72" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D72" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E72" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="31.5" customHeight="1">
+      <x:c r="A73" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+      </x:c>
+      <x:c r="B73" s="14" t="str">
+        <x:v>data.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C73" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D73" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="E73" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="31.5" customHeight="1">
+      <x:c r="A74" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+      </x:c>
+      <x:c r="B74" s="14" t="str">
+        <x:v>ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C74" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D74" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="E74" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="31.5" customHeight="1">
+      <x:c r="A75" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+      </x:c>
+      <x:c r="B75" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C75" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D75" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+      </x:c>
+      <x:c r="E75" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="31.5" customHeight="1">
+      <x:c r="A76" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+      </x:c>
+      <x:c r="B76" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C76" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D76" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+      </x:c>
+      <x:c r="E76" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="31.5" customHeight="1">
+      <x:c r="A77" s="14" t="str">
         <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
-      <x:c r="B71" s="14" t="str">
+      <x:c r="B77" s="14" t="str">
         <x:v>United Nations</x:v>
       </x:c>
-      <x:c r="C71" s="14" t="str">
+      <x:c r="C77" s="14" t="str">
         <x:v>official_reference</x:v>
       </x:c>
-      <x:c r="D71" s="14" t="str">
+      <x:c r="D77" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
-      <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="31.5" customHeight="1">
-      <x:c r="A72" s="15" t="str">
+      <x:c r="E77" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="31.5" customHeight="1">
+      <x:c r="A78" s="14" t="str">
         <x:v>UN-NON-MEMBER-STATES</x:v>
       </x:c>
-      <x:c r="B72" s="15" t="str">
+      <x:c r="B78" s="14" t="str">
         <x:v>United Nations</x:v>
       </x:c>
-      <x:c r="C72" s="15" t="str">
+      <x:c r="C78" s="14" t="str">
         <x:v>official_reference</x:v>
       </x:c>
-      <x:c r="D72" s="15" t="str">
+      <x:c r="D78" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
-      <x:c r="E72" s="15" t="str">
+      <x:c r="E78" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="31.5" customHeight="1">
+      <x:c r="A79" s="15" t="str">
+        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+      </x:c>
+      <x:c r="B79" s="15" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C79" s="15" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D79" s="15" t="str">
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
+      </x:c>
+      <x:c r="E79" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dcf706411294d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeb72f7eb4cb42f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3830,38 +3949,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
-        <x:v>NZ-2022-NOTIFIABLE-PRODUCT-REPORTED-REVENUE</x:v>
+        <x:v>CA-2019-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C3" s="14" t="str">
-        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D3" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E3" s="14" t="n">
-        <x:v>2022</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G3" s="45" t="n">
-        <x:v>404000000</x:v>
+        <x:v>477077000</x:v>
       </x:c>
       <x:c r="H3" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I3" s="45" t="n">
-        <x:v>1.6582474708171</x:v>
+        <x:v>1.485477254902</x:v>
       </x:c>
       <x:c r="J3" s="45" t="n">
         <x:f>G3/I3</x:f>
-        <x:v>243630704.7710613</x:v>
+        <x:v>321160757.20827764</x:v>
       </x:c>
       <x:c r="K3" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2022</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2019</x:v>
       </x:c>
       <x:c r="L3" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M3" s="14" t="str">
         <x:v>computed</x:v>
@@ -3875,38 +3994,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>NZ-2023-NOTIFIABLE-PRODUCT-REPORTED-REVENUE-LOWER-BOUND</x:v>
+        <x:v>CA-2020-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C4" s="14" t="str">
-        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E4" s="14" t="n">
-        <x:v>2023</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G4" s="45" t="n">
-        <x:v>374000000</x:v>
+        <x:v>520647000</x:v>
       </x:c>
       <x:c r="H4" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I4" s="45" t="n">
-        <x:v>1.762151372549</x:v>
+        <x:v>1.5299926070039</x:v>
       </x:c>
       <x:c r="J4" s="45" t="n">
         <x:f>G4/I4</x:f>
-        <x:v>212240563.33991262</x:v>
+        <x:v>340293801.1704215</x:v>
       </x:c>
       <x:c r="K4" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2023</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2020</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
         <x:v>computed</x:v>
@@ -3920,38 +4039,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>NZ-2024-SPECIALIST-RETAIL-SALES-LOWER-BOUND</x:v>
+        <x:v>CA-2021-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C5" s="14" t="str">
-        <x:v>official_specialist_retail_sales_lower_bound</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D5" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E5" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G5" s="45" t="n">
-        <x:v>280000000</x:v>
+        <x:v>992732000</x:v>
       </x:c>
       <x:c r="H5" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I5" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.4825689922481</x:v>
       </x:c>
       <x:c r="J5" s="45" t="n">
         <x:f>G5/I5</x:f>
-        <x:v>156595276.14445302</x:v>
+        <x:v>669602565.0008142</x:v>
       </x:c>
       <x:c r="K5" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
       </x:c>
       <x:c r="L5" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M5" s="14" t="str">
         <x:v>computed</x:v>
@@ -3965,38 +4084,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>NZ-2024-SPECIALIST-RETAIL-PRODUCT-SALES-RAW-FILE-SUM</x:v>
+        <x:v>CA-2022-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
-        <x:v>derived_official_workbook_sales_raw_sum</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E6" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G6" s="45" t="n">
-        <x:v>280684512.81</x:v>
+        <x:v>1277158000</x:v>
       </x:c>
       <x:c r="H6" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I6" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.3694910505837</x:v>
       </x:c>
       <x:c r="J6" s="45" t="n">
         <x:f>G6/I6</x:f>
-        <x:v>156978102.83197576</x:v>
+        <x:v>932578565.924658</x:v>
       </x:c>
       <x:c r="K6" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2022</x:v>
       </x:c>
       <x:c r="L6" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M6" s="14" t="str">
         <x:v>computed</x:v>
@@ -4010,38 +4129,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>NZ-2024-IDENTIFIED-VAPING-PRODUCT-SALES-RAW-SUM</x:v>
+        <x:v>CA-2023-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C7" s="14" t="str">
-        <x:v>derived_identified_vaping_product_sales_raw_sum</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E7" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G7" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>1530758000</x:v>
       </x:c>
       <x:c r="H7" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I7" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.459468627451</x:v>
       </x:c>
       <x:c r="J7" s="45" t="n">
         <x:f>G7/I7</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>1048846115.091565</x:v>
       </x:c>
       <x:c r="K7" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2023</x:v>
       </x:c>
       <x:c r="L7" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M7" s="14" t="str">
         <x:v>computed</x:v>
@@ -4055,44 +4174,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>EU-2023-EC-E-CIGARETTE-MARKET-BENCHMARK</x:v>
+        <x:v>CA-2024-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>institutional_market_value_benchmark</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>European Union</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E8" s="14" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G8" s="45" t="n">
-        <x:v>4990000000</x:v>
+        <x:v>1219160000</x:v>
       </x:c>
       <x:c r="H8" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I8" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.482110546875</x:v>
       </x:c>
       <x:c r="J8" s="45" t="n">
-        <x:f>G8</x:f>
-        <x:v>4990000000</x:v>
+        <x:f>G8/I8</x:f>
+        <x:v>822583715.2097555</x:v>
       </x:c>
       <x:c r="K8" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L8" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M8" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N8" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25.5" customHeight="1">
@@ -4100,44 +4219,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>DE-2023-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+        <x:v>CA-2025-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>substitutes_excise_receipts</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>Germany</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E9" s="14" t="n">
-        <x:v>2023</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G9" s="45" t="n">
-        <x:v>201000000</x:v>
+        <x:v>1266567000</x:v>
       </x:c>
       <x:c r="H9" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I9" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.5787262745098</x:v>
       </x:c>
       <x:c r="J9" s="45" t="n">
-        <x:f>G9</x:f>
-        <x:v>201000000</x:v>
+        <x:f>G9/I9</x:f>
+        <x:v>802271438.9758753</x:v>
       </x:c>
       <x:c r="K9" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L9" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M9" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N9" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25.5" customHeight="1">
@@ -4145,44 +4264,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>DE-2024-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+        <x:v>NZ-2022-NOTIFIABLE-PRODUCT-REPORTED-REVENUE</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>substitutes_excise_receipts</x:v>
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>Germany</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E10" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G10" s="45" t="n">
-        <x:v>266000000</x:v>
+        <x:v>404000000</x:v>
       </x:c>
       <x:c r="H10" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I10" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.6582474708171</x:v>
       </x:c>
       <x:c r="J10" s="45" t="n">
-        <x:f>G10</x:f>
-        <x:v>266000000</x:v>
+        <x:f>G10/I10</x:f>
+        <x:v>243630704.7710613</x:v>
       </x:c>
       <x:c r="K10" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2022</x:v>
       </x:c>
       <x:c r="L10" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M10" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N10" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25.5" customHeight="1">
@@ -4190,44 +4309,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>DE-2025-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+        <x:v>NZ-2023-NOTIFIABLE-PRODUCT-REPORTED-REVENUE-LOWER-BOUND</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>substitutes_excise_receipts</x:v>
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>Germany</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E11" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G11" s="45" t="n">
-        <x:v>404000000</x:v>
+        <x:v>374000000</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I11" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.762151372549</x:v>
       </x:c>
       <x:c r="J11" s="45" t="n">
-        <x:f>G11</x:f>
-        <x:v>404000000</x:v>
+        <x:f>G11/I11</x:f>
+        <x:v>212240563.33991262</x:v>
       </x:c>
       <x:c r="K11" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2023</x:v>
       </x:c>
       <x:c r="L11" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M11" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N11" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25.5" customHeight="1">
@@ -4235,44 +4354,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>NZ-2024-SPECIALIST-RETAIL-SALES-LOWER-BOUND</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>official_specialist_retail_sales_lower_bound</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>Finland</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E12" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G12" s="45" t="n">
-        <x:v>3540319</x:v>
+        <x:v>280000000</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I12" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J12" s="45" t="n">
-        <x:f>G12</x:f>
-        <x:v>3540319</x:v>
+        <x:f>G12/I12</x:f>
+        <x:v>156595276.14445302</x:v>
       </x:c>
       <x:c r="K12" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L12" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M12" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N12" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25.5" customHeight="1">
@@ -4280,38 +4399,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
+        <x:v>NZ-2024-SPECIALIST-RETAIL-PRODUCT-SALES-RAW-FILE-SUM</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>e_liquid_excise_amount</x:v>
+        <x:v>derived_official_workbook_sales_raw_sum</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E13" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G13" s="45" t="n">
-        <x:v>993100000</x:v>
+        <x:v>280684512.81</x:v>
       </x:c>
       <x:c r="H13" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I13" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J13" s="45" t="n">
         <x:f>G13/I13</x:f>
-        <x:v>234240611.54771507</x:v>
+        <x:v>156978102.83197576</x:v>
       </x:c>
       <x:c r="K13" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L13" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M13" s="14" t="str">
         <x:v>computed</x:v>
@@ -4325,38 +4444,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
+        <x:v>NZ-2024-IDENTIFIED-VAPING-PRODUCT-SALES-RAW-SUM</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>vaping_device_excise_amount</x:v>
+        <x:v>derived_identified_vaping_product_sales_raw_sum</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E14" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G14" s="45" t="n">
-        <x:v>175300000</x:v>
+        <x:v>274180410.21</x:v>
       </x:c>
       <x:c r="H14" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I14" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J14" s="45" t="n">
         <x:f>G14/I14</x:f>
-        <x:v>41347678.183782555</x:v>
+        <x:v>153340560.89369413</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L14" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M14" s="14" t="str">
         <x:v>computed</x:v>
@@ -4370,44 +4489,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
+        <x:v>EU-2023-EC-E-CIGARETTE-MARKET-BENCHMARK</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>vaping_component_sets_excise_amount</x:v>
+        <x:v>institutional_market_value_benchmark</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>European Union</x:v>
       </x:c>
       <x:c r="E15" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G15" s="45" t="n">
-        <x:v>2500000</x:v>
+        <x:v>4990000000</x:v>
       </x:c>
       <x:c r="H15" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I15" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J15" s="45" t="n">
-        <x:f>G15/I15</x:f>
-        <x:v>589670.2536192606</x:v>
+        <x:f>G15</x:f>
+        <x:v>4990000000</x:v>
       </x:c>
       <x:c r="K15" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L15" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M15" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N15" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25.5" customHeight="1">
@@ -4415,44 +4534,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>DE-2023-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>substitutes_excise_receipts</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>Sweden</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E16" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G16" s="45" t="n">
-        <x:v>80000000</x:v>
+        <x:v>201000000</x:v>
       </x:c>
       <x:c r="H16" s="45" t="str">
-        <x:v>SEK</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I16" s="45" t="n">
-        <x:v>11.432519140625</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J16" s="45" t="n">
-        <x:f>G16/I16</x:f>
-        <x:v>6997582.861306848</x:v>
+        <x:f>G16</x:f>
+        <x:v>201000000</x:v>
       </x:c>
       <x:c r="K16" s="14" t="str">
-        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L16" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M16" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N16" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25.5" customHeight="1">
@@ -4460,44 +4579,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>DE-2024-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>substitutes_excise_receipts</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E17" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G17" s="45" t="n">
-        <x:v>26000000000</x:v>
+        <x:v>266000000</x:v>
       </x:c>
       <x:c r="H17" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I17" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J17" s="45" t="n">
-        <x:f>G17/I17</x:f>
-        <x:v>23009192918.721367</x:v>
+        <x:f>G17</x:f>
+        <x:v>266000000</x:v>
       </x:c>
       <x:c r="K17" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L17" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M17" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N17" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25.5" customHeight="1">
@@ -4505,44 +4624,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
-        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>DE-2025-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>substitutes_excise_receipts</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E18" s="14" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G18" s="45" t="n">
-        <x:v>45700000000</x:v>
+        <x:v>404000000</x:v>
       </x:c>
       <x:c r="H18" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I18" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J18" s="45" t="n">
-        <x:f>G18/I18</x:f>
-        <x:v>40443081399.44486</x:v>
+        <x:f>G18</x:f>
+        <x:v>404000000</x:v>
       </x:c>
       <x:c r="K18" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L18" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M18" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N18" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25.5" customHeight="1">
@@ -4550,44 +4669,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Finland</x:v>
       </x:c>
       <x:c r="E19" s="14" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G19" s="45" t="n">
-        <x:v>46320000000</x:v>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="H19" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I19" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="45" t="n">
-        <x:f>G19/I19</x:f>
-        <x:v>40991762153.66052</x:v>
+        <x:f>G19</x:f>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L19" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M19" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N19" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25.5" customHeight="1">
@@ -4595,38 +4714,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_amount</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E20" s="14" t="n">
-        <x:v>2015</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G20" s="45" t="n">
-        <x:v>304170046</x:v>
+        <x:v>993100000</x:v>
       </x:c>
       <x:c r="H20" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I20" s="45" t="n">
-        <x:v>1.109512890625</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J20" s="45" t="n">
         <x:f>G20/I20</x:f>
-        <x:v>274147374.5552049</x:v>
+        <x:v>234240611.54771507</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L20" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M20" s="14" t="str">
         <x:v>computed</x:v>
@@ -4640,38 +4759,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaping_device_excise_amount</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E21" s="14" t="n">
-        <x:v>2016</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G21" s="45" t="n">
-        <x:v>485707484</x:v>
+        <x:v>175300000</x:v>
       </x:c>
       <x:c r="H21" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I21" s="45" t="n">
-        <x:v>1.1069031128405</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J21" s="45" t="n">
         <x:f>G21/I21</x:f>
-        <x:v>438798552.7961817</x:v>
+        <x:v>41347678.183782555</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L21" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M21" s="14" t="str">
         <x:v>computed</x:v>
@@ -4685,38 +4804,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaping_component_sets_excise_amount</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E22" s="14" t="n">
-        <x:v>2017</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G22" s="45" t="n">
-        <x:v>779836399</x:v>
+        <x:v>2500000</x:v>
       </x:c>
       <x:c r="H22" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I22" s="45" t="n">
-        <x:v>1.1296811764706</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J22" s="45" t="n">
         <x:f>G22/I22</x:f>
-        <x:v>690315475.943752</x:v>
+        <x:v>589670.2536192606</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L22" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M22" s="14" t="str">
         <x:v>computed</x:v>
@@ -4730,38 +4849,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Sweden</x:v>
       </x:c>
       <x:c r="E23" s="14" t="n">
-        <x:v>2018</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G23" s="45" t="n">
-        <x:v>2043703005</x:v>
+        <x:v>80000000</x:v>
       </x:c>
       <x:c r="H23" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>SEK</x:v>
       </x:c>
       <x:c r="I23" s="45" t="n">
-        <x:v>1.1809545098039</x:v>
+        <x:v>11.432519140625</x:v>
       </x:c>
       <x:c r="J23" s="45" t="n">
         <x:f>G23/I23</x:f>
-        <x:v>1730551844.3207107</x:v>
+        <x:v>6997582.861306848</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
+        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L23" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M23" s="14" t="str">
         <x:v>computed</x:v>
@@ -4775,38 +4894,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E24" s="14" t="n">
-        <x:v>2019</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G24" s="45" t="n">
-        <x:v>2702608307</x:v>
+        <x:v>26000000000</x:v>
       </x:c>
       <x:c r="H24" s="45" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="I24" s="45" t="n">
-        <x:v>1.1194745098039</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J24" s="45" t="n">
         <x:f>G24/I24</x:f>
-        <x:v>2414175832.796246</x:v>
+        <x:v>23009192918.721367</x:v>
       </x:c>
       <x:c r="K24" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L24" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M24" s="14" t="str">
         <x:v>computed</x:v>
@@ -4820,38 +4939,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E25" s="14" t="n">
-        <x:v>2020</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G25" s="45" t="n">
-        <x:v>2394423105</x:v>
+        <x:v>45700000000</x:v>
       </x:c>
       <x:c r="H25" s="45" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="I25" s="45" t="n">
-        <x:v>1.1421961089494</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J25" s="45" t="n">
         <x:f>G25/I25</x:f>
-        <x:v>2096332745.523365</x:v>
+        <x:v>40443081399.44486</x:v>
       </x:c>
       <x:c r="K25" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L25" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M25" s="14" t="str">
         <x:v>computed</x:v>
@@ -4865,38 +4984,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E26" s="14" t="n">
-        <x:v>2021</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G26" s="45" t="n">
-        <x:v>2763284338</x:v>
+        <x:v>46320000000</x:v>
       </x:c>
       <x:c r="H26" s="45" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="I26" s="45" t="n">
-        <x:v>1.1827403100775</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J26" s="45" t="n">
         <x:f>G26/I26</x:f>
-        <x:v>2336340711.866778</x:v>
+        <x:v>40991762153.66052</x:v>
       </x:c>
       <x:c r="K26" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L26" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M26" s="14" t="str">
         <x:v>computed</x:v>
@@ -4907,41 +5026,41 @@
     </x:row>
     <x:row r="27" ht="25.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>low.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E27" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G27" s="45" t="n">
-        <x:v>258327110.88</x:v>
+        <x:v>304170046</x:v>
       </x:c>
       <x:c r="H27" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I27" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.109512890625</x:v>
       </x:c>
       <x:c r="J27" s="45" t="n">
         <x:f>G27/I27</x:f>
-        <x:v>144474304.51375833</x:v>
+        <x:v>274147374.5552049</x:v>
       </x:c>
       <x:c r="K27" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
       </x:c>
       <x:c r="L27" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M27" s="14" t="str">
         <x:v>computed</x:v>
@@ -4952,41 +5071,41 @@
     </x:row>
     <x:row r="28" ht="25.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>low.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E28" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2016</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G28" s="45" t="n">
-        <x:v>275335272.8</x:v>
+        <x:v>485707484</x:v>
       </x:c>
       <x:c r="H28" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I28" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1069031128405</x:v>
       </x:c>
       <x:c r="J28" s="45" t="n">
         <x:f>G28/I28</x:f>
-        <x:v>153986439.55865824</x:v>
+        <x:v>438798552.7961817</x:v>
       </x:c>
       <x:c r="K28" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
       </x:c>
       <x:c r="L28" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M28" s="14" t="str">
         <x:v>computed</x:v>
@@ -4997,41 +5116,41 @@
     </x:row>
     <x:row r="29" ht="25.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>low.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E29" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G29" s="45" t="n">
-        <x:v>533662383.68</x:v>
+        <x:v>779836399</x:v>
       </x:c>
       <x:c r="H29" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I29" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1296811764706</x:v>
       </x:c>
       <x:c r="J29" s="45" t="n">
         <x:f>G29/I29</x:f>
-        <x:v>298460744.0724166</x:v>
+        <x:v>690315475.943752</x:v>
       </x:c>
       <x:c r="K29" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
       </x:c>
       <x:c r="L29" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M29" s="14" t="str">
         <x:v>computed</x:v>
@@ -5042,41 +5161,41 @@
     </x:row>
     <x:row r="30" ht="25.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>base.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E30" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G30" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>2043703005</x:v>
       </x:c>
       <x:c r="H30" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I30" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1809545098039</x:v>
       </x:c>
       <x:c r="J30" s="45" t="n">
         <x:f>G30/I30</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>1730551844.3207107</x:v>
       </x:c>
       <x:c r="K30" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
       </x:c>
       <x:c r="L30" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M30" s="14" t="str">
         <x:v>computed</x:v>
@@ -5087,41 +5206,41 @@
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>base.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E31" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G31" s="45" t="n">
-        <x:v>367631277.68</x:v>
+        <x:v>2702608307</x:v>
       </x:c>
       <x:c r="H31" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I31" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1194745098039</x:v>
       </x:c>
       <x:c r="J31" s="45" t="n">
         <x:f>G31/I31</x:f>
-        <x:v>205604719.4558489</x:v>
+        <x:v>2414175832.796246</x:v>
       </x:c>
       <x:c r="K31" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
       </x:c>
       <x:c r="L31" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M31" s="14" t="str">
         <x:v>computed</x:v>
@@ -5132,41 +5251,41 @@
     </x:row>
     <x:row r="32" ht="25.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>base.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E32" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G32" s="45" t="n">
-        <x:v>641811687.89</x:v>
+        <x:v>2394423105</x:v>
       </x:c>
       <x:c r="H32" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I32" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1421961089494</x:v>
       </x:c>
       <x:c r="J32" s="45" t="n">
         <x:f>G32/I32</x:f>
-        <x:v>358945280.34954304</x:v>
+        <x:v>2096332745.523365</x:v>
       </x:c>
       <x:c r="K32" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
       </x:c>
       <x:c r="L32" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M32" s="14" t="str">
         <x:v>computed</x:v>
@@ -5177,41 +5296,41 @@
     </x:row>
     <x:row r="33" ht="25.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>high.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E33" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G33" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>2763284338</x:v>
       </x:c>
       <x:c r="H33" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I33" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1827403100775</x:v>
       </x:c>
       <x:c r="J33" s="45" t="n">
         <x:f>G33/I33</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>2336340711.866778</x:v>
       </x:c>
       <x:c r="K33" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
       </x:c>
       <x:c r="L33" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M33" s="14" t="str">
         <x:v>computed</x:v>
@@ -5228,7 +5347,7 @@
         <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>high.generalRetailRpsNzd</x:v>
+        <x:v>low.specialistRetailNzd</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
         <x:v>New Zealand</x:v>
@@ -5240,7 +5359,7 @@
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G34" s="45" t="n">
-        <x:v>456995382.29</x:v>
+        <x:v>258327110.88</x:v>
       </x:c>
       <x:c r="H34" s="45" t="str">
         <x:v>NZD</x:v>
@@ -5250,7 +5369,7 @@
       </x:c>
       <x:c r="J34" s="45" t="n">
         <x:f>G34/I34</x:f>
-        <x:v>255583278.88015154</x:v>
+        <x:v>144474304.51375833</x:v>
       </x:c>
       <x:c r="K34" s="14" t="str">
         <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
@@ -5273,7 +5392,7 @@
         <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>high.combinedNzd</x:v>
+        <x:v>low.generalRetailRpsNzd</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
         <x:v>New Zealand</x:v>
@@ -5285,7 +5404,7 @@
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G35" s="45" t="n">
-        <x:v>731175792.5</x:v>
+        <x:v>275335272.8</x:v>
       </x:c>
       <x:c r="H35" s="45" t="str">
         <x:v>NZD</x:v>
@@ -5295,7 +5414,7 @@
       </x:c>
       <x:c r="J35" s="45" t="n">
         <x:f>G35/I35</x:f>
-        <x:v>408923839.7738457</x:v>
+        <x:v>153986439.55865824</x:v>
       </x:c>
       <x:c r="K35" s="14" t="str">
         <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
@@ -5312,137 +5431,452 @@
     </x:row>
     <x:row r="36" ht="25.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>scenario_component</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>low</x:v>
-      </x:c>
-      <x:c r="D36" s="14"/>
+        <x:v>low.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
       <x:c r="E36" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G36" s="45" t="n">
-        <x:v>667920000</x:v>
+        <x:v>533662383.68</x:v>
       </x:c>
       <x:c r="H36" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I36" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J36" s="45" t="n">
-        <x:f>G36</x:f>
-        <x:v>667920000</x:v>
+        <x:f>G36/I36</x:f>
+        <x:v>298460744.0724166</x:v>
       </x:c>
       <x:c r="K36" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L36" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M36" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N36" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="25.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>scenario_component</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>central</x:v>
-      </x:c>
-      <x:c r="D37" s="14"/>
+        <x:v>base.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D37" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
       <x:c r="E37" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G37" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H37" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I37" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J37" s="45" t="n">
+        <x:f>G37/I37</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K37" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L37" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M37" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N37" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="25.5" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>base.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G38" s="45" t="n">
+        <x:v>367631277.68</x:v>
+      </x:c>
+      <x:c r="H38" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I38" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J38" s="45" t="n">
+        <x:f>G38/I38</x:f>
+        <x:v>205604719.4558489</x:v>
+      </x:c>
+      <x:c r="K38" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L38" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M38" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N38" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="25.5" customHeight="1">
+      <x:c r="A39" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B39" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C39" s="14" t="str">
+        <x:v>base.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D39" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E39" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F39" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G39" s="45" t="n">
+        <x:v>641811687.89</x:v>
+      </x:c>
+      <x:c r="H39" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I39" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J39" s="45" t="n">
+        <x:f>G39/I39</x:f>
+        <x:v>358945280.34954304</x:v>
+      </x:c>
+      <x:c r="K39" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L39" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M39" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N39" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="25.5" customHeight="1">
+      <x:c r="A40" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B40" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C40" s="14" t="str">
+        <x:v>high.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D40" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E40" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F40" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G40" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H40" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I40" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J40" s="45" t="n">
+        <x:f>G40/I40</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K40" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L40" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M40" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N40" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="25.5" customHeight="1">
+      <x:c r="A41" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B41" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C41" s="14" t="str">
+        <x:v>high.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D41" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E41" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F41" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G41" s="45" t="n">
+        <x:v>456995382.29</x:v>
+      </x:c>
+      <x:c r="H41" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I41" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J41" s="45" t="n">
+        <x:f>G41/I41</x:f>
+        <x:v>255583278.88015154</x:v>
+      </x:c>
+      <x:c r="K41" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L41" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M41" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N41" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="25.5" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>high.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D42" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E42" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G42" s="45" t="n">
+        <x:v>731175792.5</x:v>
+      </x:c>
+      <x:c r="H42" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I42" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J42" s="45" t="n">
+        <x:f>G42/I42</x:f>
+        <x:v>408923839.7738457</x:v>
+      </x:c>
+      <x:c r="K42" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L42" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M42" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N42" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="25.5" customHeight="1">
+      <x:c r="A43" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B43" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C43" s="14" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="D43" s="14"/>
+      <x:c r="E43" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F43" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G43" s="45" t="n">
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="H43" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I43" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J43" s="45" t="n">
+        <x:f>G43</x:f>
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="K43" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L43" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M43" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N43" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="25.5" customHeight="1">
+      <x:c r="A44" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B44" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C44" s="14" t="str">
+        <x:v>central</x:v>
+      </x:c>
+      <x:c r="D44" s="14"/>
+      <x:c r="E44" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F44" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G44" s="45" t="n">
         <x:v>1199220000</x:v>
       </x:c>
-      <x:c r="H37" s="45" t="str">
+      <x:c r="H44" s="45" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="I37" s="45" t="n">
+      <x:c r="I44" s="45" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J37" s="45" t="n">
-        <x:f>G37</x:f>
+      <x:c r="J44" s="45" t="n">
+        <x:f>G44</x:f>
         <x:v>1199220000</x:v>
       </x:c>
-      <x:c r="K37" s="14" t="str">
+      <x:c r="K44" s="14" t="str">
         <x:v>EUR-IDENTITY</x:v>
       </x:c>
-      <x:c r="L37" s="14" t="str">
+      <x:c r="L44" s="14" t="str">
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
-      <x:c r="M37" s="14" t="str">
+      <x:c r="M44" s="14" t="str">
         <x:v>already_eur</x:v>
       </x:c>
-      <x:c r="N37" s="14" t="str">
+      <x:c r="N44" s="14" t="str">
         <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="25.5" customHeight="1">
-      <x:c r="A38" s="15" t="str">
+    <x:row r="45" ht="25.5" customHeight="1">
+      <x:c r="A45" s="15" t="str">
         <x:v>model</x:v>
       </x:c>
-      <x:c r="B38" s="15" t="str">
+      <x:c r="B45" s="15" t="str">
         <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
       </x:c>
-      <x:c r="C38" s="15" t="str">
+      <x:c r="C45" s="15" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="D38" s="15"/>
-      <x:c r="E38" s="15" t="n">
+      <x:c r="D45" s="15"/>
+      <x:c r="E45" s="15" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="F38" s="15" t="str">
+      <x:c r="F45" s="15" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
-      <x:c r="G38" s="46" t="n">
+      <x:c r="G45" s="46" t="n">
         <x:v>1654620000</x:v>
       </x:c>
-      <x:c r="H38" s="46" t="str">
+      <x:c r="H45" s="46" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="I38" s="46" t="n">
+      <x:c r="I45" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J38" s="46" t="n">
-        <x:f>G38</x:f>
+      <x:c r="J45" s="46" t="n">
+        <x:f>G45</x:f>
         <x:v>1654620000</x:v>
       </x:c>
-      <x:c r="K38" s="15" t="str">
+      <x:c r="K45" s="15" t="str">
         <x:v>EUR-IDENTITY</x:v>
       </x:c>
-      <x:c r="L38" s="15" t="str">
+      <x:c r="L45" s="15" t="str">
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
-      <x:c r="M38" s="15" t="str">
+      <x:c r="M45" s="15" t="str">
         <x:v>already_eur</x:v>
       </x:c>
-      <x:c r="N38" s="15" t="str">
+      <x:c r="N45" s="15" t="str">
         <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a0407373924926"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0554f810ee9045e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Canada retail donor sprint v19 (#17)
Add Statistics Canada retail series, donor closure actions, ECB CAD conversions, updated request/vendor states, and refreshed bilingual lender/buyer artifacts.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R74cba888082f4021"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5c44fee1a80f4349"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R4261d945d76e4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R17ceb104cfe849c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6263184a042843fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R0be318fc6c234b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7a21837fe5764959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1da2b31e28be48eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R39e5335d567a405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re44a4e909c2a433c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -351,7 +351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Record type"/>
     <x:tableColumn id="2" name="Record ID"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public package contains 27 annual observations sourced from official routes across seven countries.</x:v>
+        <x:v>The public package contains 34 annual observations sourced from official routes across seven countries.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
@@ -1160,31 +1160,31 @@
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Canada's 2024 manufacturer and importer shipment value was CAD 1.16075379678 billion.</x:v>
+        <x:v>Statistics Canada's Canada series contains seven full-year consumer-retail estimates for 2019–2025; the 2024 value is CAD 1,219,160,000.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>The official full-year series reports shipment value to wholesalers and retailers across four reported product categories. It does not measure consumer retail purchases, and Health Canada may revise the data.</x:v>
+        <x:v>The annual estimate is the sum of four RCS quarters for NAPCS 5619122. Health Canada's 2024 manufacturer/importer shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_RCS_2019_2025_RETAIL_SALES.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Sum of the four reported product categories.</x:v>
+        <x:v>CAD 1,219,160,000 − CAD 1,160,753,796.78 = CAD 58,406,203.22; RCS / Health Canada = 1.0503175, or +5.03%.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>Shipment value is not treated as consumer retail value.</x:v>
+        <x:v>Every 2024 quarter carries quality flag E. Vaping-specific channel completeness is not quantified and the vaping-excise basis is not confirmed.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Retail margins, channel structure and inventory movements must be reconciled.</x:v>
+        <x:v>The retail-to-shipment bridge does not yet explain margin, inventory, returns, timing, product scope or tax treatment; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58.5" customHeight="1">
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7aa4f32e5298488c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb43a70f44cfa4102"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-18</x:v>
+        <x:v>2026.07.24-19</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2257,7 +2257,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2266,7 +2266,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a790b47859497e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R362dc33430c844c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3370,7 +3370,7 @@
     </x:row>
     <x:row r="53" ht="31.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
+        <x:v>REGISTER-REFERENCE-BC2CDD0708D5</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3379,7 +3379,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3387,7 +3387,7 @@
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
       <x:c r="A54" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
+        <x:v>REGISTER-REFERENCE-7264539499F0</x:v>
       </x:c>
       <x:c r="B54" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3396,7 +3396,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D54" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3404,7 +3404,7 @@
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
       <x:c r="A55" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
+        <x:v>REGISTER-REFERENCE-2580DD0733C9</x:v>
       </x:c>
       <x:c r="B55" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3413,7 +3413,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D55" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3421,7 +3421,7 @@
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
       <x:c r="A56" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
+        <x:v>REGISTER-REFERENCE-38DD93023815</x:v>
       </x:c>
       <x:c r="B56" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3430,7 +3430,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D56" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3438,7 +3438,7 @@
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
       <x:c r="A57" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+        <x:v>REGISTER-REFERENCE-72D82058EA8A</x:v>
       </x:c>
       <x:c r="B57" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3447,7 +3447,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D57" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3455,7 +3455,7 @@
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
       <x:c r="A58" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
       </x:c>
       <x:c r="B58" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3464,7 +3464,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D58" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3472,7 +3472,7 @@
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
       <x:c r="A59" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+        <x:v>REGISTER-REFERENCE-ACB549D404B8</x:v>
       </x:c>
       <x:c r="B59" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3481,7 +3481,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D59" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3489,7 +3489,7 @@
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
       <x:c r="A60" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
       </x:c>
       <x:c r="B60" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3498,7 +3498,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D60" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3506,7 +3506,7 @@
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
       <x:c r="A61" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
       </x:c>
       <x:c r="B61" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3515,7 +3515,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D61" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3523,7 +3523,7 @@
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
       <x:c r="A62" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
       </x:c>
       <x:c r="B62" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3532,7 +3532,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D62" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3540,7 +3540,7 @@
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
       <x:c r="A63" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
       </x:c>
       <x:c r="B63" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3549,7 +3549,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D63" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3557,7 +3557,7 @@
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
       <x:c r="A64" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
       </x:c>
       <x:c r="B64" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3566,7 +3566,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D64" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3574,7 +3574,7 @@
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
       <x:c r="A65" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
       </x:c>
       <x:c r="B65" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3583,7 +3583,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D65" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3591,7 +3591,7 @@
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
       <x:c r="A66" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
       </x:c>
       <x:c r="B66" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3600,7 +3600,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D66" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3608,16 +3608,16 @@
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
       </x:c>
       <x:c r="B67" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C67" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D67" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3625,16 +3625,16 @@
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
       <x:c r="A68" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
       </x:c>
       <x:c r="B68" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C68" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D68" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3642,16 +3642,16 @@
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
       </x:c>
       <x:c r="B69" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C69" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D69" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3659,16 +3659,16 @@
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
       <x:c r="A70" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
       </x:c>
       <x:c r="B70" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C70" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D70" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3676,42 +3676,161 @@
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
       <x:c r="A71" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+      </x:c>
+      <x:c r="B71" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C71" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D71" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E71" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="31.5" customHeight="1">
+      <x:c r="A72" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+      </x:c>
+      <x:c r="B72" s="14" t="str">
+        <x:v>data-api.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C72" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D72" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="E72" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="31.5" customHeight="1">
+      <x:c r="A73" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+      </x:c>
+      <x:c r="B73" s="14" t="str">
+        <x:v>data.ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C73" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D73" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="E73" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="31.5" customHeight="1">
+      <x:c r="A74" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+      </x:c>
+      <x:c r="B74" s="14" t="str">
+        <x:v>ecb.europa.eu</x:v>
+      </x:c>
+      <x:c r="C74" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D74" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="E74" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="31.5" customHeight="1">
+      <x:c r="A75" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+      </x:c>
+      <x:c r="B75" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C75" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D75" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+      </x:c>
+      <x:c r="E75" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="31.5" customHeight="1">
+      <x:c r="A76" s="14" t="str">
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+      </x:c>
+      <x:c r="B76" s="14" t="str">
+        <x:v>Federal Trade Commission</x:v>
+      </x:c>
+      <x:c r="C76" s="14" t="str">
+        <x:v>official_report</x:v>
+      </x:c>
+      <x:c r="D76" s="14" t="str">
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+      </x:c>
+      <x:c r="E76" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="31.5" customHeight="1">
+      <x:c r="A77" s="14" t="str">
         <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
-      <x:c r="B71" s="14" t="str">
+      <x:c r="B77" s="14" t="str">
         <x:v>United Nations</x:v>
       </x:c>
-      <x:c r="C71" s="14" t="str">
+      <x:c r="C77" s="14" t="str">
         <x:v>official_reference</x:v>
       </x:c>
-      <x:c r="D71" s="14" t="str">
+      <x:c r="D77" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
-      <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="31.5" customHeight="1">
-      <x:c r="A72" s="15" t="str">
+      <x:c r="E77" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="31.5" customHeight="1">
+      <x:c r="A78" s="14" t="str">
         <x:v>UN-NON-MEMBER-STATES</x:v>
       </x:c>
-      <x:c r="B72" s="15" t="str">
+      <x:c r="B78" s="14" t="str">
         <x:v>United Nations</x:v>
       </x:c>
-      <x:c r="C72" s="15" t="str">
+      <x:c r="C78" s="14" t="str">
         <x:v>official_reference</x:v>
       </x:c>
-      <x:c r="D72" s="15" t="str">
+      <x:c r="D78" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
-      <x:c r="E72" s="15" t="str">
+      <x:c r="E78" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="31.5" customHeight="1">
+      <x:c r="A79" s="15" t="str">
+        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+      </x:c>
+      <x:c r="B79" s="15" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C79" s="15" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D79" s="15" t="str">
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
+      </x:c>
+      <x:c r="E79" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dcf706411294d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeb72f7eb4cb42f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3830,38 +3949,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
-        <x:v>NZ-2022-NOTIFIABLE-PRODUCT-REPORTED-REVENUE</x:v>
+        <x:v>CA-2019-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C3" s="14" t="str">
-        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D3" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E3" s="14" t="n">
-        <x:v>2022</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G3" s="45" t="n">
-        <x:v>404000000</x:v>
+        <x:v>477077000</x:v>
       </x:c>
       <x:c r="H3" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I3" s="45" t="n">
-        <x:v>1.6582474708171</x:v>
+        <x:v>1.485477254902</x:v>
       </x:c>
       <x:c r="J3" s="45" t="n">
         <x:f>G3/I3</x:f>
-        <x:v>243630704.7710613</x:v>
+        <x:v>321160757.20827764</x:v>
       </x:c>
       <x:c r="K3" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2022</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2019</x:v>
       </x:c>
       <x:c r="L3" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M3" s="14" t="str">
         <x:v>computed</x:v>
@@ -3875,38 +3994,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>NZ-2023-NOTIFIABLE-PRODUCT-REPORTED-REVENUE-LOWER-BOUND</x:v>
+        <x:v>CA-2020-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C4" s="14" t="str">
-        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E4" s="14" t="n">
-        <x:v>2023</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G4" s="45" t="n">
-        <x:v>374000000</x:v>
+        <x:v>520647000</x:v>
       </x:c>
       <x:c r="H4" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I4" s="45" t="n">
-        <x:v>1.762151372549</x:v>
+        <x:v>1.5299926070039</x:v>
       </x:c>
       <x:c r="J4" s="45" t="n">
         <x:f>G4/I4</x:f>
-        <x:v>212240563.33991262</x:v>
+        <x:v>340293801.1704215</x:v>
       </x:c>
       <x:c r="K4" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2023</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2020</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
         <x:v>computed</x:v>
@@ -3920,38 +4039,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>NZ-2024-SPECIALIST-RETAIL-SALES-LOWER-BOUND</x:v>
+        <x:v>CA-2021-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C5" s="14" t="str">
-        <x:v>official_specialist_retail_sales_lower_bound</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D5" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E5" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G5" s="45" t="n">
-        <x:v>280000000</x:v>
+        <x:v>992732000</x:v>
       </x:c>
       <x:c r="H5" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I5" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.4825689922481</x:v>
       </x:c>
       <x:c r="J5" s="45" t="n">
         <x:f>G5/I5</x:f>
-        <x:v>156595276.14445302</x:v>
+        <x:v>669602565.0008142</x:v>
       </x:c>
       <x:c r="K5" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
       </x:c>
       <x:c r="L5" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M5" s="14" t="str">
         <x:v>computed</x:v>
@@ -3965,38 +4084,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>NZ-2024-SPECIALIST-RETAIL-PRODUCT-SALES-RAW-FILE-SUM</x:v>
+        <x:v>CA-2022-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
-        <x:v>derived_official_workbook_sales_raw_sum</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E6" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G6" s="45" t="n">
-        <x:v>280684512.81</x:v>
+        <x:v>1277158000</x:v>
       </x:c>
       <x:c r="H6" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I6" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.3694910505837</x:v>
       </x:c>
       <x:c r="J6" s="45" t="n">
         <x:f>G6/I6</x:f>
-        <x:v>156978102.83197576</x:v>
+        <x:v>932578565.924658</x:v>
       </x:c>
       <x:c r="K6" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2022</x:v>
       </x:c>
       <x:c r="L6" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M6" s="14" t="str">
         <x:v>computed</x:v>
@@ -4010,38 +4129,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>NZ-2024-IDENTIFIED-VAPING-PRODUCT-SALES-RAW-SUM</x:v>
+        <x:v>CA-2023-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C7" s="14" t="str">
-        <x:v>derived_identified_vaping_product_sales_raw_sum</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E7" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G7" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>1530758000</x:v>
       </x:c>
       <x:c r="H7" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I7" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.459468627451</x:v>
       </x:c>
       <x:c r="J7" s="45" t="n">
         <x:f>G7/I7</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>1048846115.091565</x:v>
       </x:c>
       <x:c r="K7" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2023</x:v>
       </x:c>
       <x:c r="L7" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M7" s="14" t="str">
         <x:v>computed</x:v>
@@ -4055,44 +4174,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>EU-2023-EC-E-CIGARETTE-MARKET-BENCHMARK</x:v>
+        <x:v>CA-2024-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>institutional_market_value_benchmark</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>European Union</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E8" s="14" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G8" s="45" t="n">
-        <x:v>4990000000</x:v>
+        <x:v>1219160000</x:v>
       </x:c>
       <x:c r="H8" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I8" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.482110546875</x:v>
       </x:c>
       <x:c r="J8" s="45" t="n">
-        <x:f>G8</x:f>
-        <x:v>4990000000</x:v>
+        <x:f>G8/I8</x:f>
+        <x:v>822583715.2097555</x:v>
       </x:c>
       <x:c r="K8" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L8" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M8" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N8" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25.5" customHeight="1">
@@ -4100,44 +4219,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>DE-2023-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+        <x:v>CA-2025-STATCAN-RCS-VAPING-RETAIL-SALES</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>substitutes_excise_receipts</x:v>
+        <x:v>statcan_rcs_vaping_retail_sales</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>Germany</x:v>
+        <x:v>Canada</x:v>
       </x:c>
       <x:c r="E9" s="14" t="n">
-        <x:v>2023</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G9" s="45" t="n">
-        <x:v>201000000</x:v>
+        <x:v>1266567000</x:v>
       </x:c>
       <x:c r="H9" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>CAD</x:v>
       </x:c>
       <x:c r="I9" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.5787262745098</x:v>
       </x:c>
       <x:c r="J9" s="45" t="n">
-        <x:f>G9</x:f>
-        <x:v>201000000</x:v>
+        <x:f>G9/I9</x:f>
+        <x:v>802271438.9758753</x:v>
       </x:c>
       <x:c r="K9" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L9" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M9" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N9" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25.5" customHeight="1">
@@ -4145,44 +4264,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>DE-2024-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+        <x:v>NZ-2022-NOTIFIABLE-PRODUCT-REPORTED-REVENUE</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>substitutes_excise_receipts</x:v>
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>Germany</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E10" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G10" s="45" t="n">
-        <x:v>266000000</x:v>
+        <x:v>404000000</x:v>
       </x:c>
       <x:c r="H10" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I10" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.6582474708171</x:v>
       </x:c>
       <x:c r="J10" s="45" t="n">
-        <x:f>G10</x:f>
-        <x:v>266000000</x:v>
+        <x:f>G10/I10</x:f>
+        <x:v>243630704.7710613</x:v>
       </x:c>
       <x:c r="K10" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2022</x:v>
       </x:c>
       <x:c r="L10" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M10" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N10" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25.5" customHeight="1">
@@ -4190,44 +4309,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>DE-2025-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
+        <x:v>NZ-2023-NOTIFIABLE-PRODUCT-REPORTED-REVENUE-LOWER-BOUND</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>substitutes_excise_receipts</x:v>
+        <x:v>official_reported_revenue_mixed_supply_stages</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>Germany</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E11" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G11" s="45" t="n">
-        <x:v>404000000</x:v>
+        <x:v>374000000</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I11" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.762151372549</x:v>
       </x:c>
       <x:c r="J11" s="45" t="n">
-        <x:f>G11</x:f>
-        <x:v>404000000</x:v>
+        <x:f>G11/I11</x:f>
+        <x:v>212240563.33991262</x:v>
       </x:c>
       <x:c r="K11" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2023</x:v>
       </x:c>
       <x:c r="L11" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M11" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N11" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25.5" customHeight="1">
@@ -4235,44 +4354,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>NZ-2024-SPECIALIST-RETAIL-SALES-LOWER-BOUND</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>official_specialist_retail_sales_lower_bound</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>Finland</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E12" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G12" s="45" t="n">
-        <x:v>3540319</x:v>
+        <x:v>280000000</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I12" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J12" s="45" t="n">
-        <x:f>G12</x:f>
-        <x:v>3540319</x:v>
+        <x:f>G12/I12</x:f>
+        <x:v>156595276.14445302</x:v>
       </x:c>
       <x:c r="K12" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L12" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M12" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N12" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25.5" customHeight="1">
@@ -4280,38 +4399,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
+        <x:v>NZ-2024-SPECIALIST-RETAIL-PRODUCT-SALES-RAW-FILE-SUM</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>e_liquid_excise_amount</x:v>
+        <x:v>derived_official_workbook_sales_raw_sum</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E13" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G13" s="45" t="n">
-        <x:v>993100000</x:v>
+        <x:v>280684512.81</x:v>
       </x:c>
       <x:c r="H13" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I13" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J13" s="45" t="n">
         <x:f>G13/I13</x:f>
-        <x:v>234240611.54771507</x:v>
+        <x:v>156978102.83197576</x:v>
       </x:c>
       <x:c r="K13" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L13" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M13" s="14" t="str">
         <x:v>computed</x:v>
@@ -4325,38 +4444,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
+        <x:v>NZ-2024-IDENTIFIED-VAPING-PRODUCT-SALES-RAW-SUM</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>vaping_device_excise_amount</x:v>
+        <x:v>derived_identified_vaping_product_sales_raw_sum</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>New Zealand</x:v>
       </x:c>
       <x:c r="E14" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G14" s="45" t="n">
-        <x:v>175300000</x:v>
+        <x:v>274180410.21</x:v>
       </x:c>
       <x:c r="H14" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I14" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J14" s="45" t="n">
         <x:f>G14/I14</x:f>
-        <x:v>41347678.183782555</x:v>
+        <x:v>153340560.89369413</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L14" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M14" s="14" t="str">
         <x:v>computed</x:v>
@@ -4370,44 +4489,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
+        <x:v>EU-2023-EC-E-CIGARETTE-MARKET-BENCHMARK</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>vaping_component_sets_excise_amount</x:v>
+        <x:v>institutional_market_value_benchmark</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>European Union</x:v>
       </x:c>
       <x:c r="E15" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G15" s="45" t="n">
-        <x:v>2500000</x:v>
+        <x:v>4990000000</x:v>
       </x:c>
       <x:c r="H15" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I15" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J15" s="45" t="n">
-        <x:f>G15/I15</x:f>
-        <x:v>589670.2536192606</x:v>
+        <x:f>G15</x:f>
+        <x:v>4990000000</x:v>
       </x:c>
       <x:c r="K15" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L15" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M15" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N15" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25.5" customHeight="1">
@@ -4415,44 +4534,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>DE-2023-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>substitutes_excise_receipts</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>Sweden</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E16" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G16" s="45" t="n">
-        <x:v>80000000</x:v>
+        <x:v>201000000</x:v>
       </x:c>
       <x:c r="H16" s="45" t="str">
-        <x:v>SEK</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I16" s="45" t="n">
-        <x:v>11.432519140625</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J16" s="45" t="n">
-        <x:f>G16/I16</x:f>
-        <x:v>6997582.861306848</x:v>
+        <x:f>G16</x:f>
+        <x:v>201000000</x:v>
       </x:c>
       <x:c r="K16" s="14" t="str">
-        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L16" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M16" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N16" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25.5" customHeight="1">
@@ -4460,44 +4579,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>DE-2024-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>substitutes_excise_receipts</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E17" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G17" s="45" t="n">
-        <x:v>26000000000</x:v>
+        <x:v>266000000</x:v>
       </x:c>
       <x:c r="H17" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I17" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J17" s="45" t="n">
-        <x:f>G17/I17</x:f>
-        <x:v>23009192918.721367</x:v>
+        <x:f>G17</x:f>
+        <x:v>266000000</x:v>
       </x:c>
       <x:c r="K17" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L17" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M17" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N17" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25.5" customHeight="1">
@@ -4505,44 +4624,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
-        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>DE-2025-SUBSTITUTES-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>substitutes_excise_receipts</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E18" s="14" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G18" s="45" t="n">
-        <x:v>45700000000</x:v>
+        <x:v>404000000</x:v>
       </x:c>
       <x:c r="H18" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I18" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J18" s="45" t="n">
-        <x:f>G18/I18</x:f>
-        <x:v>40443081399.44486</x:v>
+        <x:f>G18</x:f>
+        <x:v>404000000</x:v>
       </x:c>
       <x:c r="K18" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L18" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M18" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N18" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25.5" customHeight="1">
@@ -4550,44 +4669,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Finland</x:v>
       </x:c>
       <x:c r="E19" s="14" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G19" s="45" t="n">
-        <x:v>46320000000</x:v>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="H19" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I19" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="45" t="n">
-        <x:f>G19/I19</x:f>
-        <x:v>40991762153.66052</x:v>
+        <x:f>G19</x:f>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L19" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M19" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N19" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25.5" customHeight="1">
@@ -4595,38 +4714,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_amount</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E20" s="14" t="n">
-        <x:v>2015</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G20" s="45" t="n">
-        <x:v>304170046</x:v>
+        <x:v>993100000</x:v>
       </x:c>
       <x:c r="H20" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I20" s="45" t="n">
-        <x:v>1.109512890625</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J20" s="45" t="n">
         <x:f>G20/I20</x:f>
-        <x:v>274147374.5552049</x:v>
+        <x:v>234240611.54771507</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L20" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M20" s="14" t="str">
         <x:v>computed</x:v>
@@ -4640,38 +4759,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaping_device_excise_amount</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E21" s="14" t="n">
-        <x:v>2016</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G21" s="45" t="n">
-        <x:v>485707484</x:v>
+        <x:v>175300000</x:v>
       </x:c>
       <x:c r="H21" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I21" s="45" t="n">
-        <x:v>1.1069031128405</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J21" s="45" t="n">
         <x:f>G21/I21</x:f>
-        <x:v>438798552.7961817</x:v>
+        <x:v>41347678.183782555</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L21" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M21" s="14" t="str">
         <x:v>computed</x:v>
@@ -4685,38 +4804,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaping_component_sets_excise_amount</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E22" s="14" t="n">
-        <x:v>2017</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G22" s="45" t="n">
-        <x:v>779836399</x:v>
+        <x:v>2500000</x:v>
       </x:c>
       <x:c r="H22" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I22" s="45" t="n">
-        <x:v>1.1296811764706</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J22" s="45" t="n">
         <x:f>G22/I22</x:f>
-        <x:v>690315475.943752</x:v>
+        <x:v>589670.2536192606</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L22" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M22" s="14" t="str">
         <x:v>computed</x:v>
@@ -4730,38 +4849,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Sweden</x:v>
       </x:c>
       <x:c r="E23" s="14" t="n">
-        <x:v>2018</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G23" s="45" t="n">
-        <x:v>2043703005</x:v>
+        <x:v>80000000</x:v>
       </x:c>
       <x:c r="H23" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>SEK</x:v>
       </x:c>
       <x:c r="I23" s="45" t="n">
-        <x:v>1.1809545098039</x:v>
+        <x:v>11.432519140625</x:v>
       </x:c>
       <x:c r="J23" s="45" t="n">
         <x:f>G23/I23</x:f>
-        <x:v>1730551844.3207107</x:v>
+        <x:v>6997582.861306848</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
+        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L23" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M23" s="14" t="str">
         <x:v>computed</x:v>
@@ -4775,38 +4894,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E24" s="14" t="n">
-        <x:v>2019</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G24" s="45" t="n">
-        <x:v>2702608307</x:v>
+        <x:v>26000000000</x:v>
       </x:c>
       <x:c r="H24" s="45" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="I24" s="45" t="n">
-        <x:v>1.1194745098039</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J24" s="45" t="n">
         <x:f>G24/I24</x:f>
-        <x:v>2414175832.796246</x:v>
+        <x:v>23009192918.721367</x:v>
       </x:c>
       <x:c r="K24" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L24" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M24" s="14" t="str">
         <x:v>computed</x:v>
@@ -4820,38 +4939,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E25" s="14" t="n">
-        <x:v>2020</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G25" s="45" t="n">
-        <x:v>2394423105</x:v>
+        <x:v>45700000000</x:v>
       </x:c>
       <x:c r="H25" s="45" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="I25" s="45" t="n">
-        <x:v>1.1421961089494</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J25" s="45" t="n">
         <x:f>G25/I25</x:f>
-        <x:v>2096332745.523365</x:v>
+        <x:v>40443081399.44486</x:v>
       </x:c>
       <x:c r="K25" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L25" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M25" s="14" t="str">
         <x:v>computed</x:v>
@@ -4865,38 +4984,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E26" s="14" t="n">
-        <x:v>2021</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G26" s="45" t="n">
-        <x:v>2763284338</x:v>
+        <x:v>46320000000</x:v>
       </x:c>
       <x:c r="H26" s="45" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="I26" s="45" t="n">
-        <x:v>1.1827403100775</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J26" s="45" t="n">
         <x:f>G26/I26</x:f>
-        <x:v>2336340711.866778</x:v>
+        <x:v>40991762153.66052</x:v>
       </x:c>
       <x:c r="K26" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L26" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M26" s="14" t="str">
         <x:v>computed</x:v>
@@ -4907,41 +5026,41 @@
     </x:row>
     <x:row r="27" ht="25.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>low.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E27" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G27" s="45" t="n">
-        <x:v>258327110.88</x:v>
+        <x:v>304170046</x:v>
       </x:c>
       <x:c r="H27" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I27" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.109512890625</x:v>
       </x:c>
       <x:c r="J27" s="45" t="n">
         <x:f>G27/I27</x:f>
-        <x:v>144474304.51375833</x:v>
+        <x:v>274147374.5552049</x:v>
       </x:c>
       <x:c r="K27" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
       </x:c>
       <x:c r="L27" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M27" s="14" t="str">
         <x:v>computed</x:v>
@@ -4952,41 +5071,41 @@
     </x:row>
     <x:row r="28" ht="25.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>low.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E28" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2016</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G28" s="45" t="n">
-        <x:v>275335272.8</x:v>
+        <x:v>485707484</x:v>
       </x:c>
       <x:c r="H28" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I28" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1069031128405</x:v>
       </x:c>
       <x:c r="J28" s="45" t="n">
         <x:f>G28/I28</x:f>
-        <x:v>153986439.55865824</x:v>
+        <x:v>438798552.7961817</x:v>
       </x:c>
       <x:c r="K28" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
       </x:c>
       <x:c r="L28" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M28" s="14" t="str">
         <x:v>computed</x:v>
@@ -4997,41 +5116,41 @@
     </x:row>
     <x:row r="29" ht="25.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>low.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E29" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G29" s="45" t="n">
-        <x:v>533662383.68</x:v>
+        <x:v>779836399</x:v>
       </x:c>
       <x:c r="H29" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I29" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1296811764706</x:v>
       </x:c>
       <x:c r="J29" s="45" t="n">
         <x:f>G29/I29</x:f>
-        <x:v>298460744.0724166</x:v>
+        <x:v>690315475.943752</x:v>
       </x:c>
       <x:c r="K29" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
       </x:c>
       <x:c r="L29" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M29" s="14" t="str">
         <x:v>computed</x:v>
@@ -5042,41 +5161,41 @@
     </x:row>
     <x:row r="30" ht="25.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>base.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E30" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G30" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>2043703005</x:v>
       </x:c>
       <x:c r="H30" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I30" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1809545098039</x:v>
       </x:c>
       <x:c r="J30" s="45" t="n">
         <x:f>G30/I30</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>1730551844.3207107</x:v>
       </x:c>
       <x:c r="K30" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
       </x:c>
       <x:c r="L30" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M30" s="14" t="str">
         <x:v>computed</x:v>
@@ -5087,41 +5206,41 @@
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>base.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E31" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G31" s="45" t="n">
-        <x:v>367631277.68</x:v>
+        <x:v>2702608307</x:v>
       </x:c>
       <x:c r="H31" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I31" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1194745098039</x:v>
       </x:c>
       <x:c r="J31" s="45" t="n">
         <x:f>G31/I31</x:f>
-        <x:v>205604719.4558489</x:v>
+        <x:v>2414175832.796246</x:v>
       </x:c>
       <x:c r="K31" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
       </x:c>
       <x:c r="L31" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M31" s="14" t="str">
         <x:v>computed</x:v>
@@ -5132,41 +5251,41 @@
     </x:row>
     <x:row r="32" ht="25.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>base.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E32" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G32" s="45" t="n">
-        <x:v>641811687.89</x:v>
+        <x:v>2394423105</x:v>
       </x:c>
       <x:c r="H32" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I32" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1421961089494</x:v>
       </x:c>
       <x:c r="J32" s="45" t="n">
         <x:f>G32/I32</x:f>
-        <x:v>358945280.34954304</x:v>
+        <x:v>2096332745.523365</x:v>
       </x:c>
       <x:c r="K32" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
       </x:c>
       <x:c r="L32" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M32" s="14" t="str">
         <x:v>computed</x:v>
@@ -5177,41 +5296,41 @@
     </x:row>
     <x:row r="33" ht="25.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>high.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E33" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G33" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>2763284338</x:v>
       </x:c>
       <x:c r="H33" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I33" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1827403100775</x:v>
       </x:c>
       <x:c r="J33" s="45" t="n">
         <x:f>G33/I33</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>2336340711.866778</x:v>
       </x:c>
       <x:c r="K33" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
       </x:c>
       <x:c r="L33" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M33" s="14" t="str">
         <x:v>computed</x:v>
@@ -5228,7 +5347,7 @@
         <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>high.generalRetailRpsNzd</x:v>
+        <x:v>low.specialistRetailNzd</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
         <x:v>New Zealand</x:v>
@@ -5240,7 +5359,7 @@
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G34" s="45" t="n">
-        <x:v>456995382.29</x:v>
+        <x:v>258327110.88</x:v>
       </x:c>
       <x:c r="H34" s="45" t="str">
         <x:v>NZD</x:v>
@@ -5250,7 +5369,7 @@
       </x:c>
       <x:c r="J34" s="45" t="n">
         <x:f>G34/I34</x:f>
-        <x:v>255583278.88015154</x:v>
+        <x:v>144474304.51375833</x:v>
       </x:c>
       <x:c r="K34" s="14" t="str">
         <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
@@ -5273,7 +5392,7 @@
         <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>high.combinedNzd</x:v>
+        <x:v>low.generalRetailRpsNzd</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
         <x:v>New Zealand</x:v>
@@ -5285,7 +5404,7 @@
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G35" s="45" t="n">
-        <x:v>731175792.5</x:v>
+        <x:v>275335272.8</x:v>
       </x:c>
       <x:c r="H35" s="45" t="str">
         <x:v>NZD</x:v>
@@ -5295,7 +5414,7 @@
       </x:c>
       <x:c r="J35" s="45" t="n">
         <x:f>G35/I35</x:f>
-        <x:v>408923839.7738457</x:v>
+        <x:v>153986439.55865824</x:v>
       </x:c>
       <x:c r="K35" s="14" t="str">
         <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
@@ -5312,137 +5431,452 @@
     </x:row>
     <x:row r="36" ht="25.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>scenario_component</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>low</x:v>
-      </x:c>
-      <x:c r="D36" s="14"/>
+        <x:v>low.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
       <x:c r="E36" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G36" s="45" t="n">
-        <x:v>667920000</x:v>
+        <x:v>533662383.68</x:v>
       </x:c>
       <x:c r="H36" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>NZD</x:v>
       </x:c>
       <x:c r="I36" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.788048828125</x:v>
       </x:c>
       <x:c r="J36" s="45" t="n">
-        <x:f>G36</x:f>
-        <x:v>667920000</x:v>
+        <x:f>G36/I36</x:f>
+        <x:v>298460744.0724166</x:v>
       </x:c>
       <x:c r="K36" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L36" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M36" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N36" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="25.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>scenario_component</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>central</x:v>
-      </x:c>
-      <x:c r="D37" s="14"/>
+        <x:v>base.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D37" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
       <x:c r="E37" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G37" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H37" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I37" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J37" s="45" t="n">
+        <x:f>G37/I37</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K37" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L37" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M37" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N37" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="25.5" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>base.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G38" s="45" t="n">
+        <x:v>367631277.68</x:v>
+      </x:c>
+      <x:c r="H38" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I38" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J38" s="45" t="n">
+        <x:f>G38/I38</x:f>
+        <x:v>205604719.4558489</x:v>
+      </x:c>
+      <x:c r="K38" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L38" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M38" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N38" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="25.5" customHeight="1">
+      <x:c r="A39" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B39" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C39" s="14" t="str">
+        <x:v>base.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D39" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E39" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F39" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G39" s="45" t="n">
+        <x:v>641811687.89</x:v>
+      </x:c>
+      <x:c r="H39" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I39" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J39" s="45" t="n">
+        <x:f>G39/I39</x:f>
+        <x:v>358945280.34954304</x:v>
+      </x:c>
+      <x:c r="K39" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L39" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M39" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N39" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="25.5" customHeight="1">
+      <x:c r="A40" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B40" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C40" s="14" t="str">
+        <x:v>high.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D40" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E40" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F40" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G40" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H40" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I40" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J40" s="45" t="n">
+        <x:f>G40/I40</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K40" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L40" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M40" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N40" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="25.5" customHeight="1">
+      <x:c r="A41" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B41" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C41" s="14" t="str">
+        <x:v>high.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D41" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E41" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F41" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G41" s="45" t="n">
+        <x:v>456995382.29</x:v>
+      </x:c>
+      <x:c r="H41" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I41" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J41" s="45" t="n">
+        <x:f>G41/I41</x:f>
+        <x:v>255583278.88015154</x:v>
+      </x:c>
+      <x:c r="K41" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L41" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M41" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N41" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="25.5" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>high.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D42" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E42" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G42" s="45" t="n">
+        <x:v>731175792.5</x:v>
+      </x:c>
+      <x:c r="H42" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I42" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J42" s="45" t="n">
+        <x:f>G42/I42</x:f>
+        <x:v>408923839.7738457</x:v>
+      </x:c>
+      <x:c r="K42" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L42" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M42" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N42" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="25.5" customHeight="1">
+      <x:c r="A43" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B43" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C43" s="14" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="D43" s="14"/>
+      <x:c r="E43" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F43" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G43" s="45" t="n">
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="H43" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I43" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J43" s="45" t="n">
+        <x:f>G43</x:f>
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="K43" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L43" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M43" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N43" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="25.5" customHeight="1">
+      <x:c r="A44" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B44" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C44" s="14" t="str">
+        <x:v>central</x:v>
+      </x:c>
+      <x:c r="D44" s="14"/>
+      <x:c r="E44" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F44" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G44" s="45" t="n">
         <x:v>1199220000</x:v>
       </x:c>
-      <x:c r="H37" s="45" t="str">
+      <x:c r="H44" s="45" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="I37" s="45" t="n">
+      <x:c r="I44" s="45" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J37" s="45" t="n">
-        <x:f>G37</x:f>
+      <x:c r="J44" s="45" t="n">
+        <x:f>G44</x:f>
         <x:v>1199220000</x:v>
       </x:c>
-      <x:c r="K37" s="14" t="str">
+      <x:c r="K44" s="14" t="str">
         <x:v>EUR-IDENTITY</x:v>
       </x:c>
-      <x:c r="L37" s="14" t="str">
+      <x:c r="L44" s="14" t="str">
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
-      <x:c r="M37" s="14" t="str">
+      <x:c r="M44" s="14" t="str">
         <x:v>already_eur</x:v>
       </x:c>
-      <x:c r="N37" s="14" t="str">
+      <x:c r="N44" s="14" t="str">
         <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="25.5" customHeight="1">
-      <x:c r="A38" s="15" t="str">
+    <x:row r="45" ht="25.5" customHeight="1">
+      <x:c r="A45" s="15" t="str">
         <x:v>model</x:v>
       </x:c>
-      <x:c r="B38" s="15" t="str">
+      <x:c r="B45" s="15" t="str">
         <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
       </x:c>
-      <x:c r="C38" s="15" t="str">
+      <x:c r="C45" s="15" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="D38" s="15"/>
-      <x:c r="E38" s="15" t="n">
+      <x:c r="D45" s="15"/>
+      <x:c r="E45" s="15" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="F38" s="15" t="str">
+      <x:c r="F45" s="15" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
-      <x:c r="G38" s="46" t="n">
+      <x:c r="G45" s="46" t="n">
         <x:v>1654620000</x:v>
       </x:c>
-      <x:c r="H38" s="46" t="str">
+      <x:c r="H45" s="46" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="I38" s="46" t="n">
+      <x:c r="I45" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J38" s="46" t="n">
-        <x:f>G38</x:f>
+      <x:c r="J45" s="46" t="n">
+        <x:f>G45</x:f>
         <x:v>1654620000</x:v>
       </x:c>
-      <x:c r="K38" s="15" t="str">
+      <x:c r="K45" s="15" t="str">
         <x:v>EUR-IDENTITY</x:v>
       </x:c>
-      <x:c r="L38" s="15" t="str">
+      <x:c r="L45" s="15" t="str">
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
-      <x:c r="M38" s="15" t="str">
+      <x:c r="M45" s="15" t="str">
         <x:v>already_eur</x:v>
       </x:c>
-      <x:c r="N38" s="15" t="str">
+      <x:c r="N45" s="15" t="str">
         <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a0407373924926"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0554f810ee9045e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish global authority research model v20
Add the reviewed v20 site, data, controls and bilingual artifacts. Workflow hardening is applied separately through the connected GitHub app.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R0be318fc6c234b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7a21837fe5764959"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1da2b31e28be48eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R39e5335d567a405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re44a4e909c2a433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rbc42c5172dd849d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R86c75d4d236440d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rce27412c960e466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra45e6db52b454fe5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R980c80a7b6634e8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb43a70f44cfa4102"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4063c20108204ca2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-19</x:v>
+        <x:v>2026.07.24-20</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R362dc33430c844c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red9df98f696f41ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3830,7 +3830,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeb72f7eb4cb42f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9674ee543d274d2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5876,7 +5876,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0554f810ee9045e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8943a9486c4b4df5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Euromonitor access clarification v21
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rbc42c5172dd849d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R86c75d4d236440d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rce27412c960e466f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra45e6db52b454fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R980c80a7b6634e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R95fdfb05d5d94552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R951205ed14ec41d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R039dc2bc096542f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf39efc4bd9d34f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R867df7e18c004fe7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4063c20108204ca2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re960c0ee9b574839"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-20</x:v>
+        <x:v>2026.07.24-21</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red9df98f696f41ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07dccd85e5174d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3830,7 +3830,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9674ee543d274d2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11e9892f8cd423f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5876,7 +5876,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8943a9486c4b4df5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553c37f21fd44196"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Sweden official structure evidence
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R95fdfb05d5d94552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R951205ed14ec41d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R039dc2bc096542f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf39efc4bd9d34f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R867df7e18c004fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Raece48a4250945a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8dcb78c39cbd450c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R0e1112c9416844e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R2c5de709e5b04675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re8ab7f83b8db4ad4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -870,13 +870,13 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public package contains 34 annual observations sourced from official routes across seven countries.</x:v>
+        <x:v>The public market dataset contains 79 observations from 21 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The countries are Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. Transaction levels, currencies and product scopes differ.</x:v>
+        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
@@ -885,10 +885,10 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Count of annual observations whose evidenceStatus begins official_.</x:v>
+        <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>Official publication does not make the metrics automatically comparable.</x:v>
+        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
@@ -1392,31 +1392,31 @@
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 34 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>Observed retail value and device data are required.</x:v>
+        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58.5" customHeight="1">
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re960c0ee9b574839"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf643be6281f7427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-21</x:v>
+        <x:v>2026.07.24-22</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07dccd85e5174d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d14286da2f4aee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3744,16 +3744,16 @@
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C75" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3761,7 +3761,7 @@
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -3770,7 +3770,7 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3778,16 +3778,16 @@
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3795,7 +3795,7 @@
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -3804,33 +3804,50 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E78" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="31.5" customHeight="1">
+      <x:c r="A79" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B79" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C79" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D79" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
-      <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="31.5" customHeight="1">
-      <x:c r="A79" s="15" t="str">
+      <x:c r="E79" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="31.5" customHeight="1">
+      <x:c r="A80" s="15" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B79" s="15" t="str">
+      <x:c r="B80" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C79" s="15" t="str">
+      <x:c r="C80" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D79" s="15" t="str">
+      <x:c r="D80" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E79" s="15" t="str">
+      <x:c r="E80" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11e9892f8cd423f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8b171022fe4227"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5876,7 +5893,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553c37f21fd44196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d77a457b99c4894"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Sweden official registration-structure evidence (#20)
Publish Sweden's official 2018–2026 registration-structure series with explicit non-sales boundaries, streamline the bilingual bank package to 6- and 30-slide decks, and retain both Evidence Registers.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R95fdfb05d5d94552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R951205ed14ec41d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R039dc2bc096542f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf39efc4bd9d34f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R867df7e18c004fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Raece48a4250945a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8dcb78c39cbd450c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R0e1112c9416844e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R2c5de709e5b04675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re8ab7f83b8db4ad4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -870,13 +870,13 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public package contains 34 annual observations sourced from official routes across seven countries.</x:v>
+        <x:v>The public market dataset contains 79 observations from 21 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The countries are Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. Transaction levels, currencies and product scopes differ.</x:v>
+        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
@@ -885,10 +885,10 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Count of annual observations whose evidenceStatus begins official_.</x:v>
+        <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>Official publication does not make the metrics automatically comparable.</x:v>
+        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
@@ -1392,31 +1392,31 @@
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024.</x:v>
+        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>Table 7.5 reports a rounded official amount. It covers nicotine liquid only, excludes devices and nicotine-free liquid, and is not retail value.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Direct use of the calculation basis stated by the government.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 34 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>Observed retail value and device data are required.</x:v>
+        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58.5" customHeight="1">
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re960c0ee9b574839"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf643be6281f7427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-21</x:v>
+        <x:v>2026.07.24-22</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07dccd85e5174d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d14286da2f4aee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3744,16 +3744,16 @@
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C75" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3761,7 +3761,7 @@
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -3770,7 +3770,7 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3778,16 +3778,16 @@
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
         <x:v>2026-07-24</x:v>
@@ -3795,7 +3795,7 @@
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -3804,33 +3804,50 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E78" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="31.5" customHeight="1">
+      <x:c r="A79" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B79" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C79" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D79" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
-      <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="31.5" customHeight="1">
-      <x:c r="A79" s="15" t="str">
+      <x:c r="E79" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="31.5" customHeight="1">
+      <x:c r="A80" s="15" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B79" s="15" t="str">
+      <x:c r="B80" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C79" s="15" t="str">
+      <x:c r="C80" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D79" s="15" t="str">
+      <x:c r="D80" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E79" s="15" t="str">
+      <x:c r="E80" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11e9892f8cd423f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8b171022fe4227"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5876,7 +5893,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553c37f21fd44196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d77a457b99c4894"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Canada donor closure and review package v24
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Raece48a4250945a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8dcb78c39cbd450c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R0e1112c9416844e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R2c5de709e5b04675"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re8ab7f83b8db4ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R69cd4a64dde34936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re1f4d6b8847f4c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R14c2612c96254fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R8e70da967504452d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rd7df7921307f4b80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -1160,60 +1160,60 @@
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Statistics Canada's Canada series contains seven full-year consumer-retail estimates for 2019–2025; the 2024 value is CAD 1,219,160,000.</x:v>
+        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>The annual estimate is the sum of four RCS quarters for NAPCS 5619122. Health Canada's 2024 manufacturer/importer shipment value is CAD 1,160,753,796.78.</x:v>
+        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_RCS_2019_2025_RETAIL_SALES.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>CAD 1,219,160,000 − CAD 1,160,753,796.78 = CAD 58,406,203.22; RCS / Health Canada = 1.0503175, or +5.03%.</x:v>
+        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>Every 2024 quarter carries quality flag E. Vaping-specific channel completeness is not quantified and the vaping-excise basis is not confirmed.</x:v>
+        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>The retail-to-shipment bridge does not yet explain margin, inventory, returns, timing, product scope or tax treatment; Canada is not an accepted donor.</x:v>
+        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
+        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
+        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Sum of the reported liquid-containing product categories.</x:v>
+        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Physical volume is not treated as market value.</x:v>
+        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
+        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf643be6281f7427c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2278f6b81af459e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-22</x:v>
+        <x:v>2026.07.25-24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2224,7 +2224,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d14286da2f4aee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R913e8a2c347d4bca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3382,7 +3382,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3399,7 +3399,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3416,7 +3416,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3433,7 +3433,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3450,7 +3450,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3467,7 +3467,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3484,7 +3484,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3501,7 +3501,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3518,7 +3518,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3552,7 +3552,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3569,7 +3569,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3586,7 +3586,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3603,7 +3603,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3620,7 +3620,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3637,7 +3637,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3654,7 +3654,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3671,7 +3671,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3688,7 +3688,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3705,7 +3705,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3722,63 +3722,63 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C74" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C75" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C76" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -3787,32 +3787,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -3821,33 +3821,67 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E79" s="14" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="31.5" customHeight="1">
+      <x:c r="A80" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B80" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C80" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D80" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
-      <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="31.5" customHeight="1">
-      <x:c r="A80" s="15" t="str">
+      <x:c r="E80" s="14" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="31.5" customHeight="1">
+      <x:c r="A81" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B80" s="15" t="str">
+      <x:c r="B81" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C80" s="15" t="str">
+      <x:c r="C81" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D80" s="15" t="str">
+      <x:c r="D81" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E80" s="15" t="str">
-        <x:v>2026-07-24</x:v>
+      <x:c r="E81" s="14" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="31.5" customHeight="1">
+      <x:c r="A82" s="15" t="str">
+        <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
+      </x:c>
+      <x:c r="B82" s="15" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C82" s="15" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D82" s="15" t="str">
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
+      </x:c>
+      <x:c r="E82" s="15" t="str">
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8b171022fe4227"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re08668c3321e412e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5893,7 +5927,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d77a457b99c4894"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323c4a23f66d4d37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Canada donor closure and review package v24 (#21)
Canada remains outside the accepted donor count at 7/10, with D5, D7 and D10 open. Refresh the bilingual review package, evidence registers, procurement controls and downloadable manifest while keeping the global estimate fail-closed.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Raece48a4250945a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8dcb78c39cbd450c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R0e1112c9416844e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R2c5de709e5b04675"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re8ab7f83b8db4ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R69cd4a64dde34936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re1f4d6b8847f4c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R14c2612c96254fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R8e70da967504452d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rd7df7921307f4b80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -1160,60 +1160,60 @@
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Statistics Canada's Canada series contains seven full-year consumer-retail estimates for 2019–2025; the 2024 value is CAD 1,219,160,000.</x:v>
+        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>The annual estimate is the sum of four RCS quarters for NAPCS 5619122. Health Canada's 2024 manufacturer/importer shipment value is CAD 1,160,753,796.78.</x:v>
+        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_RCS_2019_2025_RETAIL_SALES.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>CAD 1,219,160,000 − CAD 1,160,753,796.78 = CAD 58,406,203.22; RCS / Health Canada = 1.0503175, or +5.03%.</x:v>
+        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>Every 2024 quarter carries quality flag E. Vaping-specific channel completeness is not quantified and the vaping-excise basis is not confirmed.</x:v>
+        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>The retail-to-shipment bridge does not yet explain margin, inventory, returns, timing, product scope or tax treatment; Canada is not an accepted donor.</x:v>
+        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Canada's 2024 shipments included 1,251,843 litres.</x:v>
+        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>The total covers the reported vaporisable-substance categories. It is a physical volume, not a retail market value.</x:v>
+        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Sum of the reported liquid-containing product categories.</x:v>
+        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Physical volume is not treated as market value.</x:v>
+        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Product mix, average price and retail-channel evidence are required.</x:v>
+        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf643be6281f7427c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2278f6b81af459e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.24-22</x:v>
+        <x:v>2026.07.25-24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2224,7 +2224,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d14286da2f4aee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R913e8a2c347d4bca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3382,7 +3382,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3399,7 +3399,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3416,7 +3416,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3433,7 +3433,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3450,7 +3450,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3467,7 +3467,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3484,7 +3484,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3501,7 +3501,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3518,7 +3518,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3552,7 +3552,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3569,7 +3569,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3586,7 +3586,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3603,7 +3603,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3620,7 +3620,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3637,7 +3637,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3654,7 +3654,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3671,7 +3671,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3688,7 +3688,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3705,7 +3705,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3722,63 +3722,63 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C74" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C75" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C76" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -3787,32 +3787,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -3821,33 +3821,67 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E79" s="14" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="31.5" customHeight="1">
+      <x:c r="A80" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B80" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C80" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D80" s="14" t="str">
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
-      <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="31.5" customHeight="1">
-      <x:c r="A80" s="15" t="str">
+      <x:c r="E80" s="14" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="31.5" customHeight="1">
+      <x:c r="A81" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B80" s="15" t="str">
+      <x:c r="B81" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C80" s="15" t="str">
+      <x:c r="C81" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D80" s="15" t="str">
+      <x:c r="D81" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E80" s="15" t="str">
-        <x:v>2026-07-24</x:v>
+      <x:c r="E81" s="14" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="31.5" customHeight="1">
+      <x:c r="A82" s="15" t="str">
+        <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
+      </x:c>
+      <x:c r="B82" s="15" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C82" s="15" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D82" s="15" t="str">
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
+      </x:c>
+      <x:c r="E82" s="15" t="str">
+        <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8b171022fe4227"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re08668c3321e412e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5893,7 +5927,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d77a457b99c4894"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323c4a23f66d4d37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish New Zealand donor closure and v25 package
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R69cd4a64dde34936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re1f4d6b8847f4c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R14c2612c96254fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R8e70da967504452d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rd7df7921307f4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rf21ee583af494152"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rfeb12b565ded4f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3bd7d98170bf4aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc5f3db670fe342e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R1594c7c51cbe4836"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public market dataset contains 79 observations from 21 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The public market dataset contains 79 observations from 23 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
@@ -882,7 +882,7 @@
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
         <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
@@ -911,7 +911,7 @@
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
         <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
@@ -984,38 +984,38 @@
         <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="58.5" customHeight="1">
+    <x:row r="15" ht="93" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>A conservative text classification identifies NZD 274,180,410.21 as New Zealand 2024 vaping-product-row raw sales.</x:v>
+        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>NZD 2,137,085.24 is identified as adjacent notifiable products and NZD 4,367,017.37 as unresolved product type. The vaping exact-row-de-duplication sensitivity is NZD 258,327,110.88, but it is not a corrected estimate.</x:v>
+        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F15" s="14" t="str">
-        <x:v>Conservative Product type text classification of product rows in the official XLSX files; classification and repeated-row sensitivities are reported separately.</x:v>
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="F15" s="17" t="str">
+        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>Product-type corruption and unresolved rows prevent interpretation as a complete vaping market.</x:v>
+        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>Obtain the authority's product-code dictionary, repeat-row semantics, complete channel coverage and GST basis. The figure is not donor-eligible.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="93" customHeight="1">
+        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58.5" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>New Zealand's supported 2024 identified-vaping retail sensitivity is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
@@ -1024,12 +1024,12 @@
         <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F16" s="17" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
         <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
@@ -1056,7 +1056,7 @@
         <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
         <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
@@ -1114,7 +1114,7 @@
         <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
         <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
@@ -2100,7 +2100,7 @@
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
         <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2278f6b81af459e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf296d8b52614dce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.25-24</x:v>
+        <x:v>2026.07.26-25</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2224,7 +2224,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R913e8a2c347d4bca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde2b98a000934d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3382,7 +3382,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3399,7 +3399,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3416,7 +3416,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3433,7 +3433,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3450,7 +3450,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3467,7 +3467,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3484,7 +3484,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3501,7 +3501,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3518,7 +3518,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3552,7 +3552,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3569,7 +3569,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3586,7 +3586,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3603,7 +3603,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3620,7 +3620,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3637,7 +3637,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3654,7 +3654,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3671,7 +3671,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3688,7 +3688,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3705,7 +3705,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3722,7 +3722,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3739,7 +3739,7 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3756,7 +3756,7 @@
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3773,7 +3773,7 @@
         <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3790,7 +3790,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -3807,81 +3807,115 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B81" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C81" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D81" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E81" s="14" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="31.5" customHeight="1">
+      <x:c r="A82" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B82" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C82" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D82" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E82" s="14" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="31.5" customHeight="1">
+      <x:c r="A83" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B81" s="14" t="str">
+      <x:c r="B83" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C81" s="14" t="str">
+      <x:c r="C83" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D81" s="14" t="str">
+      <x:c r="D83" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="31.5" customHeight="1">
-      <x:c r="A82" s="15" t="str">
+      <x:c r="E83" s="14" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="31.5" customHeight="1">
+      <x:c r="A84" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B82" s="15" t="str">
+      <x:c r="B84" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C82" s="15" t="str">
+      <x:c r="C84" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D82" s="15" t="str">
+      <x:c r="D84" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E82" s="15" t="str">
-        <x:v>2026-07-25</x:v>
+      <x:c r="E84" s="15" t="str">
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re08668c3321e412e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeb896f37267429d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5927,7 +5961,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323c4a23f66d4d37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09ec33bfc42a4320"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish New Zealand donor closure and v25 package (#22)
Add a deterministic privacy-safe reconstruction of New Zealand's 29 official 2024 annual-return workbooks, publish the identified AIS/AVP vaping subtotal and donor-closure controls, and refresh the bilingual v25 dashboard, decks and Evidence Registers.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R69cd4a64dde34936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re1f4d6b8847f4c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R14c2612c96254fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R8e70da967504452d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rd7df7921307f4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rf21ee583af494152"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rfeb12b565ded4f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3bd7d98170bf4aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc5f3db670fe342e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R1594c7c51cbe4836"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public market dataset contains 79 observations from 21 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The public market dataset contains 79 observations from 23 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
@@ -882,7 +882,7 @@
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
         <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
@@ -911,7 +911,7 @@
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
         <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
@@ -984,38 +984,38 @@
         <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="58.5" customHeight="1">
+    <x:row r="15" ht="93" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>A conservative text classification identifies NZD 274,180,410.21 as New Zealand 2024 vaping-product-row raw sales.</x:v>
+        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>NZD 2,137,085.24 is identified as adjacent notifiable products and NZD 4,367,017.37 as unresolved product type. The vaping exact-row-de-duplication sensitivity is NZD 258,327,110.88, but it is not a corrected estimate.</x:v>
+        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F15" s="14" t="str">
-        <x:v>Conservative Product type text classification of product rows in the official XLSX files; classification and repeated-row sensitivities are reported separately.</x:v>
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="F15" s="17" t="str">
+        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>Product-type corruption and unresolved rows prevent interpretation as a complete vaping market.</x:v>
+        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>Obtain the authority's product-code dictionary, repeat-row semantics, complete channel coverage and GST basis. The figure is not donor-eligible.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="93" customHeight="1">
+        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58.5" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>New Zealand's supported 2024 identified-vaping retail sensitivity is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
@@ -1024,12 +1024,12 @@
         <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2026-07-24</x:v>
-      </x:c>
-      <x:c r="F16" s="17" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
         <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
@@ -1056,7 +1056,7 @@
         <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
         <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
@@ -1114,7 +1114,7 @@
         <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
         <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
@@ -2100,7 +2100,7 @@
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
         <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2278f6b81af459e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf296d8b52614dce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.25-24</x:v>
+        <x:v>2026.07.26-25</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2224,7 +2224,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R913e8a2c347d4bca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde2b98a000934d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3382,7 +3382,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3399,7 +3399,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3416,7 +3416,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3433,7 +3433,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3450,7 +3450,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3467,7 +3467,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3484,7 +3484,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3501,7 +3501,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3518,7 +3518,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3552,7 +3552,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3569,7 +3569,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3586,7 +3586,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3603,7 +3603,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3620,7 +3620,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3637,7 +3637,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3654,7 +3654,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3671,7 +3671,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3688,7 +3688,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3705,7 +3705,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3722,7 +3722,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3739,7 +3739,7 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3756,7 +3756,7 @@
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3773,7 +3773,7 @@
         <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3790,7 +3790,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -3807,81 +3807,115 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B81" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C81" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D81" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E81" s="14" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="31.5" customHeight="1">
+      <x:c r="A82" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B82" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C82" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D82" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E82" s="14" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="31.5" customHeight="1">
+      <x:c r="A83" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B81" s="14" t="str">
+      <x:c r="B83" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C81" s="14" t="str">
+      <x:c r="C83" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D81" s="14" t="str">
+      <x:c r="D83" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="31.5" customHeight="1">
-      <x:c r="A82" s="15" t="str">
+      <x:c r="E83" s="14" t="str">
+        <x:v>2026-07-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="31.5" customHeight="1">
+      <x:c r="A84" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B82" s="15" t="str">
+      <x:c r="B84" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C82" s="15" t="str">
+      <x:c r="C84" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D82" s="15" t="str">
+      <x:c r="D84" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E82" s="15" t="str">
-        <x:v>2026-07-25</x:v>
+      <x:c r="E84" s="15" t="str">
+        <x:v>2026-07-26</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re08668c3321e412e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeb896f37267429d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5927,7 +5961,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323c4a23f66d4d37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09ec33bfc42a4320"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v26 first-donor conversion sprint
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rf21ee583af494152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rfeb12b565ded4f1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3bd7d98170bf4aa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc5f3db670fe342e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R1594c7c51cbe4836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R2878885e8db54fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R59b338c037d34dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3ac4acbedbe3415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rbf3c3ff913f54346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re56da785515a4b7c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -882,7 +882,7 @@
         <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
         <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
@@ -911,7 +911,7 @@
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
         <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
@@ -995,10 +995,10 @@
         <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F15" s="17" t="str">
         <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
@@ -1111,10 +1111,10 @@
         <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/country-scenarios.json</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
         <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
@@ -1169,10 +1169,10 @@
         <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
         <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
@@ -2100,7 +2100,7 @@
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
         <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf296d8b52614dce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1cb0c6dcdb4422"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.26-25</x:v>
+        <x:v>2026.07.27-26</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2224,7 +2224,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde2b98a000934d92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5eac6d7b97d147b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3382,7 +3382,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3399,7 +3399,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3416,7 +3416,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3433,7 +3433,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3450,7 +3450,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3467,7 +3467,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3484,7 +3484,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3501,7 +3501,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3518,7 +3518,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3552,7 +3552,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3569,7 +3569,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3586,7 +3586,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3603,7 +3603,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3620,7 +3620,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3637,7 +3637,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3654,7 +3654,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3671,7 +3671,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3688,7 +3688,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3705,7 +3705,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3722,7 +3722,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3739,7 +3739,7 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3756,7 +3756,7 @@
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3773,7 +3773,7 @@
         <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3790,7 +3790,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -3807,7 +3807,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
@@ -3824,7 +3824,7 @@
         <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
@@ -3841,7 +3841,7 @@
         <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
@@ -3858,7 +3858,7 @@
         <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
@@ -3875,7 +3875,7 @@
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
@@ -3892,7 +3892,7 @@
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
@@ -3909,13 +3909,13 @@
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
       <x:c r="E84" s="15" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeb896f37267429d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc80c1d2869c42d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5961,7 +5961,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09ec33bfc42a4320"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90757052d7854dfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v27 global base and Poland reconstruction
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R2878885e8db54fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R59b338c037d34dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3ac4acbedbe3415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rbf3c3ff913f54346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re56da785515a4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7ddec210892e4a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5665e4e2128f42ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R8f338aa557ba4d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R49a48d73a8b04ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6e68c0fc9aec4ba8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -841,36 +841,36 @@
     </x:row>
     <x:row r="10" ht="58.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>The public atlas contains a fixed research universe of 195 countries.</x:v>
+        <x:v>The public 195-country open base contains 578 observed World Bank records; it contains zero vaping retail-sales observations.</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
         <x:v>Market scope</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>countryCount = 195; universe = UN193+VA+PS.</x:v>
+        <x:v>Population and population ages 15–64 each cover 194/195 countries. GDP per capita covers 190/195 countries, and all 190 observations have a EUR equivalent calculated with the ECB rate for the same source year. WHO and UN Comtrade routes are queued and missing for 195/195 countries, not zero.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states ; https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>site/data/global-base-layer.json ; site/data/global-base-layer.csv ; https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures ; https://www.un.org/en/about-us/member-states ; https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>193 UN Member States + Holy See + State of Palestine.</x:v>
+        <x:v>For each World Bank series, the latest non-null observation from 2020–2024 is selected and its real source year is retained. USD per person is divided only by the ECB rate for that same source year.</x:v>
       </x:c>
       <x:c r="G10" s="14" t="str">
-        <x:v>The research frame is not evidence of proven market coverage.</x:v>
+        <x:v>Population, GDP, user prevalence and trade flows are context or proxy measures, not vaping sales values.</x:v>
       </x:c>
       <x:c r="H10" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I10" s="14" t="str">
-        <x:v>There is no gap in the universe definition; evidence coverage is assessed separately.</x:v>
+        <x:v>Annual country device and e-liquid sales values, numeric WHO extraction and validation of the UN Comtrade classification remain missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public market dataset contains 79 observations from 23 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
@@ -885,7 +885,7 @@
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
         <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
@@ -1334,60 +1334,60 @@
     </x:row>
     <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Poland reported 805,441 litres in 2023.</x:v>
+        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
+        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
         <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2020–2023</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
+        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>A newer series and observed retail value are required.</x:v>
+        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
+        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>The tax amount is not treated as retail value.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>Finality and reconciliation to the tax base are required.</x:v>
+        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
@@ -1407,7 +1407,7 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 34 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
         <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1cb0c6dcdb4422"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb271c2d9100e4bd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-26</x:v>
+        <x:v>2026.07.27-27</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2257,7 +2257,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2266,7 +2266,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5eac6d7b97d147b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee8f348dc7f4143"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3693,7 +3693,7 @@
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
       <x:c r="A72" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
       </x:c>
       <x:c r="B72" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3702,7 +3702,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D72" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3710,16 +3710,16 @@
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
       <x:c r="A73" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
       </x:c>
       <x:c r="B73" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C73" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D73" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3727,16 +3727,16 @@
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C74" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3744,16 +3744,16 @@
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C75" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3761,16 +3761,16 @@
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>data.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C76" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3778,16 +3778,16 @@
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>datahelpdesk.worldbank.org</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3795,16 +3795,16 @@
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3812,16 +3812,16 @@
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3829,16 +3829,16 @@
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3846,16 +3846,16 @@
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3863,16 +3863,16 @@
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3880,42 +3880,127 @@
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>www150.statcan.gc.ca</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
-      <x:c r="A84" s="15" t="str">
+      <x:c r="A84" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+      </x:c>
+      <x:c r="B84" s="14" t="str">
+        <x:v>health.govt.nz</x:v>
+      </x:c>
+      <x:c r="C84" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D84" s="14" t="str">
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+      </x:c>
+      <x:c r="E84" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="31.5" customHeight="1">
+      <x:c r="A85" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+      </x:c>
+      <x:c r="B85" s="14" t="str">
+        <x:v>podatki.gov.pl</x:v>
+      </x:c>
+      <x:c r="C85" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D85" s="14" t="str">
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+      </x:c>
+      <x:c r="E85" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="31.5" customHeight="1">
+      <x:c r="A86" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B86" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C86" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D86" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E86" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="31.5" customHeight="1">
+      <x:c r="A87" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B87" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C87" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D87" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E87" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="31.5" customHeight="1">
+      <x:c r="A88" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+      </x:c>
+      <x:c r="B88" s="14" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C88" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D88" s="14" t="str">
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
+      </x:c>
+      <x:c r="E88" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="31.5" customHeight="1">
+      <x:c r="A89" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B84" s="15" t="str">
+      <x:c r="B89" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C84" s="15" t="str">
+      <x:c r="C89" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D84" s="15" t="str">
+      <x:c r="D89" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E84" s="15" t="str">
+      <x:c r="E89" s="15" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc80c1d2869c42d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41244762c5e4ff1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5961,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90757052d7854dfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ea52fdda224042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v27 global base and Poland reconstruction (#24)
Adds the 195-country open-data base, Poland official-flow reconstruction, privacy-safe vendor and customs response state, and refreshed bilingual lender artifacts with deterministic validation.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R2878885e8db54fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R59b338c037d34dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R3ac4acbedbe3415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rbf3c3ff913f54346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Re56da785515a4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7ddec210892e4a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5665e4e2128f42ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R8f338aa557ba4d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R49a48d73a8b04ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6e68c0fc9aec4ba8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -841,36 +841,36 @@
     </x:row>
     <x:row r="10" ht="58.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>The public atlas contains a fixed research universe of 195 countries.</x:v>
+        <x:v>The public 195-country open base contains 578 observed World Bank records; it contains zero vaping retail-sales observations.</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
         <x:v>Market scope</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>countryCount = 195; universe = UN193+VA+PS.</x:v>
+        <x:v>Population and population ages 15–64 each cover 194/195 countries. GDP per capita covers 190/195 countries, and all 190 observations have a EUR equivalent calculated with the ECB rate for the same source year. WHO and UN Comtrade routes are queued and missing for 195/195 countries, not zero.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states ; https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>site/data/global-base-layer.json ; site/data/global-base-layer.csv ; https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures ; https://www.un.org/en/about-us/member-states ; https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>193 UN Member States + Holy See + State of Palestine.</x:v>
+        <x:v>For each World Bank series, the latest non-null observation from 2020–2024 is selected and its real source year is retained. USD per person is divided only by the ECB rate for that same source year.</x:v>
       </x:c>
       <x:c r="G10" s="14" t="str">
-        <x:v>The research frame is not evidence of proven market coverage.</x:v>
+        <x:v>Population, GDP, user prevalence and trade flows are context or proxy measures, not vaping sales values.</x:v>
       </x:c>
       <x:c r="H10" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I10" s="14" t="str">
-        <x:v>There is no gap in the universe definition; evidence coverage is assessed separately.</x:v>
+        <x:v>Annual country device and e-liquid sales values, numeric WHO extraction and validation of the UN Comtrade classification remain missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public market dataset contains 79 observations from 23 sources; its 70 official observations split into 34 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market size</x:v>
@@ -885,7 +885,7 @@
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>79 = 43 prior observations + 36 FHM structure counts; 70 official = 34 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
         <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
@@ -1334,60 +1334,60 @@
     </x:row>
     <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Poland reported 805,441 litres in 2023.</x:v>
+        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>The official parliamentary response reports a physical volume. It excludes devices and is not an observed retail value.</x:v>
+        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
         <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2020–2023</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Coverage is interpreted within the limitations stated in the original response.</x:v>
+        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>A newer series and observed retail value are required.</x:v>
+        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Poland reported PLN 993.1 million in e-liquid excise receipts for 2025.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The official parliamentary response reports a tax amount, not sales or retail value. The amount is separate from devices and parts.</x:v>
+        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Direct use of the amount reported in the official response.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>The tax amount is not treated as retail value.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>Finality and reconciliation to the tax base are required.</x:v>
+        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
@@ -1407,7 +1407,7 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 34 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
         <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc1cb0c6dcdb4422"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb271c2d9100e4bd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-26</x:v>
+        <x:v>2026.07.27-27</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2257,7 +2257,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2266,7 +2266,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5eac6d7b97d147b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee8f348dc7f4143"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3693,7 +3693,7 @@
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
       <x:c r="A72" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
       </x:c>
       <x:c r="B72" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3702,7 +3702,7 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D72" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3710,16 +3710,16 @@
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
       <x:c r="A73" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
       </x:c>
       <x:c r="B73" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C73" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D73" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3727,16 +3727,16 @@
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C74" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3744,16 +3744,16 @@
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C75" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3761,16 +3761,16 @@
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>data.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C76" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3778,16 +3778,16 @@
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>datahelpdesk.worldbank.org</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3795,16 +3795,16 @@
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3812,16 +3812,16 @@
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3829,16 +3829,16 @@
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3846,16 +3846,16 @@
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3863,16 +3863,16 @@
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
         <x:v>2026-07-27</x:v>
@@ -3880,42 +3880,127 @@
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>www150.statcan.gc.ca</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
-      <x:c r="A84" s="15" t="str">
+      <x:c r="A84" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+      </x:c>
+      <x:c r="B84" s="14" t="str">
+        <x:v>health.govt.nz</x:v>
+      </x:c>
+      <x:c r="C84" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D84" s="14" t="str">
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+      </x:c>
+      <x:c r="E84" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="31.5" customHeight="1">
+      <x:c r="A85" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+      </x:c>
+      <x:c r="B85" s="14" t="str">
+        <x:v>podatki.gov.pl</x:v>
+      </x:c>
+      <x:c r="C85" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D85" s="14" t="str">
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+      </x:c>
+      <x:c r="E85" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="31.5" customHeight="1">
+      <x:c r="A86" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B86" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C86" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D86" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E86" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="31.5" customHeight="1">
+      <x:c r="A87" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B87" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C87" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D87" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E87" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="31.5" customHeight="1">
+      <x:c r="A88" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+      </x:c>
+      <x:c r="B88" s="14" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C88" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D88" s="14" t="str">
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
+      </x:c>
+      <x:c r="E88" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="31.5" customHeight="1">
+      <x:c r="A89" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B84" s="15" t="str">
+      <x:c r="B89" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C84" s="15" t="str">
+      <x:c r="C89" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D84" s="15" t="str">
+      <x:c r="D89" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E84" s="15" t="str">
+      <x:c r="E89" s="15" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc80c1d2869c42d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41244762c5e4ff1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5961,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90757052d7854dfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ea52fdda224042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v28 evidence integrity hotfix
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7ddec210892e4a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5665e4e2128f42ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R8f338aa557ba4d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R49a48d73a8b04ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6e68c0fc9aec4ba8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R65657e35bd124ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1986d26057304583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf6a94b77fc0c41c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9a16eca0b4144399"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb6d14e1756e4404c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb271c2d9100e4bd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R848453b7a41e4b5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-27</x:v>
+        <x:v>2026.07.27-28</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee8f348dc7f4143"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc210fc747327418b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4000,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41244762c5e4ff1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3273dcd0eaab4eec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ea52fdda224042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R457f03cd95484a9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v28 evidence integrity hotfix (#25)
Separates evidence receipt history from gate outcomes, makes the global-base headline fail closed, corrects the schema identifier, and refreshes the bilingual lender artifacts to v28.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R7ddec210892e4a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5665e4e2128f42ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R8f338aa557ba4d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R49a48d73a8b04ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R6e68c0fc9aec4ba8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R65657e35bd124ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1986d26057304583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf6a94b77fc0c41c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9a16eca0b4144399"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb6d14e1756e4404c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb271c2d9100e4bd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R848453b7a41e4b5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-27</x:v>
+        <x:v>2026.07.27-28</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee8f348dc7f4143"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc210fc747327418b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4000,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc41244762c5e4ff1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3273dcd0eaab4eec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ea52fdda224042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R457f03cd95484a9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v29 visible receipt ledger
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R65657e35bd124ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1986d26057304583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf6a94b77fc0c41c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9a16eca0b4144399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb6d14e1756e4404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rb945fabde014491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rafe7e549148a418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R390d8a44c361445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra2e13610d16a4a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Red7ae603357a4d26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R848453b7a41e4b5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1d826692a924b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-28</x:v>
+        <x:v>2026.07.27-29</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc210fc747327418b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re275b761482347f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4000,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3273dcd0eaab4eec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2e9161dd0e9440d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R457f03cd95484a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57030ab94fca424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify receipt ledger as material intake
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rb945fabde014491f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rafe7e549148a418a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R390d8a44c361445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra2e13610d16a4a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Red7ae603357a4d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rd80abb56d7464fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R4e75f234b39c4f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R7ca57c0377fd49c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf80614604b9748f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R7af70ccacaa64d6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1d826692a924b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4652e6b7f849475a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re275b761482347f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8a93af8c878495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4000,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2e9161dd0e9440d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4fd63cfd86741d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57030ab94fca424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabf073225fdf42c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v29 visible receipt ledger (#26)
Render the public vendor-document intake as a visible seven-item material-receipt ledger separate from G1–G6 outcomes. Clarify that received rights- and terms-related material does not establish completeness or gate passage. Refresh and lock the bilingual decks and Evidence Registers to release 2026.07.27-29.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R65657e35bd124ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1986d26057304583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf6a94b77fc0c41c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9a16eca0b4144399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb6d14e1756e4404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rd80abb56d7464fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R4e75f234b39c4f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R7ca57c0377fd49c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf80614604b9748f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R7af70ccacaa64d6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R848453b7a41e4b5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4652e6b7f849475a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2216,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-28</x:v>
+        <x:v>2026.07.27-29</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2468,7 +2468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc210fc747327418b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8a93af8c878495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4000,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3273dcd0eaab4eec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4fd63cfd86741d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R457f03cd95484a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabf073225fdf42c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v30 country method control
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rd80abb56d7464fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R4e75f234b39c4f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R7ca57c0377fd49c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf80614604b9748f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R7af70ccacaa64d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R49f7ab26fc4747f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1545f49e09ce4418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf7e8bdcdbb4e4d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc862fb3dcdc44ed2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Ra8bac39862534821"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I54"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I55"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -870,448 +870,448 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The 195-country method control separates 23 reviewed country plans, 5 reviewed source leads, 15 regional EU TPD reporting patterns and 152 country-unscoped proxy routes.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market scope</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
+        <x:v>Every country has a visible method class, next evidence action and provenance basis. Classification is not a sales observation: all 195 countries in the 195-country universe have eligibleForGlobalRollup=false and donorAccepted=false.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
+        <x:v>site/data/global-base-layer.json ; source/country-method-route-config.json ; source/COUNTRY_METHOD_ROUTE_MAP.md</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>195 = 23 reviewed_method_plan + 5 reviewed_source_lead + 15 regional_tpd_pattern_only + 152 proxy_only_unscoped.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
+        <x:v>Across 195 countries, only 23 have a reviewed country-specific method plan. Five source leads and 15 regional TPD patterns do not establish a national sales series; 152 routes still require country-specific scoping.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
+        <x:v>No method class replaces annual device and e-liquid sales value, tax basis, channel coverage or D1–D10 acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
+        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
+        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
+        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
+        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
+        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
+        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
+        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
-        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
+        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
+        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
+        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
+        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
+        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
+        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="93" customHeight="1">
+        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
+        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
+        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-      <x:c r="F15" s="17" t="str">
-        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
+        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="58.5" customHeight="1">
+        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="93" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
+        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="F16" s="14" t="str">
-        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="F16" s="17" t="str">
+        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
+        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
+        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
+        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
         <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
+        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
+        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
+        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
+        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2021</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
+        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
+        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
+        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
+        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
+        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
+        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
+        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
+        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
+        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
+        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
         <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
         <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
@@ -1323,224 +1323,224 @@
         <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>The observation is not treated as the full market.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2020–2023</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
+        <x:v>Observed retail sales and price evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
+        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
+        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2020–2023</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
+        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
+        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
+        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
+        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
+        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I30" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I31" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="58.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025 volume / 2026 prices</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I32" s="14" t="str">
-        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="58.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>The public data does not contain an independent IVS valuation.</x:v>
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>site/data/atlas.json (readiness)</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
+        <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
         <x:v>The absence is recorded as a readiness blocker.</x:v>
@@ -1561,366 +1561,366 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="58.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>Validation</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+        <x:v>A patent publication is not treated as a product test report.</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="58.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>IP status</x:v>
+        <x:v>Validation</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+        <x:v>site/data/evidence.csv</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
+        <x:v>Absence check against the public evidence register.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I37" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="58.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>IP status</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>Total market value is not automatically the royalty base.</x:v>
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Application of the valuation boundary stated in the framework.</x:v>
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
+        <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
+        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
+        <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I41" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>Financing principle.</x:v>
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
+        <x:v>Financing principle.</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I43" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="58.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
         <x:v>Risks</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="58.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
-        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
         <x:v>Risks</x:v>
       </x:c>
       <x:c r="C45" s="14" t="str">
-        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E45" s="14" t="str">
-        <x:v>2026-12-04</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="F45" s="14" t="str">
-        <x:v>Check of the official maintenance-fee window.</x:v>
+        <x:v>Direct observation from the official register.</x:v>
       </x:c>
       <x:c r="G45" s="14" t="str">
-        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
       </x:c>
       <x:c r="H45" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I45" s="14" t="str">
-        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
+        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="58.5" customHeight="1">
       <x:c r="A46" s="14" t="str">
-        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
+        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
       <x:c r="B46" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C46" s="14" t="str">
-        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
+        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
       <x:c r="D46" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E46" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-12-04</x:v>
       </x:c>
       <x:c r="F46" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
       <x:c r="G46" s="14" t="str">
-        <x:v>No company-level financial conclusion is drawn.</x:v>
+        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I46" s="14" t="str">
-        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
+        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="58.5" customHeight="1">
       <x:c r="A47" s="14" t="str">
-        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
       <x:c r="D47" s="14" t="str">
         <x:v>Public package scope</x:v>
@@ -1932,24 +1932,24 @@
         <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G47" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
+        <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
       <x:c r="H47" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I47" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="58.5" customHeight="1">
       <x:c r="A48" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
       </x:c>
       <x:c r="B48" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C48" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
       </x:c>
       <x:c r="D48" s="14" t="str">
         <x:v>Public package scope</x:v>
@@ -1961,204 +1961,233 @@
         <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G48" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+        <x:v>No amount, maturity or security package is assumed.</x:v>
       </x:c>
       <x:c r="H48" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I48" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="58.5" customHeight="1">
       <x:c r="A49" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
       </x:c>
       <x:c r="B49" s="14" t="str">
-        <x:v>Competition</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C49" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
+        <x:v>The public package is limited to market and patent material.</x:v>
       </x:c>
       <x:c r="D49" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E49" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F49" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G49" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
       </x:c>
       <x:c r="H49" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I49" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="58.5" customHeight="1">
       <x:c r="A50" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
       </x:c>
       <x:c r="B50" s="14" t="str">
-        <x:v>Customers</x:v>
+        <x:v>Competition</x:v>
       </x:c>
       <x:c r="C50" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+        <x:v>Patent and case materials are not a competition map.</x:v>
       </x:c>
       <x:c r="D50" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E50" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F50" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G50" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
       </x:c>
       <x:c r="H50" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I50" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="58.5" customHeight="1">
       <x:c r="A51" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
       </x:c>
       <x:c r="B51" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Customers</x:v>
       </x:c>
       <x:c r="C51" s="14" t="str">
-        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
       </x:c>
       <x:c r="D51" s="14" t="str">
-        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E51" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F51" s="14" t="str">
-        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
       </x:c>
       <x:c r="G51" s="14" t="str">
-        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
       </x:c>
       <x:c r="H51" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I51" s="14" t="str">
-        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="58.5" customHeight="1">
       <x:c r="A52" s="14" t="str">
-        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
       </x:c>
       <x:c r="B52" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C52" s="14" t="str">
-        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
       </x:c>
       <x:c r="D52" s="14" t="str">
-        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E52" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>Count of countries in each evidence grade.</x:v>
+        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+        <x:v>Other countries depend on local rights and the products examined there.</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="58.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>No global atlas estimate has been approved for publication.</x:v>
+        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C53" s="14" t="str">
-        <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
+        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
-        <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
+        <x:v>Count of countries in each evidence grade.</x:v>
       </x:c>
       <x:c r="G53" s="14" t="str">
-        <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
+        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
       </x:c>
       <x:c r="H53" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I53" s="14" t="str">
+        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="58.5" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>No global atlas estimate has been approved for publication.</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="str">
+        <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
+      </x:c>
+      <x:c r="H54" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I54" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="58.5" customHeight="1">
-      <x:c r="A54" s="15" t="str">
+    <x:row r="55" ht="58.5" customHeight="1">
+      <x:c r="A55" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B54" s="15" t="str">
+      <x:c r="B55" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C54" s="15" t="str">
+      <x:c r="C55" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D54" s="15" t="str">
+      <x:c r="D55" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E54" s="15" t="str">
+      <x:c r="E55" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
-      <x:c r="F54" s="15" t="str">
+      <x:c r="F55" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G54" s="15" t="str">
+      <x:c r="G55" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H54" s="15" t="str">
+      <x:c r="H55" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I54" s="15" t="str">
+      <x:c r="I55" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H54">
+  <x:conditionalFormatting sqref="H2:H55">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H54">
+    <x:dataValidation type="list" sqref="H2:H55">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4652e6b7f849475a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c08f8d02c4e42d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2245,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-29</x:v>
+        <x:v>2026.07.27-30</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2240,8 +2269,8 @@
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>COUNTA('Evidence Register'!$A$2:$A$54)</x:f>
-        <x:v>53</x:v>
+        <x:f>COUNTA('Evidence Register'!$A$2:$A$55)</x:f>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
@@ -2256,8 +2285,8 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A11)</x:f>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2265,7 +2294,7 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A12)</x:f>
         <x:v>12</x:v>
       </x:c>
     </x:row>
@@ -2274,7 +2303,7 @@
         <x:v>Assumption</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A13)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A13)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -2283,7 +2312,7 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A14)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -2468,7 +2497,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8a93af8c878495c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8624f172681e4db4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4029,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4fd63cfd86741d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5230952edacc4016"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6075,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabf073225fdf42c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a75602b0ac42de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v30 country method control (#27)
Add the fail-closed 195-country method-control map, current vendor gates, refreshed bilingual bank decks and 54-row Evidence Registers.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Rd80abb56d7464fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R4e75f234b39c4f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R7ca57c0377fd49c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rf80614604b9748f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R7af70ccacaa64d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R49f7ab26fc4747f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1545f49e09ce4418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf7e8bdcdbb4e4d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc862fb3dcdc44ed2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Ra8bac39862534821"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I54"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I55"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -870,448 +870,448 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The 195-country method control separates 23 reviewed country plans, 5 reviewed source leads, 15 regional EU TPD reporting patterns and 152 country-unscoped proxy routes.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market scope</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
+        <x:v>Every country has a visible method class, next evidence action and provenance basis. Classification is not a sales observation: all 195 countries in the 195-country universe have eligibleForGlobalRollup=false and donorAccepted=false.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
+        <x:v>site/data/global-base-layer.json ; source/country-method-route-config.json ; source/COUNTRY_METHOD_ROUTE_MAP.md</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>195 = 23 reviewed_method_plan + 5 reviewed_source_lead + 15 regional_tpd_pattern_only + 152 proxy_only_unscoped.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
+        <x:v>Across 195 countries, only 23 have a reviewed country-specific method plan. Five source leads and 15 regional TPD patterns do not establish a national sales series; 152 routes still require country-specific scoping.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
+        <x:v>No method class replaces annual device and e-liquid sales value, tax basis, channel coverage or D1–D10 acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
+        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
+        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
+        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
+        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
+        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
+        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
+        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
-        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
+        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
+        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
+        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
+        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
+        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
+        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="93" customHeight="1">
+        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
+        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
+        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-      <x:c r="F15" s="17" t="str">
-        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
+        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="58.5" customHeight="1">
+        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="93" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
+        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>2026-07-26</x:v>
-      </x:c>
-      <x:c r="F16" s="14" t="str">
-        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="F16" s="17" t="str">
+        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
+        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
+        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
+        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
         <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
+        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
+        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
+        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
+        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2021</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
+        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
+        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
+        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
+        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
+        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58.5" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
+        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
+        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
+        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
+        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
+        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
         <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
         <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
@@ -1323,224 +1323,224 @@
         <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>The observation is not treated as the full market.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2020–2023</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
+        <x:v>Observed retail sales and price evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
+        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
+        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2020–2023</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
+        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
+        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
+        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
+        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
+        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I30" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I31" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="58.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025 volume / 2026 prices</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I32" s="14" t="str">
-        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="58.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>The public data does not contain an independent IVS valuation.</x:v>
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>site/data/atlas.json (readiness)</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
+        <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
         <x:v>The absence is recorded as a readiness blocker.</x:v>
@@ -1561,366 +1561,366 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="58.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>Validation</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+        <x:v>A patent publication is not treated as a product test report.</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="58.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>IP status</x:v>
+        <x:v>Validation</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+        <x:v>site/data/evidence.csv</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
+        <x:v>Absence check against the public evidence register.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I37" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="58.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>IP status</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>Total market value is not automatically the royalty base.</x:v>
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Application of the valuation boundary stated in the framework.</x:v>
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
+        <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
+        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
+        <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I41" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>Financing principle.</x:v>
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
+        <x:v>Financing principle.</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I43" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="58.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
         <x:v>Risks</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="58.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
-        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
         <x:v>Risks</x:v>
       </x:c>
       <x:c r="C45" s="14" t="str">
-        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E45" s="14" t="str">
-        <x:v>2026-12-04</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="F45" s="14" t="str">
-        <x:v>Check of the official maintenance-fee window.</x:v>
+        <x:v>Direct observation from the official register.</x:v>
       </x:c>
       <x:c r="G45" s="14" t="str">
-        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
       </x:c>
       <x:c r="H45" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I45" s="14" t="str">
-        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
+        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="58.5" customHeight="1">
       <x:c r="A46" s="14" t="str">
-        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
+        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
       <x:c r="B46" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C46" s="14" t="str">
-        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
+        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
       <x:c r="D46" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E46" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-12-04</x:v>
       </x:c>
       <x:c r="F46" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
       <x:c r="G46" s="14" t="str">
-        <x:v>No company-level financial conclusion is drawn.</x:v>
+        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I46" s="14" t="str">
-        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
+        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="58.5" customHeight="1">
       <x:c r="A47" s="14" t="str">
-        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
       <x:c r="D47" s="14" t="str">
         <x:v>Public package scope</x:v>
@@ -1932,24 +1932,24 @@
         <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G47" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
+        <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
       <x:c r="H47" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I47" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="58.5" customHeight="1">
       <x:c r="A48" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
       </x:c>
       <x:c r="B48" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C48" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
       </x:c>
       <x:c r="D48" s="14" t="str">
         <x:v>Public package scope</x:v>
@@ -1961,204 +1961,233 @@
         <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G48" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+        <x:v>No amount, maturity or security package is assumed.</x:v>
       </x:c>
       <x:c r="H48" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I48" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="58.5" customHeight="1">
       <x:c r="A49" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
       </x:c>
       <x:c r="B49" s="14" t="str">
-        <x:v>Competition</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C49" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
+        <x:v>The public package is limited to market and patent material.</x:v>
       </x:c>
       <x:c r="D49" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E49" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F49" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G49" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
       </x:c>
       <x:c r="H49" s="14" t="str">
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="I49" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="58.5" customHeight="1">
       <x:c r="A50" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
       </x:c>
       <x:c r="B50" s="14" t="str">
-        <x:v>Customers</x:v>
+        <x:v>Competition</x:v>
       </x:c>
       <x:c r="C50" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+        <x:v>Patent and case materials are not a competition map.</x:v>
       </x:c>
       <x:c r="D50" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E50" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F50" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G50" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
       </x:c>
       <x:c r="H50" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I50" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="58.5" customHeight="1">
       <x:c r="A51" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
       </x:c>
       <x:c r="B51" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Customers</x:v>
       </x:c>
       <x:c r="C51" s="14" t="str">
-        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
       </x:c>
       <x:c r="D51" s="14" t="str">
-        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E51" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F51" s="14" t="str">
-        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
       </x:c>
       <x:c r="G51" s="14" t="str">
-        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
       </x:c>
       <x:c r="H51" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I51" s="14" t="str">
-        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="58.5" customHeight="1">
       <x:c r="A52" s="14" t="str">
-        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
       </x:c>
       <x:c r="B52" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C52" s="14" t="str">
-        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
       </x:c>
       <x:c r="D52" s="14" t="str">
-        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E52" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>Count of countries in each evidence grade.</x:v>
+        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+        <x:v>Other countries depend on local rights and the products examined there.</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="58.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>No global atlas estimate has been approved for publication.</x:v>
+        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C53" s="14" t="str">
-        <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
+        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
-        <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
+        <x:v>Count of countries in each evidence grade.</x:v>
       </x:c>
       <x:c r="G53" s="14" t="str">
-        <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
+        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
       </x:c>
       <x:c r="H53" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I53" s="14" t="str">
+        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="58.5" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>No global atlas estimate has been approved for publication.</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>2026-07-27</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="str">
+        <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
+      </x:c>
+      <x:c r="H54" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I54" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="58.5" customHeight="1">
-      <x:c r="A54" s="15" t="str">
+    <x:row r="55" ht="58.5" customHeight="1">
+      <x:c r="A55" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B54" s="15" t="str">
+      <x:c r="B55" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C54" s="15" t="str">
+      <x:c r="C55" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D54" s="15" t="str">
+      <x:c r="D55" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E54" s="15" t="str">
+      <x:c r="E55" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
-      <x:c r="F54" s="15" t="str">
+      <x:c r="F55" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G54" s="15" t="str">
+      <x:c r="G55" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H54" s="15" t="str">
+      <x:c r="H55" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I54" s="15" t="str">
+      <x:c r="I55" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H54">
+  <x:conditionalFormatting sqref="H2:H55">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H54">
+    <x:dataValidation type="list" sqref="H2:H55">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4652e6b7f849475a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c08f8d02c4e42d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2245,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-29</x:v>
+        <x:v>2026.07.27-30</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2240,8 +2269,8 @@
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>COUNTA('Evidence Register'!$A$2:$A$54)</x:f>
-        <x:v>53</x:v>
+        <x:f>COUNTA('Evidence Register'!$A$2:$A$55)</x:f>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
@@ -2256,8 +2285,8 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A11)</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A11)</x:f>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2265,7 +2294,7 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A12)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A12)</x:f>
         <x:v>12</x:v>
       </x:c>
     </x:row>
@@ -2274,7 +2303,7 @@
         <x:v>Assumption</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A13)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A13)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -2283,7 +2312,7 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$54,A14)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -2468,7 +2497,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8a93af8c878495c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8624f172681e4db4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4029,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4fd63cfd86741d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5230952edacc4016"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6075,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabf073225fdf42c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a75602b0ac42de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v32 daily evidence package
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R49f7ab26fc4747f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1545f49e09ce4418"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf7e8bdcdbb4e4d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc862fb3dcdc44ed2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Ra8bac39862534821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R04994ae7b0a248b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R43a72eb45d5d45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R41543393e6e24031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra98da52778db4e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R32afc492ea9547c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I55"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I61"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E90" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The 195-country method control separates 23 reviewed country plans, 5 reviewed source leads, 15 regional EU TPD reporting patterns and 152 country-unscoped proxy routes.</x:v>
+        <x:v>The 195-country method control separates 28 reviewed country plans, 0 reviewed source leads, 15 regional EU TPD reporting patterns and 152 country-unscoped proxy routes.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market scope</x:v>
@@ -879,16 +879,16 @@
         <x:v>Every country has a visible method class, next evidence action and provenance basis. Classification is not a sales observation: all 195 countries in the 195-country universe have eligibleForGlobalRollup=false and donorAccepted=false.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>site/data/global-base-layer.json ; source/country-method-route-config.json ; source/COUNTRY_METHOD_ROUTE_MAP.md</x:v>
+        <x:v>site/data/global-base-layer.json ; source/country-method-route-config.json ; source/COUNTRY_METHOD_ROUTE_MAP.md ; source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>195 = 23 reviewed_method_plan + 5 reviewed_source_lead + 15 regional_tpd_pattern_only + 152 proxy_only_unscoped.</x:v>
+        <x:v>195 = 28 reviewed_method_plan + 0 reviewed_source_lead + 15 regional_tpd_pattern_only + 152 proxy_only_unscoped.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>Across 195 countries, only 23 have a reviewed country-specific method plan. Five source leads and 15 regional TPD patterns do not establish a national sales series; 152 routes still require country-specific scoping.</x:v>
+        <x:v>Across 195 countries, only 28 have a reviewed country-specific method plan. Five leads reviewed in this sprint were promoted only after their official holder, fields, formula and limitations were documented. Classification does not establish a national sales series; 152 routes still require country-specific scoping.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
@@ -899,1295 +899,1469 @@
     </x:row>
     <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>Austria has a reviewed method plan based on statutory annual sales reporting and e-liquid excise; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Austria</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
+        <x:v>The official route requires annual prior-year volume reporting and confirms e-liquid excise starting on 2026-04-01 at EUR 200 per litre.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Austria)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>Taxed litres = e-liquid-specific net excise / applicable EUR 200 per litre for the period starting 2026-04-01.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
+        <x:v>Mixed-rate periods are separated; annual reporting and excise inversion are alternative reconciliation routes, not additive.</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
+        <x:v>No national annual aggregate, price series, coverage evidence or retail reconciliation has been received; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
+        <x:v>Belgium’s official partial-period tax figure yields only a rounded 9 month tax-volume indicator; it is not full-year sales or retail market value.</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Belgium</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
+        <x:v>The official approximate EUR 12,500,000 and EUR 0.15 per ml rate imply approximately 83,333,333 ml or 83,333 litres.</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Belgium)</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
+        <x:v>EUR 12,500,000 / EUR 0.15 per ml = approximately 83,333,333 ml ≈ 83,333 litres.</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
-        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
+        <x:v>The figure covers a 9 month period; stockpiling, cross-border purchases and collection timing may distort interpretation.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
+        <x:v>Net releases for consumption, the full year, consumer sell-through, price and channel coverage are unverified; the 9 month indicator is not accepted as a donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
+        <x:v>Switzerland has a two-rate method route that started on 2024-10-01; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Switzerland</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
+        <x:v>The official route separates CHF 1.00 per ml for disposables and CHF 0.20 per ml for reusable nicotine products; the first period is 2024-10-01–2024-12-31.</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Switzerland)</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
+        <x:v>Disposable taxed ml = category net tax / CHF 1.00; reusable-nicotine taxed ml = category net tax / CHF 0.20; litres = ml / 1,000.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
+        <x:v>The tax categories must be supplied separately and combined receipts have no unique volume solution.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
+        <x:v>Category-specific net tax or millilitres, adjustments, reusable nicotine-free liquids, prices and sell-through are missing; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
+        <x:v>Luxembourg has an excise and fiscal-mark method starting on 2024-10-01; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Luxembourg</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
+        <x:v>The official rate is EUR 0.12 per ml from 2024-10-01, and fiscal marks carry liquid volume and mandatory consumer price.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Luxembourg)</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
+        <x:v>Taxed litres = e-liquid-specific net excise / EUR 120 per litre; marked consumer-price value = sum(marked pack quantity × mandatory marked price).</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
+        <x:v>The volume and fiscal-mark calculations are not additive; foreign B2B dispatches, destruction, refunds and corrections are separated.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="93" customHeight="1">
+        <x:v>The national aggregate, fiscal-mark quantity and price fields, sell-through and period finality are missing; retailValueStatus is not_computed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58.5" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
+        <x:v>Norway has no current Article 20(7) annual-sales route; the 2026 statutory NOK 5.38 per ml rate has no practical effect and does not establish market value.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Norway</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
+        <x:v>Official guidance prohibits commercial import and sale of nicotine products and the new TPD route does not apply; SSB external-trade data are only a customs proxy.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Norway)</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
-      <x:c r="F16" s="17" t="str">
-        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Excise inversion is permitted only if category-specific net receipts with practical effect are supplied; the customs proxy does not become national consumer sell-through.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
+        <x:v>A prohibition, statutory tax rate or missing record does not establish the absence of a market.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
+        <x:v>Nicotine-free sell-through, millilitres, prices, domestic production, inventories, re-exports and illicit channels are missing; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>Italian ADM PLI consumption-tax receipts were EUR 55,910,871.89 in 2023 and EUR 84,309,841.41 in 2024; this is not retail market value.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Italy</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
+        <x:v>Table III.9 of ADM’s Libro Blu 2024 reports a 50.79 percent tax-receipt change. In 2024 the tax scope expanded to aromas intended for PLI products and taxation changed, so the percentage is not interpreted as sales or volume growth.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43 ; source/ITALY_ADM_RESPONSE_BOUNDARY_2026-07-24.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
+        <x:v>Direct table transcription: EUR 55,910,871.89 in 2023; EUR 84,309,841.41 in 2024; reported change 50.79 percent.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
+        <x:v>Tax receipts are a fiscal measure. They are not inverted into litres or retail value without separate rates, categories, adjustments and a like-for-like scope.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+        <x:v>Nicotine and nicotine-free split, litres, devices, consumer prices, refunds, cash timing and a scope-comparable series are missing; Italy is not a donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
+        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
+        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
+        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
+        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
+        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
+        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2021</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
+        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
+        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
+        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
+        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
+        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
+        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
+        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
+        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
+        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
+        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="58.5" customHeight="1">
+        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="93" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
+        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
+        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
-      <x:c r="F22" s="14" t="str">
-        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
+      <x:c r="F22" s="17" t="str">
+        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
+        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
+        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
+        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
+        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
+        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
+        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
+        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
+        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2020–2023</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
+        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
+        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
+        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
+        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
+        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
+        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
+        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
+        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I30" s="14" t="str">
-        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I31" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="58.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>The observation is not treated as the full market.</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I32" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="58.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
+        <x:v>Observed retail sales and price evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>The public data does not contain an independent IVS valuation.</x:v>
+        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2020–2023</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="58.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
+        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="58.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>Validation</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I37" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="58.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>IP status</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025 volume / 2026 prices</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>site/data/atlas.json (readiness)</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
+        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>Total market value is not automatically the royalty base.</x:v>
+        <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Application of the valuation boundary stated in the framework.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
         <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I41" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+        <x:v>A patent publication is not treated as a product test report.</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Validation</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>site/data/evidence.csv</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Financing principle.</x:v>
+        <x:v>Absence check against the public evidence register.</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I43" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="58.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>IP status</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="58.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C45" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E45" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F45" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
       </x:c>
       <x:c r="G45" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
       </x:c>
       <x:c r="H45" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I45" s="14" t="str">
-        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
+        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="58.5" customHeight="1">
       <x:c r="A46" s="14" t="str">
-        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
+        <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
       <x:c r="B46" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C46" s="14" t="str">
-        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
+        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
       <x:c r="D46" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E46" s="14" t="str">
-        <x:v>2026-12-04</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F46" s="14" t="str">
-        <x:v>Check of the official maintenance-fee window.</x:v>
+        <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
       <x:c r="G46" s="14" t="str">
-        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
+        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I46" s="14" t="str">
-        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="58.5" customHeight="1">
       <x:c r="A47" s="14" t="str">
-        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
-        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D47" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E47" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F47" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G47" s="14" t="str">
-        <x:v>No company-level financial conclusion is drawn.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H47" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I47" s="14" t="str">
-        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="58.5" customHeight="1">
       <x:c r="A48" s="14" t="str">
-        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
       </x:c>
       <x:c r="B48" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C48" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
       </x:c>
       <x:c r="D48" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
       </x:c>
       <x:c r="E48" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F48" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
       </x:c>
       <x:c r="G48" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
       </x:c>
       <x:c r="H48" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I48" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="58.5" customHeight="1">
       <x:c r="A49" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
       </x:c>
       <x:c r="B49" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C49" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
       </x:c>
       <x:c r="D49" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E49" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F49" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Financing principle.</x:v>
       </x:c>
       <x:c r="G49" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
       </x:c>
       <x:c r="H49" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I49" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="58.5" customHeight="1">
       <x:c r="A50" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
       </x:c>
       <x:c r="B50" s="14" t="str">
-        <x:v>Competition</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C50" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
       </x:c>
       <x:c r="D50" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E50" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="F50" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
       </x:c>
       <x:c r="G50" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H50" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I50" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="58.5" customHeight="1">
       <x:c r="A51" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
       </x:c>
       <x:c r="B51" s="14" t="str">
-        <x:v>Customers</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C51" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
       </x:c>
       <x:c r="D51" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E51" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="F51" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+        <x:v>Direct observation from the official register.</x:v>
       </x:c>
       <x:c r="G51" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
       </x:c>
       <x:c r="H51" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I51" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="58.5" customHeight="1">
       <x:c r="A52" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
       <x:c r="B52" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C52" s="14" t="str">
-        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
       <x:c r="D52" s="14" t="str">
-        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E52" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-12-04</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+        <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="58.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C53" s="14" t="str">
-        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
-        <x:v>Count of countries in each evidence grade.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G53" s="14" t="str">
-        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+        <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
       <x:c r="H53" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I53" s="14" t="str">
-        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="58.5" customHeight="1">
       <x:c r="A54" s="14" t="str">
+        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="str">
+        <x:v>No amount, maturity or security package is assumed.</x:v>
+      </x:c>
+      <x:c r="H54" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I54" s="14" t="str">
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="58.5" customHeight="1">
+      <x:c r="A55" s="14" t="str">
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+      </x:c>
+      <x:c r="B55" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C55" s="14" t="str">
+        <x:v>The public package is limited to market and patent material.</x:v>
+      </x:c>
+      <x:c r="D55" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E55" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F55" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G55" s="14" t="str">
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+      </x:c>
+      <x:c r="H55" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I55" s="14" t="str">
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="58.5" customHeight="1">
+      <x:c r="A56" s="14" t="str">
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+      </x:c>
+      <x:c r="B56" s="14" t="str">
+        <x:v>Competition</x:v>
+      </x:c>
+      <x:c r="C56" s="14" t="str">
+        <x:v>Patent and case materials are not a competition map.</x:v>
+      </x:c>
+      <x:c r="D56" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E56" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F56" s="14" t="str">
+        <x:v>Absence check against the public package.</x:v>
+      </x:c>
+      <x:c r="G56" s="14" t="str">
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+      </x:c>
+      <x:c r="H56" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I56" s="14" t="str">
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="58.5" customHeight="1">
+      <x:c r="A57" s="14" t="str">
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>Customers</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F57" s="14" t="str">
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+      </x:c>
+      <x:c r="G57" s="14" t="str">
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+      </x:c>
+      <x:c r="H57" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I57" s="14" t="str">
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="58.5" customHeight="1">
+      <x:c r="A58" s="14" t="str">
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F58" s="14" t="str">
+        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+      </x:c>
+      <x:c r="G58" s="14" t="str">
+        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+      </x:c>
+      <x:c r="H58" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I58" s="14" t="str">
+        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="58.5" customHeight="1">
+      <x:c r="A59" s="14" t="str">
+        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F59" s="14" t="str">
+        <x:v>Count of countries in each evidence grade.</x:v>
+      </x:c>
+      <x:c r="G59" s="14" t="str">
+        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+      </x:c>
+      <x:c r="H59" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I59" s="14" t="str">
+        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="58.5" customHeight="1">
+      <x:c r="A60" s="14" t="str">
         <x:v>No global atlas estimate has been approved for publication.</x:v>
       </x:c>
-      <x:c r="B54" s="14" t="str">
+      <x:c r="B60" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C54" s="14" t="str">
+      <x:c r="C60" s="14" t="str">
         <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
       </x:c>
-      <x:c r="D54" s="14" t="str">
+      <x:c r="D60" s="14" t="str">
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
-      <x:c r="E54" s="14" t="str">
+      <x:c r="E60" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
-      <x:c r="F54" s="14" t="str">
+      <x:c r="F60" s="14" t="str">
         <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
       </x:c>
-      <x:c r="G54" s="14" t="str">
+      <x:c r="G60" s="14" t="str">
         <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
       </x:c>
-      <x:c r="H54" s="14" t="str">
+      <x:c r="H60" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I54" s="14" t="str">
+      <x:c r="I60" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="58.5" customHeight="1">
-      <x:c r="A55" s="15" t="str">
+    <x:row r="61" ht="58.5" customHeight="1">
+      <x:c r="A61" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B55" s="15" t="str">
+      <x:c r="B61" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C55" s="15" t="str">
+      <x:c r="C61" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D55" s="15" t="str">
+      <x:c r="D61" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E55" s="15" t="str">
+      <x:c r="E61" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
-      <x:c r="F55" s="15" t="str">
+      <x:c r="F61" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G55" s="15" t="str">
+      <x:c r="G61" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H55" s="15" t="str">
+      <x:c r="H61" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I55" s="15" t="str">
+      <x:c r="I61" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H55">
+  <x:conditionalFormatting sqref="H2:H61">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H55">
+    <x:dataValidation type="list" sqref="H2:H61">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c08f8d02c4e42d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f964f126ca9443a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2245,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-30</x:v>
+        <x:v>2026.07.28-32</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2253,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2269,8 +2443,8 @@
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>COUNTA('Evidence Register'!$A$2:$A$55)</x:f>
-        <x:v>54</x:v>
+        <x:f>COUNTA('Evidence Register'!$A$2:$A$61)</x:f>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
@@ -2285,8 +2459,8 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A11)</x:f>
-        <x:v>29</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A11)</x:f>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2294,8 +2468,8 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A12)</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A12)</x:f>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2303,7 +2477,7 @@
         <x:v>Assumption</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A13)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A13)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -2312,7 +2486,7 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A14)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -2497,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8624f172681e4db4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17d2109462c24865"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3411,7 +3585,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3428,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3445,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3462,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3479,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3496,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3513,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3530,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3547,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3564,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3581,7 +3755,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3598,7 +3772,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3615,7 +3789,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3632,7 +3806,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3649,7 +3823,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3666,7 +3840,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3683,7 +3857,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3700,7 +3874,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3717,7 +3891,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3734,7 +3908,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3751,7 +3925,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3768,7 +3942,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3785,7 +3959,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3802,7 +3976,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3819,7 +3993,7 @@
         <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -3836,63 +4010,63 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -3901,32 +4075,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
         <x:v>health.govt.nz</x:v>
@@ -3935,49 +4109,49 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C85" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C86" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -3986,50 +4160,67 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B88" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C88" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D88" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E88" s="14" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="31.5" customHeight="1">
+      <x:c r="A89" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B88" s="14" t="str">
+      <x:c r="B89" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C88" s="14" t="str">
+      <x:c r="C89" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D88" s="14" t="str">
+      <x:c r="D89" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="31.5" customHeight="1">
-      <x:c r="A89" s="15" t="str">
+      <x:c r="E89" s="14" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="31.5" customHeight="1">
+      <x:c r="A90" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B89" s="15" t="str">
+      <x:c r="B90" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C89" s="15" t="str">
+      <x:c r="C90" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D89" s="15" t="str">
+      <x:c r="D90" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E89" s="15" t="str">
-        <x:v>2026-07-27</x:v>
+      <x:c r="E90" s="15" t="str">
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5230952edacc4016"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R892c33906a724eb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6075,7 +6266,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a75602b0ac42de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9552970be04e4295"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v32 daily evidence package (#29)
Publish the bilingual v32 daily evidence package, privacy-safe Italy and Poland boundaries, current vendor follow-up states, and once-daily bank-artifact cadence.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R49f7ab26fc4747f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1545f49e09ce4418"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rf7e8bdcdbb4e4d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc862fb3dcdc44ed2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Ra8bac39862534821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R04994ae7b0a248b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R43a72eb45d5d45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R41543393e6e24031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra98da52778db4e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R32afc492ea9547c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I55"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EvidenceRegisterEN" displayName="EvidenceRegisterEN" ref="A1:I61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I61"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Claim"/>
     <x:tableColumn id="2" name="Slide/section"/>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E90" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>The 195-country method control separates 23 reviewed country plans, 5 reviewed source leads, 15 regional EU TPD reporting patterns and 152 country-unscoped proxy routes.</x:v>
+        <x:v>The 195-country method control separates 28 reviewed country plans, 0 reviewed source leads, 15 regional EU TPD reporting patterns and 152 country-unscoped proxy routes.</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>Market scope</x:v>
@@ -879,16 +879,16 @@
         <x:v>Every country has a visible method class, next evidence action and provenance basis. Classification is not a sales observation: all 195 countries in the 195-country universe have eligibleForGlobalRollup=false and donorAccepted=false.</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>site/data/global-base-layer.json ; source/country-method-route-config.json ; source/COUNTRY_METHOD_ROUTE_MAP.md</x:v>
+        <x:v>site/data/global-base-layer.json ; source/country-method-route-config.json ; source/COUNTRY_METHOD_ROUTE_MAP.md ; source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>195 = 23 reviewed_method_plan + 5 reviewed_source_lead + 15 regional_tpd_pattern_only + 152 proxy_only_unscoped.</x:v>
+        <x:v>195 = 28 reviewed_method_plan + 0 reviewed_source_lead + 15 regional_tpd_pattern_only + 152 proxy_only_unscoped.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>Across 195 countries, only 23 have a reviewed country-specific method plan. Five source leads and 15 regional TPD patterns do not establish a national sales series; 152 routes still require country-specific scoping.</x:v>
+        <x:v>Across 195 countries, only 28 have a reviewed country-specific method plan. Five leads reviewed in this sprint were promoted only after their official holder, fields, formula and limitations were documented. Classification does not establish a national sales series; 152 routes still require country-specific scoping.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
         <x:v>Confirmed</x:v>
@@ -899,1295 +899,1469 @@
     </x:row>
     <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>Austria has a reviewed method plan based on statutory annual sales reporting and e-liquid excise; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Austria</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
+        <x:v>The official route requires annual prior-year volume reporting and confirms e-liquid excise starting on 2026-04-01 at EUR 200 per litre.</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Austria)</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>Taxed litres = e-liquid-specific net excise / applicable EUR 200 per litre for the period starting 2026-04-01.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
+        <x:v>Mixed-rate periods are separated; annual reporting and excise inversion are alternative reconciliation routes, not additive.</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
+        <x:v>No national annual aggregate, price series, coverage evidence or retail reconciliation has been received; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
+        <x:v>Belgium’s official partial-period tax figure yields only a rounded 9 month tax-volume indicator; it is not full-year sales or retail market value.</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Belgium</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
+        <x:v>The official approximate EUR 12,500,000 and EUR 0.15 per ml rate imply approximately 83,333,333 ml or 83,333 litres.</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Belgium)</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
+        <x:v>EUR 12,500,000 / EUR 0.15 per ml = approximately 83,333,333 ml ≈ 83,333 litres.</x:v>
       </x:c>
       <x:c r="G13" s="14" t="str">
-        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
+        <x:v>The figure covers a 9 month period; stockpiling, cross-border purchases and collection timing may distort interpretation.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
+        <x:v>Net releases for consumption, the full year, consumer sell-through, price and channel coverage are unverified; the 9 month indicator is not accepted as a donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
+        <x:v>Switzerland has a two-rate method route that started on 2024-10-01; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Switzerland</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
+        <x:v>The official route separates CHF 1.00 per ml for disposables and CHF 0.20 per ml for reusable nicotine products; the first period is 2024-10-01–2024-12-31.</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Switzerland)</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>2024</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
+        <x:v>Disposable taxed ml = category net tax / CHF 1.00; reusable-nicotine taxed ml = category net tax / CHF 0.20; litres = ml / 1,000.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
+        <x:v>The tax categories must be supplied separately and combined receipts have no unique volume solution.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
+        <x:v>Category-specific net tax or millilitres, adjustments, reusable nicotine-free liquids, prices and sell-through are missing; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
+        <x:v>Luxembourg has an excise and fiscal-mark method starting on 2024-10-01; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Luxembourg</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
+        <x:v>The official rate is EUR 0.12 per ml from 2024-10-01, and fiscal marks carry liquid volume and mandatory consumer price.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Luxembourg)</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
+        <x:v>Taxed litres = e-liquid-specific net excise / EUR 120 per litre; marked consumer-price value = sum(marked pack quantity × mandatory marked price).</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
+        <x:v>The volume and fiscal-mark calculations are not additive; foreign B2B dispatches, destruction, refunds and corrections are separated.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="93" customHeight="1">
+        <x:v>The national aggregate, fiscal-mark quantity and price fields, sell-through and period finality are missing; retailValueStatus is not_computed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58.5" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
+        <x:v>Norway has no current Article 20(7) annual-sales route; the 2026 statutory NOK 5.38 per ml rate has no practical effect and does not establish market value.</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Norway</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
+        <x:v>Official guidance prohibits commercial import and sale of nicotine products and the new TPD route does not apply; SSB external-trade data are only a customs proxy.</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Norway)</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
-      <x:c r="F16" s="17" t="str">
-        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Excise inversion is permitted only if category-specific net receipts with practical effect are supplied; the customs proxy does not become national consumer sell-through.</x:v>
       </x:c>
       <x:c r="G16" s="14" t="str">
-        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
+        <x:v>A prohibition, statutory tax rate or missing record does not establish the absence of a market.</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
+        <x:v>Nicotine-free sell-through, millilitres, prices, domestic production, inventories, re-exports and illicit channels are missing; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>Italian ADM PLI consumption-tax receipts were EUR 55,910,871.89 in 2023 and EUR 84,309,841.41 in 2024; this is not retail market value.</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Italy</x:v>
       </x:c>
       <x:c r="C17" s="14" t="str">
-        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
+        <x:v>Table III.9 of ADM’s Libro Blu 2024 reports a 50.79 percent tax-receipt change. In 2024 the tax scope expanded to aromas intended for PLI products and taxation changed, so the percentage is not interpreted as sales or volume growth.</x:v>
       </x:c>
       <x:c r="D17" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43 ; source/ITALY_ADM_RESPONSE_BOUNDARY_2026-07-24.md</x:v>
       </x:c>
       <x:c r="E17" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
+        <x:v>Direct table transcription: EUR 55,910,871.89 in 2023; EUR 84,309,841.41 in 2024; reported change 50.79 percent.</x:v>
       </x:c>
       <x:c r="G17" s="14" t="str">
-        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
+        <x:v>Tax receipts are a fiscal measure. They are not inverted into litres or retail value without separate rates, categories, adjustments and a like-for-like scope.</x:v>
       </x:c>
       <x:c r="H17" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
-        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+        <x:v>Nicotine and nicotine-free split, litres, devices, consumer prices, refunds, cash timing and a scope-comparable series are missing; Italy is not a donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
+        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
+        <x:v>The market measures cover Canada, Germany, Finland, New Zealand, Poland, Sweden and the United States. The FHM counts describe reporting entities and notified, active and withdrawn products for 2018–2026; they are not sales or market value.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
+        <x:v>site/data/market-values.json (machine-readable source file of the public site)</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
+        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
-        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
+        <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
-        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+        <x:v>Comparable annual device and liquid consumer-retail-value series are required from additional countries.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
+        <x:v>There are zero accepted full-year national consumer-retail-value donor markets.</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
+        <x:v>comparableFullYearMarketValueDonors = 0. Five candidate tests are published against the same ten-criterion protocol.</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
+        <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>2021</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
+        <x:v>A candidate enters the donor count only when D1–D10 all pass; a failed or open criterion keeps it outside the count.</x:v>
       </x:c>
       <x:c r="G19" s="14" t="str">
-        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
+        <x:v>Official lower bounds, institutional benchmarks, shipment values, tax receipts, physical volumes and models are not relabelled as complete consumer-retail value.</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
-        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+        <x:v>At least three accepted donors are required, with regional and regulatory-archetype coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
+        <x:v>New Zealand's 2024 specialist-vape-retailer sales were reported as at least NZD 280 million.</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
+        <x:v>The Ministry of Health publishes an official consumer-retail lower bound based only on incomplete specialist-vape-retailer sales. General retail is outside the figure, adjacent notifiable products are included and the Ministry does not recommend the data for in-depth research.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024</x:v>
       </x:c>
       <x:c r="E20" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
+        <x:v>Direct use of the official at-least headline; no extrapolation and no addition of other return types.</x:v>
       </x:c>
       <x:c r="G20" s="14" t="str">
-        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
+        <x:v>The figure is a lower bound, not a complete national vaping-market value.</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
-        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
+        <x:v>Obtain a complete national vaping-only retailer aggregate, GST basis and independent reconciliation.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58.5" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
+        <x:v>The raw sum of 612,765 numeric Total sales cells across New Zealand's 29 official 2024 XLSX files is NZD 280,684,512.81.</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
+        <x:v>The raw sum reconciles to the Ministry's at-least NZD 280 million headline. The files contain 95,144 exact repeated row signatures; removing occurrences after the first would produce NZD 264,561,055.05, but repeat semantics are unverified.</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_ANNUAL_RETURNS_RECONCILIATION.md</x:v>
       </x:c>
       <x:c r="E21" s="14" t="str">
-        <x:v>2023</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
+        <x:v>Direct sum of the numeric Total sales cells in all 29 official XLSX files; no de-duplication, cleaning or extrapolation.</x:v>
       </x:c>
       <x:c r="G21" s="14" t="str">
-        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
+        <x:v>Repeated rows remain in the raw sum because their business meaning is unknown.</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
-        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="58.5" customHeight="1">
+        <x:v>The raw sum is not a cleaned national market value. General retail, missing returns and GST treatment remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="93" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
+        <x:v>New Zealand's 2024 AIS/AVP specialist-retailer identified-vaping subtotal is NZD 274,180,410.21; the donor test passes 7/10 criteria, but New Zealand is not an accepted donor.</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
+        <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
-      <x:c r="F22" s="14" t="str">
-        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
+      <x:c r="F22" s="17" t="str">
+        <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
+        <x:v>D5 fails for missing national channel coverage; D8 GST basis and D10 independent reconciliation remain open. The donor gate remains 0/3.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
+        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
+        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2026-07-25</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
+        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
+        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
+        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
+        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
+        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2023–2025</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
+        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
+        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>Final 2025 data and observed retail sales are required.</x:v>
+        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Direct use of the official cash-basis observation.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58.5" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
+        <x:v>The public site separates three evidence lanes and blocks a global total while the accepted-donor gate is 0/3.</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
+        <x:v>Five candidates are assessed against the same ten D1–D10 criteria; none is accepted. The regional and regulatory-archetype coverage gates must also pass.</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>The observation is not treated as the full market.</x:v>
+        <x:v>Only reviewed public aggregates and methods enter the public lane; licensed and private material do not enter the repository.</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I26" s="14" t="str">
-        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
+        <x:v>The global value remains uncomputed until at least three donors and both coverage gates are accepted.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58.5" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
+        <x:v>The European Commission publishes a EUR 4.99 billion benchmark for the 2023 EU e-cigarette market.</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
+        <x:v>Footnote 83 on physical PDF page 25 of SWD(2026) 111 identifies Euromonitor International Tobacco 2025 as the source for the following tables; Table 4 on physical page 27 reports EUR 4.99 billion. Physical page 161 of SWD(2025) 560 describes a nearly EUR 5 billion aggregate covering devices and liquids, including nicotine-free products; page 162 states that data are unavailable for Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
+        <x:v>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2026%3A111%3AFIN ; https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=SWD%3A2025%3A0560%3AFIN</x:v>
       </x:c>
       <x:c r="E27" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
+        <x:v>Cross-document comparison of the table, page and source references in two European Commission staff working documents; the figures are not summed.</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Tax receipts are not treated as consumer sales.</x:v>
+        <x:v>The Commission publishes the benchmark, but its basis is commercial Euromonitor data. The full method, tax basis and reusable country dataset are not public, and three EU countries lack data.</x:v>
       </x:c>
       <x:c r="H27" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I27" s="14" t="str">
-        <x:v>Observed retail sales and price evidence are required.</x:v>
+        <x:v>Acquire the licensed country table and method, transaction definition, channel coverage, tax basis and an independent reconciliation; complete Cyprus, Luxembourg and Malta.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58.5" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
+        <x:v>Canada's official 2024 consumer-retail point estimate is CAD 1,219,160,000, or EUR 822,583,715.21; the donor test passes 7/10 criteria.</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
+        <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2020–2023</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
+        <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
+        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
+        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
+        <x:v>Health Canada's four 2024 categories sum to CAD 1,160,753,796.78 of net shipment value, 118,901,910 units and 1,251,843 litres.</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
+        <x:v>Value shares are: part/device without substance 2.602%, device with substance 48.154%, part with substance 27.252% and vaping substance 21.992%. These are shipments to wholesalers or retailers, not consumer purchases.</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://health-infobase.canada.ca/substance-use/vaping/sales/ ; https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html ; source/CANADA_2024_DONOR_CLOSURE_PACK.md</x:v>
       </x:c>
       <x:c r="E29" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-25</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
+        <x:v>CAD 30,207,822.87 + 558,947,200.26 + 316,329,158.83 + 255,269,614.82 = CAD 1,160,753,796.78; shares use this total.</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
+        <x:v>Net sales are sales less returns and values are reported excluding taxes and duties. A device or part containing substance combines hardware and liquid value.</x:v>
       </x:c>
       <x:c r="H29" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I29" s="14" t="str">
-        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
+        <x:v>Do not apply shipment shares to retail as a device/liquid split and do not add transaction stages.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58.5" customHeight="1">
       <x:c r="A30" s="14" t="str">
-        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
+        <x:v>Germany's taxed liquid volume increased from 1.241 million litres to 1.518 million litres in 2023–2025.</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
+        <x:v>The 2023 and 2024 observations are final, while 2025 is provisional.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2023–2025</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>Direct use of the reported net quantities without extrapolation.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
+        <x:v>The series covers taxed liquid, not devices or illicit supply.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I30" s="14" t="str">
-        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
+        <x:v>Final 2025 data and observed retail sales are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58.5" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
+        <x:v>German excise receipts from substitutes for tobacco were EUR 404 million in 2025, provisionally.</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
+        <x:v>The observation is cash-basis excise revenue, not sales revenue or retail market value.</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003</x:v>
       </x:c>
       <x:c r="E31" s="14" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
+        <x:v>Direct use of the official cash-basis observation.</x:v>
       </x:c>
       <x:c r="G31" s="14" t="str">
-        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
+        <x:v>Excise receipts are not treated as sales or retail value.</x:v>
       </x:c>
       <x:c r="H31" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I31" s="14" t="str">
-        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
+        <x:v>Final 2025 data and reconciliation of the product-category tax base are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="58.5" customHeight="1">
       <x:c r="A32" s="14" t="str">
-        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
+        <x:v>Finland taxed 11,801.062 litres of nicotine-containing e-cigarette liquid in 2025.</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
+        <x:v>This is an official full-year observation. The full-year value for nicotine-free liquid is suppressed. The figure is a physical volume, excludes devices and is not retail value.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>2025 volume / 2026 prices</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
+        <x:v>The observation is not treated as the full market.</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I32" s="14" t="str">
-        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
+        <x:v>Devices, nicotine-free liquid, tax-free channels and illicit supply are missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="58.5" customHeight="1">
       <x:c r="A33" s="14" t="str">
-        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
+        <x:v>Finland's nicotine-liquid excise receipts were EUR 3,540,319 in 2025.</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
+        <x:v>This is an official full-year observation. The nicotine-free observation is suppressed. Tax receipts are not sales or retail value.</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness)</x:v>
+        <x:v>https://vero2.stat.fi/PXWeb/api/v1/en/Vero/Valmistevero/vvt_010.px</x:v>
       </x:c>
       <x:c r="E33" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>Use of the public dataset's own readiness classification.</x:v>
+        <x:v>Direct observation from the Finnish Tax Administration PXWeb table.</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>Market data and IP value are kept analytically separate.</x:v>
+        <x:v>Tax receipts are not treated as consumer sales.</x:v>
       </x:c>
       <x:c r="H33" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I33" s="14" t="str">
-        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
+        <x:v>Observed retail sales and price evidence are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>The public data does not contain an independent IVS valuation.</x:v>
+        <x:v>Poland's official e-liquid flow was 1,451,529 litres in 2020, 277,265 litres in 2021, 416,088 litres in 2022 and 805,441 litres in 2023.</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>The ministry's parliamentary-response table combines domestic sales, intra-EU acquisitions and imports recorded in ZEFIR2/AIS. The series is a physical e-liquid flow, not consumer sales or observed retail market value.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDDEJZ5/i07255-o1.pdf</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2020–2023</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Direct reproduction of four official annual observations; years are not summed into a market value.</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The published table does not split domestic sales, intra-EU acquisitions and imports and contains no device value.</x:v>
       </x:c>
       <x:c r="H34" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I34" s="14" t="str">
-        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
+        <x:v>Consumer retail value, channel coverage, tax basis and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="58.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The absence is recorded as a readiness blocker.</x:v>
+        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>No assumptions.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
+        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
+        <x:v>Sweden's public evidence combines a 2024 tax anchor with 36 official FHM register-structure counts for 2018–2026; the register counts are not sales or market value.</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
+        <x:v>Sweden taxed 26,000 litres of nicotine liquid in 2024 and reported rounded excise receipts of SEK 80,000,000. An authority-supplied workbook received and reviewed on 24 July 2026 contains 9 year labels × 4 structure metrics: reporting entities and notified, active and withdrawn products. The public FHM page documents the notification system; it is not presented as publishing the numeric series.</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://www.regeringen.se/contentassets/1ed01e00001b42e5ad8d47433db63ece/berakningskonventioner_2026.pdf ; https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/ ; site/data/market-values.json</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>Absence check in relation to any technical performance claim.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>A patent publication is not treated as a product test report.</x:v>
+        <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
+        <x:v>Observed consumer sales in euros, device units and liquid millilitres, plus a publicly reusable numeric FHM series, are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="58.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
+        <x:v>Three commercial 2025 global estimates form a range of USD 26.0–46.32 billion.</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>Validation</x:v>
+        <x:v>Market size</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
+        <x:v>IMARC reports USD 26.0 billion, Grand View Research USD 45.7 billion and Fortune Business Insights USD 46.32 billion.</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>site/data/evidence.csv</x:v>
+        <x:v>https://www.imarcgroup.com/e-cigarette-market ; https://www.grandviewresearch.com/industry-analysis/e-cigarette-vaping-market ; https://www.fortunebusinessinsights.com/e-cigarette-and-vaping-market-114882</x:v>
       </x:c>
       <x:c r="E37" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Absence check against the public evidence register.</x:v>
+        <x:v>Minimum USD 26.0 billion; maximum USD 46.32 billion; the estimates are compared, not summed.</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
+        <x:v>The scopes and methods of the commercial estimates may not be comparable.</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I37" s="14" t="str">
-        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
+        <x:v>Full methodologies and a harmonised scope are required before relying on the range.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="58.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
+        <x:v>The 2025 German taxed-liquid retail-equivalent model gives a range of EUR 667.92–1,654.62 million.</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>IP status</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>Family publications do not establish current national post-grant status.</x:v>
+        <x:v>This is not observed sales. Provisional 2025 volume is multiplied by three individual 2026 German e-shop prices. The year mismatch, a price basket from one retailer, product-mix uncertainty and exclusions make the estimate low confidence.</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003 ; https://www.intaste.de/pfefferminz-liquid-germanflavours-liquid ; https://www.intaste.de/anstand-liquid-samurai-liquid ; https://www.intaste.de/tobacco-vanilla-nikotinsalz-revoltage-liquid</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2025 volume / 2026 prices</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Identification of the legal due-diligence limitation.</x:v>
+        <x:v>volume_litres * 1000 * retail_price_eur_per_ml</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>Checks in four registers do not establish status across the full family.</x:v>
+        <x:v>Three individual online-shop prices; input years 2025 and 2026; taxed liquid only.</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
+        <x:v>A representative price basket, product mix and channel margins, plus model-year 2025 prices, are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
+        <x:v>The atlas is not yet a lender-ready market valuation.</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>Technical differentiation</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
+        <x:v>research_dataset_not_valuation: most countries lack official annual device and liquid sales; market evidence is not yet linked to country-level patent status and claim charts; there is no independent IVS valuation or realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>site/data/atlas.json (readiness)</x:v>
       </x:c>
       <x:c r="E39" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
+        <x:v>Use of the public dataset's own readiness classification.</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
+        <x:v>Market data and IP value are kept analytically separate.</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I39" s="14" t="str">
-        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
+        <x:v>Every listed blocker must be closed before drawing collateral-value or enterprise-value conclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>Total market value is not automatically the royalty base.</x:v>
+        <x:v>The public data does not contain an independent IVS valuation.</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
         <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>Application of the valuation boundary stated in the framework.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
+        <x:v>Commission an independent IP valuation and, if relevant, an enterprise valuation with scenarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
+        <x:v>The public data does not demonstrate realised licence or damages cash flow.</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
+        <x:v>The absence is recorded as a readiness blocker.</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>site/data/atlas.json (readiness.blockers)</x:v>
       </x:c>
       <x:c r="E41" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
-        <x:v>Analytical separation of the value concepts.</x:v>
+        <x:v>Absence check against the public package.</x:v>
       </x:c>
       <x:c r="G41" s="14" t="str">
         <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H41" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I41" s="14" t="str">
-        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
+        <x:v>Provide signed agreements, invoices, proof of payment and reconciliation of receivables.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
+        <x:v>The public data does not confirm test results or independent technical validation.</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>Commercialisation model</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
+        <x:v>The patent specification describes the solution, but the package contains no separate test register.</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
+        <x:v>site/data/patent-history.json</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
-        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
+        <x:v>Absence check in relation to any technical performance claim.</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
+        <x:v>A patent publication is not treated as a product test report.</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
+        <x:v>Provide a test protocol, independent laboratory evidence, results and raw data.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
+        <x:v>The public data does not confirm pilots or named customer evidence.</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Validation</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
+        <x:v>The public evidence register contains no validated pilot or customer evidence.</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
-        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
+        <x:v>site/data/evidence.csv</x:v>
       </x:c>
       <x:c r="E43" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
-        <x:v>Financing principle.</x:v>
+        <x:v>Absence check against the public evidence register.</x:v>
       </x:c>
       <x:c r="G43" s="14" t="str">
-        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
+        <x:v>No company-level customer or pilot evidence is inferred.</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I43" s="14" t="str">
-        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
+        <x:v>Provide signed pilot documents, delivery evidence, customer references and usage data.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="58.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
+        <x:v>The public data does not confirm current country-level title, renewal-fee status or absence of encumbrances across the family.</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>IP status</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
+        <x:v>Family publications do not establish current national post-grant status.</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
-        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
+        <x:v>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=legal ; https://www.epo.org/en/applying/european/validation</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>2026-08-14</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
-        <x:v>Diligence alert derived directly from the official API record.</x:v>
+        <x:v>Identification of the legal due-diligence limitation.</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
+        <x:v>Checks in four registers do not establish status across the full family.</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
+        <x:v>Provide a counsel-signed country matrix, current official extracts, renewal receipts and encumbrance evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="58.5" customHeight="1">
       <x:c r="A45" s="14" t="str">
-        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
+        <x:v>The public data contains no country-specific product-to-claim mappings.</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Technical differentiation</x:v>
       </x:c>
       <x:c r="C45" s="14" t="str">
-        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
+        <x:v>The published guardrail requires a counsel-reviewed claim chart before infringement conclusions.</x:v>
       </x:c>
       <x:c r="D45" s="14" t="str">
-        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
+        <x:v>https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
       </x:c>
       <x:c r="E45" s="14" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F45" s="14" t="str">
-        <x:v>Direct observation from the official register.</x:v>
+        <x:v>Absence check for product-feature mapping to operative claim limitations.</x:v>
       </x:c>
       <x:c r="G45" s="14" t="str">
-        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
+        <x:v>Product similarity is not treated as evidence of infringement.</x:v>
       </x:c>
       <x:c r="H45" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I45" s="14" t="str">
-        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
+        <x:v>Obtain identified products, chain of custody, teardown evidence and counsel-reviewed claim charts.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="58.5" customHeight="1">
       <x:c r="A46" s="14" t="str">
-        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
+        <x:v>Total market value is not automatically the royalty base.</x:v>
       </x:c>
       <x:c r="B46" s="14" t="str">
-        <x:v>Risks</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C46" s="14" t="str">
-        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
+        <x:v>The valuation framework separates total market, addressable sales and cash flow.</x:v>
       </x:c>
       <x:c r="D46" s="14" t="str">
-        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E46" s="14" t="str">
-        <x:v>2026-12-04</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F46" s="14" t="str">
-        <x:v>Check of the official maintenance-fee window.</x:v>
+        <x:v>Application of the valuation boundary stated in the framework.</x:v>
       </x:c>
       <x:c r="G46" s="14" t="str">
-        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
+        <x:v>A royalty base requires geographic, temporal and product-level relevance to the claims.</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I46" s="14" t="str">
-        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
+        <x:v>Build a bridge from total market to addressable, in-scope and claim-mapped sales.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="58.5" customHeight="1">
       <x:c r="A47" s="14" t="str">
-        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
+        <x:v>Patent value, enterprise value, equity value and collateral value are distinct metrics.</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
-        <x:v>Financial model</x:v>
+        <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
-        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
+        <x:v>WIPO valuation and IP-financing frameworks, together with the published guardrail, require the value concepts to be separated.</x:v>
       </x:c>
       <x:c r="D47" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/en/web/business/ip-valuation ; https://www.wipo.int/en/web/ip-financing</x:v>
       </x:c>
       <x:c r="E47" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F47" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Analytical separation of the value concepts.</x:v>
       </x:c>
       <x:c r="G47" s="14" t="str">
-        <x:v>No company-level financial conclusion is drawn.</x:v>
+        <x:v>No assumptions.</x:v>
       </x:c>
       <x:c r="H47" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I47" s="14" t="str">
-        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
+        <x:v>Separate legal and economic analysis is required for each value concept.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="58.5" customHeight="1">
       <x:c r="A48" s="14" t="str">
-        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+        <x:v>A counsel-led limited licensing or settlement pilot is a possible commercialisation hypothesis.</x:v>
       </x:c>
       <x:c r="B48" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Commercialisation model</x:v>
       </x:c>
       <x:c r="C48" s="14" t="str">
-        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+        <x:v>The proposed route uses staged hard gates, claim charts and auditable outreach.</x:v>
       </x:c>
       <x:c r="D48" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/business/settle-ip-disputes ; https://www.epo.org/en/searching-for-patents/business/ipscore</x:v>
       </x:c>
       <x:c r="E48" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F48" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>A proposed hypothesis, not evidence of realised commercialisation.</x:v>
       </x:c>
       <x:c r="G48" s="14" t="str">
-        <x:v>No amount, maturity or security package is assumed.</x:v>
+        <x:v>Targets would be selected only after legal and evidence gates are satisfied.</x:v>
       </x:c>
       <x:c r="H48" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Assumption</x:v>
       </x:c>
       <x:c r="I48" s="14" t="str">
-        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+        <x:v>Management and patent-counsel approval are required, and cost, responses and terms must be documented.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="58.5" customHeight="1">
       <x:c r="A49" s="14" t="str">
-        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+        <x:v>Patent-backed financing should be assessed only on the basis of confirmed rights and cash flows.</x:v>
       </x:c>
       <x:c r="B49" s="14" t="str">
         <x:v>Financing thesis</x:v>
       </x:c>
       <x:c r="C49" s="14" t="str">
-        <x:v>The public package is limited to market and patent material.</x:v>
+        <x:v>WIPO IP Finance and phase 5 of the patent history.</x:v>
       </x:c>
       <x:c r="D49" s="14" t="str">
-        <x:v>Public package scope</x:v>
+        <x:v>https://www.wipo.int/en/web/ip-financing ; https://www.wipo.int/en/web/business/ip-valuation</x:v>
       </x:c>
       <x:c r="E49" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F49" s="14" t="str">
-        <x:v>Absence check against the scope of the public package.</x:v>
+        <x:v>Financing principle.</x:v>
       </x:c>
       <x:c r="G49" s="14" t="str">
-        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+        <x:v>The current material does not demonstrate an existing collateral value.</x:v>
       </x:c>
       <x:c r="H49" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I49" s="14" t="str">
-        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+        <x:v>Independent valuation, rights due diligence, realised or contracted cash flow and downside analysis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="58.5" customHeight="1">
       <x:c r="A50" s="14" t="str">
-        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+        <x:v>The next Australian renewal must be confirmed immediately.</x:v>
       </x:c>
       <x:c r="B50" s="14" t="str">
-        <x:v>Competition</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C50" s="14" t="str">
-        <x:v>Patent and case materials are not a competition map.</x:v>
+        <x:v>The official API records the patent as GRANTED, the latest renewal on 18 July 2025 and an in-force date of 14 August 2026.</x:v>
       </x:c>
       <x:c r="D50" s="14" t="str">
-        <x:v>site/data/patent-history.json</x:v>
+        <x:v>https://production.api.ipaustralia.gov.au/public/ipright-search-api/v1/patents/2014307829</x:v>
       </x:c>
       <x:c r="E50" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-08-14</x:v>
       </x:c>
       <x:c r="F50" s="14" t="str">
-        <x:v>Absence check against the public package.</x:v>
+        <x:v>Diligence alert derived directly from the official API record.</x:v>
       </x:c>
       <x:c r="G50" s="14" t="str">
-        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+        <x:v>The recorded in-force-through date is not asserted to be the statutory payment deadline.</x:v>
       </x:c>
       <x:c r="H50" s="14" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I50" s="14" t="str">
-        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+        <x:v>The patent administrator or Australian counsel must confirm the statutory date, amount, authority and payment, and archive the receipt and current extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="58.5" customHeight="1">
       <x:c r="A51" s="14" t="str">
-        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+        <x:v>The Finnish register records the 14th-year fee as due on 31 August 2026.</x:v>
       </x:c>
       <x:c r="B51" s="14" t="str">
-        <x:v>Customers</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C51" s="14" t="str">
-        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+        <x:v>PRH records the 14th-year EUR 670 fee as due on 31 August 2026, with a late-payment period through 28 February 2027.</x:v>
       </x:c>
       <x:c r="D51" s="14" t="str">
-        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+        <x:v>https://patenttitietopalvelu.prh.fi/en/patent/20135829</x:v>
       </x:c>
       <x:c r="E51" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="F51" s="14" t="str">
-        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+        <x:v>Direct observation from the official register.</x:v>
       </x:c>
       <x:c r="G51" s="14" t="str">
-        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+        <x:v>The ordinary deadline is the target rather than the late-payment period.</x:v>
       </x:c>
       <x:c r="H51" s="14" t="str">
-        <x:v>Assumption</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I51" s="14" t="str">
-        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+        <x:v>Pay by the ordinary deadline and archive the receipt and updated register extract.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="58.5" customHeight="1">
       <x:c r="A52" s="14" t="str">
-        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+        <x:v>The US 7.5-year maintenance-fee status must be confirmed.</x:v>
       </x:c>
       <x:c r="B52" s="14" t="str">
-        <x:v>Financing thesis</x:v>
+        <x:v>Risks</x:v>
       </x:c>
       <x:c r="C52" s="14" t="str">
-        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+        <x:v>The official route shows that the no-surcharge window ends on 4 December 2026. Payment was not independently confirmed from the reviewed public material.</x:v>
       </x:c>
       <x:c r="D52" s="14" t="str">
-        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+        <x:v>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</x:v>
       </x:c>
       <x:c r="E52" s="14" t="str">
-        <x:v>2026-07-24</x:v>
+        <x:v>2026-12-04</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+        <x:v>Check of the official maintenance-fee window.</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+        <x:v>The public record reviewed here does not establish whether the fee has been paid or remains unpaid.</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+        <x:v>US counsel must confirm entity status, amount and payment, and archive receipts and assignment records.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="58.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+        <x:v>The public data lacks audited historical financial statements and a cash-flow forecast.</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Financial model</x:v>
       </x:c>
       <x:c r="C53" s="14" t="str">
-        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+        <x:v>The market and patent dataset does not contain company financial statements.</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+        <x:v>Public package scope</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F53" s="14" t="str">
-        <x:v>Count of countries in each evidence grade.</x:v>
+        <x:v>Absence check against the scope of the public package.</x:v>
       </x:c>
       <x:c r="G53" s="14" t="str">
-        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+        <x:v>No company-level financial conclusion is drawn.</x:v>
       </x:c>
       <x:c r="H53" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Missing</x:v>
       </x:c>
       <x:c r="I53" s="14" t="str">
-        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+        <x:v>Provide 3–5 years of financial statements, the current general ledger, budget, cash-flow forecast, debt schedule and tax-debt certificate.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="58.5" customHeight="1">
       <x:c r="A54" s="14" t="str">
+        <x:v>The public data does not specify the funding need, use of funds or repayment source.</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>The public package does not state the requested amount, intended use or repayment structure.</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="str">
+        <x:v>No amount, maturity or security package is assumed.</x:v>
+      </x:c>
+      <x:c r="H54" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I54" s="14" t="str">
+        <x:v>Provide the amount, use of funds, maturity, amortisation, repayment source and proposed covenants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="58.5" customHeight="1">
+      <x:c r="A55" s="14" t="str">
+        <x:v>The public data does not show the share capital, cap table or share encumbrances.</x:v>
+      </x:c>
+      <x:c r="B55" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C55" s="14" t="str">
+        <x:v>The public package is limited to market and patent material.</x:v>
+      </x:c>
+      <x:c r="D55" s="14" t="str">
+        <x:v>Public package scope</x:v>
+      </x:c>
+      <x:c r="E55" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F55" s="14" t="str">
+        <x:v>Absence check against the scope of the public package.</x:v>
+      </x:c>
+      <x:c r="G55" s="14" t="str">
+        <x:v>No conclusion is drawn about ownership or vulnerability to competing claims.</x:v>
+      </x:c>
+      <x:c r="H55" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I55" s="14" t="str">
+        <x:v>Provide a certified shareholder register, articles, resolutions and a share-pledge and encumbrance statement in a closed data room.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="58.5" customHeight="1">
+      <x:c r="A56" s="14" t="str">
+        <x:v>The public data lacks a comparable analysis of competitors and alternatives.</x:v>
+      </x:c>
+      <x:c r="B56" s="14" t="str">
+        <x:v>Competition</x:v>
+      </x:c>
+      <x:c r="C56" s="14" t="str">
+        <x:v>Patent and case materials are not a competition map.</x:v>
+      </x:c>
+      <x:c r="D56" s="14" t="str">
+        <x:v>site/data/patent-history.json</x:v>
+      </x:c>
+      <x:c r="E56" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F56" s="14" t="str">
+        <x:v>Absence check against the public package.</x:v>
+      </x:c>
+      <x:c r="G56" s="14" t="str">
+        <x:v>Competition is kept separate from patent overlap and from non-patented alternatives.</x:v>
+      </x:c>
+      <x:c r="H56" s="14" t="str">
+        <x:v>Missing</x:v>
+      </x:c>
+      <x:c r="I56" s="14" t="str">
+        <x:v>Map products, manufacturers, technologies, patent families, prices and claim-map status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="58.5" customHeight="1">
+      <x:c r="A57" s="14" t="str">
+        <x:v>Manufacturers, technology providers and IP financiers are preliminary customer segments.</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>Customers</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>The reviewed commercialisation routes include licensing, assignment and IP finance.</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>https://www.wipo.int/ja/web/business/assignment-licensing ; https://www.wipo.int/en/web/ip-financing</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F57" s="14" t="str">
+        <x:v>Preliminary segmentation hypothesis based on the identified commercialisation routes.</x:v>
+      </x:c>
+      <x:c r="G57" s="14" t="str">
+        <x:v>There is no verified purchase intent or validated customer base.</x:v>
+      </x:c>
+      <x:c r="H57" s="14" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="I57" s="14" t="str">
+        <x:v>Validate the segments through 10–15 structured buyer and financier interviews and document their purchase criteria.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="58.5" customHeight="1">
+      <x:c r="A58" s="14" t="str">
+        <x:v>The German decisions can serve as an evidence anchor, not as a worldwide infringement determination.</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>Financing thesis</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>The decisions are limited to a country, products, parties and period.</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>https://www.rechtsprechung-im-internet.de/jportal/?quelle=jlink&amp;docid=JURE269032275&amp;psml=bsjrsprod.psml ; https://www.gesetze-bayern.de/Content/Document/Y-300-Z-BECKRS-B-2026-N-14206</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F58" s="14" t="str">
+        <x:v>Application of the territorial and case-specific limits of the decisions.</x:v>
+      </x:c>
+      <x:c r="G58" s="14" t="str">
+        <x:v>Other countries depend on local rights and the products examined there.</x:v>
+      </x:c>
+      <x:c r="H58" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I58" s="14" t="str">
+        <x:v>Country-specific legal and claim packages are required before outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="58.5" customHeight="1">
+      <x:c r="A59" s="14" t="str">
+        <x:v>Five countries are graded A and 158 countries are graded D.</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>Market size</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>Classes: A 5, B 13, C 19, D 158.</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>site/data/atlas.json (summary.gradeCounts)</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="F59" s="14" t="str">
+        <x:v>Count of countries in each evidence grade.</x:v>
+      </x:c>
+      <x:c r="G59" s="14" t="str">
+        <x:v>Evidence maturity is not treated as market attractiveness.</x:v>
+      </x:c>
+      <x:c r="H59" s="14" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I59" s="14" t="str">
+        <x:v>Prioritise Grade D data requests by economic size, patent relevance and regulatory fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="58.5" customHeight="1">
+      <x:c r="A60" s="14" t="str">
         <x:v>No global atlas estimate has been approved for publication.</x:v>
       </x:c>
-      <x:c r="B54" s="14" t="str">
+      <x:c r="B60" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
-      <x:c r="C54" s="14" t="str">
+      <x:c r="C60" s="14" t="str">
         <x:v>Zero accepted donors is below the minimum of three. Each of the five published New Zealand, EU, Canada, Germany and United States candidates has at least one failed or open D1–D10 criterion; the regional and regulatory-archetype coverage gates also remain unmet.</x:v>
       </x:c>
-      <x:c r="D54" s="14" t="str">
+      <x:c r="D60" s="14" t="str">
         <x:v>site/data/market-values.json (modelReadiness, donorProtocol and donorCandidates)</x:v>
       </x:c>
-      <x:c r="E54" s="14" t="str">
+      <x:c r="E60" s="14" t="str">
         <x:v>2026-07-27</x:v>
       </x:c>
-      <x:c r="F54" s="14" t="str">
+      <x:c r="F60" s="14" t="str">
         <x:v>Hard gate: every donor must pass D1–D10, and at least three compatible donors plus both coverage gates are required.</x:v>
       </x:c>
-      <x:c r="G54" s="14" t="str">
+      <x:c r="G60" s="14" t="str">
         <x:v>Official lower bounds and external benchmarks remain useful cross-checks but are not counted as accepted donors.</x:v>
       </x:c>
-      <x:c r="H54" s="14" t="str">
+      <x:c r="H60" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
-      <x:c r="I54" s="14" t="str">
+      <x:c r="I60" s="14" t="str">
         <x:v>Do not publish a single global value before the methodology gates are met.</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="58.5" customHeight="1">
-      <x:c r="A55" s="15" t="str">
+    <x:row r="61" ht="58.5" customHeight="1">
+      <x:c r="A61" s="15" t="str">
         <x:v>A high-confidence financing package requires a closed data room alongside the public package.</x:v>
       </x:c>
-      <x:c r="B55" s="15" t="str">
+      <x:c r="B61" s="15" t="str">
         <x:v>Next steps</x:v>
       </x:c>
-      <x:c r="C55" s="15" t="str">
+      <x:c r="C61" s="15" t="str">
         <x:v>The public package documents sources and gaps but does not contain confidential financial, contractual or complete title evidence.</x:v>
       </x:c>
-      <x:c r="D55" s="15" t="str">
+      <x:c r="D61" s="15" t="str">
         <x:v>Public package scope</x:v>
       </x:c>
-      <x:c r="E55" s="15" t="str">
+      <x:c r="E61" s="15" t="str">
         <x:v>2026-07-24</x:v>
       </x:c>
-      <x:c r="F55" s="15" t="str">
+      <x:c r="F61" s="15" t="str">
         <x:v>Recommendation based on the due-diligence architecture required by the identified gaps.</x:v>
       </x:c>
-      <x:c r="G55" s="15" t="str">
+      <x:c r="G61" s="15" t="str">
         <x:v>Access would be restricted and logged.</x:v>
       </x:c>
-      <x:c r="H55" s="15" t="str">
+      <x:c r="H61" s="15" t="str">
         <x:v>Supported</x:v>
       </x:c>
-      <x:c r="I55" s="15" t="str">
+      <x:c r="I61" s="15" t="str">
         <x:v>Create an indexed data room with Corporate, IP, Legal, Commercial, Finance, Valuation and Security sections.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="H2:H55">
+  <x:conditionalFormatting sqref="H2:H61">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Supported"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Assumption"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H55">
+    <x:dataValidation type="list" sqref="H2:H61">
       <x:formula1>"Confirmed,Supported,Assumption,Missing"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c08f8d02c4e42d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f964f126ca9443a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2245,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.27-30</x:v>
+        <x:v>2026.07.28-32</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2253,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2269,8 +2443,8 @@
         <x:v>Evidence rows</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>COUNTA('Evidence Register'!$A$2:$A$55)</x:f>
-        <x:v>54</x:v>
+        <x:f>COUNTA('Evidence Register'!$A$2:$A$61)</x:f>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20.25" customHeight="1"/>
@@ -2285,8 +2459,8 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A11)</x:f>
-        <x:v>29</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A11)</x:f>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2294,8 +2468,8 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A12)</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A12)</x:f>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2303,7 +2477,7 @@
         <x:v>Assumption</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A13)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A13)</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -2312,7 +2486,7 @@
         <x:v>Missing</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
-        <x:f>COUNTIF('Evidence Register'!$H$2:$H$55,A14)</x:f>
+        <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A14)</x:f>
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -2497,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8624f172681e4db4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17d2109462c24865"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3411,7 +3585,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3428,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3445,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3462,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3479,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3496,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3513,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3530,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3547,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3564,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3581,7 +3755,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3598,7 +3772,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3615,7 +3789,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3632,7 +3806,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3649,7 +3823,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3666,7 +3840,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3683,7 +3857,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3700,7 +3874,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3717,7 +3891,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3734,7 +3908,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3751,7 +3925,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3768,7 +3942,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3785,7 +3959,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3802,7 +3976,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3819,7 +3993,7 @@
         <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -3836,63 +4010,63 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -3901,32 +4075,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
         <x:v>health.govt.nz</x:v>
@@ -3935,49 +4109,49 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C85" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C86" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -3986,50 +4160,67 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B88" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C88" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D88" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E88" s="14" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="31.5" customHeight="1">
+      <x:c r="A89" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B88" s="14" t="str">
+      <x:c r="B89" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C88" s="14" t="str">
+      <x:c r="C89" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D88" s="14" t="str">
+      <x:c r="D89" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="31.5" customHeight="1">
-      <x:c r="A89" s="15" t="str">
+      <x:c r="E89" s="14" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="31.5" customHeight="1">
+      <x:c r="A90" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B89" s="15" t="str">
+      <x:c r="B90" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C89" s="15" t="str">
+      <x:c r="C90" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D89" s="15" t="str">
+      <x:c r="D90" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E89" s="15" t="str">
-        <x:v>2026-07-27</x:v>
+      <x:c r="E90" s="15" t="str">
+        <x:v>2026-07-28</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5230952edacc4016"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R892c33906a724eb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6075,7 +6266,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a75602b0ac42de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9552970be04e4295"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v35 mail and daily evidence update
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R04994ae7b0a248b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R43a72eb45d5d45da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R41543393e6e24031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra98da52778db4e33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R32afc492ea9547c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Reb6a694f75184ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re5c1182cab6e45f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1426fb9bf7804ca3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R41d70ab5aaff419c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb59fd997face46e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E90" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -986,31 +986,31 @@
     </x:row>
     <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>Luxembourg has an excise and fiscal-mark method starting on 2024-10-01; no retail market value has been computed.</x:v>
+        <x:v>Luxembourg has an excise and fiscal-mark method starting on 2024-10-01, but the official response confirms that the requested consumption-release volumes, excise revenue and category statistics are unavailable; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size / Luxembourg</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>The official rate is EUR 0.12 per ml from 2024-10-01, and fiscal marks carry liquid volume and mandatory consumer price.</x:v>
+        <x:v>The authority supplied no volume or excise-revenue series and does not distinguish the requested product categories. It identified the official registered retail-price list, which is only a price and fiscal-mark reference.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Luxembourg)</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf ; source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Luxembourg)</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Taxed litres = e-liquid-specific net excise / EUR 120 per litre; marked consumer-price value = sum(marked pack quantity × mandatory marked price).</x:v>
+        <x:v>No calculation: the price list is not multiplied by unverified pack counts, and the tax rate is not inverted without net excise receipts.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>The volume and fiscal-mark calculations are not additive; foreign B2B dispatches, destruction, refunds and corrections are separated.</x:v>
+        <x:v>A missing authority aggregate is not treated as zero. The price list does not establish sales, volume, release for consumption or consumer demand.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>The national aggregate, fiscal-mark quantity and price fields, sell-through and period finality are missing; retailValueStatus is not_computed.</x:v>
+        <x:v>Annual taxable millilitres, excise revenue, fiscal-mark pack counts, device units, sell-through and period finality are missing; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58.5" customHeight="1">
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f964f126ca9443a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7eb99bd974ab1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.28-32</x:v>
+        <x:v>2026.07.29-35</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17d2109462c24865"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref80ab36b6774155"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,7 +3585,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3602,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3619,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3636,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3653,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3670,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3687,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3704,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3721,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3738,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3755,7 +3755,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3772,7 +3772,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3789,7 +3789,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3806,7 +3806,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3823,7 +3823,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3840,7 +3840,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3857,7 +3857,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3874,7 +3874,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3891,7 +3891,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3908,7 +3908,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3925,7 +3925,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3942,7 +3942,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3959,7 +3959,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3976,7 +3976,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3993,97 +3993,97 @@
         <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>douanes.public.lu</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>adm.gov.it</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -4092,32 +4092,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C84" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
         <x:v>health.govt.nz</x:v>
@@ -4126,49 +4126,49 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C86" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C87" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B88" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -4177,50 +4177,67 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D88" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
       <x:c r="A89" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B89" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C89" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D89" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E89" s="14" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="31.5" customHeight="1">
+      <x:c r="A90" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B89" s="14" t="str">
+      <x:c r="B90" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C89" s="14" t="str">
+      <x:c r="C90" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D89" s="14" t="str">
+      <x:c r="D90" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-28</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="31.5" customHeight="1">
-      <x:c r="A90" s="15" t="str">
+      <x:c r="E90" s="14" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="31.5" customHeight="1">
+      <x:c r="A91" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B90" s="15" t="str">
+      <x:c r="B91" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C90" s="15" t="str">
+      <x:c r="C91" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D90" s="15" t="str">
+      <x:c r="D91" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E90" s="15" t="str">
-        <x:v>2026-07-28</x:v>
+      <x:c r="E91" s="15" t="str">
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R892c33906a724eb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4613b5b2125c40e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6266,7 +6283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9552970be04e4295"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cda5e154f2c4bbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v35 official-response and daily-package update (#32)
Publish the privacy-safe authority-response deltas, conditional Germany extract status, aligned v35 dashboard and six once-daily package downloads. No purchase, fee, subscription, donor decision or market total is accepted or changed.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R04994ae7b0a248b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R43a72eb45d5d45da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R41543393e6e24031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra98da52778db4e33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R32afc492ea9547c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Reb6a694f75184ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re5c1182cab6e45f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1426fb9bf7804ca3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R41d70ab5aaff419c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb59fd997face46e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E90" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -986,31 +986,31 @@
     </x:row>
     <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>Luxembourg has an excise and fiscal-mark method starting on 2024-10-01; no retail market value has been computed.</x:v>
+        <x:v>Luxembourg has an excise and fiscal-mark method starting on 2024-10-01, but the official response confirms that the requested consumption-release volumes, excise revenue and category statistics are unavailable; no retail market value has been computed.</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>Market size / Luxembourg</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>The official rate is EUR 0.12 per ml from 2024-10-01, and fiscal marks carry liquid volume and mandatory consumer price.</x:v>
+        <x:v>The authority supplied no volume or excise-revenue series and does not distinguish the requested product categories. It identified the official registered retail-price list, which is only a price and fiscal-mark reference.</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Luxembourg)</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf ; source/FIVE_COUNTRY_METHOD_SPRINT_2026-07-27.md (Luxembourg)</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Taxed litres = e-liquid-specific net excise / EUR 120 per litre; marked consumer-price value = sum(marked pack quantity × mandatory marked price).</x:v>
+        <x:v>No calculation: the price list is not multiplied by unverified pack counts, and the tax rate is not inverted without net excise receipts.</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>The volume and fiscal-mark calculations are not additive; foreign B2B dispatches, destruction, refunds and corrections are separated.</x:v>
+        <x:v>A missing authority aggregate is not treated as zero. The price list does not establish sales, volume, release for consumption or consumer demand.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>The national aggregate, fiscal-mark quantity and price fields, sell-through and period finality are missing; retailValueStatus is not_computed.</x:v>
+        <x:v>Annual taxable millilitres, excise revenue, fiscal-mark pack counts, device units, sell-through and period finality are missing; retailValueStatus is not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58.5" customHeight="1">
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f964f126ca9443a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7eb99bd974ab1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.28-32</x:v>
+        <x:v>2026.07.29-35</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17d2109462c24865"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref80ab36b6774155"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,7 +3585,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3602,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3619,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3636,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3653,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3670,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3687,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3704,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3721,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3738,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3755,7 +3755,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3772,7 +3772,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3789,7 +3789,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3806,7 +3806,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3823,7 +3823,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3840,7 +3840,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3857,7 +3857,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3874,7 +3874,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3891,7 +3891,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3908,7 +3908,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3925,7 +3925,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3942,7 +3942,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3959,7 +3959,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3976,7 +3976,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3993,97 +3993,97 @@
         <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>douanes.public.lu</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>adm.gov.it</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -4092,32 +4092,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C84" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
         <x:v>health.govt.nz</x:v>
@@ -4126,49 +4126,49 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C86" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C87" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>UN-MEMBER-STATES</x:v>
       </x:c>
       <x:c r="B88" s="14" t="str">
         <x:v>United Nations</x:v>
@@ -4177,50 +4177,67 @@
         <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D88" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
       <x:c r="A89" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B89" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C89" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D89" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E89" s="14" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="31.5" customHeight="1">
+      <x:c r="A90" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B89" s="14" t="str">
+      <x:c r="B90" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C89" s="14" t="str">
+      <x:c r="C90" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D89" s="14" t="str">
+      <x:c r="D90" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-28</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="31.5" customHeight="1">
-      <x:c r="A90" s="15" t="str">
+      <x:c r="E90" s="14" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="31.5" customHeight="1">
+      <x:c r="A91" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B90" s="15" t="str">
+      <x:c r="B91" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C90" s="15" t="str">
+      <x:c r="C91" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D90" s="15" t="str">
+      <x:c r="D91" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E90" s="15" t="str">
-        <x:v>2026-07-28</x:v>
+      <x:c r="E91" s="15" t="str">
+        <x:v>2026-07-29</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R892c33906a724eb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4613b5b2125c40e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6266,7 +6283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9552970be04e4295"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cda5e154f2c4bbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v36 Canada tax-basis clarification
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Reb6a694f75184ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re5c1182cab6e45f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1426fb9bf7804ca3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R41d70ab5aaff419c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb59fd997face46e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R3653e33f3e5a42e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R73247874e00f4b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rb921ca5a204a4012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R73b8d62659824bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rbef0ecddc797410e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1372,16 +1372,16 @@
         <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_RCS_TAX_BASIS_CLARIFICATION_2026-07-29.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>D8 passes: CAD, exclusion of GST/HST/PST/QST and inclusion of additional duties embedded in retail prices are confirmed for table 20-10-0071-01. The exact duty components and monthly and legacy-table tax bases remain under clarification. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
         <x:v>Supported</x:v>
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7eb99bd974ab1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2031e0156924472"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.29-35</x:v>
+        <x:v>2026.07.30-36</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref80ab36b6774155"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R361b2d8017b64e66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,7 +3585,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3602,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3619,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3636,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3653,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3670,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3687,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3704,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3721,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3738,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3755,7 +3755,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3772,7 +3772,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3789,7 +3789,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3806,7 +3806,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3823,7 +3823,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3840,7 +3840,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3857,7 +3857,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3874,7 +3874,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3891,7 +3891,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3908,7 +3908,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3925,7 +3925,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3942,7 +3942,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3959,7 +3959,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3976,7 +3976,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3993,7 +3993,7 @@
         <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -4010,7 +4010,7 @@
         <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
@@ -4027,7 +4027,7 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
@@ -4044,7 +4044,7 @@
         <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
@@ -4061,7 +4061,7 @@
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
@@ -4078,7 +4078,7 @@
         <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
@@ -4095,7 +4095,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
@@ -4112,7 +4112,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
@@ -4129,7 +4129,7 @@
         <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
@@ -4146,7 +4146,7 @@
         <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
@@ -4163,7 +4163,7 @@
         <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
@@ -4180,7 +4180,7 @@
         <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
@@ -4197,7 +4197,7 @@
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="31.5" customHeight="1">
@@ -4214,7 +4214,7 @@
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
       <x:c r="E90" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="31.5" customHeight="1">
@@ -4231,13 +4231,13 @@
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
       <x:c r="E91" s="15" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4613b5b2125c40e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f772ce103d44c71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6283,7 +6283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cda5e154f2c4bbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516ea67dac564bc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v36 Canada tax-basis clarification (#33)
Co-authored-by: jounirautio78-ops <jounirautio78-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Reb6a694f75184ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re5c1182cab6e45f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R1426fb9bf7804ca3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R41d70ab5aaff419c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rb59fd997face46e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R3653e33f3e5a42e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R73247874e00f4b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rb921ca5a204a4012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R73b8d62659824bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rbef0ecddc797410e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1372,16 +1372,16 @@
         <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_RCS_TAX_BASIS_CLARIFICATION_2026-07-29.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>D8 passes: CAD and exclusion of GST/HST, provincial sales taxes and excise are source-linked. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>D8 passes: CAD, exclusion of GST/HST/PST/QST and inclusion of additional duties embedded in retail prices are confirmed for table 20-10-0071-01. The exact duty components and monthly and legacy-table tax bases remain under clarification. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
         <x:v>Supported</x:v>
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7eb99bd974ab1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2031e0156924472"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.29-35</x:v>
+        <x:v>2026.07.30-36</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref80ab36b6774155"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R361b2d8017b64e66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,7 +3585,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3602,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3619,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3636,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3653,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3670,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3687,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3704,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3721,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3738,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3755,7 +3755,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
@@ -3772,7 +3772,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
@@ -3789,7 +3789,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
@@ -3806,7 +3806,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
@@ -3823,7 +3823,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
@@ -3840,7 +3840,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
@@ -3857,7 +3857,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
@@ -3874,7 +3874,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
@@ -3891,7 +3891,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
@@ -3908,7 +3908,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
@@ -3925,7 +3925,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
@@ -3942,7 +3942,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
@@ -3959,7 +3959,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
@@ -3976,7 +3976,7 @@
         <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
@@ -3993,7 +3993,7 @@
         <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
@@ -4010,7 +4010,7 @@
         <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
@@ -4027,7 +4027,7 @@
         <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
@@ -4044,7 +4044,7 @@
         <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
@@ -4061,7 +4061,7 @@
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
@@ -4078,7 +4078,7 @@
         <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
@@ -4095,7 +4095,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
@@ -4112,7 +4112,7 @@
         <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
@@ -4129,7 +4129,7 @@
         <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
@@ -4146,7 +4146,7 @@
         <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
@@ -4163,7 +4163,7 @@
         <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
@@ -4180,7 +4180,7 @@
         <x:v>https://www.un.org/en/about-us/member-states</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
@@ -4197,7 +4197,7 @@
         <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
       </x:c>
       <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="31.5" customHeight="1">
@@ -4214,7 +4214,7 @@
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
       <x:c r="E90" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="31.5" customHeight="1">
@@ -4231,13 +4231,13 @@
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
       <x:c r="E91" s="15" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-30</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4613b5b2125c40e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f772ce103d44c71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6283,7 +6283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cda5e154f2c4bbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516ea67dac564bc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v37 Canada closure and donor controls
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R3653e33f3e5a42e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R73247874e00f4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rb921ca5a204a4012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R73b8d62659824bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rbef0ecddc797410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6cfd5a0345244ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8cd41972a2f147b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rdf6fee85d1354963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5b240c5013ab4964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R21dd5aa9add24763"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -1198,16 +1198,16 @@
         <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_DONOR_FOLLOWUP_PACK_2026-08-07.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="F22" s="17" t="str">
         <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
+        <x:v>The deterministic scope rules are public. RPS collects product types and quantities but no observed retail value. The GST basis is unknown. Stats NZ's final 2024 HS10 control is a customs-stage sensitivity, not independent retail reconciliation.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Supported</x:v>
@@ -1372,22 +1372,22 @@
         <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_RCS_TAX_BASIS_CLARIFICATION_2026-07-29.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_RCS_TAX_BASIS_CLARIFICATION_2026-07-29.md ; source/CANADA_RCS_SCOPE_QUALITY_CLARIFICATION_2026-07-30.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>D8 passes: CAD, exclusion of GST/HST/PST/QST and inclusion of additional duties embedded in retail prices are confirmed for table 20-10-0071-01. The exact duty components and monthly and legacy-table tax bases remain under clarification. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>D8 passes: CAD, exclusion of GST/HST/PST/QST and inclusion of embedded additional duties are confirmed for the reviewed quarterly, monthly and archived tables. Additional duties can include federal, additional and provincial vaping duties. The monthly route is same-survey QA, not D10.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
+        <x:v>D5 failed because NAICS 459999 specialist retail is outside the confirmed 441100–459993 target range. D7 failed because exact product-class quality and annual-uncertainty information is unavailable. D10 remains open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
@@ -1566,31 +1566,31 @@
     </x:row>
     <x:row r="35" ht="58.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable broad vaporisation-device-group units and 62,500 derived taxable component sets; neither is e-cigarette-specific.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
+        <x:v>The official response reports PLN 993.1 million for e-liquids, PLN 175.3 million for the broad device group and PLN 2.5 million for component sets. The statutory group includes refillable e-cigarettes, heated-tobacco heaters and multifunction devices. Duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/ ; https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego ; https://api.sejm.gov.pl/eli/acts/DU/2025/698/text.pdf ; source/POLAND_D1_D10_PREASSESSMENT_2026-07-31.md</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable broad-group units; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. AKC-4/R requires device-type detail, but the current public aggregate does not publish it. The values do not establish consumer prices, retail sales or an e-cigarette-only count.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
+        <x:v>The AKC-4/R e-cigarette/heater/multifunction split, monthly duty profile, retail prices, channel coverage and independent reconciliation are required. Poland receives no donor score without a country-year retail value.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58.5" customHeight="1">
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2031e0156924472"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954404b7d653401c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.30-36</x:v>
+        <x:v>2026.07.31-37</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A11)</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2469,7 +2469,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A12)</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R361b2d8017b64e66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bdb2db608a14175"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3573,24 +3573,24 @@
     </x:row>
     <x:row r="53" ht="31.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-BC2CDD0708D5</x:v>
+        <x:v>REGISTER-REFERENCE-067A847A44A9</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
-        <x:v>data-api.ecb.europa.eu</x:v>
+        <x:v>api.sejm.gov.pl</x:v>
       </x:c>
       <x:c r="C53" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://api.sejm.gov.pl/eli/acts/DU/2025/698/text.pdf</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
       <x:c r="A54" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7264539499F0</x:v>
+        <x:v>REGISTER-REFERENCE-BC2CDD0708D5</x:v>
       </x:c>
       <x:c r="B54" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3599,15 +3599,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D54" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
       <x:c r="A55" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2580DD0733C9</x:v>
+        <x:v>REGISTER-REFERENCE-7264539499F0</x:v>
       </x:c>
       <x:c r="B55" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3616,15 +3616,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D55" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
       <x:c r="A56" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-38DD93023815</x:v>
+        <x:v>REGISTER-REFERENCE-2580DD0733C9</x:v>
       </x:c>
       <x:c r="B56" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3633,15 +3633,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D56" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
       <x:c r="A57" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-72D82058EA8A</x:v>
+        <x:v>REGISTER-REFERENCE-38DD93023815</x:v>
       </x:c>
       <x:c r="B57" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3650,15 +3650,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D57" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
       <x:c r="A58" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
+        <x:v>REGISTER-REFERENCE-72D82058EA8A</x:v>
       </x:c>
       <x:c r="B58" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3667,15 +3667,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D58" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
       <x:c r="A59" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-ACB549D404B8</x:v>
+        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
       </x:c>
       <x:c r="B59" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3684,15 +3684,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D59" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
       <x:c r="A60" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
+        <x:v>REGISTER-REFERENCE-ACB549D404B8</x:v>
       </x:c>
       <x:c r="B60" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3701,15 +3701,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D60" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
       <x:c r="A61" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
+        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
       </x:c>
       <x:c r="B61" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3718,15 +3718,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D61" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
       <x:c r="A62" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
+        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
       </x:c>
       <x:c r="B62" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3735,15 +3735,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D62" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
       <x:c r="A63" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
       </x:c>
       <x:c r="B63" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3752,15 +3752,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D63" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
       <x:c r="A64" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
       </x:c>
       <x:c r="B64" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3769,15 +3769,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D64" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
       <x:c r="A65" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
       </x:c>
       <x:c r="B65" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3786,15 +3786,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D65" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
       <x:c r="A66" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
       </x:c>
       <x:c r="B66" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3803,15 +3803,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D66" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
       </x:c>
       <x:c r="B67" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3820,15 +3820,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D67" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
       <x:c r="A68" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
       </x:c>
       <x:c r="B68" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3837,15 +3837,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D68" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
       </x:c>
       <x:c r="B69" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3854,15 +3854,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D69" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
       <x:c r="A70" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
       </x:c>
       <x:c r="B70" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3871,15 +3871,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D70" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
       <x:c r="A71" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
       </x:c>
       <x:c r="B71" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3888,15 +3888,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D71" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
       <x:c r="A72" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
       </x:c>
       <x:c r="B72" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3905,15 +3905,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D72" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
       <x:c r="A73" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
+        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
       </x:c>
       <x:c r="B73" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3922,15 +3922,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D73" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
+        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3939,15 +3939,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3956,151 +3956,151 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C76" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>datahelpdesk.worldbank.org</x:v>
+        <x:v>data.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
+        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>douanes.public.lu</x:v>
+        <x:v>datahelpdesk.worldbank.org</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
+        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>douanes.public.lu</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>adm.gov.it</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -4109,32 +4109,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C85" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
         <x:v>health.govt.nz</x:v>
@@ -4143,101 +4143,135 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>REGISTER-REFERENCE-1766C84ECA96</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C87" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-529570B0D6C7</x:v>
       </x:c>
       <x:c r="B88" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C88" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D88" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
       <x:c r="A89" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
       </x:c>
       <x:c r="B89" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C89" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D89" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="31.5" customHeight="1">
       <x:c r="A90" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B90" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C90" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D90" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E90" s="14" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="31.5" customHeight="1">
+      <x:c r="A91" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B91" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C91" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D91" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E91" s="14" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="31.5" customHeight="1">
+      <x:c r="A92" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B90" s="14" t="str">
+      <x:c r="B92" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C90" s="14" t="str">
+      <x:c r="C92" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D90" s="14" t="str">
+      <x:c r="D92" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E90" s="14" t="str">
-        <x:v>2026-07-30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="31.5" customHeight="1">
-      <x:c r="A91" s="15" t="str">
+      <x:c r="E92" s="14" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="31.5" customHeight="1">
+      <x:c r="A93" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B91" s="15" t="str">
+      <x:c r="B93" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C91" s="15" t="str">
+      <x:c r="C93" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D91" s="15" t="str">
+      <x:c r="D93" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E91" s="15" t="str">
-        <x:v>2026-07-30</x:v>
+      <x:c r="E93" s="15" t="str">
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f772ce103d44c71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfba39bfbba49c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5169,7 +5203,7 @@
         <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>vaping_device_excise_amount</x:v>
+        <x:v>vaporisation_device_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
         <x:v>Poland</x:v>
@@ -5214,7 +5248,7 @@
         <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>vaping_component_sets_excise_amount</x:v>
+        <x:v>vaporisation_device_component_sets_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
         <x:v>Poland</x:v>
@@ -6283,7 +6317,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516ea67dac564bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95774ccc37c49e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v37 Canada closure and donor controls (#34)
Release the verified v37 dashboard and daily lender package.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R3653e33f3e5a42e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R73247874e00f4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rb921ca5a204a4012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R73b8d62659824bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="Rbef0ecddc797410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6cfd5a0345244ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8cd41972a2f147b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rdf6fee85d1354963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5b240c5013ab4964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R21dd5aa9add24763"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -1198,16 +1198,16 @@
         <x:v>Consumables are NZD 189,402,451.96, devices/hardware NZD 84,709,409.85 and mixed systems NZD 68,548.40. Adjacent notifiable products of NZD 2,137,085.24 and unresolved product types of NZD 4,367,017.37 are separately quantified and excluded. All observed value comes from AIS/AVP workbooks; no Notifier or RPS value is added.</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return ; https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf ; source/NZ_2024_DONOR_CLOSURE_PACK.md ; source/NZ_2024_D8_D10_OFFICIAL_SOURCE_AUDIT.md ; source/NZ_DONOR_FOLLOWUP_PACK_2026-08-07.md ; source/NZ_2024_WORKBOOK_MANIFEST.json ; source/NZ_2024_PRODUCT_SCOPE_AUDIT.json ; scripts/analyze_nz_2024_returns.py</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="F22" s="17" t="str">
         <x:v>NZD 189,402,451.96 + 84,709,409.85 + 68,548.40 = NZD 274,180,410.21. Adjacent and unresolved classes are applied before the vaping subtotal and excluded. URLs, byte sizes and SHA-256 hashes for all 29 files are validated before aggregation.</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>The deterministic scope rules are public. Observed general-retail value is absent, the GST basis is unknown, exact-row-deduplication sensitivity is not a corrected estimate and no independent reconciliation has passed.</x:v>
+        <x:v>The deterministic scope rules are public. RPS collects product types and quantities but no observed retail value. The GST basis is unknown. Stats NZ's final 2024 HS10 control is a customs-stage sensitivity, not independent retail reconciliation.</x:v>
       </x:c>
       <x:c r="H22" s="14" t="str">
         <x:v>Supported</x:v>
@@ -1372,22 +1372,22 @@
         <x:v>The four-quarter sum is CAD 1,219,160,000; the same-survey sum of 12 months is CAD 1,219,161,000. Health Canada's 2024 manufacturer/importer net shipment value is CAD 1,160,753,796.78.</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_RCS_TAX_BASIS_CLARIFICATION_2026-07-29.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
+        <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101 ; https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001 ; https://health-infobase.canada.ca/substance-use/vaping/sales/ ; source/CANADA_2024_DONOR_CLOSURE_PACK.md ; source/CANADA_RCS_TAX_BASIS_CLARIFICATION_2026-07-29.md ; source/CANADA_RCS_SCOPE_QUALITY_CLARIFICATION_2026-07-30.md ; source/CANADA_2024_D5_D7_D10_OFFICIAL_SOURCE_AUDIT.md</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>Monthly − quarterly = CAD 1,000 (0.000082%). Retail − shipments = CAD 58,406,203.22; retail / shipments − 1 = 5.031748%. ECB 2024: 1,219,160,000 / 1.482110546875 = EUR 822,583,715.21.</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>D8 passes: CAD, exclusion of GST/HST/PST/QST and inclusion of additional duties embedded in retail prices are confirmed for table 20-10-0071-01. The exact duty components and monthly and legacy-table tax bases remain under clarification. The monthly route is same-survey QA, not D10; retail and shipments do not form a market range.</x:v>
+        <x:v>D8 passes: CAD, exclusion of GST/HST/PST/QST and inclusion of embedded additional duties are confirmed for the reviewed quarterly, monthly and archived tables. Additional duties can include federal, additional and provincial vaping duties. The monthly route is same-survey QA, not D10.</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>D5 NAICS 459993/459999 coverage, D7 annual error boundary and D10 retail-to-shipment reconciliation remain open; Canada is not an accepted donor.</x:v>
+        <x:v>D5 failed because NAICS 459999 specialist retail is outside the confirmed 441100–459993 target range. D7 failed because exact product-class quality and annual-uncertainty information is unavailable. D10 remains open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
@@ -1566,31 +1566,31 @@
     </x:row>
     <x:row r="35" ht="58.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable e-cigarette devices and 62,500 derived taxable component sets.</x:v>
+        <x:v>Poland's 2025 tax bridge yields 4,382,500 derived taxable broad vaporisation-device-group units and 62,500 derived taxable component sets; neither is e-cigarette-specific.</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>The official parliamentary response reports PLN 993.1 million for e-liquids, PLN 175.3 million for devices and PLN 2.5 million for component sets. The device and component-set duty was PLN 40 per unit from 1 July 2025.</x:v>
+        <x:v>The official response reports PLN 993.1 million for e-liquids, PLN 175.3 million for the broad device group and PLN 2.5 million for component sets. The statutory group includes refillable e-cigarettes, heated-tobacco heaters and multifunction devices. Duty was PLN 40 per unit from 1 July 2025.</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://api.sejm.gov.pl/sejm/term10/interpellations/attachment/ATTDVKHSJ/i17526-o1.pdf ; https://www.podatki.gov.pl/akcyza/stawki-podatkowe/ ; https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego ; https://api.sejm.gov.pl/eli/acts/DU/2025/698/text.pdf ; source/POLAND_D1_D10_PREASSESSMENT_2026-07-31.md</x:v>
       </x:c>
       <x:c r="E35" s="14" t="str">
-        <x:v>2025</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable devices; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
+        <x:v>PLN 175,300,000 / 40 = 4,382,500 taxable broad-group units; PLN 2,500,000 / 40 = 62,500 taxable component sets.</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. It does not establish consumer prices, retail sales, untaxed quantities or stock transitions.</x:v>
+        <x:v>The derived tax base covers only devices and component sets taxed from 1 July 2025. AKC-4/R requires device-type detail, but the current public aggregate does not publish it. The values do not establish consumer prices, retail sales or an e-cigarette-only count.</x:v>
       </x:c>
       <x:c r="H35" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I35" s="14" t="str">
-        <x:v>The monthly duty profile, finality, retail prices, channel coverage and independent reconciliation are required.</x:v>
+        <x:v>The AKC-4/R e-cigarette/heater/multifunction split, monthly duty profile, retail prices, channel coverage and independent reconciliation are required. Poland receives no donor score without a country-year retail value.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58.5" customHeight="1">
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2031e0156924472"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954404b7d653401c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.30-36</x:v>
+        <x:v>2026.07.31-37</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A11)</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2469,7 +2469,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A12)</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R361b2d8017b64e66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bdb2db608a14175"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3573,24 +3573,24 @@
     </x:row>
     <x:row r="53" ht="31.5" customHeight="1">
       <x:c r="A53" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-BC2CDD0708D5</x:v>
+        <x:v>REGISTER-REFERENCE-067A847A44A9</x:v>
       </x:c>
       <x:c r="B53" s="14" t="str">
-        <x:v>data-api.ecb.europa.eu</x:v>
+        <x:v>api.sejm.gov.pl</x:v>
       </x:c>
       <x:c r="C53" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D53" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://api.sejm.gov.pl/eli/acts/DU/2025/698/text.pdf</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
       <x:c r="A54" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7264539499F0</x:v>
+        <x:v>REGISTER-REFERENCE-BC2CDD0708D5</x:v>
       </x:c>
       <x:c r="B54" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3599,15 +3599,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D54" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
       <x:c r="A55" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2580DD0733C9</x:v>
+        <x:v>REGISTER-REFERENCE-7264539499F0</x:v>
       </x:c>
       <x:c r="B55" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3616,15 +3616,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D55" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
       <x:c r="A56" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-38DD93023815</x:v>
+        <x:v>REGISTER-REFERENCE-2580DD0733C9</x:v>
       </x:c>
       <x:c r="B56" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3633,15 +3633,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D56" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
       <x:c r="A57" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-72D82058EA8A</x:v>
+        <x:v>REGISTER-REFERENCE-38DD93023815</x:v>
       </x:c>
       <x:c r="B57" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3650,15 +3650,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D57" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
       <x:c r="A58" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
+        <x:v>REGISTER-REFERENCE-72D82058EA8A</x:v>
       </x:c>
       <x:c r="B58" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3667,15 +3667,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D58" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
       <x:c r="A59" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-ACB549D404B8</x:v>
+        <x:v>REGISTER-REFERENCE-E8408060156E</x:v>
       </x:c>
       <x:c r="B59" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3684,15 +3684,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D59" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
       <x:c r="A60" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
+        <x:v>REGISTER-REFERENCE-ACB549D404B8</x:v>
       </x:c>
       <x:c r="B60" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3701,15 +3701,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D60" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
       <x:c r="A61" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
+        <x:v>REGISTER-REFERENCE-2FB6E2117AD7</x:v>
       </x:c>
       <x:c r="B61" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3718,15 +3718,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D61" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
       <x:c r="A62" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
+        <x:v>REGISTER-REFERENCE-8FEBAD85B03E</x:v>
       </x:c>
       <x:c r="B62" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3735,15 +3735,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D62" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
       <x:c r="A63" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+        <x:v>REGISTER-REFERENCE-37CBB91A050A</x:v>
       </x:c>
       <x:c r="B63" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3752,15 +3752,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D63" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
       <x:c r="A64" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
       </x:c>
       <x:c r="B64" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3769,15 +3769,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D64" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
       <x:c r="A65" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
       </x:c>
       <x:c r="B65" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3786,15 +3786,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D65" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
       <x:c r="A66" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
       </x:c>
       <x:c r="B66" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3803,15 +3803,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D66" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
       </x:c>
       <x:c r="B67" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3820,15 +3820,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D67" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
       <x:c r="A68" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
       </x:c>
       <x:c r="B68" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3837,15 +3837,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D68" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
       </x:c>
       <x:c r="B69" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3854,15 +3854,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D69" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
       <x:c r="A70" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
       </x:c>
       <x:c r="B70" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3871,15 +3871,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D70" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
       <x:c r="A71" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
       </x:c>
       <x:c r="B71" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3888,15 +3888,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D71" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
       <x:c r="A72" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
       </x:c>
       <x:c r="B72" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3905,15 +3905,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D72" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
       <x:c r="A73" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
+        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
       </x:c>
       <x:c r="B73" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3922,15 +3922,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D73" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
+        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3939,15 +3939,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3956,151 +3956,151 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C76" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>datahelpdesk.worldbank.org</x:v>
+        <x:v>data.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
+        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>douanes.public.lu</x:v>
+        <x:v>datahelpdesk.worldbank.org</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
+        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>douanes.public.lu</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>adm.gov.it</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
         <x:v>Federal Trade Commission</x:v>
@@ -4109,32 +4109,32 @@
         <x:v>official_report</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C85" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-B5944DDC2320</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
         <x:v>health.govt.nz</x:v>
@@ -4143,101 +4143,135 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2024-12/2024-annual-returns-user-guide.pdf</x:v>
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>REGISTER-REFERENCE-1766C84ECA96</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C87" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-529570B0D6C7</x:v>
       </x:c>
       <x:c r="B88" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C88" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D88" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
       <x:c r="A89" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
       </x:c>
       <x:c r="B89" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>podatki.gov.pl</x:v>
       </x:c>
       <x:c r="C89" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D89" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
       </x:c>
       <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="31.5" customHeight="1">
       <x:c r="A90" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B90" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C90" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D90" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E90" s="14" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="31.5" customHeight="1">
+      <x:c r="A91" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B91" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C91" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D91" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E91" s="14" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="31.5" customHeight="1">
+      <x:c r="A92" s="14" t="str">
         <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
       </x:c>
-      <x:c r="B90" s="14" t="str">
+      <x:c r="B92" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C90" s="14" t="str">
+      <x:c r="C92" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D90" s="14" t="str">
+      <x:c r="D92" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E90" s="14" t="str">
-        <x:v>2026-07-30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="31.5" customHeight="1">
-      <x:c r="A91" s="15" t="str">
+      <x:c r="E92" s="14" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="31.5" customHeight="1">
+      <x:c r="A93" s="15" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B91" s="15" t="str">
+      <x:c r="B93" s="15" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C91" s="15" t="str">
+      <x:c r="C93" s="15" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D91" s="15" t="str">
+      <x:c r="D93" s="15" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E91" s="15" t="str">
-        <x:v>2026-07-30</x:v>
+      <x:c r="E93" s="15" t="str">
+        <x:v>2026-07-31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f772ce103d44c71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfba39bfbba49c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5169,7 +5203,7 @@
         <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>vaping_device_excise_amount</x:v>
+        <x:v>vaporisation_device_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
         <x:v>Poland</x:v>
@@ -5214,7 +5248,7 @@
         <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>vaping_component_sets_excise_amount</x:v>
+        <x:v>vaporisation_device_component_sets_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
         <x:v>Poland</x:v>
@@ -6283,7 +6317,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516ea67dac564bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95774ccc37c49e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v41 donor-control checkpoint
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6cfd5a0345244ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8cd41972a2f147b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rdf6fee85d1354963"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5b240c5013ab4964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R21dd5aa9add24763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Ra750953b0efb45e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R51debb22911341db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R8cda80fb9a3545b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R00af4b2413b44413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R2bbabee95be94804"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E102" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -351,7 +351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N76" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Record type"/>
     <x:tableColumn id="2" name="Record ID"/>
@@ -1073,7 +1073,7 @@
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The public market dataset contains 156 observations from 47 sources; its 134 official observations split into 98 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
@@ -1088,7 +1088,7 @@
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>156 = 120 market and model observations + 36 FHM structure counts; 134 official = 98 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
         <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
@@ -1218,89 +1218,89 @@
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>Stats NZ's selected 2024 HS10 control yields NZD 183,370,681 and NZD 197,070,322 net border proxies; neither is retail market value.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
+        <x:v>Selected imports are NZD 189,640,890 at value for duty and NZD 203,340,531 at CIF. Selected exports are NZD 6,270,209 FOB. The control applies a locked 2024 product-code selection rule.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.stats.govt.nz/large-datasets/csv-files-for-download/overseas-merchandise-trade-datasets/ ; https://www3.stats.govt.nz/HS10_by_Country/2024_Imports_HS10.zip ; https://www3.stats.govt.nz/HS10_by_Country/2024_Exports_HS10.zip ; source/NZ_CA_DE_DONOR_CONTROL_SPRINT_2026-08-02.md</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
+        <x:v>NZD 189,640,890 − 6,270,209 = 183,370,681; NZD 203,340,531 − 6,270,209 = 197,070,322. Candidate / proxies = 1.495224911 and 1.391282094.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
+        <x:v>Border event stage, product scope, domestic production, inventory, re-exports, margins, channels, GST and consumer sell-through do not match the retail boundary.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+        <x:v>The ratios are not margin, uplift, validation intervals or a market range. D10 remains open and New Zealand remains 7/10 NOT ACCEPTED.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
+        <x:v>Germany's prospective vendor benchmark DE-BLIND-1.0.0 was locked before any future submission is scored; it is NOT SCORED.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Germany</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
+        <x:v>Final official anchors are 1,241,000 litres for 2023 and 1,284,000 litres for 2024, or 2,525,000 litres combined. Preregistered caps are 15% annually and 10% combined.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003/ ; source/NZ_CA_DE_DONOR_CONTROL_SPRINT_2026-08-02.md</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2021</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
+        <x:v>Annual deviation = |vendor litres / official litres − 1|; combined deviation = |vendor two-year sum / 2,525,000 − 1|.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
+        <x:v>A numeric match alone does not establish matching product, unit, tax basis, channel or event stage. Thresholds are not tuned to private values.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+        <x:v>Passing does not accept Germany as a donor or authorise a purchase, licence, fee or disclosure. Germany's official retail value remains not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58.5" customHeight="1">
@@ -1317,7 +1317,7 @@
         <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
         <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
@@ -1387,7 +1387,7 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>D5 failed because NAICS 459999 specialist retail is outside the confirmed 441100–459993 target range. D7 failed because exact product-class quality and annual-uncertainty information is unavailable. D10 remains open; Canada is not an accepted donor.</x:v>
+        <x:v>D5 failed because NAICS 459999 specialist retail is outside the confirmed 441100–459993 target range; in-scope online sales do not cover excluded specialist, foreign direct or cross-border channels. D7 failed because exact NAPCS 5619122 response, imputation, CV, standard-error, confidence-interval and covariance metrics are unavailable. D10 remains open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
@@ -1610,7 +1610,7 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 98 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
         <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954404b7d653401c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdecff32e9b034609"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.31-37</x:v>
+        <x:v>2026.08.02-41</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A11)</x:f>
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2469,7 +2469,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A12)</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bdb2db608a14175"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda256a45c5674ce7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,7 +3585,7 @@
         <x:v>https://api.sejm.gov.pl/eli/acts/DU/2025/698/text.pdf</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3602,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3619,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3636,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3653,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3670,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3687,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3704,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3721,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3738,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3755,12 +3755,12 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
       <x:c r="A64" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+        <x:v>REGISTER-REFERENCE-BCE59F2D3F9D</x:v>
       </x:c>
       <x:c r="B64" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3769,15 +3769,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D64" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
       <x:c r="A65" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+        <x:v>REGISTER-REFERENCE-2267B190A073</x:v>
       </x:c>
       <x:c r="B65" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3786,15 +3786,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D65" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
       <x:c r="A66" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+        <x:v>REGISTER-REFERENCE-957871D9CB33</x:v>
       </x:c>
       <x:c r="B66" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3803,15 +3803,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D66" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+        <x:v>REGISTER-REFERENCE-5C7194247112</x:v>
       </x:c>
       <x:c r="B67" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3820,15 +3820,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D67" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
       <x:c r="A68" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+        <x:v>REGISTER-REFERENCE-75BF634166B2</x:v>
       </x:c>
       <x:c r="B68" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3837,15 +3837,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D68" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
       </x:c>
       <x:c r="B69" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3854,15 +3854,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D69" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
       <x:c r="A70" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
       </x:c>
       <x:c r="B70" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3871,15 +3871,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D70" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
       <x:c r="A71" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
       </x:c>
       <x:c r="B71" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3888,15 +3888,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D71" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
       <x:c r="A72" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
       </x:c>
       <x:c r="B72" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3905,15 +3905,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D72" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
       <x:c r="A73" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
       </x:c>
       <x:c r="B73" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3922,15 +3922,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D73" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3939,15 +3939,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3956,15 +3956,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3973,305 +3973,458 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
+        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>datahelpdesk.worldbank.org</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
+        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>douanes.public.lu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>adm.gov.it</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>data.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>datahelpdesk.worldbank.org</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>douanes.public.lu</x:v>
       </x:c>
       <x:c r="C84" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>REGISTER-REFERENCE-25E8C2FC0150</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>genesis.destatis.de</x:v>
       </x:c>
       <x:c r="C85" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003/</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C86" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-1766C84ECA96</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C87" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-529570B0D6C7</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B88" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C88" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D88" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
       <x:c r="A89" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B89" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C89" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D89" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="31.5" customHeight="1">
       <x:c r="A90" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B90" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C90" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D90" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E90" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="31.5" customHeight="1">
       <x:c r="A91" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B91" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C91" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D91" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E91" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="31.5" customHeight="1">
       <x:c r="A92" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B92" s="14" t="str">
-        <x:v>www150.statcan.gc.ca</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C92" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D92" s="14" t="str">
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+      </x:c>
+      <x:c r="E92" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="31.5" customHeight="1">
+      <x:c r="A93" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-1766C84ECA96</x:v>
+      </x:c>
+      <x:c r="B93" s="14" t="str">
+        <x:v>health.govt.nz</x:v>
+      </x:c>
+      <x:c r="C93" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D93" s="14" t="str">
+        <x:v>https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf</x:v>
+      </x:c>
+      <x:c r="E93" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="31.5" customHeight="1">
+      <x:c r="A94" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-529570B0D6C7</x:v>
+      </x:c>
+      <x:c r="B94" s="14" t="str">
+        <x:v>podatki.gov.pl</x:v>
+      </x:c>
+      <x:c r="C94" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D94" s="14" t="str">
+        <x:v>https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego</x:v>
+      </x:c>
+      <x:c r="E94" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="31.5" customHeight="1">
+      <x:c r="A95" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+      </x:c>
+      <x:c r="B95" s="14" t="str">
+        <x:v>podatki.gov.pl</x:v>
+      </x:c>
+      <x:c r="C95" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D95" s="14" t="str">
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+      </x:c>
+      <x:c r="E95" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="31.5" customHeight="1">
+      <x:c r="A96" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-645255DD4B34</x:v>
+      </x:c>
+      <x:c r="B96" s="14" t="str">
+        <x:v>stats.govt.nz</x:v>
+      </x:c>
+      <x:c r="C96" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D96" s="14" t="str">
+        <x:v>https://www.stats.govt.nz/large-datasets/csv-files-for-download/overseas-merchandise-trade-datasets/</x:v>
+      </x:c>
+      <x:c r="E96" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="31.5" customHeight="1">
+      <x:c r="A97" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B97" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C97" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D97" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E97" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="31.5" customHeight="1">
+      <x:c r="A98" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B98" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C98" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D98" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E98" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="31.5" customHeight="1">
+      <x:c r="A99" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+      </x:c>
+      <x:c r="B99" s="14" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C99" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D99" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E92" s="14" t="str">
-        <x:v>2026-07-31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="31.5" customHeight="1">
-      <x:c r="A93" s="15" t="str">
+      <x:c r="E99" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="31.5" customHeight="1">
+      <x:c r="A100" s="14" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B93" s="15" t="str">
+      <x:c r="B100" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C93" s="15" t="str">
+      <x:c r="C100" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D93" s="15" t="str">
+      <x:c r="D100" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E93" s="15" t="str">
-        <x:v>2026-07-31</x:v>
+      <x:c r="E100" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="31.5" customHeight="1">
+      <x:c r="A101" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9479B1548E50</x:v>
+      </x:c>
+      <x:c r="B101" s="14" t="str">
+        <x:v>www3.stats.govt.nz</x:v>
+      </x:c>
+      <x:c r="C101" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D101" s="14" t="str">
+        <x:v>https://www3.stats.govt.nz/HS10_by_Country/2024_Exports_HS10.zip</x:v>
+      </x:c>
+      <x:c r="E101" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="31.5" customHeight="1">
+      <x:c r="A102" s="15" t="str">
+        <x:v>REGISTER-REFERENCE-94B1312153E9</x:v>
+      </x:c>
+      <x:c r="B102" s="15" t="str">
+        <x:v>www3.stats.govt.nz</x:v>
+      </x:c>
+      <x:c r="C102" s="15" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D102" s="15" t="str">
+        <x:v>https://www3.stats.govt.nz/HS10_by_Country/2024_Imports_HS10.zip</x:v>
+      </x:c>
+      <x:c r="E102" s="15" t="str">
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfba39bfbba49c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5824c78453646dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5110,22 +5263,22 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>DE-2019-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Finland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E19" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G19" s="45" t="n">
-        <x:v>3540319</x:v>
+        <x:v>2247267035</x:v>
       </x:c>
       <x:c r="H19" s="45" t="str">
         <x:v>EUR</x:v>
@@ -5135,7 +5288,7 @@
       </x:c>
       <x:c r="J19" s="45" t="n">
         <x:f>G19</x:f>
-        <x:v>3540319</x:v>
+        <x:v>2247267035</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
         <x:v>EUR-IDENTITY</x:v>
@@ -5155,44 +5308,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
+        <x:v>DE-2020-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>e_liquid_excise_amount</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E20" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G20" s="45" t="n">
-        <x:v>993100000</x:v>
+        <x:v>2444948000</x:v>
       </x:c>
       <x:c r="H20" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I20" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J20" s="45" t="n">
-        <x:f>G20/I20</x:f>
-        <x:v>234240611.54771507</x:v>
+        <x:f>G20</x:f>
+        <x:v>2444948000</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L20" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M20" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N20" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25.5" customHeight="1">
@@ -5200,44 +5353,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
+        <x:v>DE-2021-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>vaporisation_device_broad_group_excise_amount</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E21" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G21" s="45" t="n">
-        <x:v>175300000</x:v>
+        <x:v>2325648577</x:v>
       </x:c>
       <x:c r="H21" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I21" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J21" s="45" t="n">
-        <x:f>G21/I21</x:f>
-        <x:v>41347678.183782555</x:v>
+        <x:f>G21</x:f>
+        <x:v>2325648577</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L21" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M21" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N21" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25.5" customHeight="1">
@@ -5245,44 +5398,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
+        <x:v>DE-2022-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>vaporisation_device_component_sets_broad_group_excise_amount</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E22" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G22" s="45" t="n">
-        <x:v>2500000</x:v>
+        <x:v>2510888578</x:v>
       </x:c>
       <x:c r="H22" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I22" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J22" s="45" t="n">
-        <x:f>G22/I22</x:f>
-        <x:v>589670.2536192606</x:v>
+        <x:f>G22</x:f>
+        <x:v>2510888578</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L22" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M22" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N22" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25.5" customHeight="1">
@@ -5290,44 +5443,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>DE-2023-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>Sweden</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E23" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G23" s="45" t="n">
-        <x:v>80000000</x:v>
+        <x:v>2581608198</x:v>
       </x:c>
       <x:c r="H23" s="45" t="str">
-        <x:v>SEK</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I23" s="45" t="n">
-        <x:v>11.432519140625</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J23" s="45" t="n">
-        <x:f>G23/I23</x:f>
-        <x:v>6997582.861306848</x:v>
+        <x:f>G23</x:f>
+        <x:v>2581608198</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
-        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L23" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M23" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N23" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25.5" customHeight="1">
@@ -5335,44 +5488,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>DE-2024-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E24" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G24" s="45" t="n">
-        <x:v>26000000000</x:v>
+        <x:v>2687776000</x:v>
       </x:c>
       <x:c r="H24" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I24" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J24" s="45" t="n">
-        <x:f>G24/I24</x:f>
-        <x:v>23009192918.721367</x:v>
+        <x:f>G24</x:f>
+        <x:v>2687776000</x:v>
       </x:c>
       <x:c r="K24" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L24" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M24" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N24" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="25.5" customHeight="1">
@@ -5380,44 +5533,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Finland</x:v>
       </x:c>
       <x:c r="E25" s="14" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G25" s="45" t="n">
-        <x:v>45700000000</x:v>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="H25" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I25" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J25" s="45" t="n">
-        <x:f>G25/I25</x:f>
-        <x:v>40443081399.44486</x:v>
+        <x:f>G25</x:f>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="K25" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L25" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M25" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N25" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25.5" customHeight="1">
@@ -5425,38 +5578,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>PL-2021-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E26" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G26" s="45" t="n">
-        <x:v>46320000000</x:v>
+        <x:v>179500000</x:v>
       </x:c>
       <x:c r="H26" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I26" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>4.5651786821705</x:v>
       </x:c>
       <x:c r="J26" s="45" t="n">
         <x:f>G26/I26</x:f>
-        <x:v>40991762153.66052</x:v>
+        <x:v>39319381.01372568</x:v>
       </x:c>
       <x:c r="K26" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2021</x:v>
       </x:c>
       <x:c r="L26" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M26" s="14" t="str">
         <x:v>computed</x:v>
@@ -5470,38 +5623,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2022-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E27" s="14" t="n">
-        <x:v>2015</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G27" s="45" t="n">
-        <x:v>304170046</x:v>
+        <x:v>229900000</x:v>
       </x:c>
       <x:c r="H27" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I27" s="45" t="n">
-        <x:v>1.109512890625</x:v>
+        <x:v>4.686106614786</x:v>
       </x:c>
       <x:c r="J27" s="45" t="n">
         <x:f>G27/I27</x:f>
-        <x:v>274147374.5552049</x:v>
+        <x:v>49059916.66399566</x:v>
       </x:c>
       <x:c r="K27" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2022</x:v>
       </x:c>
       <x:c r="L27" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M27" s="14" t="str">
         <x:v>computed</x:v>
@@ -5515,38 +5668,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2023-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E28" s="14" t="n">
-        <x:v>2016</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G28" s="45" t="n">
-        <x:v>485707484</x:v>
+        <x:v>443600000</x:v>
       </x:c>
       <x:c r="H28" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I28" s="45" t="n">
-        <x:v>1.1069031128405</x:v>
+        <x:v>4.5419658823529</x:v>
       </x:c>
       <x:c r="J28" s="45" t="n">
         <x:f>G28/I28</x:f>
-        <x:v>438798552.7961817</x:v>
+        <x:v>97666959.96628653</x:v>
       </x:c>
       <x:c r="K28" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2023</x:v>
       </x:c>
       <x:c r="L28" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M28" s="14" t="str">
         <x:v>computed</x:v>
@@ -5560,38 +5713,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2024-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E29" s="14" t="n">
-        <x:v>2017</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G29" s="45" t="n">
-        <x:v>779836399</x:v>
+        <x:v>561400000</x:v>
       </x:c>
       <x:c r="H29" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I29" s="45" t="n">
-        <x:v>1.1296811764706</x:v>
+        <x:v>4.305795703125</x:v>
       </x:c>
       <x:c r="J29" s="45" t="n">
         <x:f>G29/I29</x:f>
-        <x:v>690315475.943752</x:v>
+        <x:v>130382405.18298511</x:v>
       </x:c>
       <x:c r="K29" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L29" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M29" s="14" t="str">
         <x:v>computed</x:v>
@@ -5605,44 +5758,37 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2015-UOKIK-E-CIGARETTE-MARKET-VALUE-ESTIMATE</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>institutional_market_value_benchmark</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E30" s="14" t="n">
-        <x:v>2018</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>study_reference_period_may_2015</x:v>
       </x:c>
       <x:c r="G30" s="45" t="n">
-        <x:v>2043703005</x:v>
+        <x:v>500000000</x:v>
       </x:c>
       <x:c r="H30" s="45" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="I30" s="45" t="n">
-        <x:v>1.1809545098039</x:v>
-      </x:c>
-      <x:c r="J30" s="45" t="n">
-        <x:f>G30/I30</x:f>
-        <x:v>1730551844.3207107</x:v>
-      </x:c>
-      <x:c r="K30" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
-      </x:c>
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I30" s="45"/>
+      <x:c r="J30" s="45"/>
+      <x:c r="K30" s="14"/>
       <x:c r="L30" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="M30" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>not_computed</x:v>
       </x:c>
       <x:c r="N30" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>period_not_compatible_with_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1">
@@ -5650,38 +5796,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E31" s="14" t="n">
-        <x:v>2019</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G31" s="45" t="n">
-        <x:v>2702608307</x:v>
+        <x:v>993100000</x:v>
       </x:c>
       <x:c r="H31" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I31" s="45" t="n">
-        <x:v>1.1194745098039</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J31" s="45" t="n">
         <x:f>G31/I31</x:f>
-        <x:v>2414175832.796246</x:v>
+        <x:v>234240611.54771507</x:v>
       </x:c>
       <x:c r="K31" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L31" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M31" s="14" t="str">
         <x:v>computed</x:v>
@@ -5695,38 +5841,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaporisation_device_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E32" s="14" t="n">
-        <x:v>2020</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G32" s="45" t="n">
-        <x:v>2394423105</x:v>
+        <x:v>175300000</x:v>
       </x:c>
       <x:c r="H32" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I32" s="45" t="n">
-        <x:v>1.1421961089494</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J32" s="45" t="n">
         <x:f>G32/I32</x:f>
-        <x:v>2096332745.523365</x:v>
+        <x:v>41347678.183782555</x:v>
       </x:c>
       <x:c r="K32" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L32" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M32" s="14" t="str">
         <x:v>computed</x:v>
@@ -5740,38 +5886,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaporisation_device_component_sets_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E33" s="14" t="n">
-        <x:v>2021</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G33" s="45" t="n">
-        <x:v>2763284338</x:v>
+        <x:v>2500000</x:v>
       </x:c>
       <x:c r="H33" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I33" s="45" t="n">
-        <x:v>1.1827403100775</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J33" s="45" t="n">
         <x:f>G33/I33</x:f>
-        <x:v>2336340711.866778</x:v>
+        <x:v>589670.2536192606</x:v>
       </x:c>
       <x:c r="K33" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L33" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M33" s="14" t="str">
         <x:v>computed</x:v>
@@ -5782,16 +5928,16 @@
     </x:row>
     <x:row r="34" ht="25.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>low.specialistRetailNzd</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Sweden</x:v>
       </x:c>
       <x:c r="E34" s="14" t="n">
         <x:v>2024</x:v>
@@ -5800,23 +5946,23 @@
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G34" s="45" t="n">
-        <x:v>258327110.88</x:v>
+        <x:v>80000000</x:v>
       </x:c>
       <x:c r="H34" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>SEK</x:v>
       </x:c>
       <x:c r="I34" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>11.432519140625</x:v>
       </x:c>
       <x:c r="J34" s="45" t="n">
         <x:f>G34/I34</x:f>
-        <x:v>144474304.51375833</x:v>
+        <x:v>6997582.861306848</x:v>
       </x:c>
       <x:c r="K34" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L34" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M34" s="14" t="str">
         <x:v>computed</x:v>
@@ -5827,41 +5973,41 @@
     </x:row>
     <x:row r="35" ht="25.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>low.generalRetailRpsNzd</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E35" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G35" s="45" t="n">
-        <x:v>275335272.8</x:v>
+        <x:v>26000000000</x:v>
       </x:c>
       <x:c r="H35" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I35" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J35" s="45" t="n">
         <x:f>G35/I35</x:f>
-        <x:v>153986439.55865824</x:v>
+        <x:v>23009192918.721367</x:v>
       </x:c>
       <x:c r="K35" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L35" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M35" s="14" t="str">
         <x:v>computed</x:v>
@@ -5872,41 +6018,41 @@
     </x:row>
     <x:row r="36" ht="25.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>low.combinedNzd</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E36" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G36" s="45" t="n">
-        <x:v>533662383.68</x:v>
+        <x:v>45700000000</x:v>
       </x:c>
       <x:c r="H36" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I36" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J36" s="45" t="n">
         <x:f>G36/I36</x:f>
-        <x:v>298460744.0724166</x:v>
+        <x:v>40443081399.44486</x:v>
       </x:c>
       <x:c r="K36" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L36" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M36" s="14" t="str">
         <x:v>computed</x:v>
@@ -5917,41 +6063,41 @@
     </x:row>
     <x:row r="37" ht="25.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>base.specialistRetailNzd</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E37" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G37" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>46320000000</x:v>
       </x:c>
       <x:c r="H37" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I37" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J37" s="45" t="n">
         <x:f>G37/I37</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>40991762153.66052</x:v>
       </x:c>
       <x:c r="K37" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L37" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M37" s="14" t="str">
         <x:v>computed</x:v>
@@ -5962,41 +6108,41 @@
     </x:row>
     <x:row r="38" ht="25.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>base.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E38" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G38" s="45" t="n">
-        <x:v>367631277.68</x:v>
+        <x:v>304170046</x:v>
       </x:c>
       <x:c r="H38" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I38" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.109512890625</x:v>
       </x:c>
       <x:c r="J38" s="45" t="n">
         <x:f>G38/I38</x:f>
-        <x:v>205604719.4558489</x:v>
+        <x:v>274147374.5552049</x:v>
       </x:c>
       <x:c r="K38" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
       </x:c>
       <x:c r="L38" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M38" s="14" t="str">
         <x:v>computed</x:v>
@@ -6007,41 +6153,41 @@
     </x:row>
     <x:row r="39" ht="25.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>base.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E39" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2016</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G39" s="45" t="n">
-        <x:v>641811687.89</x:v>
+        <x:v>485707484</x:v>
       </x:c>
       <x:c r="H39" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I39" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1069031128405</x:v>
       </x:c>
       <x:c r="J39" s="45" t="n">
         <x:f>G39/I39</x:f>
-        <x:v>358945280.34954304</x:v>
+        <x:v>438798552.7961817</x:v>
       </x:c>
       <x:c r="K39" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
       </x:c>
       <x:c r="L39" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M39" s="14" t="str">
         <x:v>computed</x:v>
@@ -6052,41 +6198,41 @@
     </x:row>
     <x:row r="40" ht="25.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>high.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E40" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G40" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>779836399</x:v>
       </x:c>
       <x:c r="H40" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I40" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1296811764706</x:v>
       </x:c>
       <x:c r="J40" s="45" t="n">
         <x:f>G40/I40</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>690315475.943752</x:v>
       </x:c>
       <x:c r="K40" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
       </x:c>
       <x:c r="L40" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M40" s="14" t="str">
         <x:v>computed</x:v>
@@ -6097,41 +6243,41 @@
     </x:row>
     <x:row r="41" ht="25.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>high.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E41" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G41" s="45" t="n">
-        <x:v>456995382.29</x:v>
+        <x:v>2043703005</x:v>
       </x:c>
       <x:c r="H41" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I41" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1809545098039</x:v>
       </x:c>
       <x:c r="J41" s="45" t="n">
         <x:f>G41/I41</x:f>
-        <x:v>255583278.88015154</x:v>
+        <x:v>1730551844.3207107</x:v>
       </x:c>
       <x:c r="K41" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
       </x:c>
       <x:c r="L41" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M41" s="14" t="str">
         <x:v>computed</x:v>
@@ -6142,41 +6288,41 @@
     </x:row>
     <x:row r="42" ht="25.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>high.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E42" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G42" s="45" t="n">
-        <x:v>731175792.5</x:v>
+        <x:v>2702608307</x:v>
       </x:c>
       <x:c r="H42" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I42" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1194745098039</x:v>
       </x:c>
       <x:c r="J42" s="45" t="n">
         <x:f>G42/I42</x:f>
-        <x:v>408923839.7738457</x:v>
+        <x:v>2414175832.796246</x:v>
       </x:c>
       <x:c r="K42" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
       </x:c>
       <x:c r="L42" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M42" s="14" t="str">
         <x:v>computed</x:v>
@@ -6187,137 +6333,1490 @@
     </x:row>
     <x:row r="43" ht="25.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>low</x:v>
-      </x:c>
-      <x:c r="D43" s="14"/>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D43" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
       <x:c r="E43" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G43" s="45" t="n">
-        <x:v>667920000</x:v>
+        <x:v>2394423105</x:v>
       </x:c>
       <x:c r="H43" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I43" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.1421961089494</x:v>
       </x:c>
       <x:c r="J43" s="45" t="n">
-        <x:f>G43</x:f>
-        <x:v>667920000</x:v>
+        <x:f>G43/I43</x:f>
+        <x:v>2096332745.523365</x:v>
       </x:c>
       <x:c r="K43" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
       </x:c>
       <x:c r="L43" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M43" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N43" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="25.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>central</x:v>
-      </x:c>
-      <x:c r="D44" s="14"/>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D44" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
       <x:c r="E44" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G44" s="45" t="n">
+        <x:v>2763284338</x:v>
+      </x:c>
+      <x:c r="H44" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I44" s="45" t="n">
+        <x:v>1.1827403100775</x:v>
+      </x:c>
+      <x:c r="J44" s="45" t="n">
+        <x:f>G44/I44</x:f>
+        <x:v>2336340711.866778</x:v>
+      </x:c>
+      <x:c r="K44" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L44" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M44" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N44" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="25.5" customHeight="1">
+      <x:c r="A45" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B45" s="14" t="str">
+        <x:v>NZ-2019-HES-E-CIGARETTES-AND-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C45" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D45" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E45" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F45" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G45" s="45" t="n">
+        <x:v>42276000</x:v>
+      </x:c>
+      <x:c r="H45" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I45" s="45"/>
+      <x:c r="J45" s="45"/>
+      <x:c r="K45" s="14"/>
+      <x:c r="L45" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M45" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N45" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="25.5" customHeight="1">
+      <x:c r="A46" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>NZ-2019-HES-E-CIGARETTE-DEVICES-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G46" s="45" t="n">
+        <x:v>18034000</x:v>
+      </x:c>
+      <x:c r="H46" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I46" s="45"/>
+      <x:c r="J46" s="45"/>
+      <x:c r="K46" s="14"/>
+      <x:c r="L46" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M46" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N46" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="25.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="str">
+        <x:v>NZ-2019-HES-E-CIGARETTE-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G47" s="45" t="n">
+        <x:v>24242000</x:v>
+      </x:c>
+      <x:c r="H47" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I47" s="45"/>
+      <x:c r="J47" s="45"/>
+      <x:c r="K47" s="14"/>
+      <x:c r="L47" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M47" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N47" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="25.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>NZ-2023-HES-E-CIGARETTES-AND-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G48" s="45" t="n">
+        <x:v>186980000</x:v>
+      </x:c>
+      <x:c r="H48" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I48" s="45"/>
+      <x:c r="J48" s="45"/>
+      <x:c r="K48" s="14"/>
+      <x:c r="L48" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M48" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N48" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="25.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="str">
+        <x:v>NZ-2023-HES-E-CIGARETTE-DEVICES-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G49" s="45" t="n">
+        <x:v>22488000</x:v>
+      </x:c>
+      <x:c r="H49" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I49" s="45"/>
+      <x:c r="J49" s="45"/>
+      <x:c r="K49" s="14"/>
+      <x:c r="L49" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M49" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N49" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="25.5" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>NZ-2023-HES-E-CIGARETTE-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G50" s="45" t="n">
+        <x:v>164492000</x:v>
+      </x:c>
+      <x:c r="H50" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I50" s="45"/>
+      <x:c r="J50" s="45"/>
+      <x:c r="K50" s="14"/>
+      <x:c r="L50" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M50" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N50" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="25.5" customHeight="1">
+      <x:c r="A51" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B51" s="14" t="str">
+        <x:v>CA-2021-HC-VAPING-MARKET-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C51" s="14" t="str">
+        <x:v>institutional_market_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D51" s="14" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E51" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F51" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G51" s="45" t="n">
+        <x:v>2040000000</x:v>
+      </x:c>
+      <x:c r="H51" s="45" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I51" s="45" t="n">
+        <x:v>1.4825689922481</x:v>
+      </x:c>
+      <x:c r="J51" s="45" t="n">
+        <x:f>G51/I51</x:f>
+        <x:v>1375989927.3939602</x:v>
+      </x:c>
+      <x:c r="K51" s="14" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L51" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M51" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N51" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="25.5" customHeight="1">
+      <x:c r="A52" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B52" s="14" t="str">
+        <x:v>CA-2021-HC-GAS-CONVENIENCE-VAPING-SALES-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C52" s="14" t="str">
+        <x:v>institutional_channel_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D52" s="14" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E52" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F52" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G52" s="45" t="n">
+        <x:v>631000000</x:v>
+      </x:c>
+      <x:c r="H52" s="45" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I52" s="45" t="n">
+        <x:v>1.4825689922481</x:v>
+      </x:c>
+      <x:c r="J52" s="45" t="n">
+        <x:f>G52/I52</x:f>
+        <x:v>425612570.67921025</x:v>
+      </x:c>
+      <x:c r="K52" s="14" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L52" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M52" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N52" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="25.5" customHeight="1">
+      <x:c r="A53" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B53" s="14" t="str">
+        <x:v>CA-2021-HC-ONLINE-VAPING-SALES-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C53" s="14" t="str">
+        <x:v>institutional_channel_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D53" s="14" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E53" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F53" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G53" s="45" t="n">
+        <x:v>436000000</x:v>
+      </x:c>
+      <x:c r="H53" s="45" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I53" s="45" t="n">
+        <x:v>1.4825689922481</x:v>
+      </x:c>
+      <x:c r="J53" s="45" t="n">
+        <x:f>G53/I53</x:f>
+        <x:v>294084121.73714054</x:v>
+      </x:c>
+      <x:c r="K53" s="14" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L53" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M53" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N53" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="25.5" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-SOLD-PRODUCTION-EUR</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>prodcom_20595980_sold_production_value</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G54" s="45" t="n">
+        <x:v>39078000</x:v>
+      </x:c>
+      <x:c r="H54" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I54" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J54" s="45" t="n">
+        <x:f>G54</x:f>
+        <x:v>39078000</x:v>
+      </x:c>
+      <x:c r="K54" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L54" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M54" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N54" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="25.5" customHeight="1">
+      <x:c r="A55" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B55" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-IMPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C55" s="14" t="str">
+        <x:v>prodcom_20595980_import_value</x:v>
+      </x:c>
+      <x:c r="D55" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E55" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F55" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G55" s="45" t="n">
+        <x:v>400843037</x:v>
+      </x:c>
+      <x:c r="H55" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I55" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J55" s="45" t="n">
+        <x:f>G55</x:f>
+        <x:v>400843037</x:v>
+      </x:c>
+      <x:c r="K55" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L55" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M55" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N55" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="25.5" customHeight="1">
+      <x:c r="A56" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B56" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-EXPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C56" s="14" t="str">
+        <x:v>prodcom_20595980_export_value</x:v>
+      </x:c>
+      <x:c r="D56" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E56" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F56" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G56" s="45" t="n">
+        <x:v>120676188</x:v>
+      </x:c>
+      <x:c r="H56" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I56" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J56" s="45" t="n">
+        <x:f>G56</x:f>
+        <x:v>120676188</x:v>
+      </x:c>
+      <x:c r="K56" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L56" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M56" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N56" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="25.5" customHeight="1">
+      <x:c r="A57" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-SOLD-PRODUCTION-EUR</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>prodcom_27901152_sold_production_value</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F57" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G57" s="45" t="n">
+        <x:v>99890000</x:v>
+      </x:c>
+      <x:c r="H57" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I57" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J57" s="45" t="n">
+        <x:f>G57</x:f>
+        <x:v>99890000</x:v>
+      </x:c>
+      <x:c r="K57" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L57" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M57" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N57" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="25.5" customHeight="1">
+      <x:c r="A58" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-IMPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>prodcom_27901152_import_value</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F58" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G58" s="45" t="n">
+        <x:v>490580247</x:v>
+      </x:c>
+      <x:c r="H58" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I58" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J58" s="45" t="n">
+        <x:f>G58</x:f>
+        <x:v>490580247</x:v>
+      </x:c>
+      <x:c r="K58" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L58" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M58" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N58" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="25.5" customHeight="1">
+      <x:c r="A59" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-EXPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>prodcom_27901152_export_value</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F59" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G59" s="45" t="n">
+        <x:v>301380538</x:v>
+      </x:c>
+      <x:c r="H59" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I59" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J59" s="45" t="n">
+        <x:f>G59</x:f>
+        <x:v>301380538</x:v>
+      </x:c>
+      <x:c r="K59" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L59" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M59" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N59" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="25.5" customHeight="1">
+      <x:c r="A60" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B60" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-APPARENT-SUPPLY-EUR</x:v>
+      </x:c>
+      <x:c r="C60" s="14" t="str">
+        <x:v>prodcom_20595980_apparent_supply_value</x:v>
+      </x:c>
+      <x:c r="D60" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E60" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F60" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G60" s="45" t="n">
+        <x:v>319244849</x:v>
+      </x:c>
+      <x:c r="H60" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I60" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J60" s="45" t="n">
+        <x:f>G60</x:f>
+        <x:v>319244849</x:v>
+      </x:c>
+      <x:c r="K60" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L60" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M60" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N60" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="25.5" customHeight="1">
+      <x:c r="A61" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B61" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-APPARENT-SUPPLY-EUR</x:v>
+      </x:c>
+      <x:c r="C61" s="14" t="str">
+        <x:v>prodcom_27901152_apparent_supply_value</x:v>
+      </x:c>
+      <x:c r="D61" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E61" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F61" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G61" s="45" t="n">
+        <x:v>289089709</x:v>
+      </x:c>
+      <x:c r="H61" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I61" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J61" s="45" t="n">
+        <x:f>G61</x:f>
+        <x:v>289089709</x:v>
+      </x:c>
+      <x:c r="K61" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L61" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M61" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N61" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="25.5" customHeight="1">
+      <x:c r="A62" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B62" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-COMBINED-APPARENT-SUPPLY-EUR</x:v>
+      </x:c>
+      <x:c r="C62" s="14" t="str">
+        <x:v>combined_prodcom_apparent_supply_value</x:v>
+      </x:c>
+      <x:c r="D62" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E62" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F62" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G62" s="45" t="n">
+        <x:v>608334558</x:v>
+      </x:c>
+      <x:c r="H62" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I62" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J62" s="45" t="n">
+        <x:f>G62</x:f>
+        <x:v>608334558</x:v>
+      </x:c>
+      <x:c r="K62" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L62" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M62" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N62" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="25.5" customHeight="1">
+      <x:c r="A63" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B63" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-APPARENT-SUPPLY-EXCISE-VAT-BRIDGE-EUR</x:v>
+      </x:c>
+      <x:c r="C63" s="14" t="str">
+        <x:v>mechanical_apparent_supply_excise_vat_bridge</x:v>
+      </x:c>
+      <x:c r="D63" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E63" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F63" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G63" s="45" t="n">
+        <x:v>1040458124.02</x:v>
+      </x:c>
+      <x:c r="H63" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I63" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J63" s="45" t="n">
+        <x:f>G63</x:f>
+        <x:v>1040458124.02</x:v>
+      </x:c>
+      <x:c r="K63" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L63" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M63" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N63" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="25.5" customHeight="1">
+      <x:c r="A64" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B64" s="14" t="str">
+        <x:v>PL-2023-CMR-DISPOSABLE-E-CIGARETTE-RETAIL-SALES-VALUE</x:v>
+      </x:c>
+      <x:c r="C64" s="14" t="str">
+        <x:v>commercial_disposable_e_cigarette_retail_sales_value</x:v>
+      </x:c>
+      <x:c r="D64" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E64" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F64" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G64" s="45" t="n">
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="H64" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I64" s="45" t="n">
+        <x:v>4.5419658823529</x:v>
+      </x:c>
+      <x:c r="J64" s="45" t="n">
+        <x:f>G64/I64</x:f>
+        <x:v>440337961.9760439</x:v>
+      </x:c>
+      <x:c r="K64" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2023</x:v>
+      </x:c>
+      <x:c r="L64" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M64" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N64" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="25.5" customHeight="1">
+      <x:c r="A65" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B65" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C65" s="14" t="str">
+        <x:v>low.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D65" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E65" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F65" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G65" s="45" t="n">
+        <x:v>258327110.88</x:v>
+      </x:c>
+      <x:c r="H65" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I65" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J65" s="45" t="n">
+        <x:f>G65/I65</x:f>
+        <x:v>144474304.51375833</x:v>
+      </x:c>
+      <x:c r="K65" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L65" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M65" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N65" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="25.5" customHeight="1">
+      <x:c r="A66" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B66" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C66" s="14" t="str">
+        <x:v>low.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D66" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E66" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F66" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G66" s="45" t="n">
+        <x:v>275335272.8</x:v>
+      </x:c>
+      <x:c r="H66" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I66" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J66" s="45" t="n">
+        <x:f>G66/I66</x:f>
+        <x:v>153986439.55865824</x:v>
+      </x:c>
+      <x:c r="K66" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L66" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M66" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N66" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="25.5" customHeight="1">
+      <x:c r="A67" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B67" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C67" s="14" t="str">
+        <x:v>low.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D67" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E67" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F67" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G67" s="45" t="n">
+        <x:v>533662383.68</x:v>
+      </x:c>
+      <x:c r="H67" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I67" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J67" s="45" t="n">
+        <x:f>G67/I67</x:f>
+        <x:v>298460744.0724166</x:v>
+      </x:c>
+      <x:c r="K67" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L67" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M67" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N67" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="25.5" customHeight="1">
+      <x:c r="A68" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B68" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C68" s="14" t="str">
+        <x:v>base.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D68" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E68" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F68" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G68" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H68" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I68" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J68" s="45" t="n">
+        <x:f>G68/I68</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K68" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L68" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M68" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N68" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="25.5" customHeight="1">
+      <x:c r="A69" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B69" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C69" s="14" t="str">
+        <x:v>base.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D69" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E69" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F69" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G69" s="45" t="n">
+        <x:v>367631277.68</x:v>
+      </x:c>
+      <x:c r="H69" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I69" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J69" s="45" t="n">
+        <x:f>G69/I69</x:f>
+        <x:v>205604719.4558489</x:v>
+      </x:c>
+      <x:c r="K69" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L69" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M69" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N69" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="25.5" customHeight="1">
+      <x:c r="A70" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B70" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C70" s="14" t="str">
+        <x:v>base.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D70" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E70" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F70" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G70" s="45" t="n">
+        <x:v>641811687.89</x:v>
+      </x:c>
+      <x:c r="H70" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I70" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J70" s="45" t="n">
+        <x:f>G70/I70</x:f>
+        <x:v>358945280.34954304</x:v>
+      </x:c>
+      <x:c r="K70" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L70" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M70" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N70" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="25.5" customHeight="1">
+      <x:c r="A71" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B71" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C71" s="14" t="str">
+        <x:v>high.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D71" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E71" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F71" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G71" s="45" t="n">
+        <x:v>274180410.21</x:v>
+      </x:c>
+      <x:c r="H71" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I71" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J71" s="45" t="n">
+        <x:f>G71/I71</x:f>
+        <x:v>153340560.89369413</x:v>
+      </x:c>
+      <x:c r="K71" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L71" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M71" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N71" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="25.5" customHeight="1">
+      <x:c r="A72" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B72" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C72" s="14" t="str">
+        <x:v>high.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D72" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E72" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F72" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G72" s="45" t="n">
+        <x:v>456995382.29</x:v>
+      </x:c>
+      <x:c r="H72" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I72" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J72" s="45" t="n">
+        <x:f>G72/I72</x:f>
+        <x:v>255583278.88015154</x:v>
+      </x:c>
+      <x:c r="K72" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L72" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M72" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N72" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="25.5" customHeight="1">
+      <x:c r="A73" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B73" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C73" s="14" t="str">
+        <x:v>high.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D73" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E73" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F73" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G73" s="45" t="n">
+        <x:v>731175792.5</x:v>
+      </x:c>
+      <x:c r="H73" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I73" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J73" s="45" t="n">
+        <x:f>G73/I73</x:f>
+        <x:v>408923839.7738457</x:v>
+      </x:c>
+      <x:c r="K73" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L73" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M73" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N73" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="25.5" customHeight="1">
+      <x:c r="A74" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B74" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C74" s="14" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="D74" s="14"/>
+      <x:c r="E74" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F74" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G74" s="45" t="n">
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="H74" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I74" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J74" s="45" t="n">
+        <x:f>G74</x:f>
+        <x:v>667920000</x:v>
+      </x:c>
+      <x:c r="K74" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L74" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M74" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N74" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="25.5" customHeight="1">
+      <x:c r="A75" s="14" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B75" s="14" t="str">
+        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+      </x:c>
+      <x:c r="C75" s="14" t="str">
+        <x:v>central</x:v>
+      </x:c>
+      <x:c r="D75" s="14"/>
+      <x:c r="E75" s="14" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="F75" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G75" s="45" t="n">
         <x:v>1199220000</x:v>
       </x:c>
-      <x:c r="H44" s="45" t="str">
+      <x:c r="H75" s="45" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="I44" s="45" t="n">
+      <x:c r="I75" s="45" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J44" s="45" t="n">
-        <x:f>G44</x:f>
+      <x:c r="J75" s="45" t="n">
+        <x:f>G75</x:f>
         <x:v>1199220000</x:v>
       </x:c>
-      <x:c r="K44" s="14" t="str">
+      <x:c r="K75" s="14" t="str">
         <x:v>EUR-IDENTITY</x:v>
       </x:c>
-      <x:c r="L44" s="14" t="str">
+      <x:c r="L75" s="14" t="str">
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
-      <x:c r="M44" s="14" t="str">
+      <x:c r="M75" s="14" t="str">
         <x:v>already_eur</x:v>
       </x:c>
-      <x:c r="N44" s="14" t="str">
+      <x:c r="N75" s="14" t="str">
         <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="25.5" customHeight="1">
-      <x:c r="A45" s="15" t="str">
+    <x:row r="76" ht="25.5" customHeight="1">
+      <x:c r="A76" s="15" t="str">
         <x:v>model</x:v>
       </x:c>
-      <x:c r="B45" s="15" t="str">
+      <x:c r="B76" s="15" t="str">
         <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
       </x:c>
-      <x:c r="C45" s="15" t="str">
+      <x:c r="C76" s="15" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="D45" s="15"/>
-      <x:c r="E45" s="15" t="n">
+      <x:c r="D76" s="15"/>
+      <x:c r="E76" s="15" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="F45" s="15" t="str">
+      <x:c r="F76" s="15" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
-      <x:c r="G45" s="46" t="n">
+      <x:c r="G76" s="46" t="n">
         <x:v>1654620000</x:v>
       </x:c>
-      <x:c r="H45" s="46" t="str">
+      <x:c r="H76" s="46" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="I45" s="46" t="n">
+      <x:c r="I76" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J45" s="46" t="n">
-        <x:f>G45</x:f>
+      <x:c r="J76" s="46" t="n">
+        <x:f>G76</x:f>
         <x:v>1654620000</x:v>
       </x:c>
-      <x:c r="K45" s="15" t="str">
+      <x:c r="K76" s="15" t="str">
         <x:v>EUR-IDENTITY</x:v>
       </x:c>
-      <x:c r="L45" s="15" t="str">
+      <x:c r="L76" s="15" t="str">
         <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
-      <x:c r="M45" s="15" t="str">
+      <x:c r="M76" s="15" t="str">
         <x:v>already_eur</x:v>
       </x:c>
-      <x:c r="N45" s="15" t="str">
+      <x:c r="N76" s="15" t="str">
         <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95774ccc37c49e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe581b66afbf4775"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish v41 donor-control checkpoint (#38)
Co-authored-by: jounirautio78-ops <jounirautio78-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-en.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-en.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="R6cfd5a0345244ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8cd41972a2f147b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="Rdf6fee85d1354963"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5b240c5013ab4964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R21dd5aa9add24763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="1" r:id="Ra750953b0efb45e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R51debb22911341db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer questions" sheetId="3" r:id="R8cda80fb9a3545b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R00af4b2413b44413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR equivalents" sheetId="5" r:id="R2bbabee95be94804"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourcesEN" displayName="SourcesEN" ref="A1:E102" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Publisher"/>
@@ -351,7 +351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EurEquivalentsEN" displayName="EurEquivalentsEN" ref="A1:N76" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Record type"/>
     <x:tableColumn id="2" name="Record ID"/>
@@ -1073,7 +1073,7 @@
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>The public market dataset contains 84 observations from 24 sources; its 75 official observations split into 39 market measures and 36 Swedish FHM register-structure counts.</x:v>
+        <x:v>The public market dataset contains 156 observations from 47 sources; its 134 official observations split into 98 market measures and 36 Swedish FHM register-structure counts.</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Market size</x:v>
@@ -1088,7 +1088,7 @@
         <x:v>2026-07-27</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>84 = 48 market and model observations + 36 FHM structure counts; 75 official = 39 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
+        <x:v>156 = 120 market and model observations + 36 FHM structure counts; 134 official = 98 market measures + 36 structure counts. The roles remain separate and are not summed into a market.</x:v>
       </x:c>
       <x:c r="G18" s="14" t="str">
         <x:v>The 2018–2025 figures are authority-supplied year labels, not assumed calendar-year flows or year-end snapshots. The 2026 FHM records are a current snapshot, not a completed annual period. Official sourcing does not make unlike metrics comparable.</x:v>
@@ -1218,89 +1218,89 @@
     </x:row>
     <x:row r="23" ht="58.5" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>New Zealand's separate supported 2024 RPS retail-sensitivity model is NZD 533,662,383.68–731,175,792.50, with a base case of NZD 641,811,687.89.</x:v>
+        <x:v>Stats NZ's selected 2024 HS10 control yields NZD 183,370,681 and NZD 197,070,322 net border proxies; neither is retail market value.</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>The combined low, base and high cases are NZD 533,662,383.68 / 641,811,687.89 / 731,175,792.50. The model combines the specialist-retailer anchor with a general-retailer quantity-and-price model.</x:v>
+        <x:v>Selected imports are NZD 189,640,890 at value for duty and NZD 203,340,531 at CIF. Selected exports are NZD 6,270,209 FOB. The control applies a locked 2024 product-code selection rule.</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2024 ; source/NZ_2024_RPS_RETAIL_VALUE_SENSITIVITY.md ; source/NZ_2024_DONOR_CLOSURE_PACK.md</x:v>
+        <x:v>https://www.stats.govt.nz/large-datasets/csv-files-for-download/overseas-merchandise-trade-datasets/ ; https://www3.stats.govt.nz/HS10_by_Country/2024_Imports_HS10.zip ; https://www3.stats.govt.nz/HS10_by_Country/2024_Exports_HS10.zip ; source/NZ_CA_DE_DONOR_CONTROL_SPRINT_2026-08-02.md</x:v>
       </x:c>
       <x:c r="E23" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Low (exact-row deduplication): NZD 258,327,110.88 + 275,335,272.80 = 533,662,383.68. Base (reported/raw rows): NZD 274,180,410.21 + 367,631,277.68 = 641,811,687.89. High (reported/raw rows): NZD 274,180,410.21 + 456,995,382.29 = 731,175,792.50.</x:v>
+        <x:v>NZD 189,640,890 − 6,270,209 = 183,370,681; NZD 203,340,531 − 6,270,209 = 197,070,322. Candidate / proxies = 1.495224911 and 1.391282094.</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>GST treatment, return completeness and independent reconciliation are open; notifier supply-stage values are excluded.</x:v>
+        <x:v>Border event stage, product scope, domestic production, inventory, re-exports, margins, channels, GST and consumer sell-through do not match the retail boundary.</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I23" s="14" t="str">
-        <x:v>Not an observed national value or accepted donor. Authority confirmation of scope and GST plus independent reproduction are required.</x:v>
+        <x:v>The ratios are not margin, uplift, validation intervals or a market range. D10 remains open and New Zealand remains 7/10 NOT ACCEPTED.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58.5" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>The new numerical reconstruction from the six official 2023 workbooks is intentionally not computed.</x:v>
+        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>Market size</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>The Ministry's published aggregate is at least NZD 374 million and 2,570 returns. It covers all notifiable products, including heated tobacco, and the Ministry warns about data quality.</x:v>
+        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return/annual-returns-2023 ; source/NZ_2023_ANNUAL_RETURNS_FAIL_CLOSED.md</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>2026-07-26</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Six official files are integrity-hashed; every new computation returns not_computed.</x:v>
+        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
       </x:c>
       <x:c r="G24" s="14" t="str">
-        <x:v>Product scope, quantity fields, duplication, supply-chain level, tax basis and independent reconciliation remain unresolved.</x:v>
+        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
       </x:c>
       <x:c r="H24" s="14" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Supported</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
-        <x:v>A new 2023 vaping-only value is missing, and NZD 374 million must not be relabelled as a pure vaping market.</x:v>
+        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58.5" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Official FTC tables yield USD 2,763,284,338 of reported cartridge-system-plus-disposable sales in 2021.</x:v>
+        <x:v>Germany's prospective vendor benchmark DE-BLIND-1.0.0 was locked before any future submission is scored; it is NOT SCORED.</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>Market size</x:v>
+        <x:v>Market size / Germany</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>The seven-year 2015–2021 series sums the cartridge-system and disposable rows annually. The corrected 2020 table covers five prior recipients plus three of four new recipients; 2021 covers all nine recipients.</x:v>
+        <x:v>Final official anchors are 1,241,000 litres for 2023 and 1,284,000 litres for 2024, or 2,525,000 litres combined. Preregistered caps are 15% annually and 10% combined.</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018 ; https://www.ftc.gov/reports/e-cigarette-report-2021 ; source/US_FTC_2015_2021_REPORTED_SALES.md</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003/ ; source/NZ_CA_DE_DONOR_CONTROL_SPRINT_2026-08-02.md</x:v>
       </x:c>
       <x:c r="E25" s="14" t="str">
-        <x:v>2021</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Annual sum of FTC-table cartridge systems + disposable e-cigarette sales.</x:v>
+        <x:v>Annual deviation = |vendor litres / official litres − 1|; combined deviation = |vendor two-year sum / 2,525,000 − 1|.</x:v>
       </x:c>
       <x:c r="G25" s="14" t="str">
-        <x:v>The reporting population changes, open-system products are excluded, the level is manufacturer reporting and the tax basis is unstated.</x:v>
+        <x:v>A numeric match alone does not establish matching product, unit, tax basis, channel or event stage. Thresholds are not tuned to private values.</x:v>
       </x:c>
       <x:c r="H25" s="14" t="str">
-        <x:v>Supported</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
-        <x:v>Not complete national consumer-retail value or an accepted donor; an open POS or consumer-sales series and tax basis are required.</x:v>
+        <x:v>Passing does not accept Germany as a donor or authorise a purchase, licence, fee or disclosure. Germany's official retail value remains not_computed.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58.5" customHeight="1">
@@ -1317,7 +1317,7 @@
         <x:v>site/data/evidence-lanes.json ; site/data/donor-cockpit.json ; site/data/third-donor-screen.json ; site/data/country-scenarios.json</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>2026-07-27</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
         <x:v>Fail-closed gates: a missing or invalid input returns not_computed rather than zero.</x:v>
@@ -1387,7 +1387,7 @@
         <x:v>Supported</x:v>
       </x:c>
       <x:c r="I28" s="14" t="str">
-        <x:v>D5 failed because NAICS 459999 specialist retail is outside the confirmed 441100–459993 target range. D7 failed because exact product-class quality and annual-uncertainty information is unavailable. D10 remains open; Canada is not an accepted donor.</x:v>
+        <x:v>D5 failed because NAICS 459999 specialist retail is outside the confirmed 441100–459993 target range; in-scope online sales do not cover excluded specialist, foreign direct or cross-border channels. D7 failed because exact NAPCS 5619122 response, imputation, CV, standard-error, confidence-interval and covariance metrics are unavailable. D10 remains open; Canada is not an accepted donor.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58.5" customHeight="1">
@@ -1610,7 +1610,7 @@
         <x:v>2026-07-24</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 39 market measures and 36 structure counts remain separate.</x:v>
+        <x:v>36 = 9 years (2018–2026) × 4 register-structure metrics. The tax anchor, 98 market measures and 36 structure counts remain separate.</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
         <x:v>No sales value, sales volume or market share is inferred from the structure counts. The 2018–2025 figures are authority-supplied year labels, not assumed annual flows or year-end snapshots. The 2026 records are a current snapshot and are not annualised.</x:v>
@@ -2361,7 +2361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954404b7d653401c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdecff32e9b034609"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>2026.07.31-37</x:v>
+        <x:v>2026.08.02-41</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20.25" customHeight="1">
@@ -2427,7 +2427,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -2460,7 +2460,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A11)</x:f>
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
@@ -2469,7 +2469,7 @@
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>COUNTIF('Evidence Register'!$H$2:$H$61,A12)</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">
@@ -2671,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bdb2db608a14175"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda256a45c5674ce7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,7 +3585,7 @@
         <x:v>https://api.sejm.gov.pl/eli/acts/DU/2025/698/text.pdf</x:v>
       </x:c>
       <x:c r="E53" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="31.5" customHeight="1">
@@ -3602,7 +3602,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="31.5" customHeight="1">
@@ -3619,7 +3619,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E55" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="31.5" customHeight="1">
@@ -3636,7 +3636,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E56" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="31.5" customHeight="1">
@@ -3653,7 +3653,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E57" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="31.5" customHeight="1">
@@ -3670,7 +3670,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E58" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="31.5" customHeight="1">
@@ -3687,7 +3687,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E59" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="31.5" customHeight="1">
@@ -3704,7 +3704,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E60" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="31.5" customHeight="1">
@@ -3721,7 +3721,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
@@ -3738,7 +3738,7 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E62" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="31.5" customHeight="1">
@@ -3755,12 +3755,12 @@
         <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E63" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="31.5" customHeight="1">
       <x:c r="A64" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
+        <x:v>REGISTER-REFERENCE-BCE59F2D3F9D</x:v>
       </x:c>
       <x:c r="B64" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3769,15 +3769,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D64" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E64" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="31.5" customHeight="1">
       <x:c r="A65" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
+        <x:v>REGISTER-REFERENCE-2267B190A073</x:v>
       </x:c>
       <x:c r="B65" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3786,15 +3786,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D65" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="31.5" customHeight="1">
       <x:c r="A66" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
+        <x:v>REGISTER-REFERENCE-957871D9CB33</x:v>
       </x:c>
       <x:c r="B66" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3803,15 +3803,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D66" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="31.5" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
+        <x:v>REGISTER-REFERENCE-5C7194247112</x:v>
       </x:c>
       <x:c r="B67" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3820,15 +3820,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D67" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E67" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="31.5" customHeight="1">
       <x:c r="A68" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
+        <x:v>REGISTER-REFERENCE-75BF634166B2</x:v>
       </x:c>
       <x:c r="B68" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3837,15 +3837,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D68" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E68" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="31.5" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
+        <x:v>REGISTER-REFERENCE-54AB30A87D3D</x:v>
       </x:c>
       <x:c r="B69" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3854,15 +3854,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D69" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E69" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="31.5" customHeight="1">
       <x:c r="A70" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
+        <x:v>REGISTER-REFERENCE-4B9D48C385C9</x:v>
       </x:c>
       <x:c r="B70" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3871,15 +3871,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D70" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E70" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="31.5" customHeight="1">
       <x:c r="A71" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
+        <x:v>REGISTER-REFERENCE-97704C5CE7D4</x:v>
       </x:c>
       <x:c r="B71" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3888,15 +3888,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D71" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E71" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="31.5" customHeight="1">
       <x:c r="A72" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
+        <x:v>REGISTER-REFERENCE-EF5511CEAE3C</x:v>
       </x:c>
       <x:c r="B72" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3905,15 +3905,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D72" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E72" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="31.5" customHeight="1">
       <x:c r="A73" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
+        <x:v>REGISTER-REFERENCE-15452EF50F15</x:v>
       </x:c>
       <x:c r="B73" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3922,15 +3922,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D73" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E73" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="31.5" customHeight="1">
       <x:c r="A74" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
+        <x:v>REGISTER-REFERENCE-9C7C0F0FD33F</x:v>
       </x:c>
       <x:c r="B74" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3939,15 +3939,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D74" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E74" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="31.5" customHeight="1">
       <x:c r="A75" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
+        <x:v>REGISTER-REFERENCE-82A9C0A0E9C4</x:v>
       </x:c>
       <x:c r="B75" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3956,15 +3956,15 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D75" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="31.5" customHeight="1">
       <x:c r="A76" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
+        <x:v>REGISTER-REFERENCE-25E2E410922F</x:v>
       </x:c>
       <x:c r="B76" s="14" t="str">
         <x:v>data-api.ecb.europa.eu</x:v>
@@ -3973,305 +3973,458 @@
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D76" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="31.5" customHeight="1">
       <x:c r="A77" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
+        <x:v>REGISTER-REFERENCE-74211110370B</x:v>
       </x:c>
       <x:c r="B77" s="14" t="str">
-        <x:v>data.ecb.europa.eu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C77" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D77" s="14" t="str">
-        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E77" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="31.5" customHeight="1">
       <x:c r="A78" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
+        <x:v>REGISTER-REFERENCE-59446D8EB279</x:v>
       </x:c>
       <x:c r="B78" s="14" t="str">
-        <x:v>datahelpdesk.worldbank.org</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C78" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D78" s="14" t="str">
-        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E78" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="31.5" customHeight="1">
       <x:c r="A79" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
+        <x:v>REGISTER-REFERENCE-BFB2E2E1B4A3</x:v>
       </x:c>
       <x:c r="B79" s="14" t="str">
-        <x:v>douanes.public.lu</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C79" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D79" s="14" t="str">
-        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E79" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="31.5" customHeight="1">
       <x:c r="A80" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
+        <x:v>REGISTER-REFERENCE-D26C27B033B0</x:v>
       </x:c>
       <x:c r="B80" s="14" t="str">
-        <x:v>laws-lois.justice.gc.ca</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C80" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D80" s="14" t="str">
-        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E80" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="31.5" customHeight="1">
       <x:c r="A81" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
+        <x:v>REGISTER-REFERENCE-32690599750D</x:v>
       </x:c>
       <x:c r="B81" s="14" t="str">
-        <x:v>adm.gov.it</x:v>
+        <x:v>data-api.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C81" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D81" s="14" t="str">
-        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="E81" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="31.5" customHeight="1">
       <x:c r="A82" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
+        <x:v>REGISTER-REFERENCE-9B93C76EF890</x:v>
       </x:c>
       <x:c r="B82" s="14" t="str">
-        <x:v>ecb.europa.eu</x:v>
+        <x:v>data.ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C82" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D82" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="E82" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="31.5" customHeight="1">
       <x:c r="A83" s="14" t="str">
-        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
+        <x:v>REGISTER-REFERENCE-2DA87527D51F</x:v>
       </x:c>
       <x:c r="B83" s="14" t="str">
-        <x:v>Public Health Agency of Sweden</x:v>
+        <x:v>datahelpdesk.worldbank.org</x:v>
       </x:c>
       <x:c r="C83" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D83" s="14" t="str">
-        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
+        <x:v>https://datahelpdesk.worldbank.org/knowledgebase/articles/898581-api-basic-call-structures</x:v>
       </x:c>
       <x:c r="E83" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="31.5" customHeight="1">
       <x:c r="A84" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
+        <x:v>REGISTER-REFERENCE-1208D3C8F46C</x:v>
       </x:c>
       <x:c r="B84" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>douanes.public.lu</x:v>
       </x:c>
       <x:c r="C84" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D84" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
+        <x:v>https://douanes.public.lu/dam-assets/fr/accises/signes-fiscaux/2024/s48/bareme-e-liquide-s48.pdf</x:v>
       </x:c>
       <x:c r="E84" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="31.5" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
+        <x:v>REGISTER-REFERENCE-25E8C2FC0150</x:v>
       </x:c>
       <x:c r="B85" s="14" t="str">
-        <x:v>Federal Trade Commission</x:v>
+        <x:v>genesis.destatis.de</x:v>
       </x:c>
       <x:c r="C85" s="14" t="str">
-        <x:v>official_report</x:v>
+        <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D85" s="14" t="str">
-        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
+        <x:v>https://genesis.destatis.de/datenbank/online/statistic/73411/table/73411-0003/</x:v>
       </x:c>
       <x:c r="E85" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="31.5" customHeight="1">
       <x:c r="A86" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
+        <x:v>REGISTER-REFERENCE-77110A089CB9</x:v>
       </x:c>
       <x:c r="B86" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>laws-lois.justice.gc.ca</x:v>
       </x:c>
       <x:c r="C86" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D86" s="14" t="str">
-        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+        <x:v>https://laws-lois.justice.gc.ca/eng/regulations/SOR-2023-123/FullText.html</x:v>
       </x:c>
       <x:c r="E86" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="31.5" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-1766C84ECA96</x:v>
+        <x:v>REGISTER-REFERENCE-A3B80D981A8D</x:v>
       </x:c>
       <x:c r="B87" s="14" t="str">
-        <x:v>health.govt.nz</x:v>
+        <x:v>adm.gov.it</x:v>
       </x:c>
       <x:c r="C87" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D87" s="14" t="str">
-        <x:v>https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf</x:v>
+        <x:v>https://www.adm.gov.it/portale/documents/20182/261920520/Libro+blu+2024+-+Relazione.pdf/e46989ce-b39f-a404-3b4b-2af3196cba43</x:v>
       </x:c>
       <x:c r="E87" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="31.5" customHeight="1">
       <x:c r="A88" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-529570B0D6C7</x:v>
+        <x:v>REGISTER-REFERENCE-50ED634F402A</x:v>
       </x:c>
       <x:c r="B88" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>ecb.europa.eu</x:v>
       </x:c>
       <x:c r="C88" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D88" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="E88" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="31.5" customHeight="1">
       <x:c r="A89" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+        <x:v>SE-FHM-PUBLIC-RECORD-RESPONSE-2026-07-24</x:v>
       </x:c>
       <x:c r="B89" s="14" t="str">
-        <x:v>podatki.gov.pl</x:v>
+        <x:v>Public Health Agency of Sweden</x:v>
       </x:c>
       <x:c r="C89" s="14" t="str">
-        <x:v>register_reference</x:v>
+        <x:v>official_reference</x:v>
       </x:c>
       <x:c r="D89" s="14" t="str">
-        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+        <x:v>https://www.folkhalsomyndigheten.se/regler-och-tillsyn/tobak-och-nikotinprodukter-regler-for-tillverkning-handel-och-hantering/elektroniska-cigaretter-och-pafyllningsbehallare-sa-foljer-du-reglerna/</x:v>
       </x:c>
       <x:c r="E89" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="31.5" customHeight="1">
       <x:c r="A90" s="14" t="str">
-        <x:v>UN-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2015-2018</x:v>
       </x:c>
       <x:c r="B90" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C90" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D90" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2015-2018</x:v>
       </x:c>
       <x:c r="E90" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="31.5" customHeight="1">
       <x:c r="A91" s="14" t="str">
-        <x:v>UN-NON-MEMBER-STATES</x:v>
+        <x:v>US-FTC-E-CIGARETTE-REPORT-2021</x:v>
       </x:c>
       <x:c r="B91" s="14" t="str">
-        <x:v>United Nations</x:v>
+        <x:v>Federal Trade Commission</x:v>
       </x:c>
       <x:c r="C91" s="14" t="str">
-        <x:v>official_reference</x:v>
+        <x:v>official_report</x:v>
       </x:c>
       <x:c r="D91" s="14" t="str">
-        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+        <x:v>https://www.ftc.gov/reports/e-cigarette-report-2021</x:v>
       </x:c>
       <x:c r="E91" s="14" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="31.5" customHeight="1">
       <x:c r="A92" s="14" t="str">
-        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+        <x:v>REGISTER-REFERENCE-E034CF64F670</x:v>
       </x:c>
       <x:c r="B92" s="14" t="str">
-        <x:v>www150.statcan.gc.ca</x:v>
+        <x:v>health.govt.nz</x:v>
       </x:c>
       <x:c r="C92" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
       <x:c r="D92" s="14" t="str">
+        <x:v>https://www.health.govt.nz/regulation-legislation/vaping-herbal-smoking-and-smokeless-tobacco/requirements/complete-a-notifiable-product-annual-return</x:v>
+      </x:c>
+      <x:c r="E92" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="31.5" customHeight="1">
+      <x:c r="A93" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-1766C84ECA96</x:v>
+      </x:c>
+      <x:c r="B93" s="14" t="str">
+        <x:v>health.govt.nz</x:v>
+      </x:c>
+      <x:c r="C93" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D93" s="14" t="str">
+        <x:v>https://www.health.govt.nz/system/files/2025-11/notifiable-products-annual-sales-return-2025-user-guide.pdf</x:v>
+      </x:c>
+      <x:c r="E93" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="31.5" customHeight="1">
+      <x:c r="A94" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-529570B0D6C7</x:v>
+      </x:c>
+      <x:c r="B94" s="14" t="str">
+        <x:v>podatki.gov.pl</x:v>
+      </x:c>
+      <x:c r="C94" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D94" s="14" t="str">
+        <x:v>https://www.podatki.gov.pl/akcyza/komunikaty-w-zakresie-podatku-akcyzowego</x:v>
+      </x:c>
+      <x:c r="E94" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="31.5" customHeight="1">
+      <x:c r="A95" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-7AD3E1157197</x:v>
+      </x:c>
+      <x:c r="B95" s="14" t="str">
+        <x:v>podatki.gov.pl</x:v>
+      </x:c>
+      <x:c r="C95" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D95" s="14" t="str">
+        <x:v>https://www.podatki.gov.pl/akcyza/stawki-podatkowe/</x:v>
+      </x:c>
+      <x:c r="E95" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="31.5" customHeight="1">
+      <x:c r="A96" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-645255DD4B34</x:v>
+      </x:c>
+      <x:c r="B96" s="14" t="str">
+        <x:v>stats.govt.nz</x:v>
+      </x:c>
+      <x:c r="C96" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D96" s="14" t="str">
+        <x:v>https://www.stats.govt.nz/large-datasets/csv-files-for-download/overseas-merchandise-trade-datasets/</x:v>
+      </x:c>
+      <x:c r="E96" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="31.5" customHeight="1">
+      <x:c r="A97" s="14" t="str">
+        <x:v>UN-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B97" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C97" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D97" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/member-states</x:v>
+      </x:c>
+      <x:c r="E97" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="31.5" customHeight="1">
+      <x:c r="A98" s="14" t="str">
+        <x:v>UN-NON-MEMBER-STATES</x:v>
+      </x:c>
+      <x:c r="B98" s="14" t="str">
+        <x:v>United Nations</x:v>
+      </x:c>
+      <x:c r="C98" s="14" t="str">
+        <x:v>official_reference</x:v>
+      </x:c>
+      <x:c r="D98" s="14" t="str">
+        <x:v>https://www.un.org/en/about-us/non-member-states</x:v>
+      </x:c>
+      <x:c r="E98" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="31.5" customHeight="1">
+      <x:c r="A99" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-3332B0031C1D</x:v>
+      </x:c>
+      <x:c r="B99" s="14" t="str">
+        <x:v>www150.statcan.gc.ca</x:v>
+      </x:c>
+      <x:c r="C99" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D99" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010007101</x:v>
       </x:c>
-      <x:c r="E92" s="14" t="str">
-        <x:v>2026-07-31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="31.5" customHeight="1">
-      <x:c r="A93" s="15" t="str">
+      <x:c r="E99" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="31.5" customHeight="1">
+      <x:c r="A100" s="14" t="str">
         <x:v>REGISTER-REFERENCE-D61AFC87FA19</x:v>
       </x:c>
-      <x:c r="B93" s="15" t="str">
+      <x:c r="B100" s="14" t="str">
         <x:v>www150.statcan.gc.ca</x:v>
       </x:c>
-      <x:c r="C93" s="15" t="str">
+      <x:c r="C100" s="14" t="str">
         <x:v>register_reference</x:v>
       </x:c>
-      <x:c r="D93" s="15" t="str">
+      <x:c r="D100" s="14" t="str">
         <x:v>https://www150.statcan.gc.ca/t1/tbl1/en/tv.action?pid=2010008001</x:v>
       </x:c>
-      <x:c r="E93" s="15" t="str">
-        <x:v>2026-07-31</x:v>
+      <x:c r="E100" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="31.5" customHeight="1">
+      <x:c r="A101" s="14" t="str">
+        <x:v>REGISTER-REFERENCE-9479B1548E50</x:v>
+      </x:c>
+      <x:c r="B101" s="14" t="str">
+        <x:v>www3.stats.govt.nz</x:v>
+      </x:c>
+      <x:c r="C101" s="14" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D101" s="14" t="str">
+        <x:v>https://www3.stats.govt.nz/HS10_by_Country/2024_Exports_HS10.zip</x:v>
+      </x:c>
+      <x:c r="E101" s="14" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="31.5" customHeight="1">
+      <x:c r="A102" s="15" t="str">
+        <x:v>REGISTER-REFERENCE-94B1312153E9</x:v>
+      </x:c>
+      <x:c r="B102" s="15" t="str">
+        <x:v>www3.stats.govt.nz</x:v>
+      </x:c>
+      <x:c r="C102" s="15" t="str">
+        <x:v>register_reference</x:v>
+      </x:c>
+      <x:c r="D102" s="15" t="str">
+        <x:v>https://www3.stats.govt.nz/HS10_by_Country/2024_Imports_HS10.zip</x:v>
+      </x:c>
+      <x:c r="E102" s="15" t="str">
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfba39bfbba49c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5824c78453646dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5110,22 +5263,22 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
-        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>DE-2019-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
-        <x:v>Finland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E19" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G19" s="45" t="n">
-        <x:v>3540319</x:v>
+        <x:v>2247267035</x:v>
       </x:c>
       <x:c r="H19" s="45" t="str">
         <x:v>EUR</x:v>
@@ -5135,7 +5288,7 @@
       </x:c>
       <x:c r="J19" s="45" t="n">
         <x:f>G19</x:f>
-        <x:v>3540319</x:v>
+        <x:v>2247267035</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
         <x:v>EUR-IDENTITY</x:v>
@@ -5155,44 +5308,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
+        <x:v>DE-2020-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>e_liquid_excise_amount</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E20" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G20" s="45" t="n">
-        <x:v>993100000</x:v>
+        <x:v>2444948000</x:v>
       </x:c>
       <x:c r="H20" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I20" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J20" s="45" t="n">
-        <x:f>G20/I20</x:f>
-        <x:v>234240611.54771507</x:v>
+        <x:f>G20</x:f>
+        <x:v>2444948000</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L20" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M20" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N20" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25.5" customHeight="1">
@@ -5200,44 +5353,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
-        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
+        <x:v>DE-2021-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>vaporisation_device_broad_group_excise_amount</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E21" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G21" s="45" t="n">
-        <x:v>175300000</x:v>
+        <x:v>2325648577</x:v>
       </x:c>
       <x:c r="H21" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I21" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J21" s="45" t="n">
-        <x:f>G21/I21</x:f>
-        <x:v>41347678.183782555</x:v>
+        <x:f>G21</x:f>
+        <x:v>2325648577</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L21" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M21" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N21" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25.5" customHeight="1">
@@ -5245,44 +5398,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
-        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
+        <x:v>DE-2022-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>vaporisation_device_component_sets_broad_group_excise_amount</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
-        <x:v>Poland</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E22" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G22" s="45" t="n">
-        <x:v>2500000</x:v>
+        <x:v>2510888578</x:v>
       </x:c>
       <x:c r="H22" s="45" t="str">
-        <x:v>PLN</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I22" s="45" t="n">
-        <x:v>4.2396576470588</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J22" s="45" t="n">
-        <x:f>G22/I22</x:f>
-        <x:v>589670.2536192606</x:v>
+        <x:f>G22</x:f>
+        <x:v>2510888578</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
-        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L22" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M22" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N22" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25.5" customHeight="1">
@@ -5290,44 +5443,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
-        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
+        <x:v>DE-2023-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>nicotine_e_liquid_excise_receipts</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
-        <x:v>Sweden</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E23" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G23" s="45" t="n">
-        <x:v>80000000</x:v>
+        <x:v>2581608198</x:v>
       </x:c>
       <x:c r="H23" s="45" t="str">
-        <x:v>SEK</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I23" s="45" t="n">
-        <x:v>11.432519140625</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J23" s="45" t="n">
-        <x:f>G23/I23</x:f>
-        <x:v>6997582.861306848</x:v>
+        <x:f>G23</x:f>
+        <x:v>2581608198</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
-        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L23" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M23" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N23" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25.5" customHeight="1">
@@ -5335,44 +5488,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
-        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>DE-2024-WZ4726-TAXABLE-TURNOVER-EUR</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>wz4726_tobacco_specialist_taxable_supplies_and_services_turnover</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Germany</x:v>
       </x:c>
       <x:c r="E24" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G24" s="45" t="n">
-        <x:v>26000000000</x:v>
+        <x:v>2687776000</x:v>
       </x:c>
       <x:c r="H24" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I24" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J24" s="45" t="n">
-        <x:f>G24/I24</x:f>
-        <x:v>23009192918.721367</x:v>
+        <x:f>G24</x:f>
+        <x:v>2687776000</x:v>
       </x:c>
       <x:c r="K24" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L24" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M24" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N24" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="25.5" customHeight="1">
@@ -5380,44 +5533,44 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B25" s="14" t="str">
-        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>FI-2025-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Finland</x:v>
       </x:c>
       <x:c r="E25" s="14" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G25" s="45" t="n">
-        <x:v>45700000000</x:v>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="H25" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>EUR</x:v>
       </x:c>
       <x:c r="I25" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J25" s="45" t="n">
-        <x:f>G25/I25</x:f>
-        <x:v>40443081399.44486</x:v>
+        <x:f>G25</x:f>
+        <x:v>3540319</x:v>
       </x:c>
       <x:c r="K25" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>EUR-IDENTITY</x:v>
       </x:c>
       <x:c r="L25" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
       </x:c>
       <x:c r="M25" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>already_eur</x:v>
       </x:c>
       <x:c r="N25" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>original_currency_already_eur</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25.5" customHeight="1">
@@ -5425,38 +5578,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
+        <x:v>PL-2021-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>commercial_market_estimate</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
-        <x:v>Global</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E26" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>calendar_year_estimate</x:v>
+        <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G26" s="45" t="n">
-        <x:v>46320000000</x:v>
+        <x:v>179500000</x:v>
       </x:c>
       <x:c r="H26" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I26" s="45" t="n">
-        <x:v>1.1299831372549</x:v>
+        <x:v>4.5651786821705</x:v>
       </x:c>
       <x:c r="J26" s="45" t="n">
         <x:f>G26/I26</x:f>
-        <x:v>40991762153.66052</x:v>
+        <x:v>39319381.01372568</x:v>
       </x:c>
       <x:c r="K26" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2021</x:v>
       </x:c>
       <x:c r="L26" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M26" s="14" t="str">
         <x:v>computed</x:v>
@@ -5470,38 +5623,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B27" s="14" t="str">
-        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2022-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E27" s="14" t="n">
-        <x:v>2015</x:v>
+        <x:v>2022</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G27" s="45" t="n">
-        <x:v>304170046</x:v>
+        <x:v>229900000</x:v>
       </x:c>
       <x:c r="H27" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I27" s="45" t="n">
-        <x:v>1.109512890625</x:v>
+        <x:v>4.686106614786</x:v>
       </x:c>
       <x:c r="J27" s="45" t="n">
         <x:f>G27/I27</x:f>
-        <x:v>274147374.5552049</x:v>
+        <x:v>49059916.66399566</x:v>
       </x:c>
       <x:c r="K27" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2022</x:v>
       </x:c>
       <x:c r="L27" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2022&amp;endPeriod=2022&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M27" s="14" t="str">
         <x:v>computed</x:v>
@@ -5515,38 +5668,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2023-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E28" s="14" t="n">
-        <x:v>2016</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G28" s="45" t="n">
-        <x:v>485707484</x:v>
+        <x:v>443600000</x:v>
       </x:c>
       <x:c r="H28" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I28" s="45" t="n">
-        <x:v>1.1069031128405</x:v>
+        <x:v>4.5419658823529</x:v>
       </x:c>
       <x:c r="J28" s="45" t="n">
         <x:f>G28/I28</x:f>
-        <x:v>438798552.7961817</x:v>
+        <x:v>97666959.96628653</x:v>
       </x:c>
       <x:c r="K28" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2023</x:v>
       </x:c>
       <x:c r="L28" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M28" s="14" t="str">
         <x:v>computed</x:v>
@@ -5560,38 +5713,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B29" s="14" t="str">
-        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2024-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E29" s="14" t="n">
-        <x:v>2017</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G29" s="45" t="n">
-        <x:v>779836399</x:v>
+        <x:v>561400000</x:v>
       </x:c>
       <x:c r="H29" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I29" s="45" t="n">
-        <x:v>1.1296811764706</x:v>
+        <x:v>4.305795703125</x:v>
       </x:c>
       <x:c r="J29" s="45" t="n">
         <x:f>G29/I29</x:f>
-        <x:v>690315475.943752</x:v>
+        <x:v>130382405.18298511</x:v>
       </x:c>
       <x:c r="K29" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L29" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M29" s="14" t="str">
         <x:v>computed</x:v>
@@ -5605,44 +5758,37 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2015-UOKIK-E-CIGARETTE-MARKET-VALUE-ESTIMATE</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>institutional_market_value_benchmark</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E30" s="14" t="n">
-        <x:v>2018</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>study_reference_period_may_2015</x:v>
       </x:c>
       <x:c r="G30" s="45" t="n">
-        <x:v>2043703005</x:v>
+        <x:v>500000000</x:v>
       </x:c>
       <x:c r="H30" s="45" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="I30" s="45" t="n">
-        <x:v>1.1809545098039</x:v>
-      </x:c>
-      <x:c r="J30" s="45" t="n">
-        <x:f>G30/I30</x:f>
-        <x:v>1730551844.3207107</x:v>
-      </x:c>
-      <x:c r="K30" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
-      </x:c>
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I30" s="45"/>
+      <x:c r="J30" s="45"/>
+      <x:c r="K30" s="14"/>
       <x:c r="L30" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
       </x:c>
       <x:c r="M30" s="14" t="str">
-        <x:v>computed</x:v>
+        <x:v>not_computed</x:v>
       </x:c>
       <x:c r="N30" s="14" t="str">
-        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+        <x:v>period_not_compatible_with_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1">
@@ -5650,38 +5796,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B31" s="14" t="str">
-        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-E-LIQUID-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E31" s="14" t="n">
-        <x:v>2019</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G31" s="45" t="n">
-        <x:v>2702608307</x:v>
+        <x:v>993100000</x:v>
       </x:c>
       <x:c r="H31" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I31" s="45" t="n">
-        <x:v>1.1194745098039</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J31" s="45" t="n">
         <x:f>G31/I31</x:f>
-        <x:v>2414175832.796246</x:v>
+        <x:v>234240611.54771507</x:v>
       </x:c>
       <x:c r="K31" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L31" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M31" s="14" t="str">
         <x:v>computed</x:v>
@@ -5695,38 +5841,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B32" s="14" t="str">
-        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-DEVICE-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaporisation_device_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E32" s="14" t="n">
-        <x:v>2020</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G32" s="45" t="n">
-        <x:v>2394423105</x:v>
+        <x:v>175300000</x:v>
       </x:c>
       <x:c r="H32" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I32" s="45" t="n">
-        <x:v>1.1421961089494</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J32" s="45" t="n">
         <x:f>G32/I32</x:f>
-        <x:v>2096332745.523365</x:v>
+        <x:v>41347678.183782555</x:v>
       </x:c>
       <x:c r="K32" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L32" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M32" s="14" t="str">
         <x:v>computed</x:v>
@@ -5740,38 +5886,38 @@
         <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B33" s="14" t="str">
-        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
+        <x:v>PL-2025-VAPING-COMPONENT-SETS-EXCISE-AMOUNT</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+        <x:v>vaporisation_device_component_sets_broad_group_excise_amount</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
-        <x:v>United States</x:v>
+        <x:v>Poland</x:v>
       </x:c>
       <x:c r="E33" s="14" t="n">
-        <x:v>2021</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G33" s="45" t="n">
-        <x:v>2763284338</x:v>
+        <x:v>2500000</x:v>
       </x:c>
       <x:c r="H33" s="45" t="str">
-        <x:v>USD</x:v>
+        <x:v>PLN</x:v>
       </x:c>
       <x:c r="I33" s="45" t="n">
-        <x:v>1.1827403100775</x:v>
+        <x:v>4.2396576470588</x:v>
       </x:c>
       <x:c r="J33" s="45" t="n">
         <x:f>G33/I33</x:f>
-        <x:v>2336340711.866778</x:v>
+        <x:v>589670.2536192606</x:v>
       </x:c>
       <x:c r="K33" s="14" t="str">
-        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L33" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M33" s="14" t="str">
         <x:v>computed</x:v>
@@ -5782,16 +5928,16 @@
     </x:row>
     <x:row r="34" ht="25.5" customHeight="1">
       <x:c r="A34" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B34" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>SE-2024-NICOTINE-E-LIQUID-EXCISE-RECEIPTS</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>low.specialistRetailNzd</x:v>
+        <x:v>nicotine_e_liquid_excise_receipts</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Sweden</x:v>
       </x:c>
       <x:c r="E34" s="14" t="n">
         <x:v>2024</x:v>
@@ -5800,23 +5946,23 @@
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G34" s="45" t="n">
-        <x:v>258327110.88</x:v>
+        <x:v>80000000</x:v>
       </x:c>
       <x:c r="H34" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>SEK</x:v>
       </x:c>
       <x:c r="I34" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>11.432519140625</x:v>
       </x:c>
       <x:c r="J34" s="45" t="n">
         <x:f>G34/I34</x:f>
-        <x:v>144474304.51375833</x:v>
+        <x:v>6997582.861306848</x:v>
       </x:c>
       <x:c r="K34" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-SEK-EUR-SP00-A-2024</x:v>
       </x:c>
       <x:c r="L34" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.SEK.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M34" s="14" t="str">
         <x:v>computed</x:v>
@@ -5827,41 +5973,41 @@
     </x:row>
     <x:row r="35" ht="25.5" customHeight="1">
       <x:c r="A35" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B35" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>GLOBAL-2025-IMARC-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>low.generalRetailRpsNzd</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E35" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G35" s="45" t="n">
-        <x:v>275335272.8</x:v>
+        <x:v>26000000000</x:v>
       </x:c>
       <x:c r="H35" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I35" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J35" s="45" t="n">
         <x:f>G35/I35</x:f>
-        <x:v>153986439.55865824</x:v>
+        <x:v>23009192918.721367</x:v>
       </x:c>
       <x:c r="K35" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L35" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M35" s="14" t="str">
         <x:v>computed</x:v>
@@ -5872,41 +6018,41 @@
     </x:row>
     <x:row r="36" ht="25.5" customHeight="1">
       <x:c r="A36" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B36" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>GLOBAL-2025-GVR-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>low.combinedNzd</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E36" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G36" s="45" t="n">
-        <x:v>533662383.68</x:v>
+        <x:v>45700000000</x:v>
       </x:c>
       <x:c r="H36" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I36" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J36" s="45" t="n">
         <x:f>G36/I36</x:f>
-        <x:v>298460744.0724166</x:v>
+        <x:v>40443081399.44486</x:v>
       </x:c>
       <x:c r="K36" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L36" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M36" s="14" t="str">
         <x:v>computed</x:v>
@@ -5917,41 +6063,41 @@
     </x:row>
     <x:row r="37" ht="25.5" customHeight="1">
       <x:c r="A37" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>GLOBAL-2025-FORTUNE-COMMERCIAL-ESTIMATE</x:v>
       </x:c>
       <x:c r="C37" s="14" t="str">
-        <x:v>base.specialistRetailNzd</x:v>
+        <x:v>commercial_market_estimate</x:v>
       </x:c>
       <x:c r="D37" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>Global</x:v>
       </x:c>
       <x:c r="E37" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>calendar_year</x:v>
+        <x:v>calendar_year_estimate</x:v>
       </x:c>
       <x:c r="G37" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>46320000000</x:v>
       </x:c>
       <x:c r="H37" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I37" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1299831372549</x:v>
       </x:c>
       <x:c r="J37" s="45" t="n">
         <x:f>G37/I37</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>40991762153.66052</x:v>
       </x:c>
       <x:c r="K37" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2025</x:v>
       </x:c>
       <x:c r="L37" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2025&amp;endPeriod=2025&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M37" s="14" t="str">
         <x:v>computed</x:v>
@@ -5962,41 +6108,41 @@
     </x:row>
     <x:row r="38" ht="25.5" customHeight="1">
       <x:c r="A38" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2015-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>base.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E38" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G38" s="45" t="n">
-        <x:v>367631277.68</x:v>
+        <x:v>304170046</x:v>
       </x:c>
       <x:c r="H38" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I38" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.109512890625</x:v>
       </x:c>
       <x:c r="J38" s="45" t="n">
         <x:f>G38/I38</x:f>
-        <x:v>205604719.4558489</x:v>
+        <x:v>274147374.5552049</x:v>
       </x:c>
       <x:c r="K38" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2015</x:v>
       </x:c>
       <x:c r="L38" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2015&amp;endPeriod=2015&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M38" s="14" t="str">
         <x:v>computed</x:v>
@@ -6007,41 +6153,41 @@
     </x:row>
     <x:row r="39" ht="25.5" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B39" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2016-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>base.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E39" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2016</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G39" s="45" t="n">
-        <x:v>641811687.89</x:v>
+        <x:v>485707484</x:v>
       </x:c>
       <x:c r="H39" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I39" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1069031128405</x:v>
       </x:c>
       <x:c r="J39" s="45" t="n">
         <x:f>G39/I39</x:f>
-        <x:v>358945280.34954304</x:v>
+        <x:v>438798552.7961817</x:v>
       </x:c>
       <x:c r="K39" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2016</x:v>
       </x:c>
       <x:c r="L39" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2016&amp;endPeriod=2016&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M39" s="14" t="str">
         <x:v>computed</x:v>
@@ -6052,41 +6198,41 @@
     </x:row>
     <x:row r="40" ht="25.5" customHeight="1">
       <x:c r="A40" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B40" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2017-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C40" s="14" t="str">
-        <x:v>high.specialistRetailNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D40" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E40" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G40" s="45" t="n">
-        <x:v>274180410.21</x:v>
+        <x:v>779836399</x:v>
       </x:c>
       <x:c r="H40" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I40" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1296811764706</x:v>
       </x:c>
       <x:c r="J40" s="45" t="n">
         <x:f>G40/I40</x:f>
-        <x:v>153340560.89369413</x:v>
+        <x:v>690315475.943752</x:v>
       </x:c>
       <x:c r="K40" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2017</x:v>
       </x:c>
       <x:c r="L40" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2017&amp;endPeriod=2017&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M40" s="14" t="str">
         <x:v>computed</x:v>
@@ -6097,41 +6243,41 @@
     </x:row>
     <x:row r="41" ht="25.5" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B41" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2018-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>high.generalRetailRpsNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E41" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="F41" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G41" s="45" t="n">
-        <x:v>456995382.29</x:v>
+        <x:v>2043703005</x:v>
       </x:c>
       <x:c r="H41" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I41" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1809545098039</x:v>
       </x:c>
       <x:c r="J41" s="45" t="n">
         <x:f>G41/I41</x:f>
-        <x:v>255583278.88015154</x:v>
+        <x:v>1730551844.3207107</x:v>
       </x:c>
       <x:c r="K41" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2018</x:v>
       </x:c>
       <x:c r="L41" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2018&amp;endPeriod=2018&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M41" s="14" t="str">
         <x:v>computed</x:v>
@@ -6142,41 +6288,41 @@
     </x:row>
     <x:row r="42" ht="25.5" customHeight="1">
       <x:c r="A42" s="14" t="str">
-        <x:v>scenario_component</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B42" s="14" t="str">
-        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+        <x:v>US-2019-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C42" s="14" t="str">
-        <x:v>high.combinedNzd</x:v>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
       </x:c>
       <x:c r="D42" s="14" t="str">
-        <x:v>New Zealand</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="E42" s="14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G42" s="45" t="n">
-        <x:v>731175792.5</x:v>
+        <x:v>2702608307</x:v>
       </x:c>
       <x:c r="H42" s="45" t="str">
-        <x:v>NZD</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I42" s="45" t="n">
-        <x:v>1.788048828125</x:v>
+        <x:v>1.1194745098039</x:v>
       </x:c>
       <x:c r="J42" s="45" t="n">
         <x:f>G42/I42</x:f>
-        <x:v>408923839.7738457</x:v>
+        <x:v>2414175832.796246</x:v>
       </x:c>
       <x:c r="K42" s="14" t="str">
-        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2019</x:v>
       </x:c>
       <x:c r="L42" s="14" t="str">
-        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2019&amp;endPeriod=2019&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M42" s="14" t="str">
         <x:v>computed</x:v>
@@ -6187,137 +6333,1490 @@
     </x:row>
     <x:row r="43" ht="25.5" customHeight="1">
       <x:c r="A43" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>US-2020-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>low</x:v>
-      </x:c>
-      <x:c r="D43" s="14"/>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D43" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
       <x:c r="E43" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2020</x:v>
       </x:c>
       <x:c r="F43" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G43" s="45" t="n">
-        <x:v>667920000</x:v>
+        <x:v>2394423105</x:v>
       </x:c>
       <x:c r="H43" s="45" t="str">
-        <x:v>EUR</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="I43" s="45" t="n">
-        <x:v>1</x:v>
+        <x:v>1.1421961089494</x:v>
       </x:c>
       <x:c r="J43" s="45" t="n">
-        <x:f>G43</x:f>
-        <x:v>667920000</x:v>
+        <x:f>G43/I43</x:f>
+        <x:v>2096332745.523365</x:v>
       </x:c>
       <x:c r="K43" s="14" t="str">
-        <x:v>EUR-IDENTITY</x:v>
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2020</x:v>
       </x:c>
       <x:c r="L43" s="14" t="str">
-        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2020&amp;endPeriod=2020&amp;format=csvdata</x:v>
       </x:c>
       <x:c r="M43" s="14" t="str">
-        <x:v>already_eur</x:v>
+        <x:v>computed</x:v>
       </x:c>
       <x:c r="N43" s="14" t="str">
-        <x:v>original_currency_already_eur</x:v>
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="25.5" customHeight="1">
       <x:c r="A44" s="14" t="str">
-        <x:v>model</x:v>
+        <x:v>market_observation</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>DE-2025-LIQUID-RETAIL-EQUIVALENT-RANGE</x:v>
+        <x:v>US-2021-FTC-CARTRIDGE-DISPOSABLE-REPORTED-SALES</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>central</x:v>
-      </x:c>
-      <x:c r="D44" s="14"/>
+        <x:v>ftc_reported_cartridge_and_disposable_sales</x:v>
+      </x:c>
+      <x:c r="D44" s="14" t="str">
+        <x:v>United States</x:v>
+      </x:c>
       <x:c r="E44" s="14" t="n">
-        <x:v>2025</x:v>
+        <x:v>2021</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
         <x:v>calendar_year</x:v>
       </x:c>
       <x:c r="G44" s="45" t="n">
+        <x:v>2763284338</x:v>
+      </x:c>
+      <x:c r="H44" s="45" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I44" s="45" t="n">
+        <x:v>1.1827403100775</x:v>
+      </x:c>
+      <x:c r="J44" s="45" t="n">
+        <x:f>G44/I44</x:f>
+        <x:v>2336340711.866778</x:v>
+      </x:c>
+      <x:c r="K44" s="14" t="str">
+        <x:v>ECB-EXR-A-USD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L44" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.USD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M44" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N44" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="25.5" customHeight="1">
+      <x:c r="A45" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B45" s="14" t="str">
+        <x:v>NZ-2019-HES-E-CIGARETTES-AND-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C45" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D45" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E45" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F45" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G45" s="45" t="n">
+        <x:v>42276000</x:v>
+      </x:c>
+      <x:c r="H45" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I45" s="45"/>
+      <x:c r="J45" s="45"/>
+      <x:c r="K45" s="14"/>
+      <x:c r="L45" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M45" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N45" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="25.5" customHeight="1">
+      <x:c r="A46" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>NZ-2019-HES-E-CIGARETTE-DEVICES-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G46" s="45" t="n">
+        <x:v>18034000</x:v>
+      </x:c>
+      <x:c r="H46" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I46" s="45"/>
+      <x:c r="J46" s="45"/>
+      <x:c r="K46" s="14"/>
+      <x:c r="L46" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M46" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N46" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="25.5" customHeight="1">
+      <x:c r="A47" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B47" s="14" t="str">
+        <x:v>NZ-2019-HES-E-CIGARETTE-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C47" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D47" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E47" s="14" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G47" s="45" t="n">
+        <x:v>24242000</x:v>
+      </x:c>
+      <x:c r="H47" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I47" s="45"/>
+      <x:c r="J47" s="45"/>
+      <x:c r="K47" s="14"/>
+      <x:c r="L47" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M47" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N47" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="25.5" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>NZ-2023-HES-E-CIGARETTES-AND-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G48" s="45" t="n">
+        <x:v>186980000</x:v>
+      </x:c>
+      <x:c r="H48" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I48" s="45"/>
+      <x:c r="J48" s="45"/>
+      <x:c r="K48" s="14"/>
+      <x:c r="L48" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M48" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N48" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="25.5" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B49" s="14" t="str">
+        <x:v>NZ-2023-HES-E-CIGARETTE-DEVICES-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C49" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D49" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E49" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G49" s="45" t="n">
+        <x:v>22488000</x:v>
+      </x:c>
+      <x:c r="H49" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I49" s="45"/>
+      <x:c r="J49" s="45"/>
+      <x:c r="K49" s="14"/>
+      <x:c r="L49" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M49" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N49" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="25.5" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>NZ-2023-HES-E-CIGARETTE-REFILLS-EXPENDITURE-NZD</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>household_expenditure_estimate</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>year_ended_june</x:v>
+      </x:c>
+      <x:c r="G50" s="45" t="n">
+        <x:v>164492000</x:v>
+      </x:c>
+      <x:c r="H50" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I50" s="45"/>
+      <x:c r="J50" s="45"/>
+      <x:c r="K50" s="14"/>
+      <x:c r="L50" s="14" t="str">
+        <x:v>https://data.ecb.europa.eu/data/datasets/exr/data-information</x:v>
+      </x:c>
+      <x:c r="M50" s="14" t="str">
+        <x:v>not_computed</x:v>
+      </x:c>
+      <x:c r="N50" s="14" t="str">
+        <x:v>period_not_compatible_with_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="25.5" customHeight="1">
+      <x:c r="A51" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B51" s="14" t="str">
+        <x:v>CA-2021-HC-VAPING-MARKET-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C51" s="14" t="str">
+        <x:v>institutional_market_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D51" s="14" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E51" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F51" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G51" s="45" t="n">
+        <x:v>2040000000</x:v>
+      </x:c>
+      <x:c r="H51" s="45" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I51" s="45" t="n">
+        <x:v>1.4825689922481</x:v>
+      </x:c>
+      <x:c r="J51" s="45" t="n">
+        <x:f>G51/I51</x:f>
+        <x:v>1375989927.3939602</x:v>
+      </x:c>
+      <x:c r="K51" s="14" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L51" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M51" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N51" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="25.5" customHeight="1">
+      <x:c r="A52" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B52" s="14" t="str">
+        <x:v>CA-2021-HC-GAS-CONVENIENCE-VAPING-SALES-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C52" s="14" t="str">
+        <x:v>institutional_channel_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D52" s="14" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E52" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F52" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G52" s="45" t="n">
+        <x:v>631000000</x:v>
+      </x:c>
+      <x:c r="H52" s="45" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I52" s="45" t="n">
+        <x:v>1.4825689922481</x:v>
+      </x:c>
+      <x:c r="J52" s="45" t="n">
+        <x:f>G52/I52</x:f>
+        <x:v>425612570.67921025</x:v>
+      </x:c>
+      <x:c r="K52" s="14" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L52" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M52" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N52" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="25.5" customHeight="1">
+      <x:c r="A53" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B53" s="14" t="str">
+        <x:v>CA-2021-HC-ONLINE-VAPING-SALES-BENCHMARK</x:v>
+      </x:c>
+      <x:c r="C53" s="14" t="str">
+        <x:v>institutional_channel_value_benchmark</x:v>
+      </x:c>
+      <x:c r="D53" s="14" t="str">
+        <x:v>Canada</x:v>
+      </x:c>
+      <x:c r="E53" s="14" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F53" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G53" s="45" t="n">
+        <x:v>436000000</x:v>
+      </x:c>
+      <x:c r="H53" s="45" t="str">
+        <x:v>CAD</x:v>
+      </x:c>
+      <x:c r="I53" s="45" t="n">
+        <x:v>1.4825689922481</x:v>
+      </x:c>
+      <x:c r="J53" s="45" t="n">
+        <x:f>G53/I53</x:f>
+        <x:v>294084121.73714054</x:v>
+      </x:c>
+      <x:c r="K53" s="14" t="str">
+        <x:v>ECB-EXR-A-CAD-EUR-SP00-A-2021</x:v>
+      </x:c>
+      <x:c r="L53" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.CAD.EUR.SP00.A?startPeriod=2021&amp;endPeriod=2021&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M53" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N53" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="25.5" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-SOLD-PRODUCTION-EUR</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>prodcom_20595980_sold_production_value</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G54" s="45" t="n">
+        <x:v>39078000</x:v>
+      </x:c>
+      <x:c r="H54" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I54" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J54" s="45" t="n">
+        <x:f>G54</x:f>
+        <x:v>39078000</x:v>
+      </x:c>
+      <x:c r="K54" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L54" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M54" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N54" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="25.5" customHeight="1">
+      <x:c r="A55" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B55" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-IMPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C55" s="14" t="str">
+        <x:v>prodcom_20595980_import_value</x:v>
+      </x:c>
+      <x:c r="D55" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E55" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F55" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G55" s="45" t="n">
+        <x:v>400843037</x:v>
+      </x:c>
+      <x:c r="H55" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I55" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J55" s="45" t="n">
+        <x:f>G55</x:f>
+        <x:v>400843037</x:v>
+      </x:c>
+      <x:c r="K55" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L55" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M55" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N55" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="25.5" customHeight="1">
+      <x:c r="A56" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B56" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-EXPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C56" s="14" t="str">
+        <x:v>prodcom_20595980_export_value</x:v>
+      </x:c>
+      <x:c r="D56" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E56" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F56" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G56" s="45" t="n">
+        <x:v>120676188</x:v>
+      </x:c>
+      <x:c r="H56" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I56" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J56" s="45" t="n">
+        <x:f>G56</x:f>
+        <x:v>120676188</x:v>
+      </x:c>
+      <x:c r="K56" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L56" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M56" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N56" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="25.5" customHeight="1">
+      <x:c r="A57" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-SOLD-PRODUCTION-EUR</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>prodcom_27901152_sold_production_value</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F57" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G57" s="45" t="n">
+        <x:v>99890000</x:v>
+      </x:c>
+      <x:c r="H57" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I57" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J57" s="45" t="n">
+        <x:f>G57</x:f>
+        <x:v>99890000</x:v>
+      </x:c>
+      <x:c r="K57" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L57" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M57" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N57" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="25.5" customHeight="1">
+      <x:c r="A58" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-IMPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>prodcom_27901152_import_value</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F58" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G58" s="45" t="n">
+        <x:v>490580247</x:v>
+      </x:c>
+      <x:c r="H58" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I58" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J58" s="45" t="n">
+        <x:f>G58</x:f>
+        <x:v>490580247</x:v>
+      </x:c>
+      <x:c r="K58" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L58" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M58" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N58" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="25.5" customHeight="1">
+      <x:c r="A59" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-EXPORTS-EUR</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>prodcom_27901152_export_value</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F59" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G59" s="45" t="n">
+        <x:v>301380538</x:v>
+      </x:c>
+      <x:c r="H59" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I59" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J59" s="45" t="n">
+        <x:f>G59</x:f>
+        <x:v>301380538</x:v>
+      </x:c>
+      <x:c r="K59" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L59" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M59" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N59" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="25.5" customHeight="1">
+      <x:c r="A60" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B60" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-20595980-APPARENT-SUPPLY-EUR</x:v>
+      </x:c>
+      <x:c r="C60" s="14" t="str">
+        <x:v>prodcom_20595980_apparent_supply_value</x:v>
+      </x:c>
+      <x:c r="D60" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E60" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F60" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G60" s="45" t="n">
+        <x:v>319244849</x:v>
+      </x:c>
+      <x:c r="H60" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I60" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J60" s="45" t="n">
+        <x:f>G60</x:f>
+        <x:v>319244849</x:v>
+      </x:c>
+      <x:c r="K60" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L60" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M60" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N60" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="25.5" customHeight="1">
+      <x:c r="A61" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B61" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-27901152-APPARENT-SUPPLY-EUR</x:v>
+      </x:c>
+      <x:c r="C61" s="14" t="str">
+        <x:v>prodcom_27901152_apparent_supply_value</x:v>
+      </x:c>
+      <x:c r="D61" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E61" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F61" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G61" s="45" t="n">
+        <x:v>289089709</x:v>
+      </x:c>
+      <x:c r="H61" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I61" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J61" s="45" t="n">
+        <x:f>G61</x:f>
+        <x:v>289089709</x:v>
+      </x:c>
+      <x:c r="K61" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L61" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M61" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N61" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="25.5" customHeight="1">
+      <x:c r="A62" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B62" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-COMBINED-APPARENT-SUPPLY-EUR</x:v>
+      </x:c>
+      <x:c r="C62" s="14" t="str">
+        <x:v>combined_prodcom_apparent_supply_value</x:v>
+      </x:c>
+      <x:c r="D62" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E62" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F62" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G62" s="45" t="n">
+        <x:v>608334558</x:v>
+      </x:c>
+      <x:c r="H62" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I62" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J62" s="45" t="n">
+        <x:f>G62</x:f>
+        <x:v>608334558</x:v>
+      </x:c>
+      <x:c r="K62" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L62" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M62" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N62" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="25.5" customHeight="1">
+      <x:c r="A63" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B63" s="14" t="str">
+        <x:v>DE-2024-EUROSTAT-APPARENT-SUPPLY-EXCISE-VAT-BRIDGE-EUR</x:v>
+      </x:c>
+      <x:c r="C63" s="14" t="str">
+        <x:v>mechanical_apparent_supply_excise_vat_bridge</x:v>
+      </x:c>
+      <x:c r="D63" s="14" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="E63" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F63" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G63" s="45" t="n">
+        <x:v>1040458124.02</x:v>
+      </x:c>
+      <x:c r="H63" s="45" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I63" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J63" s="45" t="n">
+        <x:f>G63</x:f>
+        <x:v>1040458124.02</x:v>
+      </x:c>
+      <x:c r="K63" s="14" t="str">
+        <x:v>EUR-IDENTITY</x:v>
+      </x:c>
+      <x:c r="L63" s="14" t="str">
+        <x:v>https://www.ecb.europa.eu/stats/policy_and_exchange_rates/euro_reference_exchange_rates/html/index.en.html</x:v>
+      </x:c>
+      <x:c r="M63" s="14" t="str">
+        <x:v>already_eur</x:v>
+      </x:c>
+      <x:c r="N63" s="14" t="str">
+        <x:v>original_currency_already_eur</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="25.5" customHeight="1">
+      <x:c r="A64" s="14" t="str">
+        <x:v>market_observation</x:v>
+      </x:c>
+      <x:c r="B64" s="14" t="str">
+        <x:v>PL-2023-CMR-DISPOSABLE-E-CIGARETTE-RETAIL-SALES-VALUE</x:v>
+      </x:c>
+      <x:c r="C64" s="14" t="str">
+        <x:v>commercial_disposable_e_cigarette_retail_sales_value</x:v>
+      </x:c>
+      <x:c r="D64" s="14" t="str">
+        <x:v>Poland</x:v>
+      </x:c>
+      <x:c r="E64" s="14" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F64" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G64" s="45" t="n">
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="H64" s="45" t="str">
+        <x:v>PLN</x:v>
+      </x:c>
+      <x:c r="I64" s="45" t="n">
+        <x:v>4.5419658823529</x:v>
+      </x:c>
+      <x:c r="J64" s="45" t="n">
+        <x:f>G64/I64</x:f>
+        <x:v>440337961.9760439</x:v>
+      </x:c>
+      <x:c r="K64" s="14" t="str">
+        <x:v>ECB-EXR-A-PLN-EUR-SP00-A-2023</x:v>
+      </x:c>
+      <x:c r="L64" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.PLN.EUR.SP00.A?startPeriod=2023&amp;endPeriod=2023&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M64" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N64" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="25.5" customHeight="1">
+      <x:c r="A65" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B65" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C65" s="14" t="str">
+        <x:v>low.specialistRetailNzd</x:v>
+      </x:c>
+      <x:c r="D65" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E65" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F65" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G65" s="45" t="n">
+        <x:v>258327110.88</x:v>
+      </x:c>
+      <x:c r="H65" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I65" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J65" s="45" t="n">
+        <x:f>G65/I65</x:f>
+        <x:v>144474304.51375833</x:v>
+      </x:c>
+      <x:c r="K65" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L65" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M65" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N65" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="25.5" customHeight="1">
+      <x:c r="A66" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B66" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C66" s="14" t="str">
+        <x:v>low.generalRetailRpsNzd</x:v>
+      </x:c>
+      <x:c r="D66" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E66" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F66" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G66" s="45" t="n">
+        <x:v>275335272.8</x:v>
+      </x:c>
+      <x:c r="H66" s="45" t="str">
+        <x:v>NZD</x:v>
+      </x:c>
+      <x:c r="I66" s="45" t="n">
+        <x:v>1.788048828125</x:v>
+      </x:c>
+      <x:c r="J66" s="45" t="n">
+        <x:f>G66/I66</x:f>
+        <x:v>153986439.55865824</x:v>
+      </x:c>
+      <x:c r="K66" s="14" t="str">
+        <x:v>ECB-EXR-A-NZD-EUR-SP00-A-2024</x:v>
+      </x:c>
+      <x:c r="L66" s="14" t="str">
+        <x:v>https://data-api.ecb.europa.eu/service/data/EXR/A.NZD.EUR.SP00.A?startPeriod=2024&amp;endPeriod=2024&amp;format=csvdata</x:v>
+      </x:c>
+      <x:c r="M66" s="14" t="str">
+        <x:v>computed</x:v>
+      </x:c>
+      <x:c r="N66" s="14" t="str">
+        <x:v>original_amount_divided_by_ecb_annual_average</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="25.5" customHeight="1">
+      <x:c r="A67" s="14" t="str">
+        <x:v>scenario_component</x:v>
+      </x:c>
+      <x:c r="B67" s="14" t="str">
+        <x:v>NZ-2024-RETAIL-RANGE</x:v>
+      </x:c>
+      <x:c r="C67" s="14" t="str">
+        <x:v>low.combinedNzd</x:v>
+      </x:c>
+      <x:c r="D67" s="14" t="str">
+        <x:v>New Zealand</x:v>
+      </x:c>
+      <x:c r="E67" s="14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="F67" s="14" t="str">
+        <x:v>calendar_year</x:v>
+      </x:c>
+      <x:c r="G67" s="45" t="n">
+        <x:v>533662383.68</x:v>
+      </x:c>
+      <x:c r="H67